<commit_message>
Feedgas backfill: [ 2/119] 2026-09-26 ~ 14/17 meters metered 12.64 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Plaquemines (CGT) | elapsed 0:02 ~2:12 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80553,9 +80553,39 @@
       <c r="A2462" s="4" t="n">
         <v>46291</v>
       </c>
+      <c r="B2462" t="n">
+        <v>3.361</v>
+      </c>
+      <c r="C2462" t="n">
+        <v>3.372</v>
+      </c>
+      <c r="D2462" t="n">
+        <v>1.406</v>
+      </c>
+      <c r="E2462" t="n">
+        <v>0.569</v>
+      </c>
+      <c r="F2462" t="n">
+        <v>2.417</v>
+      </c>
+      <c r="G2462" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H2462" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I2462" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J2462" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K2462" t="n">
+        <v>12.642</v>
+      </c>
       <c r="L2462" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80610,7 +80640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80675,22 +80705,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B2" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C2" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D2" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F2" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G2" t="n">
         <v>0.395</v>
@@ -80705,6 +80735,41 @@
         <v>0.014</v>
       </c>
       <c r="K2" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K3" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -80719,7 +80784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80789,22 +80854,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B2" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C2" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D2" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F2" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G2" t="n">
         <v>0.395</v>
@@ -80819,9 +80884,47 @@
         <v>0.014</v>
       </c>
       <c r="K2" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L2" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K3" t="n">
         <v>12.277</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L3" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81262,7 +81365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81362,40 +81465,40 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B2" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C2" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D2" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E2" t="n">
         <v>9100</v>
       </c>
       <c r="F2" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G2" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I2" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K2" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M2" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N2" t="n">
         <v>189475</v>
       </c>
       <c r="O2" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P2" t="n">
         <v>375660</v>
@@ -81404,6 +81507,53 @@
         <v>773586</v>
       </c>
       <c r="R2" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C3" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K3" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N3" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O3" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P3" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R3" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 3/119] 2026-09-25 ~ 14/17 meters metered 12.37 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Plaquemines (CGT) | elapsed 0:03 ~2:04 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80543,9 +80543,39 @@
       <c r="A2461" s="4" t="n">
         <v>46290</v>
       </c>
+      <c r="B2461" t="n">
+        <v>3.412</v>
+      </c>
+      <c r="C2461" t="n">
+        <v>3.251</v>
+      </c>
+      <c r="D2461" t="n">
+        <v>1.484</v>
+      </c>
+      <c r="E2461" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="F2461" t="n">
+        <v>2.274</v>
+      </c>
+      <c r="G2461" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="H2461" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="I2461" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="J2461" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K2461" t="n">
+        <v>12.373</v>
+      </c>
       <c r="L2461" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80640,7 +80670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80705,57 +80735,57 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B2" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C2" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D2" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E2" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F2" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G2" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H2" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I2" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J2" t="n">
         <v>0.014</v>
       </c>
       <c r="K2" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B3" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C3" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D3" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F3" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G3" t="n">
         <v>0.395</v>
@@ -80770,6 +80800,41 @@
         <v>0.014</v>
       </c>
       <c r="K3" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K4" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -80784,7 +80849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80854,60 +80919,60 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B2" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C2" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D2" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E2" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F2" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G2" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H2" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I2" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J2" t="n">
         <v>0.014</v>
       </c>
       <c r="K2" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L2" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B3" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C3" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D3" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F3" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G3" t="n">
         <v>0.395</v>
@@ -80922,9 +80987,47 @@
         <v>0.014</v>
       </c>
       <c r="K3" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L3" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K4" t="n">
         <v>12.277</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L4" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81365,7 +81468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81465,46 +81568,46 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B2" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C2" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D2" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E2" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F2" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G2" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I2" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K2" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M2" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N2" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O2" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P2" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q2" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R2" t="n">
         <v>15000</v>
@@ -81512,40 +81615,40 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B3" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C3" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D3" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E3" t="n">
         <v>9100</v>
       </c>
       <c r="F3" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G3" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I3" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K3" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M3" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N3" t="n">
         <v>189475</v>
       </c>
       <c r="O3" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P3" t="n">
         <v>375660</v>
@@ -81554,6 +81657,53 @@
         <v>773586</v>
       </c>
       <c r="R3" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C4" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K4" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M4" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N4" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O4" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P4" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R4" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 4/119] 2026-09-24 ~ 13/17 meters metered 12.12 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:04 ~2:01 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80533,9 +80533,36 @@
       <c r="A2460" s="4" t="n">
         <v>46289</v>
       </c>
+      <c r="B2460" t="n">
+        <v>3.365</v>
+      </c>
+      <c r="C2460" t="n">
+        <v>3.197</v>
+      </c>
+      <c r="D2460" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="E2460" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="F2460" t="n">
+        <v>2.354</v>
+      </c>
+      <c r="G2460" t="n">
+        <v>0.462</v>
+      </c>
+      <c r="H2460" t="n">
+        <v>0.343</v>
+      </c>
+      <c r="I2460" t="n">
+        <v>0.704</v>
+      </c>
+      <c r="K2460" t="n">
+        <v>12.118</v>
+      </c>
       <c r="L2460" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80670,7 +80697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80735,92 +80762,89 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B2" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C2" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D2" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E2" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F2" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G2" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H2" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I2" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K2" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B3" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C3" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D3" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E3" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F3" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G3" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H3" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I3" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J3" t="n">
         <v>0.014</v>
       </c>
       <c r="K3" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B4" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C4" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D4" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F4" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G4" t="n">
         <v>0.395</v>
@@ -80835,6 +80859,41 @@
         <v>0.014</v>
       </c>
       <c r="K4" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K5" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -80849,7 +80908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80919,98 +80978,95 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B2" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C2" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D2" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E2" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F2" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G2" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H2" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I2" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K2" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L2" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B3" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C3" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D3" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E3" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F3" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G3" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H3" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I3" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J3" t="n">
         <v>0.014</v>
       </c>
       <c r="K3" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L3" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B4" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C4" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D4" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F4" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G4" t="n">
         <v>0.395</v>
@@ -81025,9 +81081,47 @@
         <v>0.014</v>
       </c>
       <c r="K4" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L4" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K5" t="n">
         <v>12.277</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L5" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81468,7 +81562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81568,93 +81662,90 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B2" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C2" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D2" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E2" t="n">
         <v>9300</v>
       </c>
       <c r="F2" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G2" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I2" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K2" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M2" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N2" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P2" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q2" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R2" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B3" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C3" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D3" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E3" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F3" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G3" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I3" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K3" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M3" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N3" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O3" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P3" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q3" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R3" t="n">
         <v>15000</v>
@@ -81662,40 +81753,40 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B4" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C4" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D4" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E4" t="n">
         <v>9100</v>
       </c>
       <c r="F4" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G4" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I4" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K4" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M4" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N4" t="n">
         <v>189475</v>
       </c>
       <c r="O4" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P4" t="n">
         <v>375660</v>
@@ -81704,6 +81795,53 @@
         <v>773586</v>
       </c>
       <c r="R4" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C5" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E5" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K5" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N5" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O5" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P5" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R5" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 5/119] 2026-09-23 ~ 13/17 meters metered 12.08 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:05 ~1:55 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80523,9 +80523,36 @@
       <c r="A2459" s="4" t="n">
         <v>46288</v>
       </c>
+      <c r="B2459" t="n">
+        <v>3.277</v>
+      </c>
+      <c r="C2459" t="n">
+        <v>3.153</v>
+      </c>
+      <c r="D2459" t="n">
+        <v>1.426</v>
+      </c>
+      <c r="E2459" t="n">
+        <v>0.237</v>
+      </c>
+      <c r="F2459" t="n">
+        <v>2.454</v>
+      </c>
+      <c r="G2459" t="n">
+        <v>0.462</v>
+      </c>
+      <c r="H2459" t="n">
+        <v>0.343</v>
+      </c>
+      <c r="I2459" t="n">
+        <v>0.728</v>
+      </c>
+      <c r="K2459" t="n">
+        <v>12.08</v>
+      </c>
       <c r="L2459" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80697,7 +80724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80762,22 +80789,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B2" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C2" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D2" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E2" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F2" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G2" t="n">
         <v>0.462</v>
@@ -80786,100 +80813,97 @@
         <v>0.343</v>
       </c>
       <c r="I2" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K2" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B3" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C3" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D3" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E3" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F3" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G3" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H3" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I3" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K3" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B4" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C4" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D4" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E4" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F4" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G4" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H4" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I4" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J4" t="n">
         <v>0.014</v>
       </c>
       <c r="K4" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B5" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C5" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D5" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F5" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G5" t="n">
         <v>0.395</v>
@@ -80894,6 +80918,41 @@
         <v>0.014</v>
       </c>
       <c r="K5" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K6" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -80908,7 +80967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80978,22 +81037,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B2" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C2" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D2" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E2" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F2" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G2" t="n">
         <v>0.462</v>
@@ -81002,109 +81061,106 @@
         <v>0.343</v>
       </c>
       <c r="I2" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K2" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L2" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B3" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C3" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D3" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E3" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F3" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G3" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H3" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I3" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K3" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L3" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B4" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C4" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D4" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E4" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F4" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G4" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H4" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I4" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J4" t="n">
         <v>0.014</v>
       </c>
       <c r="K4" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L4" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B5" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C5" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D5" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F5" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G5" t="n">
         <v>0.395</v>
@@ -81119,9 +81175,47 @@
         <v>0.014</v>
       </c>
       <c r="K5" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L5" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K6" t="n">
         <v>12.277</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L6" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81562,7 +81656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81662,34 +81756,34 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B2" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C2" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D2" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E2" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F2" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G2" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I2" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K2" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M2" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
@@ -81698,101 +81792,98 @@
         <v>264857</v>
       </c>
       <c r="P2" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q2" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B3" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C3" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D3" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E3" t="n">
         <v>9300</v>
       </c>
       <c r="F3" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G3" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I3" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K3" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M3" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N3" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P3" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q3" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R3" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B4" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C4" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D4" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E4" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F4" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G4" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I4" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K4" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M4" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N4" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O4" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P4" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q4" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R4" t="n">
         <v>15000</v>
@@ -81800,40 +81891,40 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B5" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C5" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D5" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E5" t="n">
         <v>9100</v>
       </c>
       <c r="F5" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G5" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I5" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K5" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M5" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N5" t="n">
         <v>189475</v>
       </c>
       <c r="O5" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P5" t="n">
         <v>375660</v>
@@ -81842,6 +81933,53 @@
         <v>773586</v>
       </c>
       <c r="R5" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C6" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E6" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K6" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N6" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O6" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P6" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R6" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 6/119] 2026-09-22 ~ 13/17 meters metered 12.19 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:05 ~1:51 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80513,9 +80513,36 @@
       <c r="A2458" s="4" t="n">
         <v>46287</v>
       </c>
+      <c r="B2458" t="n">
+        <v>3.259</v>
+      </c>
+      <c r="C2458" t="n">
+        <v>3.268</v>
+      </c>
+      <c r="D2458" t="n">
+        <v>1.449</v>
+      </c>
+      <c r="E2458" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="F2458" t="n">
+        <v>2.276</v>
+      </c>
+      <c r="G2458" t="n">
+        <v>0.462</v>
+      </c>
+      <c r="H2458" t="n">
+        <v>0.343</v>
+      </c>
+      <c r="I2458" t="n">
+        <v>0.731</v>
+      </c>
+      <c r="K2458" t="n">
+        <v>12.187</v>
+      </c>
       <c r="L2458" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80724,7 +80751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80789,22 +80816,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B2" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C2" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D2" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E2" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F2" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G2" t="n">
         <v>0.462</v>
@@ -80813,30 +80840,30 @@
         <v>0.343</v>
       </c>
       <c r="I2" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K2" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B3" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C3" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D3" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E3" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F3" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G3" t="n">
         <v>0.462</v>
@@ -80845,100 +80872,97 @@
         <v>0.343</v>
       </c>
       <c r="I3" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K3" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B4" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C4" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D4" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E4" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F4" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G4" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H4" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I4" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K4" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B5" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C5" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D5" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E5" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F5" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G5" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H5" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I5" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J5" t="n">
         <v>0.014</v>
       </c>
       <c r="K5" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B6" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C6" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D6" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F6" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G6" t="n">
         <v>0.395</v>
@@ -80953,6 +80977,41 @@
         <v>0.014</v>
       </c>
       <c r="K6" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K7" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -80967,7 +81026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81037,22 +81096,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B2" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C2" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D2" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E2" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F2" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G2" t="n">
         <v>0.462</v>
@@ -81061,33 +81120,33 @@
         <v>0.343</v>
       </c>
       <c r="I2" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K2" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L2" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B3" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C3" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D3" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E3" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F3" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G3" t="n">
         <v>0.462</v>
@@ -81096,109 +81155,106 @@
         <v>0.343</v>
       </c>
       <c r="I3" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K3" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L3" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B4" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C4" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D4" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E4" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F4" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G4" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H4" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I4" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K4" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L4" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B5" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C5" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D5" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E5" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F5" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G5" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H5" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I5" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J5" t="n">
         <v>0.014</v>
       </c>
       <c r="K5" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L5" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B6" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C6" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D6" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F6" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G6" t="n">
         <v>0.395</v>
@@ -81213,9 +81269,47 @@
         <v>0.014</v>
       </c>
       <c r="K6" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L6" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K7" t="n">
         <v>12.277</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L7" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81656,7 +81750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81756,34 +81850,34 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B2" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C2" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D2" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E2" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G2" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I2" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K2" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M2" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
@@ -81792,42 +81886,42 @@
         <v>264857</v>
       </c>
       <c r="P2" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q2" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B3" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C3" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D3" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E3" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F3" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G3" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I3" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K3" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M3" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
@@ -81836,101 +81930,98 @@
         <v>264857</v>
       </c>
       <c r="P3" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q3" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B4" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C4" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D4" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E4" t="n">
         <v>9300</v>
       </c>
       <c r="F4" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G4" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I4" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K4" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M4" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N4" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P4" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q4" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R4" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B5" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C5" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D5" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E5" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F5" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G5" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I5" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K5" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M5" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N5" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O5" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P5" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q5" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R5" t="n">
         <v>15000</v>
@@ -81938,40 +82029,40 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B6" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C6" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D6" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E6" t="n">
         <v>9100</v>
       </c>
       <c r="F6" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G6" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I6" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K6" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M6" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N6" t="n">
         <v>189475</v>
       </c>
       <c r="O6" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P6" t="n">
         <v>375660</v>
@@ -81980,6 +82071,53 @@
         <v>773586</v>
       </c>
       <c r="R6" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C7" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E7" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K7" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M7" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N7" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O7" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P7" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R7" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 7/119] 2026-09-21 ~ 13/17 meters metered 12.22 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:06 ~1:49 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80503,9 +80503,36 @@
       <c r="A2457" s="4" t="n">
         <v>46286</v>
       </c>
+      <c r="B2457" t="n">
+        <v>3.263</v>
+      </c>
+      <c r="C2457" t="n">
+        <v>3.261</v>
+      </c>
+      <c r="D2457" t="n">
+        <v>1.435</v>
+      </c>
+      <c r="E2457" t="n">
+        <v>0.554</v>
+      </c>
+      <c r="F2457" t="n">
+        <v>2.197</v>
+      </c>
+      <c r="G2457" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="H2457" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="I2457" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="K2457" t="n">
+        <v>12.224</v>
+      </c>
       <c r="L2457" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80751,7 +80778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80816,54 +80843,54 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B2" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C2" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D2" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E2" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F2" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G2" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H2" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I2" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K2" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B3" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C3" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D3" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E3" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F3" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G3" t="n">
         <v>0.462</v>
@@ -80872,30 +80899,30 @@
         <v>0.343</v>
       </c>
       <c r="I3" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K3" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B4" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C4" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D4" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E4" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F4" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G4" t="n">
         <v>0.462</v>
@@ -80904,100 +80931,97 @@
         <v>0.343</v>
       </c>
       <c r="I4" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K4" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B5" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C5" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D5" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E5" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F5" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G5" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H5" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I5" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K5" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B6" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C6" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D6" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E6" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F6" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G6" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H6" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I6" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J6" t="n">
         <v>0.014</v>
       </c>
       <c r="K6" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B7" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C7" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D7" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F7" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G7" t="n">
         <v>0.395</v>
@@ -81012,6 +81036,41 @@
         <v>0.014</v>
       </c>
       <c r="K7" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K8" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81026,7 +81085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81096,57 +81155,57 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B2" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C2" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D2" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E2" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F2" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G2" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H2" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I2" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K2" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L2" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B3" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C3" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D3" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E3" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F3" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G3" t="n">
         <v>0.462</v>
@@ -81155,33 +81214,33 @@
         <v>0.343</v>
       </c>
       <c r="I3" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K3" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L3" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B4" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C4" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D4" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E4" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F4" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G4" t="n">
         <v>0.462</v>
@@ -81190,109 +81249,106 @@
         <v>0.343</v>
       </c>
       <c r="I4" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K4" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L4" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B5" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C5" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D5" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E5" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F5" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G5" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H5" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I5" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K5" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L5" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B6" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C6" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D6" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E6" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F6" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G6" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H6" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I6" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J6" t="n">
         <v>0.014</v>
       </c>
       <c r="K6" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L6" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B7" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C7" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D7" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F7" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G7" t="n">
         <v>0.395</v>
@@ -81307,9 +81363,47 @@
         <v>0.014</v>
       </c>
       <c r="K7" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L7" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K8" t="n">
         <v>12.277</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L8" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81750,7 +81844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81850,78 +81944,78 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B2" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C2" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D2" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E2" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F2" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G2" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I2" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K2" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M2" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P2" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q2" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B3" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C3" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D3" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E3" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G3" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I3" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K3" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M3" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
@@ -81930,42 +82024,42 @@
         <v>264857</v>
       </c>
       <c r="P3" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q3" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B4" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C4" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D4" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E4" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F4" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G4" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I4" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K4" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M4" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
@@ -81974,101 +82068,98 @@
         <v>264857</v>
       </c>
       <c r="P4" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q4" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B5" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C5" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D5" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E5" t="n">
         <v>9300</v>
       </c>
       <c r="F5" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G5" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I5" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K5" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M5" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N5" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P5" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q5" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R5" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B6" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C6" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D6" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E6" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F6" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G6" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I6" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K6" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M6" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N6" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O6" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P6" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q6" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R6" t="n">
         <v>15000</v>
@@ -82076,40 +82167,40 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B7" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C7" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D7" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E7" t="n">
         <v>9100</v>
       </c>
       <c r="F7" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G7" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I7" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K7" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M7" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N7" t="n">
         <v>189475</v>
       </c>
       <c r="O7" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P7" t="n">
         <v>375660</v>
@@ -82118,6 +82209,53 @@
         <v>773586</v>
       </c>
       <c r="R7" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C8" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K8" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N8" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O8" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P8" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R8" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 8/119] 2026-09-20 ~ 13/17 meters metered 12.28 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:07 ~1:49 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80493,9 +80493,36 @@
       <c r="A2456" s="4" t="n">
         <v>46285</v>
       </c>
+      <c r="B2456" t="n">
+        <v>3.232</v>
+      </c>
+      <c r="C2456" t="n">
+        <v>3.162</v>
+      </c>
+      <c r="D2456" t="n">
+        <v>1.435</v>
+      </c>
+      <c r="E2456" t="n">
+        <v>0.609</v>
+      </c>
+      <c r="F2456" t="n">
+        <v>2.324</v>
+      </c>
+      <c r="G2456" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="H2456" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="I2456" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="K2456" t="n">
+        <v>12.276</v>
+      </c>
       <c r="L2456" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80778,7 +80805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80843,22 +80870,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B2" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C2" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D2" t="n">
         <v>1.435</v>
       </c>
       <c r="E2" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F2" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G2" t="n">
         <v>0.446</v>
@@ -80870,59 +80897,59 @@
         <v>0.712</v>
       </c>
       <c r="K2" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B3" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C3" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D3" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E3" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F3" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G3" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H3" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I3" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K3" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B4" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C4" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D4" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E4" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F4" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G4" t="n">
         <v>0.462</v>
@@ -80931,30 +80958,30 @@
         <v>0.343</v>
       </c>
       <c r="I4" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K4" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B5" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C5" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D5" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E5" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F5" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G5" t="n">
         <v>0.462</v>
@@ -80963,100 +80990,97 @@
         <v>0.343</v>
       </c>
       <c r="I5" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K5" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B6" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C6" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D6" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E6" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F6" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G6" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H6" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I6" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K6" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B7" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C7" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D7" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E7" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F7" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G7" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H7" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I7" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J7" t="n">
         <v>0.014</v>
       </c>
       <c r="K7" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B8" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C8" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D8" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F8" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G8" t="n">
         <v>0.395</v>
@@ -81071,6 +81095,41 @@
         <v>0.014</v>
       </c>
       <c r="K8" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K9" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81085,7 +81144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81155,22 +81214,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B2" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C2" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D2" t="n">
         <v>1.435</v>
       </c>
       <c r="E2" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F2" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G2" t="n">
         <v>0.446</v>
@@ -81182,65 +81241,65 @@
         <v>0.712</v>
       </c>
       <c r="K2" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L2" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B3" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C3" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D3" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E3" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F3" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G3" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H3" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I3" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K3" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L3" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B4" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C4" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D4" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E4" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F4" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G4" t="n">
         <v>0.462</v>
@@ -81249,33 +81308,33 @@
         <v>0.343</v>
       </c>
       <c r="I4" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K4" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L4" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B5" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C5" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D5" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E5" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F5" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G5" t="n">
         <v>0.462</v>
@@ -81284,109 +81343,106 @@
         <v>0.343</v>
       </c>
       <c r="I5" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K5" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L5" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B6" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C6" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D6" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E6" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F6" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G6" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H6" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I6" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K6" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L6" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B7" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C7" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D7" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E7" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F7" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G7" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H7" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I7" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J7" t="n">
         <v>0.014</v>
       </c>
       <c r="K7" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L7" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B8" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C8" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D8" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F8" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G8" t="n">
         <v>0.395</v>
@@ -81401,9 +81457,47 @@
         <v>0.014</v>
       </c>
       <c r="K8" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L8" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K9" t="n">
         <v>12.277</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L9" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81844,7 +81938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81944,34 +82038,34 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B2" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C2" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D2" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E2" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G2" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I2" t="n">
         <v>1488515</v>
       </c>
       <c r="K2" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M2" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
@@ -81980,7 +82074,7 @@
         <v>247857</v>
       </c>
       <c r="P2" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q2" t="n">
         <v>738429</v>
@@ -81988,78 +82082,78 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B3" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C3" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D3" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E3" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F3" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G3" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I3" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K3" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M3" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P3" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q3" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B4" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C4" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D4" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E4" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G4" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I4" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K4" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M4" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
@@ -82068,42 +82162,42 @@
         <v>264857</v>
       </c>
       <c r="P4" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q4" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B5" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C5" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D5" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E5" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F5" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G5" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I5" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K5" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M5" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
@@ -82112,101 +82206,98 @@
         <v>264857</v>
       </c>
       <c r="P5" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q5" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B6" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C6" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D6" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E6" t="n">
         <v>9300</v>
       </c>
       <c r="F6" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G6" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I6" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K6" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M6" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N6" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P6" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q6" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R6" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B7" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C7" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D7" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E7" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F7" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G7" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I7" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K7" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M7" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N7" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O7" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P7" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q7" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R7" t="n">
         <v>15000</v>
@@ -82214,40 +82305,40 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B8" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C8" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D8" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E8" t="n">
         <v>9100</v>
       </c>
       <c r="F8" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G8" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I8" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K8" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M8" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N8" t="n">
         <v>189475</v>
       </c>
       <c r="O8" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P8" t="n">
         <v>375660</v>
@@ -82256,6 +82347,53 @@
         <v>773586</v>
       </c>
       <c r="R8" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C9" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E9" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K9" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N9" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O9" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P9" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R9" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 9/119] 2026-09-19 ~ 13/17 meters metered 12.57 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:08 ~1:46 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80483,9 +80483,36 @@
       <c r="A2455" s="4" t="n">
         <v>46284</v>
       </c>
+      <c r="B2455" t="n">
+        <v>3.176</v>
+      </c>
+      <c r="C2455" t="n">
+        <v>3.163</v>
+      </c>
+      <c r="D2455" t="n">
+        <v>1.435</v>
+      </c>
+      <c r="E2455" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="F2455" t="n">
+        <v>2.607</v>
+      </c>
+      <c r="G2455" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="H2455" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="I2455" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="K2455" t="n">
+        <v>12.569</v>
+      </c>
       <c r="L2455" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80805,7 +80832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80870,22 +80897,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B2" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C2" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D2" t="n">
         <v>1.435</v>
       </c>
       <c r="E2" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F2" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G2" t="n">
         <v>0.446</v>
@@ -80897,27 +80924,27 @@
         <v>0.712</v>
       </c>
       <c r="K2" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B3" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C3" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D3" t="n">
         <v>1.435</v>
       </c>
       <c r="E3" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F3" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G3" t="n">
         <v>0.446</v>
@@ -80929,59 +80956,59 @@
         <v>0.712</v>
       </c>
       <c r="K3" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B4" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C4" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D4" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E4" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F4" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G4" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H4" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I4" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K4" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B5" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C5" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D5" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E5" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F5" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G5" t="n">
         <v>0.462</v>
@@ -80990,30 +81017,30 @@
         <v>0.343</v>
       </c>
       <c r="I5" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K5" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B6" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C6" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D6" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E6" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F6" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G6" t="n">
         <v>0.462</v>
@@ -81022,100 +81049,97 @@
         <v>0.343</v>
       </c>
       <c r="I6" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K6" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B7" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C7" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D7" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E7" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F7" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G7" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H7" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I7" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K7" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B8" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C8" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D8" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E8" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F8" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G8" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H8" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I8" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J8" t="n">
         <v>0.014</v>
       </c>
       <c r="K8" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B9" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C9" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D9" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F9" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G9" t="n">
         <v>0.395</v>
@@ -81130,6 +81154,41 @@
         <v>0.014</v>
       </c>
       <c r="K9" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K10" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81144,7 +81203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81214,22 +81273,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B2" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C2" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D2" t="n">
         <v>1.435</v>
       </c>
       <c r="E2" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F2" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G2" t="n">
         <v>0.446</v>
@@ -81241,30 +81300,30 @@
         <v>0.712</v>
       </c>
       <c r="K2" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L2" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B3" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C3" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D3" t="n">
         <v>1.435</v>
       </c>
       <c r="E3" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F3" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G3" t="n">
         <v>0.446</v>
@@ -81276,65 +81335,65 @@
         <v>0.712</v>
       </c>
       <c r="K3" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L3" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B4" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C4" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D4" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E4" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F4" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G4" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H4" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I4" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K4" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L4" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B5" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C5" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D5" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E5" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F5" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G5" t="n">
         <v>0.462</v>
@@ -81343,33 +81402,33 @@
         <v>0.343</v>
       </c>
       <c r="I5" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K5" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L5" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B6" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C6" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D6" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E6" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F6" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G6" t="n">
         <v>0.462</v>
@@ -81378,109 +81437,106 @@
         <v>0.343</v>
       </c>
       <c r="I6" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K6" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L6" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B7" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C7" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D7" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E7" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F7" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G7" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H7" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I7" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K7" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L7" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B8" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C8" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D8" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E8" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F8" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G8" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H8" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I8" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J8" t="n">
         <v>0.014</v>
       </c>
       <c r="K8" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L8" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B9" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C9" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D9" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F9" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G9" t="n">
         <v>0.395</v>
@@ -81495,9 +81551,47 @@
         <v>0.014</v>
       </c>
       <c r="K9" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L9" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K10" t="n">
         <v>12.277</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L10" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -81938,7 +82032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82038,34 +82132,34 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B2" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C2" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D2" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G2" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I2" t="n">
         <v>1488515</v>
       </c>
       <c r="K2" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M2" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
@@ -82074,7 +82168,7 @@
         <v>247857</v>
       </c>
       <c r="P2" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q2" t="n">
         <v>738429</v>
@@ -82082,34 +82176,34 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B3" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C3" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D3" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E3" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G3" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I3" t="n">
         <v>1488515</v>
       </c>
       <c r="K3" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M3" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
@@ -82118,7 +82212,7 @@
         <v>247857</v>
       </c>
       <c r="P3" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q3" t="n">
         <v>738429</v>
@@ -82126,78 +82220,78 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B4" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C4" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D4" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E4" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F4" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G4" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I4" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K4" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M4" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P4" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q4" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B5" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C5" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D5" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E5" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G5" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I5" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K5" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M5" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
@@ -82206,42 +82300,42 @@
         <v>264857</v>
       </c>
       <c r="P5" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q5" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B6" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C6" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D6" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E6" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F6" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G6" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I6" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K6" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M6" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
@@ -82250,101 +82344,98 @@
         <v>264857</v>
       </c>
       <c r="P6" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q6" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B7" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C7" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D7" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E7" t="n">
         <v>9300</v>
       </c>
       <c r="F7" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G7" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I7" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K7" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M7" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N7" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P7" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q7" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R7" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B8" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C8" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D8" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E8" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F8" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G8" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I8" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K8" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M8" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N8" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O8" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P8" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q8" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R8" t="n">
         <v>15000</v>
@@ -82352,40 +82443,40 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B9" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C9" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D9" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E9" t="n">
         <v>9100</v>
       </c>
       <c r="F9" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G9" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I9" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K9" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M9" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N9" t="n">
         <v>189475</v>
       </c>
       <c r="O9" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P9" t="n">
         <v>375660</v>
@@ -82394,6 +82485,53 @@
         <v>773586</v>
       </c>
       <c r="R9" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C10" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K10" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N10" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O10" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P10" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R10" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 10/119] 2026-09-18 ~ 13/17 meters metered 12.63 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:09 ~1:45 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80473,9 +80473,36 @@
       <c r="A2454" s="4" t="n">
         <v>46283</v>
       </c>
+      <c r="B2454" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C2454" t="n">
+        <v>3.232</v>
+      </c>
+      <c r="D2454" t="n">
+        <v>1.484</v>
+      </c>
+      <c r="E2454" t="n">
+        <v>0.6889999999999999</v>
+      </c>
+      <c r="F2454" t="n">
+        <v>2.598</v>
+      </c>
+      <c r="G2454" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="H2454" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I2454" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="K2454" t="n">
+        <v>12.634</v>
+      </c>
       <c r="L2454" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80832,7 +80859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80897,54 +80924,54 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B2" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C2" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D2" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E2" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G2" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H2" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I2" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K2" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B3" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C3" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D3" t="n">
         <v>1.435</v>
       </c>
       <c r="E3" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F3" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G3" t="n">
         <v>0.446</v>
@@ -80956,27 +80983,27 @@
         <v>0.712</v>
       </c>
       <c r="K3" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B4" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C4" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D4" t="n">
         <v>1.435</v>
       </c>
       <c r="E4" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F4" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G4" t="n">
         <v>0.446</v>
@@ -80988,59 +81015,59 @@
         <v>0.712</v>
       </c>
       <c r="K4" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B5" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C5" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D5" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E5" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F5" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G5" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H5" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I5" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K5" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B6" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C6" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D6" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E6" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F6" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G6" t="n">
         <v>0.462</v>
@@ -81049,30 +81076,30 @@
         <v>0.343</v>
       </c>
       <c r="I6" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K6" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B7" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C7" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D7" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E7" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F7" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G7" t="n">
         <v>0.462</v>
@@ -81081,100 +81108,97 @@
         <v>0.343</v>
       </c>
       <c r="I7" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K7" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B8" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C8" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D8" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E8" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F8" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G8" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H8" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I8" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K8" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B9" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C9" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D9" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E9" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F9" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G9" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H9" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I9" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J9" t="n">
         <v>0.014</v>
       </c>
       <c r="K9" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B10" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C10" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D10" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F10" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G10" t="n">
         <v>0.395</v>
@@ -81189,6 +81213,41 @@
         <v>0.014</v>
       </c>
       <c r="K10" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K11" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81203,7 +81262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81273,57 +81332,57 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B2" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C2" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D2" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E2" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G2" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H2" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I2" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K2" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L2" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B3" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C3" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D3" t="n">
         <v>1.435</v>
       </c>
       <c r="E3" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F3" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G3" t="n">
         <v>0.446</v>
@@ -81335,30 +81394,30 @@
         <v>0.712</v>
       </c>
       <c r="K3" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L3" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B4" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C4" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D4" t="n">
         <v>1.435</v>
       </c>
       <c r="E4" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F4" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G4" t="n">
         <v>0.446</v>
@@ -81370,65 +81429,65 @@
         <v>0.712</v>
       </c>
       <c r="K4" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L4" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B5" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C5" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D5" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E5" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F5" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G5" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H5" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I5" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K5" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L5" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B6" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C6" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D6" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E6" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F6" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G6" t="n">
         <v>0.462</v>
@@ -81437,33 +81496,33 @@
         <v>0.343</v>
       </c>
       <c r="I6" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K6" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L6" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B7" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C7" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D7" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E7" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F7" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G7" t="n">
         <v>0.462</v>
@@ -81472,109 +81531,106 @@
         <v>0.343</v>
       </c>
       <c r="I7" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K7" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L7" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B8" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C8" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D8" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E8" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F8" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G8" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H8" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I8" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K8" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L8" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B9" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C9" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D9" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E9" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F9" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G9" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H9" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I9" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J9" t="n">
         <v>0.014</v>
       </c>
       <c r="K9" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L9" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B10" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C10" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D10" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F10" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G10" t="n">
         <v>0.395</v>
@@ -81589,9 +81645,47 @@
         <v>0.014</v>
       </c>
       <c r="K10" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L10" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K11" t="n">
         <v>12.277</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L11" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82032,7 +82126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82132,78 +82226,78 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B2" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C2" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D2" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G2" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I2" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K2" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M2" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N2" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O2" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P2" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q2" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B3" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C3" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D3" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G3" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I3" t="n">
         <v>1488515</v>
       </c>
       <c r="K3" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M3" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
@@ -82212,7 +82306,7 @@
         <v>247857</v>
       </c>
       <c r="P3" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q3" t="n">
         <v>738429</v>
@@ -82220,34 +82314,34 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B4" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C4" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D4" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E4" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G4" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I4" t="n">
         <v>1488515</v>
       </c>
       <c r="K4" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M4" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
@@ -82256,7 +82350,7 @@
         <v>247857</v>
       </c>
       <c r="P4" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q4" t="n">
         <v>738429</v>
@@ -82264,78 +82358,78 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B5" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C5" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D5" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E5" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F5" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G5" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I5" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K5" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M5" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P5" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q5" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B6" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C6" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D6" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E6" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G6" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I6" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K6" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M6" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
@@ -82344,42 +82438,42 @@
         <v>264857</v>
       </c>
       <c r="P6" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q6" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B7" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C7" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D7" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E7" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F7" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G7" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I7" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K7" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M7" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
@@ -82388,101 +82482,98 @@
         <v>264857</v>
       </c>
       <c r="P7" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q7" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B8" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C8" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D8" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E8" t="n">
         <v>9300</v>
       </c>
       <c r="F8" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G8" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I8" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K8" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M8" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N8" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P8" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q8" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R8" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B9" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C9" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D9" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E9" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F9" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G9" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I9" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K9" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M9" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N9" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O9" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P9" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q9" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R9" t="n">
         <v>15000</v>
@@ -82490,40 +82581,40 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B10" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C10" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D10" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E10" t="n">
         <v>9100</v>
       </c>
       <c r="F10" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G10" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I10" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K10" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M10" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N10" t="n">
         <v>189475</v>
       </c>
       <c r="O10" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P10" t="n">
         <v>375660</v>
@@ -82532,6 +82623,53 @@
         <v>773586</v>
       </c>
       <c r="R10" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C11" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K11" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N11" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O11" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P11" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R11" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 11/119] 2026-09-17 ~ 13/17 meters metered 12.27 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:10 ~1:43 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80463,9 +80463,36 @@
       <c r="A2453" s="4" t="n">
         <v>46282</v>
       </c>
+      <c r="B2453" t="n">
+        <v>3.196</v>
+      </c>
+      <c r="C2453" t="n">
+        <v>3.232</v>
+      </c>
+      <c r="D2453" t="n">
+        <v>1.246</v>
+      </c>
+      <c r="E2453" t="n">
+        <v>0.677</v>
+      </c>
+      <c r="F2453" t="n">
+        <v>2.543</v>
+      </c>
+      <c r="G2453" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="H2453" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="I2453" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="K2453" t="n">
+        <v>12.272</v>
+      </c>
       <c r="L2453" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80859,7 +80886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80924,86 +80951,86 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B2" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C2" t="n">
         <v>3.232</v>
       </c>
       <c r="D2" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F2" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G2" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H2" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K2" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B3" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C3" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D3" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E3" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G3" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H3" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I3" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K3" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B4" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C4" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D4" t="n">
         <v>1.435</v>
       </c>
       <c r="E4" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F4" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G4" t="n">
         <v>0.446</v>
@@ -81015,27 +81042,27 @@
         <v>0.712</v>
       </c>
       <c r="K4" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B5" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C5" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D5" t="n">
         <v>1.435</v>
       </c>
       <c r="E5" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F5" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G5" t="n">
         <v>0.446</v>
@@ -81047,59 +81074,59 @@
         <v>0.712</v>
       </c>
       <c r="K5" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B6" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C6" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D6" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E6" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F6" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G6" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H6" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I6" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K6" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B7" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C7" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D7" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E7" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F7" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G7" t="n">
         <v>0.462</v>
@@ -81108,30 +81135,30 @@
         <v>0.343</v>
       </c>
       <c r="I7" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K7" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B8" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C8" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D8" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E8" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F8" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G8" t="n">
         <v>0.462</v>
@@ -81140,100 +81167,97 @@
         <v>0.343</v>
       </c>
       <c r="I8" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K8" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B9" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C9" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D9" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E9" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F9" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G9" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H9" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I9" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K9" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B10" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C10" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D10" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E10" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F10" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G10" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H10" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I10" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J10" t="n">
         <v>0.014</v>
       </c>
       <c r="K10" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B11" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C11" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D11" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F11" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G11" t="n">
         <v>0.395</v>
@@ -81248,6 +81272,41 @@
         <v>0.014</v>
       </c>
       <c r="K11" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K12" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81262,7 +81321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81332,92 +81391,92 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B2" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C2" t="n">
         <v>3.232</v>
       </c>
       <c r="D2" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F2" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G2" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H2" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K2" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L2" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B3" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C3" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D3" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E3" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G3" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H3" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I3" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K3" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L3" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B4" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C4" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D4" t="n">
         <v>1.435</v>
       </c>
       <c r="E4" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F4" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G4" t="n">
         <v>0.446</v>
@@ -81429,30 +81488,30 @@
         <v>0.712</v>
       </c>
       <c r="K4" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L4" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B5" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C5" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D5" t="n">
         <v>1.435</v>
       </c>
       <c r="E5" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F5" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G5" t="n">
         <v>0.446</v>
@@ -81464,65 +81523,65 @@
         <v>0.712</v>
       </c>
       <c r="K5" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L5" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B6" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C6" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D6" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E6" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F6" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G6" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H6" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I6" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K6" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L6" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B7" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C7" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D7" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E7" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F7" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G7" t="n">
         <v>0.462</v>
@@ -81531,33 +81590,33 @@
         <v>0.343</v>
       </c>
       <c r="I7" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K7" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L7" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B8" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C8" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D8" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E8" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F8" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G8" t="n">
         <v>0.462</v>
@@ -81566,109 +81625,106 @@
         <v>0.343</v>
       </c>
       <c r="I8" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K8" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L8" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B9" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C9" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D9" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E9" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F9" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G9" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H9" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I9" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K9" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L9" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B10" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C10" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D10" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E10" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F10" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G10" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H10" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I10" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J10" t="n">
         <v>0.014</v>
       </c>
       <c r="K10" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L10" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B11" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C11" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D11" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F11" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G11" t="n">
         <v>0.395</v>
@@ -81683,9 +81739,47 @@
         <v>0.014</v>
       </c>
       <c r="K11" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L11" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K12" t="n">
         <v>12.277</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L12" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82126,7 +82220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82226,13 +82320,13 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B2" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C2" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D2" t="n">
         <v>1438502</v>
@@ -82241,107 +82335,107 @@
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G2" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I2" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K2" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M2" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N2" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O2" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P2" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q2" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B3" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C3" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D3" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G3" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I3" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K3" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M3" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N3" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O3" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P3" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q3" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B4" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C4" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D4" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G4" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I4" t="n">
         <v>1488515</v>
       </c>
       <c r="K4" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M4" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
@@ -82350,7 +82444,7 @@
         <v>247857</v>
       </c>
       <c r="P4" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q4" t="n">
         <v>738429</v>
@@ -82358,34 +82452,34 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B5" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C5" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D5" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E5" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G5" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I5" t="n">
         <v>1488515</v>
       </c>
       <c r="K5" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M5" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
@@ -82394,7 +82488,7 @@
         <v>247857</v>
       </c>
       <c r="P5" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q5" t="n">
         <v>738429</v>
@@ -82402,78 +82496,78 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B6" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C6" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D6" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E6" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F6" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G6" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I6" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K6" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M6" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P6" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q6" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B7" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C7" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D7" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E7" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G7" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I7" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K7" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M7" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
@@ -82482,42 +82576,42 @@
         <v>264857</v>
       </c>
       <c r="P7" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q7" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B8" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C8" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D8" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E8" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F8" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G8" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I8" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K8" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M8" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
@@ -82526,101 +82620,98 @@
         <v>264857</v>
       </c>
       <c r="P8" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q8" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B9" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C9" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D9" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E9" t="n">
         <v>9300</v>
       </c>
       <c r="F9" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G9" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I9" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K9" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M9" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N9" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P9" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q9" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R9" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B10" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C10" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D10" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E10" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F10" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G10" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I10" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K10" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M10" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N10" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O10" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P10" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q10" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R10" t="n">
         <v>15000</v>
@@ -82628,40 +82719,40 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B11" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C11" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D11" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E11" t="n">
         <v>9100</v>
       </c>
       <c r="F11" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G11" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I11" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K11" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M11" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N11" t="n">
         <v>189475</v>
       </c>
       <c r="O11" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P11" t="n">
         <v>375660</v>
@@ -82670,6 +82761,53 @@
         <v>773586</v>
       </c>
       <c r="R11" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C12" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E12" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K12" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M12" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N12" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O12" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P12" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R12" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 12/119] 2026-09-16 ~ 13/17 meters metered 12.11 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:11 ~1:41 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80453,9 +80453,36 @@
       <c r="A2452" s="4" t="n">
         <v>46281</v>
       </c>
+      <c r="B2452" t="n">
+        <v>3.195</v>
+      </c>
+      <c r="C2452" t="n">
+        <v>3.193</v>
+      </c>
+      <c r="D2452" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="E2452" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="F2452" t="n">
+        <v>2.577</v>
+      </c>
+      <c r="G2452" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="H2452" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="I2452" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="K2452" t="n">
+        <v>12.108</v>
+      </c>
       <c r="L2452" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80886,7 +80913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80951,118 +80978,118 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B2" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C2" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D2" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E2" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G2" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H2" t="n">
         <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K2" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B3" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C3" t="n">
         <v>3.232</v>
       </c>
       <c r="D3" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F3" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G3" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H3" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K3" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B4" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C4" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D4" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E4" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G4" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H4" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I4" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K4" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B5" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C5" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D5" t="n">
         <v>1.435</v>
       </c>
       <c r="E5" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F5" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G5" t="n">
         <v>0.446</v>
@@ -81074,27 +81101,27 @@
         <v>0.712</v>
       </c>
       <c r="K5" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B6" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C6" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D6" t="n">
         <v>1.435</v>
       </c>
       <c r="E6" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F6" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G6" t="n">
         <v>0.446</v>
@@ -81106,59 +81133,59 @@
         <v>0.712</v>
       </c>
       <c r="K6" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B7" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C7" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D7" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E7" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F7" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G7" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H7" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I7" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K7" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B8" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C8" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D8" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E8" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F8" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G8" t="n">
         <v>0.462</v>
@@ -81167,30 +81194,30 @@
         <v>0.343</v>
       </c>
       <c r="I8" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K8" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B9" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C9" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D9" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E9" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F9" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G9" t="n">
         <v>0.462</v>
@@ -81199,100 +81226,97 @@
         <v>0.343</v>
       </c>
       <c r="I9" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K9" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B10" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C10" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D10" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E10" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F10" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G10" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H10" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I10" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K10" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B11" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C11" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D11" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E11" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F11" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G11" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H11" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I11" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J11" t="n">
         <v>0.014</v>
       </c>
       <c r="K11" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B12" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C12" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D12" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F12" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G12" t="n">
         <v>0.395</v>
@@ -81307,6 +81331,41 @@
         <v>0.014</v>
       </c>
       <c r="K12" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K13" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81321,7 +81380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81391,127 +81450,127 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B2" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C2" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D2" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E2" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G2" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H2" t="n">
         <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K2" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L2" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B3" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C3" t="n">
         <v>3.232</v>
       </c>
       <c r="D3" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F3" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G3" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H3" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K3" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L3" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B4" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C4" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D4" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E4" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G4" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H4" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I4" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K4" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L4" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B5" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C5" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D5" t="n">
         <v>1.435</v>
       </c>
       <c r="E5" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F5" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G5" t="n">
         <v>0.446</v>
@@ -81523,30 +81582,30 @@
         <v>0.712</v>
       </c>
       <c r="K5" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L5" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B6" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C6" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D6" t="n">
         <v>1.435</v>
       </c>
       <c r="E6" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F6" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G6" t="n">
         <v>0.446</v>
@@ -81558,65 +81617,65 @@
         <v>0.712</v>
       </c>
       <c r="K6" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L6" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B7" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C7" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D7" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E7" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F7" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G7" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H7" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I7" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K7" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L7" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B8" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C8" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D8" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E8" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F8" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G8" t="n">
         <v>0.462</v>
@@ -81625,33 +81684,33 @@
         <v>0.343</v>
       </c>
       <c r="I8" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K8" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L8" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B9" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C9" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D9" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E9" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F9" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G9" t="n">
         <v>0.462</v>
@@ -81660,109 +81719,106 @@
         <v>0.343</v>
       </c>
       <c r="I9" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K9" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L9" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B10" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C10" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D10" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E10" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F10" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G10" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H10" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I10" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K10" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L10" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B11" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C11" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D11" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E11" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F11" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G11" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H11" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I11" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J11" t="n">
         <v>0.014</v>
       </c>
       <c r="K11" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L11" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B12" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C12" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D12" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F12" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G12" t="n">
         <v>0.395</v>
@@ -81777,9 +81833,47 @@
         <v>0.014</v>
       </c>
       <c r="K12" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L12" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K13" t="n">
         <v>12.277</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L13" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82220,7 +82314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82320,57 +82414,57 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B2" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C2" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D2" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G2" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I2" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K2" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M2" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N2" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P2" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q2" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B3" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C3" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D3" t="n">
         <v>1438502</v>
@@ -82379,107 +82473,107 @@
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G3" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I3" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K3" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M3" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N3" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O3" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P3" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q3" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B4" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C4" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D4" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G4" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I4" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K4" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M4" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N4" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O4" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P4" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q4" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B5" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C5" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D5" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G5" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I5" t="n">
         <v>1488515</v>
       </c>
       <c r="K5" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M5" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
@@ -82488,7 +82582,7 @@
         <v>247857</v>
       </c>
       <c r="P5" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q5" t="n">
         <v>738429</v>
@@ -82496,34 +82590,34 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B6" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C6" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D6" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E6" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G6" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I6" t="n">
         <v>1488515</v>
       </c>
       <c r="K6" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M6" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
@@ -82532,7 +82626,7 @@
         <v>247857</v>
       </c>
       <c r="P6" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q6" t="n">
         <v>738429</v>
@@ -82540,78 +82634,78 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B7" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C7" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D7" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E7" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F7" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G7" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I7" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K7" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M7" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P7" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q7" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B8" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C8" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D8" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E8" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G8" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I8" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K8" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M8" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
@@ -82620,42 +82714,42 @@
         <v>264857</v>
       </c>
       <c r="P8" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q8" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B9" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C9" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D9" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E9" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F9" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G9" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I9" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K9" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M9" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
@@ -82664,101 +82758,98 @@
         <v>264857</v>
       </c>
       <c r="P9" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q9" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B10" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C10" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D10" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E10" t="n">
         <v>9300</v>
       </c>
       <c r="F10" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G10" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I10" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K10" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M10" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N10" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P10" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q10" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R10" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B11" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C11" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D11" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E11" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F11" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G11" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I11" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K11" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M11" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N11" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O11" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P11" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q11" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R11" t="n">
         <v>15000</v>
@@ -82766,40 +82857,40 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B12" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C12" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D12" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E12" t="n">
         <v>9100</v>
       </c>
       <c r="F12" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G12" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I12" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K12" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M12" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N12" t="n">
         <v>189475</v>
       </c>
       <c r="O12" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P12" t="n">
         <v>375660</v>
@@ -82808,6 +82899,53 @@
         <v>773586</v>
       </c>
       <c r="R12" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C13" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K13" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N13" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O13" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P13" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R13" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 13/119] 2026-09-15 ~ 13/17 meters metered 12.02 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:12 ~1:40 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80443,9 +80443,36 @@
       <c r="A2451" s="4" t="n">
         <v>46280</v>
       </c>
+      <c r="B2451" t="n">
+        <v>3.223</v>
+      </c>
+      <c r="C2451" t="n">
+        <v>3.299</v>
+      </c>
+      <c r="D2451" t="n">
+        <v>1.188</v>
+      </c>
+      <c r="E2451" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="F2451" t="n">
+        <v>2.549</v>
+      </c>
+      <c r="G2451" t="n">
+        <v>0.371</v>
+      </c>
+      <c r="H2451" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="I2451" t="n">
+        <v>0.703</v>
+      </c>
+      <c r="K2451" t="n">
+        <v>12.02</v>
+      </c>
       <c r="L2451" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80913,7 +80940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80978,150 +81005,150 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B2" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C2" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D2" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F2" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G2" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H2" t="n">
         <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K2" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B3" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C3" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D3" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E3" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G3" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H3" t="n">
         <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K3" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B4" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C4" t="n">
         <v>3.232</v>
       </c>
       <c r="D4" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F4" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G4" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H4" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K4" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B5" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C5" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D5" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E5" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G5" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H5" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I5" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K5" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B6" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C6" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D6" t="n">
         <v>1.435</v>
       </c>
       <c r="E6" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F6" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G6" t="n">
         <v>0.446</v>
@@ -81133,27 +81160,27 @@
         <v>0.712</v>
       </c>
       <c r="K6" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B7" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C7" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D7" t="n">
         <v>1.435</v>
       </c>
       <c r="E7" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F7" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G7" t="n">
         <v>0.446</v>
@@ -81165,59 +81192,59 @@
         <v>0.712</v>
       </c>
       <c r="K7" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B8" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C8" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D8" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E8" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F8" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G8" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H8" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I8" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K8" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B9" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C9" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D9" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E9" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F9" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G9" t="n">
         <v>0.462</v>
@@ -81226,30 +81253,30 @@
         <v>0.343</v>
       </c>
       <c r="I9" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K9" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B10" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C10" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D10" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E10" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F10" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G10" t="n">
         <v>0.462</v>
@@ -81258,100 +81285,97 @@
         <v>0.343</v>
       </c>
       <c r="I10" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K10" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B11" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C11" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D11" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E11" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F11" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G11" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H11" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I11" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K11" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B12" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C12" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D12" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E12" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F12" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G12" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H12" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I12" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J12" t="n">
         <v>0.014</v>
       </c>
       <c r="K12" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B13" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C13" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D13" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F13" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G13" t="n">
         <v>0.395</v>
@@ -81366,6 +81390,41 @@
         <v>0.014</v>
       </c>
       <c r="K13" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K14" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81380,7 +81439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81450,162 +81509,162 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B2" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C2" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D2" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F2" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G2" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H2" t="n">
         <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K2" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L2" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B3" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C3" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D3" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E3" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G3" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H3" t="n">
         <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K3" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L3" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B4" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C4" t="n">
         <v>3.232</v>
       </c>
       <c r="D4" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F4" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G4" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H4" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K4" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L4" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B5" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C5" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D5" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E5" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G5" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H5" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I5" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K5" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L5" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B6" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C6" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D6" t="n">
         <v>1.435</v>
       </c>
       <c r="E6" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F6" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G6" t="n">
         <v>0.446</v>
@@ -81617,30 +81676,30 @@
         <v>0.712</v>
       </c>
       <c r="K6" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L6" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B7" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C7" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D7" t="n">
         <v>1.435</v>
       </c>
       <c r="E7" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F7" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G7" t="n">
         <v>0.446</v>
@@ -81652,65 +81711,65 @@
         <v>0.712</v>
       </c>
       <c r="K7" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L7" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B8" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C8" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D8" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E8" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F8" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G8" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H8" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I8" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K8" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L8" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B9" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C9" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D9" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E9" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F9" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G9" t="n">
         <v>0.462</v>
@@ -81719,33 +81778,33 @@
         <v>0.343</v>
       </c>
       <c r="I9" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K9" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L9" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B10" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C10" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D10" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E10" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F10" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G10" t="n">
         <v>0.462</v>
@@ -81754,109 +81813,106 @@
         <v>0.343</v>
       </c>
       <c r="I10" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K10" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L10" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B11" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C11" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D11" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E11" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F11" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G11" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H11" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I11" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K11" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L11" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B12" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C12" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D12" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E12" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F12" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G12" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H12" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I12" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J12" t="n">
         <v>0.014</v>
       </c>
       <c r="K12" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L12" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B13" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C13" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D13" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F13" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G13" t="n">
         <v>0.395</v>
@@ -81871,9 +81927,47 @@
         <v>0.014</v>
       </c>
       <c r="K13" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L13" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K14" t="n">
         <v>12.277</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L14" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82314,7 +82408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82414,101 +82508,101 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B2" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C2" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D2" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E2" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F2" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G2" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I2" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K2" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M2" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N2" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O2" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P2" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q2" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B3" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C3" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D3" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G3" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I3" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K3" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M3" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N3" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P3" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q3" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B4" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C4" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D4" t="n">
         <v>1438502</v>
@@ -82517,107 +82611,107 @@
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G4" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I4" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K4" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M4" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N4" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O4" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P4" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q4" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B5" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C5" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D5" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G5" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I5" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K5" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M5" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N5" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O5" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P5" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q5" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B6" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C6" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D6" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G6" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I6" t="n">
         <v>1488515</v>
       </c>
       <c r="K6" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M6" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
@@ -82626,7 +82720,7 @@
         <v>247857</v>
       </c>
       <c r="P6" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q6" t="n">
         <v>738429</v>
@@ -82634,34 +82728,34 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B7" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C7" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D7" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E7" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G7" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I7" t="n">
         <v>1488515</v>
       </c>
       <c r="K7" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M7" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
@@ -82670,7 +82764,7 @@
         <v>247857</v>
       </c>
       <c r="P7" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q7" t="n">
         <v>738429</v>
@@ -82678,78 +82772,78 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B8" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C8" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D8" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E8" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F8" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G8" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I8" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K8" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M8" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P8" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q8" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B9" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C9" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D9" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E9" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G9" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I9" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K9" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M9" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
@@ -82758,42 +82852,42 @@
         <v>264857</v>
       </c>
       <c r="P9" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q9" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B10" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C10" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D10" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E10" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F10" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G10" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I10" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K10" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M10" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
@@ -82802,101 +82896,98 @@
         <v>264857</v>
       </c>
       <c r="P10" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q10" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B11" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C11" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D11" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E11" t="n">
         <v>9300</v>
       </c>
       <c r="F11" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G11" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I11" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K11" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M11" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N11" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P11" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q11" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R11" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B12" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C12" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D12" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E12" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F12" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G12" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I12" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K12" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M12" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N12" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O12" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P12" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q12" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R12" t="n">
         <v>15000</v>
@@ -82904,40 +82995,40 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B13" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C13" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D13" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E13" t="n">
         <v>9100</v>
       </c>
       <c r="F13" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G13" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I13" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K13" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M13" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N13" t="n">
         <v>189475</v>
       </c>
       <c r="O13" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P13" t="n">
         <v>375660</v>
@@ -82946,6 +83037,53 @@
         <v>773586</v>
       </c>
       <c r="R13" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C14" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E14" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K14" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M14" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N14" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O14" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P14" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R14" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 14/119] 2026-09-14 ~ 13/17 meters metered 12.23 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:13 ~1:38 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80433,9 +80433,36 @@
       <c r="A2450" s="4" t="n">
         <v>46279</v>
       </c>
+      <c r="B2450" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="C2450" t="n">
+        <v>3.219</v>
+      </c>
+      <c r="D2450" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="E2450" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F2450" t="n">
+        <v>2.609</v>
+      </c>
+      <c r="G2450" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="H2450" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="I2450" t="n">
+        <v>0.671</v>
+      </c>
+      <c r="K2450" t="n">
+        <v>12.229</v>
+      </c>
       <c r="L2450" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80940,7 +80967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81005,182 +81032,182 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B2" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C2" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D2" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E2" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F2" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G2" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H2" t="n">
         <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K2" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B3" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C3" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D3" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F3" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G3" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H3" t="n">
         <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K3" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B4" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C4" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D4" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E4" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G4" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H4" t="n">
         <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K4" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B5" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C5" t="n">
         <v>3.232</v>
       </c>
       <c r="D5" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F5" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G5" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H5" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K5" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B6" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C6" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D6" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E6" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G6" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H6" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I6" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K6" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B7" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C7" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D7" t="n">
         <v>1.435</v>
       </c>
       <c r="E7" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F7" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G7" t="n">
         <v>0.446</v>
@@ -81192,27 +81219,27 @@
         <v>0.712</v>
       </c>
       <c r="K7" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B8" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C8" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D8" t="n">
         <v>1.435</v>
       </c>
       <c r="E8" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F8" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G8" t="n">
         <v>0.446</v>
@@ -81224,59 +81251,59 @@
         <v>0.712</v>
       </c>
       <c r="K8" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B9" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C9" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D9" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E9" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F9" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G9" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H9" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I9" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K9" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B10" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C10" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D10" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E10" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F10" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G10" t="n">
         <v>0.462</v>
@@ -81285,30 +81312,30 @@
         <v>0.343</v>
       </c>
       <c r="I10" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K10" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B11" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C11" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D11" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E11" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F11" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G11" t="n">
         <v>0.462</v>
@@ -81317,100 +81344,97 @@
         <v>0.343</v>
       </c>
       <c r="I11" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K11" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B12" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C12" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D12" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E12" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F12" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G12" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H12" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I12" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K12" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B13" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C13" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D13" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E13" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F13" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G13" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H13" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I13" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J13" t="n">
         <v>0.014</v>
       </c>
       <c r="K13" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B14" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C14" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D14" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F14" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G14" t="n">
         <v>0.395</v>
@@ -81425,6 +81449,41 @@
         <v>0.014</v>
       </c>
       <c r="K14" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K15" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81439,7 +81498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81509,197 +81568,197 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B2" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C2" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D2" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E2" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F2" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G2" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H2" t="n">
         <v>0.365</v>
       </c>
       <c r="I2" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K2" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L2" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B3" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C3" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D3" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F3" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G3" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H3" t="n">
         <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K3" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L3" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B4" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C4" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D4" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E4" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G4" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H4" t="n">
         <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K4" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L4" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B5" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C5" t="n">
         <v>3.232</v>
       </c>
       <c r="D5" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F5" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G5" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H5" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K5" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L5" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B6" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C6" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D6" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E6" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G6" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H6" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I6" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K6" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L6" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B7" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C7" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D7" t="n">
         <v>1.435</v>
       </c>
       <c r="E7" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F7" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G7" t="n">
         <v>0.446</v>
@@ -81711,30 +81770,30 @@
         <v>0.712</v>
       </c>
       <c r="K7" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L7" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B8" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C8" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D8" t="n">
         <v>1.435</v>
       </c>
       <c r="E8" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F8" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G8" t="n">
         <v>0.446</v>
@@ -81746,65 +81805,65 @@
         <v>0.712</v>
       </c>
       <c r="K8" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L8" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B9" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C9" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D9" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E9" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F9" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G9" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H9" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I9" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K9" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L9" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B10" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C10" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D10" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E10" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F10" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G10" t="n">
         <v>0.462</v>
@@ -81813,33 +81872,33 @@
         <v>0.343</v>
       </c>
       <c r="I10" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K10" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L10" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B11" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C11" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D11" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E11" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F11" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G11" t="n">
         <v>0.462</v>
@@ -81848,109 +81907,106 @@
         <v>0.343</v>
       </c>
       <c r="I11" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K11" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L11" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B12" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C12" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D12" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E12" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F12" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G12" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H12" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I12" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K12" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L12" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B13" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C13" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D13" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E13" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F13" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G13" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H13" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I13" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J13" t="n">
         <v>0.014</v>
       </c>
       <c r="K13" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L13" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B14" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C14" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D14" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F14" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G14" t="n">
         <v>0.395</v>
@@ -81965,9 +82021,47 @@
         <v>0.014</v>
       </c>
       <c r="K14" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L14" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K15" t="n">
         <v>12.277</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L15" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82408,7 +82502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82508,145 +82602,145 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B2" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C2" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D2" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E2" t="n">
         <v>9400</v>
       </c>
       <c r="F2" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G2" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I2" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K2" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M2" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N2" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P2" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q2" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B3" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C3" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D3" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E3" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F3" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G3" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I3" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K3" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M3" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N3" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O3" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P3" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q3" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B4" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C4" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D4" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G4" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I4" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K4" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M4" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N4" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P4" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q4" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B5" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C5" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D5" t="n">
         <v>1438502</v>
@@ -82655,107 +82749,107 @@
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G5" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I5" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K5" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M5" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N5" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O5" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P5" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q5" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B6" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C6" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D6" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G6" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I6" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K6" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M6" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N6" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O6" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P6" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q6" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B7" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C7" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D7" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G7" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I7" t="n">
         <v>1488515</v>
       </c>
       <c r="K7" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M7" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
@@ -82764,7 +82858,7 @@
         <v>247857</v>
       </c>
       <c r="P7" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q7" t="n">
         <v>738429</v>
@@ -82772,34 +82866,34 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B8" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C8" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D8" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E8" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G8" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I8" t="n">
         <v>1488515</v>
       </c>
       <c r="K8" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M8" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
@@ -82808,7 +82902,7 @@
         <v>247857</v>
       </c>
       <c r="P8" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q8" t="n">
         <v>738429</v>
@@ -82816,78 +82910,78 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B9" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C9" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D9" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E9" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F9" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G9" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I9" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K9" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M9" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P9" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q9" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B10" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C10" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D10" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E10" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G10" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I10" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K10" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M10" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
@@ -82896,42 +82990,42 @@
         <v>264857</v>
       </c>
       <c r="P10" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q10" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B11" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C11" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D11" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E11" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F11" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G11" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I11" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K11" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M11" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
@@ -82940,101 +83034,98 @@
         <v>264857</v>
       </c>
       <c r="P11" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q11" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B12" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C12" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D12" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E12" t="n">
         <v>9300</v>
       </c>
       <c r="F12" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G12" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I12" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K12" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M12" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N12" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P12" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q12" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R12" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B13" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C13" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D13" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E13" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F13" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G13" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I13" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K13" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M13" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N13" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O13" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P13" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q13" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R13" t="n">
         <v>15000</v>
@@ -83042,40 +83133,40 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B14" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C14" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D14" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E14" t="n">
         <v>9100</v>
       </c>
       <c r="F14" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G14" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I14" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K14" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M14" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N14" t="n">
         <v>189475</v>
       </c>
       <c r="O14" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P14" t="n">
         <v>375660</v>
@@ -83084,6 +83175,53 @@
         <v>773586</v>
       </c>
       <c r="R14" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B15" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C15" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E15" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K15" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N15" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O15" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P15" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R15" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 15/119] 2026-09-13 ~ 13/17 meters metered 12.23 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:13 ~1:36 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80423,9 +80423,36 @@
       <c r="A2449" s="4" t="n">
         <v>46278</v>
       </c>
+      <c r="B2449" t="n">
+        <v>3.218</v>
+      </c>
+      <c r="C2449" t="n">
+        <v>3.218</v>
+      </c>
+      <c r="D2449" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="E2449" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="F2449" t="n">
+        <v>2.635</v>
+      </c>
+      <c r="G2449" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="H2449" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2449" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="K2449" t="n">
+        <v>12.233</v>
+      </c>
       <c r="L2449" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80967,7 +80994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81032,214 +81059,214 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B2" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C2" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D2" t="n">
         <v>1.44</v>
       </c>
       <c r="E2" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F2" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G2" t="n">
         <v>0.435</v>
       </c>
       <c r="H2" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K2" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B3" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C3" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D3" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E3" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F3" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G3" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H3" t="n">
         <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K3" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B4" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C4" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D4" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F4" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G4" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H4" t="n">
         <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K4" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B5" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C5" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D5" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E5" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G5" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H5" t="n">
         <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K5" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B6" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C6" t="n">
         <v>3.232</v>
       </c>
       <c r="D6" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F6" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G6" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H6" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K6" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B7" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C7" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D7" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E7" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G7" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H7" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I7" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K7" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B8" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C8" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D8" t="n">
         <v>1.435</v>
       </c>
       <c r="E8" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F8" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G8" t="n">
         <v>0.446</v>
@@ -81251,27 +81278,27 @@
         <v>0.712</v>
       </c>
       <c r="K8" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B9" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C9" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D9" t="n">
         <v>1.435</v>
       </c>
       <c r="E9" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F9" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G9" t="n">
         <v>0.446</v>
@@ -81283,59 +81310,59 @@
         <v>0.712</v>
       </c>
       <c r="K9" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B10" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C10" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D10" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E10" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F10" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G10" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H10" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I10" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K10" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B11" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C11" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D11" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E11" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F11" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G11" t="n">
         <v>0.462</v>
@@ -81344,30 +81371,30 @@
         <v>0.343</v>
       </c>
       <c r="I11" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K11" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B12" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C12" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D12" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E12" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F12" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G12" t="n">
         <v>0.462</v>
@@ -81376,100 +81403,97 @@
         <v>0.343</v>
       </c>
       <c r="I12" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K12" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B13" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C13" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D13" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E13" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F13" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G13" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H13" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I13" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K13" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B14" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C14" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D14" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E14" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F14" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G14" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H14" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I14" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J14" t="n">
         <v>0.014</v>
       </c>
       <c r="K14" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B15" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C15" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D15" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F15" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G15" t="n">
         <v>0.395</v>
@@ -81484,6 +81508,41 @@
         <v>0.014</v>
       </c>
       <c r="K15" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K16" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81498,7 +81557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81568,232 +81627,232 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B2" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C2" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D2" t="n">
         <v>1.44</v>
       </c>
       <c r="E2" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F2" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G2" t="n">
         <v>0.435</v>
       </c>
       <c r="H2" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K2" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L2" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B3" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C3" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D3" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E3" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F3" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G3" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H3" t="n">
         <v>0.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K3" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L3" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B4" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C4" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D4" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F4" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G4" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H4" t="n">
         <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K4" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L4" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B5" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C5" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D5" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E5" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G5" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H5" t="n">
         <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K5" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L5" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B6" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C6" t="n">
         <v>3.232</v>
       </c>
       <c r="D6" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F6" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G6" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H6" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K6" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L6" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B7" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C7" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D7" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E7" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G7" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H7" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I7" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K7" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L7" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B8" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C8" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D8" t="n">
         <v>1.435</v>
       </c>
       <c r="E8" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F8" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G8" t="n">
         <v>0.446</v>
@@ -81805,30 +81864,30 @@
         <v>0.712</v>
       </c>
       <c r="K8" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L8" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B9" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C9" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D9" t="n">
         <v>1.435</v>
       </c>
       <c r="E9" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F9" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G9" t="n">
         <v>0.446</v>
@@ -81840,65 +81899,65 @@
         <v>0.712</v>
       </c>
       <c r="K9" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L9" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B10" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C10" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D10" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E10" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F10" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G10" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H10" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I10" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K10" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L10" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B11" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C11" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D11" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E11" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F11" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G11" t="n">
         <v>0.462</v>
@@ -81907,33 +81966,33 @@
         <v>0.343</v>
       </c>
       <c r="I11" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K11" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L11" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B12" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C12" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D12" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E12" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F12" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G12" t="n">
         <v>0.462</v>
@@ -81942,109 +82001,106 @@
         <v>0.343</v>
       </c>
       <c r="I12" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K12" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L12" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B13" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C13" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D13" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E13" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F13" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G13" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H13" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I13" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K13" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L13" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B14" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C14" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D14" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E14" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F14" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G14" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H14" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I14" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J14" t="n">
         <v>0.014</v>
       </c>
       <c r="K14" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L14" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B15" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C15" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D15" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F15" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G15" t="n">
         <v>0.395</v>
@@ -82059,9 +82115,47 @@
         <v>0.014</v>
       </c>
       <c r="K15" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L15" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K16" t="n">
         <v>12.277</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L16" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82502,7 +82596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82602,34 +82696,34 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B2" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C2" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D2" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E2" t="n">
         <v>9400</v>
       </c>
       <c r="F2" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G2" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I2" t="n">
         <v>1493578</v>
       </c>
       <c r="K2" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M2" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
@@ -82638,153 +82732,153 @@
         <v>236857</v>
       </c>
       <c r="P2" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q2" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B3" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C3" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D3" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E3" t="n">
         <v>9400</v>
       </c>
       <c r="F3" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G3" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I3" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K3" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M3" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N3" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P3" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q3" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B4" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C4" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D4" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E4" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F4" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G4" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I4" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K4" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M4" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N4" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O4" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P4" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q4" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B5" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C5" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D5" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G5" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I5" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K5" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M5" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N5" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P5" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q5" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B6" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C6" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D6" t="n">
         <v>1438502</v>
@@ -82793,107 +82887,107 @@
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G6" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I6" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K6" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M6" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N6" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O6" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P6" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q6" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B7" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C7" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D7" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G7" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I7" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K7" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M7" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N7" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O7" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P7" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q7" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B8" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C8" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D8" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G8" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I8" t="n">
         <v>1488515</v>
       </c>
       <c r="K8" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M8" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
@@ -82902,7 +82996,7 @@
         <v>247857</v>
       </c>
       <c r="P8" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q8" t="n">
         <v>738429</v>
@@ -82910,34 +83004,34 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B9" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C9" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D9" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E9" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G9" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I9" t="n">
         <v>1488515</v>
       </c>
       <c r="K9" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M9" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
@@ -82946,7 +83040,7 @@
         <v>247857</v>
       </c>
       <c r="P9" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q9" t="n">
         <v>738429</v>
@@ -82954,78 +83048,78 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B10" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C10" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D10" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E10" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F10" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G10" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I10" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K10" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M10" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P10" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q10" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B11" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C11" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D11" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E11" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G11" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I11" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K11" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M11" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
@@ -83034,42 +83128,42 @@
         <v>264857</v>
       </c>
       <c r="P11" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q11" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B12" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C12" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D12" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E12" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F12" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G12" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I12" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K12" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M12" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
@@ -83078,101 +83172,98 @@
         <v>264857</v>
       </c>
       <c r="P12" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q12" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B13" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C13" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D13" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E13" t="n">
         <v>9300</v>
       </c>
       <c r="F13" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G13" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I13" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K13" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M13" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N13" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O13" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P13" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q13" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R13" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B14" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C14" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D14" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E14" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F14" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G14" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I14" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K14" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M14" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N14" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O14" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P14" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q14" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R14" t="n">
         <v>15000</v>
@@ -83180,40 +83271,40 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B15" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C15" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D15" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E15" t="n">
         <v>9100</v>
       </c>
       <c r="F15" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G15" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I15" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K15" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M15" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N15" t="n">
         <v>189475</v>
       </c>
       <c r="O15" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P15" t="n">
         <v>375660</v>
@@ -83222,6 +83313,53 @@
         <v>773586</v>
       </c>
       <c r="R15" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B16" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C16" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E16" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K16" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M16" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N16" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O16" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P16" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R16" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 16/119] 2026-09-12 ~ 13/17 meters metered 12.29 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:14 ~1:34 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80413,9 +80413,36 @@
       <c r="A2448" s="4" t="n">
         <v>46277</v>
       </c>
+      <c r="B2448" t="n">
+        <v>3.244</v>
+      </c>
+      <c r="C2448" t="n">
+        <v>3.247</v>
+      </c>
+      <c r="D2448" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="E2448" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="F2448" t="n">
+        <v>2.638</v>
+      </c>
+      <c r="G2448" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="H2448" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2448" t="n">
+        <v>0.662</v>
+      </c>
+      <c r="K2448" t="n">
+        <v>12.294</v>
+      </c>
       <c r="L2448" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -80994,7 +81021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81059,13 +81086,13 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B2" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C2" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D2" t="n">
         <v>1.44</v>
@@ -81074,7 +81101,7 @@
         <v>0.261</v>
       </c>
       <c r="F2" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G2" t="n">
         <v>0.435</v>
@@ -81083,222 +81110,222 @@
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K2" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B3" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C3" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D3" t="n">
         <v>1.44</v>
       </c>
       <c r="E3" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F3" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G3" t="n">
         <v>0.435</v>
       </c>
       <c r="H3" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K3" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B4" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C4" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D4" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E4" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F4" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G4" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H4" t="n">
         <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K4" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B5" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C5" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D5" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F5" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G5" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H5" t="n">
         <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K5" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B6" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C6" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D6" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E6" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G6" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H6" t="n">
         <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K6" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B7" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C7" t="n">
         <v>3.232</v>
       </c>
       <c r="D7" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F7" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G7" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H7" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K7" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B8" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C8" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D8" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E8" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G8" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H8" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I8" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K8" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B9" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C9" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D9" t="n">
         <v>1.435</v>
       </c>
       <c r="E9" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F9" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G9" t="n">
         <v>0.446</v>
@@ -81310,27 +81337,27 @@
         <v>0.712</v>
       </c>
       <c r="K9" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B10" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C10" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D10" t="n">
         <v>1.435</v>
       </c>
       <c r="E10" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F10" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G10" t="n">
         <v>0.446</v>
@@ -81342,59 +81369,59 @@
         <v>0.712</v>
       </c>
       <c r="K10" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B11" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C11" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D11" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E11" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F11" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G11" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H11" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I11" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K11" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B12" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C12" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D12" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E12" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F12" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G12" t="n">
         <v>0.462</v>
@@ -81403,30 +81430,30 @@
         <v>0.343</v>
       </c>
       <c r="I12" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K12" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B13" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C13" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D13" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E13" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F13" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G13" t="n">
         <v>0.462</v>
@@ -81435,100 +81462,97 @@
         <v>0.343</v>
       </c>
       <c r="I13" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K13" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B14" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C14" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D14" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E14" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F14" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G14" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H14" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I14" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K14" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B15" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C15" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D15" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E15" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F15" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G15" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H15" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I15" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J15" t="n">
         <v>0.014</v>
       </c>
       <c r="K15" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B16" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C16" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D16" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F16" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G16" t="n">
         <v>0.395</v>
@@ -81543,6 +81567,41 @@
         <v>0.014</v>
       </c>
       <c r="K16" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K17" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81557,7 +81616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81627,13 +81686,13 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B2" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C2" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D2" t="n">
         <v>1.44</v>
@@ -81642,7 +81701,7 @@
         <v>0.261</v>
       </c>
       <c r="F2" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G2" t="n">
         <v>0.435</v>
@@ -81651,243 +81710,243 @@
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K2" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L2" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B3" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C3" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D3" t="n">
         <v>1.44</v>
       </c>
       <c r="E3" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F3" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G3" t="n">
         <v>0.435</v>
       </c>
       <c r="H3" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K3" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L3" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B4" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C4" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D4" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E4" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F4" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G4" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H4" t="n">
         <v>0.365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K4" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L4" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B5" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C5" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D5" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F5" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G5" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H5" t="n">
         <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K5" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L5" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B6" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C6" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D6" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E6" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G6" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H6" t="n">
         <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K6" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L6" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B7" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C7" t="n">
         <v>3.232</v>
       </c>
       <c r="D7" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F7" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G7" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H7" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K7" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L7" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B8" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C8" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D8" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E8" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G8" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H8" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I8" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K8" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L8" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B9" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C9" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D9" t="n">
         <v>1.435</v>
       </c>
       <c r="E9" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F9" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G9" t="n">
         <v>0.446</v>
@@ -81899,30 +81958,30 @@
         <v>0.712</v>
       </c>
       <c r="K9" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L9" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B10" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C10" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D10" t="n">
         <v>1.435</v>
       </c>
       <c r="E10" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F10" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G10" t="n">
         <v>0.446</v>
@@ -81934,65 +81993,65 @@
         <v>0.712</v>
       </c>
       <c r="K10" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L10" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B11" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C11" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D11" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E11" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F11" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G11" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H11" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I11" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K11" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L11" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B12" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C12" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D12" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E12" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F12" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G12" t="n">
         <v>0.462</v>
@@ -82001,33 +82060,33 @@
         <v>0.343</v>
       </c>
       <c r="I12" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K12" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L12" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B13" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C13" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D13" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E13" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F13" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G13" t="n">
         <v>0.462</v>
@@ -82036,109 +82095,106 @@
         <v>0.343</v>
       </c>
       <c r="I13" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K13" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L13" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B14" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C14" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D14" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E14" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F14" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G14" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H14" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I14" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K14" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L14" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B15" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C15" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D15" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E15" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F15" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G15" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H15" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I15" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J15" t="n">
         <v>0.014</v>
       </c>
       <c r="K15" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L15" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B16" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C16" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D16" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F16" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G16" t="n">
         <v>0.395</v>
@@ -82153,9 +82209,47 @@
         <v>0.014</v>
       </c>
       <c r="K16" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L16" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K17" t="n">
         <v>12.277</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L17" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82596,7 +82690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82696,25 +82790,25 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B2" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C2" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D2" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E2" t="n">
         <v>9400</v>
       </c>
       <c r="F2" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G2" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I2" t="n">
         <v>1493578</v>
@@ -82723,7 +82817,7 @@
         <v>270165</v>
       </c>
       <c r="M2" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
@@ -82735,39 +82829,39 @@
         <v>380581</v>
       </c>
       <c r="Q2" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B3" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C3" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D3" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E3" t="n">
         <v>9400</v>
       </c>
       <c r="F3" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G3" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I3" t="n">
         <v>1493578</v>
       </c>
       <c r="K3" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M3" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
@@ -82776,153 +82870,153 @@
         <v>236857</v>
       </c>
       <c r="P3" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q3" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B4" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C4" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D4" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E4" t="n">
         <v>9400</v>
       </c>
       <c r="F4" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G4" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I4" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K4" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M4" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N4" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P4" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q4" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B5" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C5" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D5" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E5" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F5" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G5" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I5" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K5" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M5" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N5" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O5" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P5" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q5" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B6" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C6" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D6" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G6" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I6" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K6" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M6" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N6" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P6" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q6" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B7" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C7" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D7" t="n">
         <v>1438502</v>
@@ -82931,107 +83025,107 @@
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G7" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I7" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K7" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M7" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N7" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O7" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P7" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q7" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B8" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C8" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D8" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G8" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I8" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K8" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M8" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N8" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O8" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P8" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q8" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B9" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C9" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D9" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G9" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I9" t="n">
         <v>1488515</v>
       </c>
       <c r="K9" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M9" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
@@ -83040,7 +83134,7 @@
         <v>247857</v>
       </c>
       <c r="P9" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q9" t="n">
         <v>738429</v>
@@ -83048,34 +83142,34 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B10" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C10" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D10" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E10" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G10" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I10" t="n">
         <v>1488515</v>
       </c>
       <c r="K10" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M10" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
@@ -83084,7 +83178,7 @@
         <v>247857</v>
       </c>
       <c r="P10" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q10" t="n">
         <v>738429</v>
@@ -83092,78 +83186,78 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B11" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C11" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D11" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E11" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F11" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G11" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I11" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K11" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M11" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P11" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q11" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B12" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C12" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D12" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E12" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G12" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I12" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K12" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M12" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
@@ -83172,42 +83266,42 @@
         <v>264857</v>
       </c>
       <c r="P12" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q12" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B13" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C13" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D13" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E13" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F13" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G13" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I13" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K13" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M13" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
@@ -83216,101 +83310,98 @@
         <v>264857</v>
       </c>
       <c r="P13" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q13" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B14" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C14" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D14" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E14" t="n">
         <v>9300</v>
       </c>
       <c r="F14" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G14" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I14" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K14" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M14" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N14" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O14" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P14" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q14" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R14" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B15" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C15" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D15" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E15" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F15" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G15" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I15" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K15" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M15" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N15" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O15" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P15" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q15" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R15" t="n">
         <v>15000</v>
@@ -83318,40 +83409,40 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B16" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C16" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D16" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E16" t="n">
         <v>9100</v>
       </c>
       <c r="F16" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G16" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I16" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K16" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M16" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N16" t="n">
         <v>189475</v>
       </c>
       <c r="O16" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P16" t="n">
         <v>375660</v>
@@ -83360,6 +83451,53 @@
         <v>773586</v>
       </c>
       <c r="R16" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C17" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E17" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K17" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M17" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N17" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O17" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P17" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R17" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 17/119] 2026-09-11 ~ 13/17 meters metered 12.17 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:15 ~1:33 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80403,9 +80403,36 @@
       <c r="A2447" s="4" t="n">
         <v>46276</v>
       </c>
+      <c r="B2447" t="n">
+        <v>3.287</v>
+      </c>
+      <c r="C2447" t="n">
+        <v>3.198</v>
+      </c>
+      <c r="D2447" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="E2447" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="F2447" t="n">
+        <v>2.607</v>
+      </c>
+      <c r="G2447" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="H2447" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2447" t="n">
+        <v>0.666</v>
+      </c>
+      <c r="K2447" t="n">
+        <v>12.171</v>
+      </c>
       <c r="L2447" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81021,7 +81048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81086,45 +81113,45 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B2" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C2" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D2" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E2" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F2" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G2" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K2" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B3" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C3" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D3" t="n">
         <v>1.44</v>
@@ -81133,7 +81160,7 @@
         <v>0.261</v>
       </c>
       <c r="F3" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G3" t="n">
         <v>0.435</v>
@@ -81142,222 +81169,222 @@
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K3" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B4" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C4" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D4" t="n">
         <v>1.44</v>
       </c>
       <c r="E4" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F4" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G4" t="n">
         <v>0.435</v>
       </c>
       <c r="H4" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K4" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B5" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C5" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D5" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E5" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F5" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G5" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H5" t="n">
         <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K5" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B6" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C6" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D6" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F6" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G6" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H6" t="n">
         <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K6" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B7" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C7" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D7" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E7" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G7" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H7" t="n">
         <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K7" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B8" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C8" t="n">
         <v>3.232</v>
       </c>
       <c r="D8" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F8" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G8" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H8" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K8" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B9" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C9" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D9" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E9" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G9" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H9" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I9" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K9" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B10" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C10" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D10" t="n">
         <v>1.435</v>
       </c>
       <c r="E10" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F10" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G10" t="n">
         <v>0.446</v>
@@ -81369,27 +81396,27 @@
         <v>0.712</v>
       </c>
       <c r="K10" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B11" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C11" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D11" t="n">
         <v>1.435</v>
       </c>
       <c r="E11" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F11" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G11" t="n">
         <v>0.446</v>
@@ -81401,59 +81428,59 @@
         <v>0.712</v>
       </c>
       <c r="K11" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B12" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C12" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D12" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E12" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F12" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G12" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H12" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I12" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K12" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B13" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C13" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D13" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E13" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F13" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G13" t="n">
         <v>0.462</v>
@@ -81462,30 +81489,30 @@
         <v>0.343</v>
       </c>
       <c r="I13" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K13" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B14" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C14" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D14" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E14" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F14" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G14" t="n">
         <v>0.462</v>
@@ -81494,100 +81521,97 @@
         <v>0.343</v>
       </c>
       <c r="I14" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K14" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B15" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C15" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D15" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E15" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F15" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G15" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H15" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I15" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K15" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B16" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C16" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D16" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E16" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F16" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G16" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H16" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I16" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J16" t="n">
         <v>0.014</v>
       </c>
       <c r="K16" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B17" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C17" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D17" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F17" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G17" t="n">
         <v>0.395</v>
@@ -81602,6 +81626,41 @@
         <v>0.014</v>
       </c>
       <c r="K17" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K18" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81616,7 +81675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81686,48 +81745,48 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B2" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C2" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D2" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E2" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F2" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G2" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K2" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L2" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B3" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C3" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D3" t="n">
         <v>1.44</v>
@@ -81736,7 +81795,7 @@
         <v>0.261</v>
       </c>
       <c r="F3" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G3" t="n">
         <v>0.435</v>
@@ -81745,243 +81804,243 @@
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K3" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L3" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B4" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C4" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D4" t="n">
         <v>1.44</v>
       </c>
       <c r="E4" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F4" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G4" t="n">
         <v>0.435</v>
       </c>
       <c r="H4" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K4" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L4" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B5" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C5" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D5" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E5" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F5" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G5" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H5" t="n">
         <v>0.365</v>
       </c>
       <c r="I5" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K5" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L5" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B6" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C6" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D6" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F6" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G6" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H6" t="n">
         <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K6" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L6" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B7" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C7" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D7" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E7" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G7" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H7" t="n">
         <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K7" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L7" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B8" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C8" t="n">
         <v>3.232</v>
       </c>
       <c r="D8" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F8" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G8" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H8" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K8" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L8" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B9" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C9" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D9" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E9" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G9" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H9" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I9" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K9" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L9" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B10" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C10" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D10" t="n">
         <v>1.435</v>
       </c>
       <c r="E10" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F10" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G10" t="n">
         <v>0.446</v>
@@ -81993,30 +82052,30 @@
         <v>0.712</v>
       </c>
       <c r="K10" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L10" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B11" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C11" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D11" t="n">
         <v>1.435</v>
       </c>
       <c r="E11" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F11" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G11" t="n">
         <v>0.446</v>
@@ -82028,65 +82087,65 @@
         <v>0.712</v>
       </c>
       <c r="K11" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L11" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B12" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C12" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D12" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E12" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F12" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G12" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H12" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I12" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K12" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L12" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B13" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C13" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D13" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E13" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F13" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G13" t="n">
         <v>0.462</v>
@@ -82095,33 +82154,33 @@
         <v>0.343</v>
       </c>
       <c r="I13" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K13" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L13" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B14" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C14" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D14" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E14" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F14" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G14" t="n">
         <v>0.462</v>
@@ -82130,109 +82189,106 @@
         <v>0.343</v>
       </c>
       <c r="I14" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K14" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L14" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B15" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C15" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D15" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E15" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F15" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G15" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H15" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I15" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K15" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L15" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B16" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C16" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D16" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E16" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F16" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G16" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H16" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I16" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J16" t="n">
         <v>0.014</v>
       </c>
       <c r="K16" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L16" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B17" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C17" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D17" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F17" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G17" t="n">
         <v>0.395</v>
@@ -82247,9 +82303,47 @@
         <v>0.014</v>
       </c>
       <c r="K17" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L17" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K18" t="n">
         <v>12.277</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82690,7 +82784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82790,69 +82884,69 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B2" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C2" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D2" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E2" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G2" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I2" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K2" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M2" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N2" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O2" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P2" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q2" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B3" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C3" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D3" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E3" t="n">
         <v>9400</v>
       </c>
       <c r="F3" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G3" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I3" t="n">
         <v>1493578</v>
@@ -82861,7 +82955,7 @@
         <v>270165</v>
       </c>
       <c r="M3" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
@@ -82873,39 +82967,39 @@
         <v>380581</v>
       </c>
       <c r="Q3" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B4" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C4" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D4" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E4" t="n">
         <v>9400</v>
       </c>
       <c r="F4" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G4" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I4" t="n">
         <v>1493578</v>
       </c>
       <c r="K4" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M4" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
@@ -82914,153 +83008,153 @@
         <v>236857</v>
       </c>
       <c r="P4" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q4" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B5" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C5" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D5" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E5" t="n">
         <v>9400</v>
       </c>
       <c r="F5" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G5" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I5" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K5" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M5" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N5" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P5" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q5" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B6" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C6" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D6" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E6" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F6" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G6" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I6" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K6" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M6" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N6" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O6" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P6" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q6" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B7" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C7" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D7" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G7" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I7" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K7" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M7" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N7" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P7" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q7" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B8" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C8" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D8" t="n">
         <v>1438502</v>
@@ -83069,107 +83163,107 @@
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G8" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I8" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K8" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M8" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N8" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O8" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P8" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q8" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B9" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C9" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D9" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G9" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I9" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K9" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M9" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N9" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O9" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P9" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q9" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B10" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C10" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D10" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G10" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I10" t="n">
         <v>1488515</v>
       </c>
       <c r="K10" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M10" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
@@ -83178,7 +83272,7 @@
         <v>247857</v>
       </c>
       <c r="P10" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q10" t="n">
         <v>738429</v>
@@ -83186,34 +83280,34 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B11" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C11" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D11" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E11" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G11" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I11" t="n">
         <v>1488515</v>
       </c>
       <c r="K11" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M11" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
@@ -83222,7 +83316,7 @@
         <v>247857</v>
       </c>
       <c r="P11" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q11" t="n">
         <v>738429</v>
@@ -83230,78 +83324,78 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B12" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C12" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D12" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E12" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F12" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G12" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I12" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K12" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M12" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P12" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q12" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B13" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C13" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D13" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E13" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G13" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I13" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K13" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M13" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
@@ -83310,42 +83404,42 @@
         <v>264857</v>
       </c>
       <c r="P13" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q13" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B14" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C14" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D14" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E14" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F14" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G14" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I14" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K14" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M14" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
@@ -83354,101 +83448,98 @@
         <v>264857</v>
       </c>
       <c r="P14" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q14" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B15" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C15" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D15" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E15" t="n">
         <v>9300</v>
       </c>
       <c r="F15" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G15" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I15" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K15" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M15" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N15" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O15" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P15" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q15" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R15" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B16" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C16" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D16" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E16" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F16" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G16" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I16" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K16" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M16" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N16" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O16" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P16" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q16" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R16" t="n">
         <v>15000</v>
@@ -83456,40 +83547,40 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B17" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C17" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D17" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E17" t="n">
         <v>9100</v>
       </c>
       <c r="F17" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G17" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I17" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K17" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M17" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N17" t="n">
         <v>189475</v>
       </c>
       <c r="O17" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P17" t="n">
         <v>375660</v>
@@ -83498,6 +83589,53 @@
         <v>773586</v>
       </c>
       <c r="R17" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C18" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E18" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K18" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M18" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N18" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O18" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P18" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R18" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 18/119] 2026-09-10 ~ 13/17 meters metered 12.35 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:16 ~1:31 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80393,9 +80393,36 @@
       <c r="A2446" s="4" t="n">
         <v>46275</v>
       </c>
+      <c r="B2446" t="n">
+        <v>3.334</v>
+      </c>
+      <c r="C2446" t="n">
+        <v>3.234</v>
+      </c>
+      <c r="D2446" t="n">
+        <v>1.361</v>
+      </c>
+      <c r="E2446" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F2446" t="n">
+        <v>2.609</v>
+      </c>
+      <c r="G2446" t="n">
+        <v>0.457</v>
+      </c>
+      <c r="H2446" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2446" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="K2446" t="n">
+        <v>12.347</v>
+      </c>
       <c r="L2446" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81048,7 +81075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81113,77 +81140,77 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B2" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C2" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D2" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E2" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F2" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G2" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B3" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C3" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D3" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E3" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F3" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G3" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K3" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B4" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C4" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D4" t="n">
         <v>1.44</v>
@@ -81192,7 +81219,7 @@
         <v>0.261</v>
       </c>
       <c r="F4" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G4" t="n">
         <v>0.435</v>
@@ -81201,222 +81228,222 @@
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K4" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B5" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C5" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D5" t="n">
         <v>1.44</v>
       </c>
       <c r="E5" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F5" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G5" t="n">
         <v>0.435</v>
       </c>
       <c r="H5" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K5" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B6" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C6" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D6" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E6" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F6" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G6" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H6" t="n">
         <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K6" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B7" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C7" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D7" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F7" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G7" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H7" t="n">
         <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K7" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B8" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C8" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D8" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E8" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G8" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H8" t="n">
         <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K8" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B9" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C9" t="n">
         <v>3.232</v>
       </c>
       <c r="D9" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F9" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G9" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H9" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K9" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B10" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C10" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D10" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E10" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G10" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H10" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I10" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K10" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B11" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C11" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D11" t="n">
         <v>1.435</v>
       </c>
       <c r="E11" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F11" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G11" t="n">
         <v>0.446</v>
@@ -81428,27 +81455,27 @@
         <v>0.712</v>
       </c>
       <c r="K11" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B12" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C12" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D12" t="n">
         <v>1.435</v>
       </c>
       <c r="E12" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F12" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G12" t="n">
         <v>0.446</v>
@@ -81460,59 +81487,59 @@
         <v>0.712</v>
       </c>
       <c r="K12" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B13" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C13" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D13" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E13" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F13" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G13" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H13" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I13" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K13" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B14" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C14" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D14" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E14" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F14" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G14" t="n">
         <v>0.462</v>
@@ -81521,30 +81548,30 @@
         <v>0.343</v>
       </c>
       <c r="I14" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K14" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B15" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C15" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D15" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E15" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F15" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G15" t="n">
         <v>0.462</v>
@@ -81553,100 +81580,97 @@
         <v>0.343</v>
       </c>
       <c r="I15" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K15" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B16" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C16" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D16" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E16" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F16" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G16" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H16" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I16" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K16" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B17" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C17" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D17" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E17" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F17" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G17" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H17" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I17" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J17" t="n">
         <v>0.014</v>
       </c>
       <c r="K17" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B18" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C18" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D18" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F18" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G18" t="n">
         <v>0.395</v>
@@ -81661,6 +81685,41 @@
         <v>0.014</v>
       </c>
       <c r="K18" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K19" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81675,7 +81734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81745,83 +81804,83 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B2" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C2" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D2" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E2" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F2" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G2" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L2" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B3" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C3" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D3" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E3" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F3" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G3" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K3" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L3" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B4" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C4" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D4" t="n">
         <v>1.44</v>
@@ -81830,7 +81889,7 @@
         <v>0.261</v>
       </c>
       <c r="F4" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G4" t="n">
         <v>0.435</v>
@@ -81839,243 +81898,243 @@
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K4" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L4" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B5" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C5" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D5" t="n">
         <v>1.44</v>
       </c>
       <c r="E5" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F5" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G5" t="n">
         <v>0.435</v>
       </c>
       <c r="H5" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K5" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L5" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B6" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C6" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D6" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E6" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F6" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G6" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H6" t="n">
         <v>0.365</v>
       </c>
       <c r="I6" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K6" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L6" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B7" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C7" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D7" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F7" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G7" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H7" t="n">
         <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K7" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L7" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B8" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C8" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D8" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E8" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G8" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H8" t="n">
         <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K8" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L8" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B9" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C9" t="n">
         <v>3.232</v>
       </c>
       <c r="D9" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F9" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G9" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H9" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K9" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L9" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B10" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C10" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D10" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E10" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G10" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H10" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I10" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K10" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L10" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B11" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C11" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D11" t="n">
         <v>1.435</v>
       </c>
       <c r="E11" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F11" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G11" t="n">
         <v>0.446</v>
@@ -82087,30 +82146,30 @@
         <v>0.712</v>
       </c>
       <c r="K11" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L11" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B12" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C12" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D12" t="n">
         <v>1.435</v>
       </c>
       <c r="E12" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F12" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G12" t="n">
         <v>0.446</v>
@@ -82122,65 +82181,65 @@
         <v>0.712</v>
       </c>
       <c r="K12" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L12" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B13" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C13" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D13" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E13" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F13" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G13" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H13" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I13" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K13" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L13" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B14" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C14" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D14" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E14" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F14" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G14" t="n">
         <v>0.462</v>
@@ -82189,33 +82248,33 @@
         <v>0.343</v>
       </c>
       <c r="I14" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K14" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L14" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B15" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C15" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D15" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E15" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F15" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G15" t="n">
         <v>0.462</v>
@@ -82224,109 +82283,106 @@
         <v>0.343</v>
       </c>
       <c r="I15" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K15" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L15" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B16" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C16" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D16" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E16" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F16" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G16" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H16" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I16" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K16" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L16" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B17" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C17" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D17" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E17" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F17" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G17" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H17" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I17" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J17" t="n">
         <v>0.014</v>
       </c>
       <c r="K17" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L17" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B18" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C18" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D18" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F18" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G18" t="n">
         <v>0.395</v>
@@ -82341,9 +82397,47 @@
         <v>0.014</v>
       </c>
       <c r="K18" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L18" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K19" t="n">
         <v>12.277</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L19" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82784,7 +82878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82884,113 +82978,113 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B2" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C2" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D2" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G2" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I2" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K2" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M2" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N2" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P2" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q2" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B3" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C3" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D3" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E3" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G3" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I3" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K3" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M3" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N3" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O3" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P3" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q3" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B4" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C4" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D4" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E4" t="n">
         <v>9400</v>
       </c>
       <c r="F4" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G4" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I4" t="n">
         <v>1493578</v>
@@ -82999,7 +83093,7 @@
         <v>270165</v>
       </c>
       <c r="M4" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
@@ -83011,39 +83105,39 @@
         <v>380581</v>
       </c>
       <c r="Q4" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B5" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C5" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D5" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E5" t="n">
         <v>9400</v>
       </c>
       <c r="F5" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G5" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I5" t="n">
         <v>1493578</v>
       </c>
       <c r="K5" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M5" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
@@ -83052,153 +83146,153 @@
         <v>236857</v>
       </c>
       <c r="P5" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q5" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B6" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C6" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D6" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E6" t="n">
         <v>9400</v>
       </c>
       <c r="F6" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G6" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I6" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K6" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M6" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N6" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P6" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q6" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B7" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C7" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D7" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E7" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F7" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G7" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I7" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K7" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M7" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N7" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O7" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P7" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q7" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B8" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C8" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D8" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G8" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I8" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K8" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M8" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N8" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P8" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q8" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B9" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C9" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D9" t="n">
         <v>1438502</v>
@@ -83207,107 +83301,107 @@
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G9" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I9" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K9" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M9" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N9" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O9" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P9" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q9" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B10" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C10" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D10" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G10" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I10" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K10" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M10" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N10" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O10" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P10" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q10" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B11" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C11" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D11" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G11" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I11" t="n">
         <v>1488515</v>
       </c>
       <c r="K11" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M11" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
@@ -83316,7 +83410,7 @@
         <v>247857</v>
       </c>
       <c r="P11" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q11" t="n">
         <v>738429</v>
@@ -83324,34 +83418,34 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B12" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C12" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D12" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E12" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G12" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I12" t="n">
         <v>1488515</v>
       </c>
       <c r="K12" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M12" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
@@ -83360,7 +83454,7 @@
         <v>247857</v>
       </c>
       <c r="P12" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q12" t="n">
         <v>738429</v>
@@ -83368,78 +83462,78 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B13" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C13" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D13" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E13" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F13" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G13" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I13" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K13" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M13" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
       </c>
       <c r="O13" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P13" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q13" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B14" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C14" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D14" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E14" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G14" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I14" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K14" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M14" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
@@ -83448,42 +83542,42 @@
         <v>264857</v>
       </c>
       <c r="P14" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q14" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B15" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C15" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D15" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E15" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F15" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G15" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I15" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K15" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M15" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
@@ -83492,101 +83586,98 @@
         <v>264857</v>
       </c>
       <c r="P15" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q15" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B16" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C16" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D16" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E16" t="n">
         <v>9300</v>
       </c>
       <c r="F16" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G16" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I16" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K16" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M16" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N16" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O16" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P16" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q16" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R16" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B17" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C17" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D17" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E17" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F17" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G17" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I17" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K17" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M17" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N17" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O17" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P17" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q17" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R17" t="n">
         <v>15000</v>
@@ -83594,40 +83685,40 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B18" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C18" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D18" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E18" t="n">
         <v>9100</v>
       </c>
       <c r="F18" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G18" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I18" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K18" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M18" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N18" t="n">
         <v>189475</v>
       </c>
       <c r="O18" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P18" t="n">
         <v>375660</v>
@@ -83636,6 +83727,53 @@
         <v>773586</v>
       </c>
       <c r="R18" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B19" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C19" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E19" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K19" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M19" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N19" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O19" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P19" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R19" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 19/119] 2026-09-09 ~ 13/17 meters metered 12.13 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:17 ~1:29 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80383,9 +80383,36 @@
       <c r="A2445" s="4" t="n">
         <v>46274</v>
       </c>
+      <c r="B2445" t="n">
+        <v>3.215</v>
+      </c>
+      <c r="C2445" t="n">
+        <v>3.214</v>
+      </c>
+      <c r="D2445" t="n">
+        <v>1.464</v>
+      </c>
+      <c r="E2445" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="F2445" t="n">
+        <v>2.594</v>
+      </c>
+      <c r="G2445" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="H2445" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2445" t="n">
+        <v>0.627</v>
+      </c>
+      <c r="K2445" t="n">
+        <v>12.126</v>
+      </c>
       <c r="L2445" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81075,7 +81102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81140,109 +81167,109 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B2" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C2" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D2" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F2" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G2" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K2" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B3" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C3" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D3" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E3" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F3" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G3" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B4" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C4" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D4" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E4" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F4" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G4" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K4" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B5" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C5" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D5" t="n">
         <v>1.44</v>
@@ -81251,7 +81278,7 @@
         <v>0.261</v>
       </c>
       <c r="F5" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G5" t="n">
         <v>0.435</v>
@@ -81260,222 +81287,222 @@
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K5" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B6" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C6" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D6" t="n">
         <v>1.44</v>
       </c>
       <c r="E6" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F6" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G6" t="n">
         <v>0.435</v>
       </c>
       <c r="H6" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K6" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B7" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C7" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D7" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E7" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F7" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G7" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H7" t="n">
         <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K7" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B8" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C8" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D8" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F8" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G8" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H8" t="n">
         <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K8" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B9" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C9" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D9" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E9" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G9" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H9" t="n">
         <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K9" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B10" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C10" t="n">
         <v>3.232</v>
       </c>
       <c r="D10" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F10" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G10" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H10" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K10" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B11" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C11" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D11" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E11" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G11" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H11" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I11" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K11" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B12" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C12" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D12" t="n">
         <v>1.435</v>
       </c>
       <c r="E12" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F12" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G12" t="n">
         <v>0.446</v>
@@ -81487,27 +81514,27 @@
         <v>0.712</v>
       </c>
       <c r="K12" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B13" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C13" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D13" t="n">
         <v>1.435</v>
       </c>
       <c r="E13" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F13" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G13" t="n">
         <v>0.446</v>
@@ -81519,59 +81546,59 @@
         <v>0.712</v>
       </c>
       <c r="K13" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B14" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C14" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D14" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E14" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F14" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G14" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H14" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I14" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K14" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B15" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C15" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D15" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E15" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F15" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G15" t="n">
         <v>0.462</v>
@@ -81580,30 +81607,30 @@
         <v>0.343</v>
       </c>
       <c r="I15" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K15" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B16" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C16" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D16" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E16" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F16" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G16" t="n">
         <v>0.462</v>
@@ -81612,100 +81639,97 @@
         <v>0.343</v>
       </c>
       <c r="I16" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K16" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B17" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C17" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D17" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E17" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F17" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G17" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H17" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I17" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K17" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B18" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C18" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D18" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E18" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F18" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G18" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H18" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I18" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J18" t="n">
         <v>0.014</v>
       </c>
       <c r="K18" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B19" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C19" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D19" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F19" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G19" t="n">
         <v>0.395</v>
@@ -81720,6 +81744,41 @@
         <v>0.014</v>
       </c>
       <c r="K19" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K20" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81734,7 +81793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81804,118 +81863,118 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B2" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C2" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D2" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F2" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G2" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K2" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L2" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B3" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C3" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D3" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E3" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F3" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G3" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L3" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B4" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C4" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D4" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E4" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F4" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G4" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K4" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L4" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B5" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C5" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D5" t="n">
         <v>1.44</v>
@@ -81924,7 +81983,7 @@
         <v>0.261</v>
       </c>
       <c r="F5" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G5" t="n">
         <v>0.435</v>
@@ -81933,243 +81992,243 @@
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K5" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L5" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B6" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C6" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D6" t="n">
         <v>1.44</v>
       </c>
       <c r="E6" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F6" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G6" t="n">
         <v>0.435</v>
       </c>
       <c r="H6" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K6" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L6" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B7" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C7" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D7" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E7" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F7" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G7" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H7" t="n">
         <v>0.365</v>
       </c>
       <c r="I7" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K7" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L7" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B8" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C8" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D8" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F8" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G8" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H8" t="n">
         <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K8" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L8" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B9" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C9" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D9" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E9" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G9" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H9" t="n">
         <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K9" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L9" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B10" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C10" t="n">
         <v>3.232</v>
       </c>
       <c r="D10" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F10" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G10" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H10" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K10" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L10" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B11" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C11" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D11" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E11" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G11" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H11" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I11" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K11" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L11" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B12" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C12" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D12" t="n">
         <v>1.435</v>
       </c>
       <c r="E12" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F12" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G12" t="n">
         <v>0.446</v>
@@ -82181,30 +82240,30 @@
         <v>0.712</v>
       </c>
       <c r="K12" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L12" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B13" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C13" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D13" t="n">
         <v>1.435</v>
       </c>
       <c r="E13" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F13" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G13" t="n">
         <v>0.446</v>
@@ -82216,65 +82275,65 @@
         <v>0.712</v>
       </c>
       <c r="K13" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L13" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B14" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C14" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D14" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E14" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F14" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G14" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H14" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I14" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K14" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L14" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B15" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C15" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D15" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E15" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F15" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G15" t="n">
         <v>0.462</v>
@@ -82283,33 +82342,33 @@
         <v>0.343</v>
       </c>
       <c r="I15" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K15" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L15" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B16" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C16" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D16" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E16" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F16" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G16" t="n">
         <v>0.462</v>
@@ -82318,109 +82377,106 @@
         <v>0.343</v>
       </c>
       <c r="I16" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K16" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L16" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B17" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C17" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D17" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E17" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F17" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G17" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H17" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I17" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K17" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L17" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B18" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C18" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D18" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E18" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F18" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G18" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H18" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I18" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J18" t="n">
         <v>0.014</v>
       </c>
       <c r="K18" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L18" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B19" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C19" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D19" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F19" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G19" t="n">
         <v>0.395</v>
@@ -82435,9 +82491,47 @@
         <v>0.014</v>
       </c>
       <c r="K19" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L19" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K20" t="n">
         <v>12.277</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L20" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82878,7 +82972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82978,157 +83072,157 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B2" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C2" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D2" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G2" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I2" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K2" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M2" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N2" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O2" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P2" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q2" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B3" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C3" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D3" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G3" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I3" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K3" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M3" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N3" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P3" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q3" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B4" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C4" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D4" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E4" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G4" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I4" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K4" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M4" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N4" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O4" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P4" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q4" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B5" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C5" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D5" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E5" t="n">
         <v>9400</v>
       </c>
       <c r="F5" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G5" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I5" t="n">
         <v>1493578</v>
@@ -83137,7 +83231,7 @@
         <v>270165</v>
       </c>
       <c r="M5" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
@@ -83149,39 +83243,39 @@
         <v>380581</v>
       </c>
       <c r="Q5" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B6" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C6" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D6" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E6" t="n">
         <v>9400</v>
       </c>
       <c r="F6" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G6" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I6" t="n">
         <v>1493578</v>
       </c>
       <c r="K6" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M6" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
@@ -83190,153 +83284,153 @@
         <v>236857</v>
       </c>
       <c r="P6" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q6" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B7" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C7" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D7" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E7" t="n">
         <v>9400</v>
       </c>
       <c r="F7" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G7" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I7" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K7" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M7" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N7" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P7" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q7" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B8" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C8" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D8" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E8" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F8" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G8" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I8" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K8" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M8" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N8" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O8" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P8" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q8" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B9" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C9" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D9" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G9" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I9" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K9" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M9" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N9" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P9" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q9" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B10" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C10" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D10" t="n">
         <v>1438502</v>
@@ -83345,107 +83439,107 @@
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G10" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I10" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K10" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M10" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N10" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O10" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P10" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q10" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B11" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C11" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D11" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G11" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I11" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K11" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M11" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N11" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O11" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P11" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q11" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B12" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C12" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D12" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G12" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I12" t="n">
         <v>1488515</v>
       </c>
       <c r="K12" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M12" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
@@ -83454,7 +83548,7 @@
         <v>247857</v>
       </c>
       <c r="P12" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q12" t="n">
         <v>738429</v>
@@ -83462,34 +83556,34 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B13" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C13" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D13" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E13" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G13" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I13" t="n">
         <v>1488515</v>
       </c>
       <c r="K13" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M13" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
@@ -83498,7 +83592,7 @@
         <v>247857</v>
       </c>
       <c r="P13" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q13" t="n">
         <v>738429</v>
@@ -83506,78 +83600,78 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B14" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C14" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D14" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E14" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F14" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G14" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I14" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K14" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M14" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
       </c>
       <c r="O14" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P14" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q14" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B15" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C15" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D15" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E15" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G15" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I15" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K15" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M15" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
@@ -83586,42 +83680,42 @@
         <v>264857</v>
       </c>
       <c r="P15" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q15" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B16" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C16" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D16" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E16" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F16" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G16" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I16" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K16" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M16" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N16" t="n">
         <v>214475</v>
@@ -83630,101 +83724,98 @@
         <v>264857</v>
       </c>
       <c r="P16" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q16" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B17" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C17" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D17" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E17" t="n">
         <v>9300</v>
       </c>
       <c r="F17" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G17" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I17" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K17" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M17" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N17" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O17" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P17" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q17" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R17" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B18" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C18" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D18" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E18" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F18" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G18" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I18" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K18" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M18" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N18" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O18" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P18" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q18" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R18" t="n">
         <v>15000</v>
@@ -83732,40 +83823,40 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B19" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C19" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D19" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E19" t="n">
         <v>9100</v>
       </c>
       <c r="F19" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G19" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I19" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K19" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M19" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N19" t="n">
         <v>189475</v>
       </c>
       <c r="O19" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P19" t="n">
         <v>375660</v>
@@ -83774,6 +83865,53 @@
         <v>773586</v>
       </c>
       <c r="R19" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C20" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E20" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K20" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M20" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N20" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O20" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P20" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R20" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 20/119] 2026-09-08 ~ 13/17 meters metered 11.96 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:17 ~1:28 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80373,9 +80373,36 @@
       <c r="A2444" s="4" t="n">
         <v>46273</v>
       </c>
+      <c r="B2444" t="n">
+        <v>3.205</v>
+      </c>
+      <c r="C2444" t="n">
+        <v>3.213</v>
+      </c>
+      <c r="D2444" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="E2444" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="F2444" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="G2444" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="H2444" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="I2444" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="K2444" t="n">
+        <v>11.961</v>
+      </c>
       <c r="L2444" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81102,7 +81129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81167,141 +81194,141 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B2" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C2" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D2" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E2" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F2" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G2" t="n">
         <v>0.437</v>
       </c>
       <c r="H2" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I2" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B3" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C3" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D3" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F3" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G3" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K3" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B4" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C4" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D4" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E4" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F4" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G4" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B5" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C5" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D5" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E5" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F5" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G5" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K5" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B6" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C6" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D6" t="n">
         <v>1.44</v>
@@ -81310,7 +81337,7 @@
         <v>0.261</v>
       </c>
       <c r="F6" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G6" t="n">
         <v>0.435</v>
@@ -81319,222 +81346,222 @@
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K6" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B7" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C7" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D7" t="n">
         <v>1.44</v>
       </c>
       <c r="E7" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F7" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G7" t="n">
         <v>0.435</v>
       </c>
       <c r="H7" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K7" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B8" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C8" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D8" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E8" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F8" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G8" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H8" t="n">
         <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K8" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B9" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C9" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D9" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F9" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G9" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H9" t="n">
         <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K9" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B10" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C10" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D10" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E10" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G10" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H10" t="n">
         <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K10" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B11" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C11" t="n">
         <v>3.232</v>
       </c>
       <c r="D11" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F11" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G11" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H11" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K11" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B12" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C12" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D12" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E12" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F12" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G12" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H12" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I12" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K12" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B13" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C13" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D13" t="n">
         <v>1.435</v>
       </c>
       <c r="E13" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F13" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G13" t="n">
         <v>0.446</v>
@@ -81546,27 +81573,27 @@
         <v>0.712</v>
       </c>
       <c r="K13" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B14" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C14" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D14" t="n">
         <v>1.435</v>
       </c>
       <c r="E14" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F14" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G14" t="n">
         <v>0.446</v>
@@ -81578,59 +81605,59 @@
         <v>0.712</v>
       </c>
       <c r="K14" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B15" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C15" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D15" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E15" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F15" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G15" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H15" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I15" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K15" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B16" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C16" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D16" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E16" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F16" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G16" t="n">
         <v>0.462</v>
@@ -81639,30 +81666,30 @@
         <v>0.343</v>
       </c>
       <c r="I16" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K16" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B17" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C17" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D17" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E17" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F17" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G17" t="n">
         <v>0.462</v>
@@ -81671,100 +81698,97 @@
         <v>0.343</v>
       </c>
       <c r="I17" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K17" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B18" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C18" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D18" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E18" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F18" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G18" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H18" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I18" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K18" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B19" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C19" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D19" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E19" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F19" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G19" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H19" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I19" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J19" t="n">
         <v>0.014</v>
       </c>
       <c r="K19" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B20" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C20" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D20" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F20" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G20" t="n">
         <v>0.395</v>
@@ -81779,6 +81803,41 @@
         <v>0.014</v>
       </c>
       <c r="K20" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B21" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K21" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81793,7 +81852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81863,153 +81922,153 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B2" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C2" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D2" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E2" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F2" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G2" t="n">
         <v>0.437</v>
       </c>
       <c r="H2" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I2" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L2" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B3" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C3" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D3" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F3" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G3" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K3" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L3" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B4" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C4" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D4" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E4" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F4" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G4" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L4" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B5" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C5" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D5" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E5" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F5" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G5" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K5" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L5" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B6" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C6" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D6" t="n">
         <v>1.44</v>
@@ -82018,7 +82077,7 @@
         <v>0.261</v>
       </c>
       <c r="F6" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G6" t="n">
         <v>0.435</v>
@@ -82027,243 +82086,243 @@
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K6" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L6" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B7" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C7" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D7" t="n">
         <v>1.44</v>
       </c>
       <c r="E7" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F7" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G7" t="n">
         <v>0.435</v>
       </c>
       <c r="H7" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K7" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L7" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B8" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C8" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D8" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E8" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F8" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G8" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H8" t="n">
         <v>0.365</v>
       </c>
       <c r="I8" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K8" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L8" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B9" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C9" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D9" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F9" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G9" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H9" t="n">
         <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K9" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L9" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B10" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C10" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D10" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E10" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G10" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H10" t="n">
         <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K10" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L10" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B11" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C11" t="n">
         <v>3.232</v>
       </c>
       <c r="D11" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F11" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G11" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H11" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K11" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L11" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B12" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C12" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D12" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E12" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F12" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G12" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H12" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I12" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K12" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L12" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B13" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C13" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D13" t="n">
         <v>1.435</v>
       </c>
       <c r="E13" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F13" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G13" t="n">
         <v>0.446</v>
@@ -82275,30 +82334,30 @@
         <v>0.712</v>
       </c>
       <c r="K13" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L13" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B14" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C14" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D14" t="n">
         <v>1.435</v>
       </c>
       <c r="E14" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F14" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G14" t="n">
         <v>0.446</v>
@@ -82310,65 +82369,65 @@
         <v>0.712</v>
       </c>
       <c r="K14" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L14" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B15" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C15" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D15" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E15" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F15" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G15" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H15" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I15" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K15" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L15" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B16" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C16" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D16" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E16" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F16" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G16" t="n">
         <v>0.462</v>
@@ -82377,33 +82436,33 @@
         <v>0.343</v>
       </c>
       <c r="I16" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K16" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L16" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B17" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C17" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D17" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E17" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F17" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G17" t="n">
         <v>0.462</v>
@@ -82412,109 +82471,106 @@
         <v>0.343</v>
       </c>
       <c r="I17" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K17" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L17" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B18" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C18" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D18" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E18" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F18" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G18" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H18" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I18" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K18" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L18" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B19" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C19" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D19" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E19" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F19" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G19" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H19" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I19" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J19" t="n">
         <v>0.014</v>
       </c>
       <c r="K19" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L19" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B20" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C20" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D20" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F20" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G20" t="n">
         <v>0.395</v>
@@ -82529,9 +82585,47 @@
         <v>0.014</v>
       </c>
       <c r="K20" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L20" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B21" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K21" t="n">
         <v>12.277</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L21" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -82972,7 +83066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83072,201 +83166,201 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B2" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C2" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D2" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G2" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I2" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K2" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M2" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N2" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O2" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P2" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q2" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B3" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C3" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D3" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G3" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I3" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K3" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M3" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N3" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O3" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P3" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q3" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B4" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C4" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D4" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G4" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I4" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K4" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M4" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N4" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P4" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q4" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B5" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C5" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D5" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E5" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G5" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I5" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K5" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M5" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N5" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O5" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P5" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q5" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B6" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C6" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D6" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E6" t="n">
         <v>9400</v>
       </c>
       <c r="F6" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G6" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I6" t="n">
         <v>1493578</v>
@@ -83275,7 +83369,7 @@
         <v>270165</v>
       </c>
       <c r="M6" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
@@ -83287,39 +83381,39 @@
         <v>380581</v>
       </c>
       <c r="Q6" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B7" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C7" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D7" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E7" t="n">
         <v>9400</v>
       </c>
       <c r="F7" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G7" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I7" t="n">
         <v>1493578</v>
       </c>
       <c r="K7" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M7" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
@@ -83328,153 +83422,153 @@
         <v>236857</v>
       </c>
       <c r="P7" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q7" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B8" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C8" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D8" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E8" t="n">
         <v>9400</v>
       </c>
       <c r="F8" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G8" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I8" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K8" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M8" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N8" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P8" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q8" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B9" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C9" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D9" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E9" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F9" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G9" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I9" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K9" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M9" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N9" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O9" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P9" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q9" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B10" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C10" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D10" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G10" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I10" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K10" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M10" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N10" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P10" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q10" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B11" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C11" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D11" t="n">
         <v>1438502</v>
@@ -83483,107 +83577,107 @@
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G11" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I11" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K11" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M11" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N11" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O11" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P11" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q11" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B12" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C12" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D12" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G12" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I12" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K12" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M12" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N12" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O12" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P12" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q12" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B13" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C13" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D13" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G13" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I13" t="n">
         <v>1488515</v>
       </c>
       <c r="K13" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M13" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
@@ -83592,7 +83686,7 @@
         <v>247857</v>
       </c>
       <c r="P13" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q13" t="n">
         <v>738429</v>
@@ -83600,34 +83694,34 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B14" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C14" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D14" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E14" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G14" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I14" t="n">
         <v>1488515</v>
       </c>
       <c r="K14" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M14" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
@@ -83636,7 +83730,7 @@
         <v>247857</v>
       </c>
       <c r="P14" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q14" t="n">
         <v>738429</v>
@@ -83644,78 +83738,78 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B15" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C15" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D15" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E15" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F15" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G15" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I15" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K15" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M15" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
       </c>
       <c r="O15" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P15" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q15" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B16" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C16" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D16" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E16" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G16" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I16" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K16" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M16" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N16" t="n">
         <v>214475</v>
@@ -83724,42 +83818,42 @@
         <v>264857</v>
       </c>
       <c r="P16" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q16" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B17" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C17" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D17" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E17" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F17" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G17" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I17" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K17" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M17" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N17" t="n">
         <v>214475</v>
@@ -83768,101 +83862,98 @@
         <v>264857</v>
       </c>
       <c r="P17" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q17" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B18" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C18" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D18" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E18" t="n">
         <v>9300</v>
       </c>
       <c r="F18" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G18" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I18" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K18" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M18" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N18" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O18" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P18" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q18" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R18" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B19" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C19" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D19" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E19" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F19" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G19" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I19" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K19" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M19" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N19" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O19" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P19" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q19" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R19" t="n">
         <v>15000</v>
@@ -83870,40 +83961,40 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B20" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C20" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D20" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E20" t="n">
         <v>9100</v>
       </c>
       <c r="F20" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G20" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I20" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K20" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M20" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N20" t="n">
         <v>189475</v>
       </c>
       <c r="O20" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P20" t="n">
         <v>375660</v>
@@ -83912,6 +84003,53 @@
         <v>773586</v>
       </c>
       <c r="R20" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B21" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C21" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E21" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K21" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M21" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N21" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O21" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P21" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R21" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -83979,7 +84117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E650"/>
+  <dimension ref="A1:E658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91229,8 +91367,93 @@
         <v>4.436</v>
       </c>
     </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Calcasieu Pass</t>
+        </is>
+      </c>
+      <c r="D651" t="n">
+        <v>0.408</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Cameron</t>
+        </is>
+      </c>
+      <c r="D652" t="n">
+        <v>1.383</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Corpus Christi</t>
+        </is>
+      </c>
+      <c r="D653" t="n">
+        <v>2.494</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Elba Island</t>
+        </is>
+      </c>
+      <c r="D654" t="n">
+        <v>0.359</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Freeport</t>
+        </is>
+      </c>
+      <c r="D655" t="n">
+        <v>0.413</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Golden Pass</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>0.701</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Plaquemines</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>3.234</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Sabine Pass</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>3.264</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="106">
+  <mergeCells count="107">
     <mergeCell ref="A544:A551"/>
     <mergeCell ref="A584:A591"/>
     <mergeCell ref="A88:A91"/>
@@ -91283,6 +91506,7 @@
     <mergeCell ref="A73:A75"/>
     <mergeCell ref="A82:A84"/>
     <mergeCell ref="A63:A64"/>
+    <mergeCell ref="A651:A658"/>
     <mergeCell ref="A616:A623"/>
     <mergeCell ref="A426:A432"/>
     <mergeCell ref="A184:A189"/>

</xml_diff>

<commit_message>
Feedgas backfill: [ 21/119] 2026-09-07 ~ 13/17 meters metered 11.94 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:18 ~1:26 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80363,9 +80363,36 @@
       <c r="A2443" s="4" t="n">
         <v>46272</v>
       </c>
+      <c r="B2443" t="n">
+        <v>3.227</v>
+      </c>
+      <c r="C2443" t="n">
+        <v>3.139</v>
+      </c>
+      <c r="D2443" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="E2443" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="F2443" t="n">
+        <v>2.554</v>
+      </c>
+      <c r="G2443" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="H2443" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2443" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="K2443" t="n">
+        <v>11.936</v>
+      </c>
       <c r="L2443" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81129,7 +81156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81194,173 +81221,173 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B2" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C2" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D2" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E2" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F2" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G2" t="n">
         <v>0.437</v>
       </c>
       <c r="H2" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I2" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B3" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C3" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D3" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E3" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F3" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G3" t="n">
         <v>0.437</v>
       </c>
       <c r="H3" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I3" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B4" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C4" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D4" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F4" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G4" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K4" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B5" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C5" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D5" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E5" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F5" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G5" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B6" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C6" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D6" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E6" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F6" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G6" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K6" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B7" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C7" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D7" t="n">
         <v>1.44</v>
@@ -81369,7 +81396,7 @@
         <v>0.261</v>
       </c>
       <c r="F7" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G7" t="n">
         <v>0.435</v>
@@ -81378,222 +81405,222 @@
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K7" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B8" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C8" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D8" t="n">
         <v>1.44</v>
       </c>
       <c r="E8" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F8" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G8" t="n">
         <v>0.435</v>
       </c>
       <c r="H8" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K8" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B9" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C9" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D9" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E9" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F9" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G9" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H9" t="n">
         <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K9" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B10" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C10" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D10" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F10" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G10" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H10" t="n">
         <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K10" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B11" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C11" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D11" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E11" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G11" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H11" t="n">
         <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K11" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B12" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C12" t="n">
         <v>3.232</v>
       </c>
       <c r="D12" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F12" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G12" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H12" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K12" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B13" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C13" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D13" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E13" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G13" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H13" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I13" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K13" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B14" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C14" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D14" t="n">
         <v>1.435</v>
       </c>
       <c r="E14" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F14" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G14" t="n">
         <v>0.446</v>
@@ -81605,27 +81632,27 @@
         <v>0.712</v>
       </c>
       <c r="K14" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B15" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C15" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D15" t="n">
         <v>1.435</v>
       </c>
       <c r="E15" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F15" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G15" t="n">
         <v>0.446</v>
@@ -81637,59 +81664,59 @@
         <v>0.712</v>
       </c>
       <c r="K15" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B16" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C16" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D16" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E16" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F16" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G16" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H16" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I16" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K16" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B17" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C17" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D17" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E17" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F17" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G17" t="n">
         <v>0.462</v>
@@ -81698,30 +81725,30 @@
         <v>0.343</v>
       </c>
       <c r="I17" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K17" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B18" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C18" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D18" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E18" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F18" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G18" t="n">
         <v>0.462</v>
@@ -81730,100 +81757,97 @@
         <v>0.343</v>
       </c>
       <c r="I18" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K18" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B19" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C19" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D19" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E19" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F19" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G19" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H19" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I19" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K19" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B20" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C20" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D20" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E20" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F20" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G20" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H20" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I20" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J20" t="n">
         <v>0.014</v>
       </c>
       <c r="K20" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B21" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C21" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D21" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E21" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F21" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G21" t="n">
         <v>0.395</v>
@@ -81838,6 +81862,41 @@
         <v>0.014</v>
       </c>
       <c r="K21" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C22" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K22" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81852,7 +81911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81922,188 +81981,188 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B2" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C2" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D2" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E2" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F2" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G2" t="n">
         <v>0.437</v>
       </c>
       <c r="H2" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I2" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L2" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B3" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C3" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D3" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E3" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F3" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G3" t="n">
         <v>0.437</v>
       </c>
       <c r="H3" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I3" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L3" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B4" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C4" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D4" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F4" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G4" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K4" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L4" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B5" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C5" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D5" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E5" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F5" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G5" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L5" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B6" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C6" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D6" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E6" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F6" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G6" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K6" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L6" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B7" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C7" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D7" t="n">
         <v>1.44</v>
@@ -82112,7 +82171,7 @@
         <v>0.261</v>
       </c>
       <c r="F7" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G7" t="n">
         <v>0.435</v>
@@ -82121,243 +82180,243 @@
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K7" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L7" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B8" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C8" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D8" t="n">
         <v>1.44</v>
       </c>
       <c r="E8" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F8" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G8" t="n">
         <v>0.435</v>
       </c>
       <c r="H8" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K8" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L8" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B9" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C9" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D9" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E9" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F9" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G9" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H9" t="n">
         <v>0.365</v>
       </c>
       <c r="I9" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K9" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L9" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B10" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C10" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D10" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F10" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G10" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H10" t="n">
         <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K10" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L10" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B11" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C11" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D11" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E11" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G11" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H11" t="n">
         <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K11" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L11" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B12" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C12" t="n">
         <v>3.232</v>
       </c>
       <c r="D12" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F12" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G12" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H12" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K12" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L12" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B13" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C13" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D13" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E13" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G13" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H13" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I13" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K13" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L13" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B14" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C14" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D14" t="n">
         <v>1.435</v>
       </c>
       <c r="E14" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F14" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G14" t="n">
         <v>0.446</v>
@@ -82369,30 +82428,30 @@
         <v>0.712</v>
       </c>
       <c r="K14" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L14" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B15" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C15" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D15" t="n">
         <v>1.435</v>
       </c>
       <c r="E15" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F15" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G15" t="n">
         <v>0.446</v>
@@ -82404,65 +82463,65 @@
         <v>0.712</v>
       </c>
       <c r="K15" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L15" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B16" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C16" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D16" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E16" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F16" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G16" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H16" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I16" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K16" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L16" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B17" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C17" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D17" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E17" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F17" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G17" t="n">
         <v>0.462</v>
@@ -82471,33 +82530,33 @@
         <v>0.343</v>
       </c>
       <c r="I17" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K17" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L17" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B18" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C18" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D18" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E18" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F18" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G18" t="n">
         <v>0.462</v>
@@ -82506,109 +82565,106 @@
         <v>0.343</v>
       </c>
       <c r="I18" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K18" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L18" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B19" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C19" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D19" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E19" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F19" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G19" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H19" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I19" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K19" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L19" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B20" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C20" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D20" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E20" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F20" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G20" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H20" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I20" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J20" t="n">
         <v>0.014</v>
       </c>
       <c r="K20" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L20" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B21" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C21" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D21" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E21" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F21" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G21" t="n">
         <v>0.395</v>
@@ -82623,9 +82679,47 @@
         <v>0.014</v>
       </c>
       <c r="K21" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L21" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C22" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K22" t="n">
         <v>12.277</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L22" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83066,7 +83160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83166,43 +83260,43 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B2" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C2" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D2" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G2" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I2" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K2" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M2" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N2" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P2" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q2" t="n">
         <v>710782</v>
@@ -83210,201 +83304,201 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B3" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C3" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D3" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G3" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I3" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K3" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M3" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N3" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O3" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P3" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q3" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B4" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C4" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D4" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G4" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I4" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K4" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M4" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N4" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O4" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P4" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q4" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B5" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C5" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D5" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G5" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I5" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K5" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M5" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N5" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P5" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q5" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B6" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C6" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D6" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E6" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G6" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I6" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K6" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M6" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N6" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O6" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P6" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q6" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B7" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C7" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D7" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E7" t="n">
         <v>9400</v>
       </c>
       <c r="F7" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G7" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I7" t="n">
         <v>1493578</v>
@@ -83413,7 +83507,7 @@
         <v>270165</v>
       </c>
       <c r="M7" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
@@ -83425,39 +83519,39 @@
         <v>380581</v>
       </c>
       <c r="Q7" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B8" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C8" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D8" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E8" t="n">
         <v>9400</v>
       </c>
       <c r="F8" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G8" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I8" t="n">
         <v>1493578</v>
       </c>
       <c r="K8" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M8" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
@@ -83466,153 +83560,153 @@
         <v>236857</v>
       </c>
       <c r="P8" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q8" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B9" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C9" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D9" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E9" t="n">
         <v>9400</v>
       </c>
       <c r="F9" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G9" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I9" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K9" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M9" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N9" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P9" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q9" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B10" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C10" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D10" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E10" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F10" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G10" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I10" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K10" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M10" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N10" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O10" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P10" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q10" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B11" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C11" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D11" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G11" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I11" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K11" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M11" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N11" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P11" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q11" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B12" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C12" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D12" t="n">
         <v>1438502</v>
@@ -83621,107 +83715,107 @@
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G12" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I12" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K12" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M12" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N12" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O12" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P12" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q12" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B13" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C13" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D13" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G13" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I13" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K13" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M13" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N13" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O13" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P13" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q13" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B14" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C14" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D14" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G14" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I14" t="n">
         <v>1488515</v>
       </c>
       <c r="K14" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M14" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
@@ -83730,7 +83824,7 @@
         <v>247857</v>
       </c>
       <c r="P14" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q14" t="n">
         <v>738429</v>
@@ -83738,34 +83832,34 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B15" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C15" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D15" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E15" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G15" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I15" t="n">
         <v>1488515</v>
       </c>
       <c r="K15" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M15" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
@@ -83774,7 +83868,7 @@
         <v>247857</v>
       </c>
       <c r="P15" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q15" t="n">
         <v>738429</v>
@@ -83782,78 +83876,78 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B16" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C16" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D16" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E16" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F16" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G16" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I16" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K16" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M16" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N16" t="n">
         <v>214475</v>
       </c>
       <c r="O16" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P16" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q16" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B17" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C17" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D17" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E17" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G17" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I17" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K17" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M17" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N17" t="n">
         <v>214475</v>
@@ -83862,42 +83956,42 @@
         <v>264857</v>
       </c>
       <c r="P17" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q17" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B18" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C18" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D18" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E18" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F18" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G18" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I18" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K18" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M18" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N18" t="n">
         <v>214475</v>
@@ -83906,101 +84000,98 @@
         <v>264857</v>
       </c>
       <c r="P18" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q18" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B19" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C19" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D19" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E19" t="n">
         <v>9300</v>
       </c>
       <c r="F19" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G19" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I19" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K19" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M19" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N19" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O19" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P19" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q19" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R19" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B20" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C20" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D20" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E20" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F20" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G20" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I20" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K20" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M20" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N20" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O20" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P20" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q20" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R20" t="n">
         <v>15000</v>
@@ -84008,40 +84099,40 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B21" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C21" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D21" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E21" t="n">
         <v>9100</v>
       </c>
       <c r="F21" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G21" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I21" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K21" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M21" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N21" t="n">
         <v>189475</v>
       </c>
       <c r="O21" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P21" t="n">
         <v>375660</v>
@@ -84050,6 +84141,53 @@
         <v>773586</v>
       </c>
       <c r="R21" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C22" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E22" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K22" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M22" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N22" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O22" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P22" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R22" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -91379,7 +91517,7 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>0.408</v>
+        <v>0.403</v>
       </c>
     </row>
     <row r="652">
@@ -91389,7 +91527,7 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>1.383</v>
+        <v>1.376</v>
       </c>
     </row>
     <row r="653">
@@ -91399,7 +91537,7 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.494</v>
+        <v>2.497</v>
       </c>
     </row>
     <row r="654">
@@ -91419,7 +91557,7 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>0.413</v>
+        <v>0.414</v>
       </c>
     </row>
     <row r="656">
@@ -91429,7 +91567,7 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>0.701</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="657">
@@ -91439,7 +91577,7 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>3.234</v>
+        <v>3.229</v>
       </c>
     </row>
     <row r="658">
@@ -91449,7 +91587,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.264</v>
+        <v>3.263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feedgas backfill: [ 22/119] 2026-09-06 ~ 13/17 meters metered 11.93 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:19 ~1:27 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80353,9 +80353,36 @@
       <c r="A2442" s="4" t="n">
         <v>46271</v>
       </c>
+      <c r="B2442" t="n">
+        <v>3.177</v>
+      </c>
+      <c r="C2442" t="n">
+        <v>2.859</v>
+      </c>
+      <c r="D2442" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="E2442" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="F2442" t="n">
+        <v>2.586</v>
+      </c>
+      <c r="G2442" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="H2442" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2442" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="K2442" t="n">
+        <v>11.931</v>
+      </c>
       <c r="L2442" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81156,7 +81183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81221,22 +81248,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B2" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C2" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D2" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E2" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F2" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G2" t="n">
         <v>0.437</v>
@@ -81248,178 +81275,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B3" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C3" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D3" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E3" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F3" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G3" t="n">
         <v>0.437</v>
       </c>
       <c r="H3" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I3" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B4" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C4" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D4" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E4" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F4" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G4" t="n">
         <v>0.437</v>
       </c>
       <c r="H4" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I4" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B5" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C5" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D5" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F5" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G5" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K5" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B6" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C6" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D6" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E6" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F6" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G6" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B7" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C7" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D7" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E7" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F7" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G7" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K7" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B8" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C8" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D8" t="n">
         <v>1.44</v>
@@ -81428,7 +81455,7 @@
         <v>0.261</v>
       </c>
       <c r="F8" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G8" t="n">
         <v>0.435</v>
@@ -81437,222 +81464,222 @@
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K8" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B9" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C9" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D9" t="n">
         <v>1.44</v>
       </c>
       <c r="E9" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F9" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G9" t="n">
         <v>0.435</v>
       </c>
       <c r="H9" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K9" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B10" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C10" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D10" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E10" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F10" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G10" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H10" t="n">
         <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K10" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B11" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C11" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D11" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F11" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G11" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H11" t="n">
         <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K11" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B12" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C12" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D12" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E12" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G12" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H12" t="n">
         <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K12" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B13" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C13" t="n">
         <v>3.232</v>
       </c>
       <c r="D13" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E13" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F13" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G13" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H13" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K13" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B14" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C14" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D14" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E14" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G14" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H14" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I14" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K14" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B15" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C15" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D15" t="n">
         <v>1.435</v>
       </c>
       <c r="E15" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F15" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G15" t="n">
         <v>0.446</v>
@@ -81664,27 +81691,27 @@
         <v>0.712</v>
       </c>
       <c r="K15" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B16" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C16" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D16" t="n">
         <v>1.435</v>
       </c>
       <c r="E16" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F16" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G16" t="n">
         <v>0.446</v>
@@ -81696,59 +81723,59 @@
         <v>0.712</v>
       </c>
       <c r="K16" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B17" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C17" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D17" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E17" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F17" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G17" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H17" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I17" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K17" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B18" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C18" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D18" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E18" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F18" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G18" t="n">
         <v>0.462</v>
@@ -81757,30 +81784,30 @@
         <v>0.343</v>
       </c>
       <c r="I18" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K18" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B19" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C19" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D19" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E19" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F19" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G19" t="n">
         <v>0.462</v>
@@ -81789,100 +81816,97 @@
         <v>0.343</v>
       </c>
       <c r="I19" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K19" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B20" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C20" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D20" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E20" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F20" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G20" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H20" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I20" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K20" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B21" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C21" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D21" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E21" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F21" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G21" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H21" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I21" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J21" t="n">
         <v>0.014</v>
       </c>
       <c r="K21" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B22" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C22" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D22" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F22" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G22" t="n">
         <v>0.395</v>
@@ -81897,6 +81921,41 @@
         <v>0.014</v>
       </c>
       <c r="K22" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B23" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K23" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81911,7 +81970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81981,22 +82040,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B2" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C2" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D2" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E2" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F2" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G2" t="n">
         <v>0.437</v>
@@ -82008,196 +82067,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L2" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B3" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C3" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D3" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E3" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F3" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G3" t="n">
         <v>0.437</v>
       </c>
       <c r="H3" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I3" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L3" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B4" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C4" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D4" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E4" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F4" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G4" t="n">
         <v>0.437</v>
       </c>
       <c r="H4" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I4" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L4" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B5" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C5" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D5" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F5" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G5" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K5" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L5" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B6" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C6" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D6" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E6" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F6" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G6" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L6" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B7" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C7" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D7" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E7" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F7" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G7" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K7" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L7" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B8" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C8" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D8" t="n">
         <v>1.44</v>
@@ -82206,7 +82265,7 @@
         <v>0.261</v>
       </c>
       <c r="F8" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G8" t="n">
         <v>0.435</v>
@@ -82215,243 +82274,243 @@
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K8" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L8" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B9" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C9" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D9" t="n">
         <v>1.44</v>
       </c>
       <c r="E9" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F9" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G9" t="n">
         <v>0.435</v>
       </c>
       <c r="H9" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K9" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L9" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B10" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C10" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D10" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E10" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F10" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G10" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H10" t="n">
         <v>0.365</v>
       </c>
       <c r="I10" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K10" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L10" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B11" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C11" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D11" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F11" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G11" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H11" t="n">
         <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K11" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L11" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B12" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C12" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D12" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E12" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G12" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H12" t="n">
         <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K12" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L12" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B13" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C13" t="n">
         <v>3.232</v>
       </c>
       <c r="D13" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E13" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F13" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G13" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H13" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K13" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L13" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B14" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C14" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D14" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E14" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G14" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H14" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I14" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K14" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L14" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B15" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C15" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D15" t="n">
         <v>1.435</v>
       </c>
       <c r="E15" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F15" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G15" t="n">
         <v>0.446</v>
@@ -82463,30 +82522,30 @@
         <v>0.712</v>
       </c>
       <c r="K15" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L15" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B16" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C16" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D16" t="n">
         <v>1.435</v>
       </c>
       <c r="E16" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F16" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G16" t="n">
         <v>0.446</v>
@@ -82498,65 +82557,65 @@
         <v>0.712</v>
       </c>
       <c r="K16" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L16" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B17" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C17" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D17" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E17" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F17" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G17" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H17" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I17" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K17" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L17" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B18" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C18" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D18" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E18" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F18" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G18" t="n">
         <v>0.462</v>
@@ -82565,33 +82624,33 @@
         <v>0.343</v>
       </c>
       <c r="I18" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K18" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L18" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B19" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C19" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D19" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E19" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F19" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G19" t="n">
         <v>0.462</v>
@@ -82600,109 +82659,106 @@
         <v>0.343</v>
       </c>
       <c r="I19" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K19" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L19" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B20" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C20" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D20" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E20" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F20" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G20" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H20" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I20" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K20" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L20" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B21" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C21" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D21" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E21" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F21" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G21" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H21" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I21" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J21" t="n">
         <v>0.014</v>
       </c>
       <c r="K21" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L21" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B22" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C22" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D22" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F22" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G22" t="n">
         <v>0.395</v>
@@ -82717,9 +82773,47 @@
         <v>0.014</v>
       </c>
       <c r="K22" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L22" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B23" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K23" t="n">
         <v>12.277</v>
       </c>
-      <c r="L22" t="n">
+      <c r="L23" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83160,7 +83254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83260,34 +83354,34 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B2" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C2" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D2" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G2" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I2" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K2" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M2" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
@@ -83296,7 +83390,7 @@
         <v>238857</v>
       </c>
       <c r="P2" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q2" t="n">
         <v>710782</v>
@@ -83304,43 +83398,43 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B3" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C3" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D3" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G3" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I3" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K3" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M3" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N3" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P3" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q3" t="n">
         <v>710782</v>
@@ -83348,201 +83442,201 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B4" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C4" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D4" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G4" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I4" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K4" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M4" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N4" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O4" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P4" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q4" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B5" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C5" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D5" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G5" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I5" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K5" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M5" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N5" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O5" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P5" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q5" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B6" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C6" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D6" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G6" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I6" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K6" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M6" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N6" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P6" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q6" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B7" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C7" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D7" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E7" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G7" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I7" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K7" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M7" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N7" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O7" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P7" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q7" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B8" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C8" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D8" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E8" t="n">
         <v>9400</v>
       </c>
       <c r="F8" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G8" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I8" t="n">
         <v>1493578</v>
@@ -83551,7 +83645,7 @@
         <v>270165</v>
       </c>
       <c r="M8" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
@@ -83563,39 +83657,39 @@
         <v>380581</v>
       </c>
       <c r="Q8" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B9" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C9" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D9" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E9" t="n">
         <v>9400</v>
       </c>
       <c r="F9" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G9" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I9" t="n">
         <v>1493578</v>
       </c>
       <c r="K9" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M9" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
@@ -83604,153 +83698,153 @@
         <v>236857</v>
       </c>
       <c r="P9" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q9" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B10" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C10" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D10" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E10" t="n">
         <v>9400</v>
       </c>
       <c r="F10" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G10" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I10" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K10" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M10" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N10" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P10" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q10" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B11" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C11" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D11" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E11" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F11" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G11" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I11" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K11" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M11" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N11" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O11" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P11" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q11" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B12" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C12" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D12" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G12" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I12" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K12" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M12" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N12" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P12" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q12" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B13" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C13" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D13" t="n">
         <v>1438502</v>
@@ -83759,107 +83853,107 @@
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G13" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I13" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K13" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M13" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N13" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O13" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P13" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q13" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B14" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C14" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D14" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G14" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I14" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K14" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M14" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N14" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O14" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P14" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q14" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B15" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C15" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D15" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G15" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I15" t="n">
         <v>1488515</v>
       </c>
       <c r="K15" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M15" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
@@ -83868,7 +83962,7 @@
         <v>247857</v>
       </c>
       <c r="P15" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q15" t="n">
         <v>738429</v>
@@ -83876,34 +83970,34 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B16" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C16" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D16" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E16" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G16" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I16" t="n">
         <v>1488515</v>
       </c>
       <c r="K16" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M16" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N16" t="n">
         <v>214475</v>
@@ -83912,7 +84006,7 @@
         <v>247857</v>
       </c>
       <c r="P16" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q16" t="n">
         <v>738429</v>
@@ -83920,78 +84014,78 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B17" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C17" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D17" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E17" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F17" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G17" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I17" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K17" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M17" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N17" t="n">
         <v>214475</v>
       </c>
       <c r="O17" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P17" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q17" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B18" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C18" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D18" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E18" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G18" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I18" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K18" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M18" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N18" t="n">
         <v>214475</v>
@@ -84000,42 +84094,42 @@
         <v>264857</v>
       </c>
       <c r="P18" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q18" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B19" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C19" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D19" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E19" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F19" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G19" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I19" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K19" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M19" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N19" t="n">
         <v>214475</v>
@@ -84044,101 +84138,98 @@
         <v>264857</v>
       </c>
       <c r="P19" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q19" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B20" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C20" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D20" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E20" t="n">
         <v>9300</v>
       </c>
       <c r="F20" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G20" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I20" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K20" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M20" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N20" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O20" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P20" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q20" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R20" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B21" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C21" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D21" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E21" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F21" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G21" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I21" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K21" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M21" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N21" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O21" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P21" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q21" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R21" t="n">
         <v>15000</v>
@@ -84146,40 +84237,40 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B22" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C22" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D22" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E22" t="n">
         <v>9100</v>
       </c>
       <c r="F22" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G22" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I22" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K22" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M22" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N22" t="n">
         <v>189475</v>
       </c>
       <c r="O22" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P22" t="n">
         <v>375660</v>
@@ -84188,6 +84279,53 @@
         <v>773586</v>
       </c>
       <c r="R22" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C23" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E23" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K23" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M23" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N23" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O23" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P23" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R23" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -91517,7 +91655,7 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>0.403</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="652">
@@ -91527,7 +91665,7 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>1.376</v>
+        <v>1.381</v>
       </c>
     </row>
     <row r="653">
@@ -91537,7 +91675,7 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.497</v>
+        <v>2.501</v>
       </c>
     </row>
     <row r="654">
@@ -91547,7 +91685,7 @@
         </is>
       </c>
       <c r="D654" t="n">
-        <v>0.359</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="655">
@@ -91557,7 +91695,7 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>0.414</v>
+        <v>0.415</v>
       </c>
     </row>
     <row r="656">
@@ -91567,7 +91705,7 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>0.7</v>
+        <v>0.699</v>
       </c>
     </row>
     <row r="657">
@@ -91577,7 +91715,7 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>3.229</v>
+        <v>3.212</v>
       </c>
     </row>
     <row r="658">
@@ -91587,7 +91725,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.263</v>
+        <v>3.259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feedgas backfill: [ 23/119] 2026-09-05 ~ 13/17 meters metered 12.34 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:20 ~1:27 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80343,9 +80343,36 @@
       <c r="A2441" s="4" t="n">
         <v>46270</v>
       </c>
+      <c r="B2441" t="n">
+        <v>3.391</v>
+      </c>
+      <c r="C2441" t="n">
+        <v>3.261</v>
+      </c>
+      <c r="D2441" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="E2441" t="n">
+        <v>0.297</v>
+      </c>
+      <c r="F2441" t="n">
+        <v>2.592</v>
+      </c>
+      <c r="G2441" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="H2441" t="n">
+        <v>0.367</v>
+      </c>
+      <c r="I2441" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="K2441" t="n">
+        <v>12.341</v>
+      </c>
       <c r="L2441" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81183,7 +81210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81248,25 +81275,25 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B2" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C2" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D2" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E2" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F2" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G2" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
@@ -81275,27 +81302,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B3" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C3" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D3" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E3" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F3" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G3" t="n">
         <v>0.437</v>
@@ -81307,178 +81334,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B4" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C4" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D4" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E4" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F4" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G4" t="n">
         <v>0.437</v>
       </c>
       <c r="H4" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I4" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B5" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C5" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D5" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E5" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F5" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G5" t="n">
         <v>0.437</v>
       </c>
       <c r="H5" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I5" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B6" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C6" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D6" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F6" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G6" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K6" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B7" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C7" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D7" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E7" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F7" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G7" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B8" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C8" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D8" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E8" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F8" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G8" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K8" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B9" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C9" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D9" t="n">
         <v>1.44</v>
@@ -81487,7 +81514,7 @@
         <v>0.261</v>
       </c>
       <c r="F9" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G9" t="n">
         <v>0.435</v>
@@ -81496,222 +81523,222 @@
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K9" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B10" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C10" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D10" t="n">
         <v>1.44</v>
       </c>
       <c r="E10" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F10" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G10" t="n">
         <v>0.435</v>
       </c>
       <c r="H10" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K10" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B11" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C11" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D11" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E11" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F11" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G11" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H11" t="n">
         <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K11" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B12" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C12" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D12" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F12" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G12" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H12" t="n">
         <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K12" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B13" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C13" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D13" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E13" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G13" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H13" t="n">
         <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K13" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B14" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C14" t="n">
         <v>3.232</v>
       </c>
       <c r="D14" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F14" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G14" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H14" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K14" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B15" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C15" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D15" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E15" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G15" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H15" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I15" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K15" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B16" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C16" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D16" t="n">
         <v>1.435</v>
       </c>
       <c r="E16" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F16" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G16" t="n">
         <v>0.446</v>
@@ -81723,27 +81750,27 @@
         <v>0.712</v>
       </c>
       <c r="K16" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B17" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C17" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D17" t="n">
         <v>1.435</v>
       </c>
       <c r="E17" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F17" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G17" t="n">
         <v>0.446</v>
@@ -81755,59 +81782,59 @@
         <v>0.712</v>
       </c>
       <c r="K17" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B18" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C18" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D18" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E18" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F18" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G18" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H18" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I18" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K18" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B19" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C19" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D19" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E19" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F19" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G19" t="n">
         <v>0.462</v>
@@ -81816,30 +81843,30 @@
         <v>0.343</v>
       </c>
       <c r="I19" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K19" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B20" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C20" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D20" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E20" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F20" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G20" t="n">
         <v>0.462</v>
@@ -81848,100 +81875,97 @@
         <v>0.343</v>
       </c>
       <c r="I20" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K20" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B21" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C21" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D21" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E21" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F21" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G21" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H21" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I21" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K21" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B22" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C22" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D22" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E22" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F22" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G22" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H22" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I22" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J22" t="n">
         <v>0.014</v>
       </c>
       <c r="K22" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B23" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C23" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D23" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E23" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F23" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G23" t="n">
         <v>0.395</v>
@@ -81956,6 +81980,41 @@
         <v>0.014</v>
       </c>
       <c r="K23" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K24" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -81970,7 +82029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82040,25 +82099,25 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B2" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C2" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D2" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E2" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F2" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G2" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H2" t="n">
         <v>0.367</v>
@@ -82067,30 +82126,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L2" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B3" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C3" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D3" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E3" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F3" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G3" t="n">
         <v>0.437</v>
@@ -82102,196 +82161,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L3" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B4" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C4" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D4" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E4" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F4" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G4" t="n">
         <v>0.437</v>
       </c>
       <c r="H4" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I4" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L4" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B5" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C5" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D5" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E5" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F5" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G5" t="n">
         <v>0.437</v>
       </c>
       <c r="H5" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I5" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L5" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B6" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C6" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D6" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F6" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G6" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K6" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L6" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B7" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C7" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D7" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E7" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F7" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G7" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L7" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B8" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C8" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D8" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E8" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F8" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G8" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K8" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L8" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B9" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C9" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D9" t="n">
         <v>1.44</v>
@@ -82300,7 +82359,7 @@
         <v>0.261</v>
       </c>
       <c r="F9" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G9" t="n">
         <v>0.435</v>
@@ -82309,243 +82368,243 @@
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K9" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L9" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B10" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C10" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D10" t="n">
         <v>1.44</v>
       </c>
       <c r="E10" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F10" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G10" t="n">
         <v>0.435</v>
       </c>
       <c r="H10" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K10" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L10" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B11" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C11" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D11" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E11" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F11" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G11" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H11" t="n">
         <v>0.365</v>
       </c>
       <c r="I11" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K11" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L11" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B12" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C12" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D12" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F12" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G12" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H12" t="n">
         <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K12" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L12" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B13" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C13" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D13" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E13" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G13" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H13" t="n">
         <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K13" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L13" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B14" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C14" t="n">
         <v>3.232</v>
       </c>
       <c r="D14" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F14" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G14" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H14" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K14" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L14" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B15" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C15" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D15" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E15" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G15" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H15" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I15" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K15" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L15" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B16" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C16" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D16" t="n">
         <v>1.435</v>
       </c>
       <c r="E16" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F16" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G16" t="n">
         <v>0.446</v>
@@ -82557,30 +82616,30 @@
         <v>0.712</v>
       </c>
       <c r="K16" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L16" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B17" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C17" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D17" t="n">
         <v>1.435</v>
       </c>
       <c r="E17" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F17" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G17" t="n">
         <v>0.446</v>
@@ -82592,65 +82651,65 @@
         <v>0.712</v>
       </c>
       <c r="K17" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L17" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B18" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C18" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D18" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E18" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F18" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G18" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H18" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I18" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K18" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L18" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B19" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C19" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D19" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E19" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F19" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G19" t="n">
         <v>0.462</v>
@@ -82659,33 +82718,33 @@
         <v>0.343</v>
       </c>
       <c r="I19" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K19" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L19" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B20" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C20" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D20" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E20" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F20" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G20" t="n">
         <v>0.462</v>
@@ -82694,109 +82753,106 @@
         <v>0.343</v>
       </c>
       <c r="I20" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K20" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L20" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B21" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C21" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D21" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E21" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F21" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G21" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H21" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I21" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K21" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L21" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B22" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C22" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D22" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E22" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F22" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G22" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H22" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I22" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J22" t="n">
         <v>0.014</v>
       </c>
       <c r="K22" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L22" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B23" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C23" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D23" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E23" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F23" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G23" t="n">
         <v>0.395</v>
@@ -82811,9 +82867,47 @@
         <v>0.014</v>
       </c>
       <c r="K23" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L23" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K24" t="n">
         <v>12.277</v>
       </c>
-      <c r="L23" t="n">
+      <c r="L24" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83254,7 +83348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83354,13 +83448,13 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B2" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C2" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D2" t="n">
         <v>1336369</v>
@@ -83369,28 +83463,28 @@
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G2" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I2" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K2" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M2" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N2" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O2" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P2" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q2" t="n">
         <v>710782</v>
@@ -83398,34 +83492,34 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B3" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C3" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D3" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G3" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I3" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K3" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M3" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
@@ -83434,7 +83528,7 @@
         <v>238857</v>
       </c>
       <c r="P3" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q3" t="n">
         <v>710782</v>
@@ -83442,43 +83536,43 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B4" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C4" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D4" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G4" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I4" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K4" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M4" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N4" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P4" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q4" t="n">
         <v>710782</v>
@@ -83486,201 +83580,201 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B5" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C5" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D5" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G5" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I5" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K5" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M5" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N5" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O5" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P5" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q5" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B6" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C6" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D6" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G6" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I6" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K6" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M6" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N6" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O6" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P6" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q6" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B7" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C7" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D7" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G7" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I7" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K7" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M7" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N7" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P7" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q7" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B8" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C8" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D8" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E8" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G8" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I8" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K8" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M8" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N8" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O8" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P8" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q8" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B9" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C9" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D9" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E9" t="n">
         <v>9400</v>
       </c>
       <c r="F9" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G9" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I9" t="n">
         <v>1493578</v>
@@ -83689,7 +83783,7 @@
         <v>270165</v>
       </c>
       <c r="M9" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
@@ -83701,39 +83795,39 @@
         <v>380581</v>
       </c>
       <c r="Q9" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B10" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C10" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D10" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E10" t="n">
         <v>9400</v>
       </c>
       <c r="F10" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G10" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I10" t="n">
         <v>1493578</v>
       </c>
       <c r="K10" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M10" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
@@ -83742,153 +83836,153 @@
         <v>236857</v>
       </c>
       <c r="P10" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q10" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B11" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C11" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D11" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E11" t="n">
         <v>9400</v>
       </c>
       <c r="F11" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G11" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I11" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K11" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M11" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N11" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P11" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q11" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B12" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C12" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D12" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E12" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F12" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G12" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I12" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K12" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M12" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N12" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O12" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P12" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q12" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B13" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C13" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D13" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G13" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I13" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K13" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M13" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N13" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O13" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P13" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q13" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B14" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C14" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D14" t="n">
         <v>1438502</v>
@@ -83897,107 +83991,107 @@
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G14" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I14" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K14" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M14" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N14" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O14" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P14" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q14" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B15" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C15" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D15" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G15" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I15" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K15" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M15" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N15" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O15" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P15" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q15" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B16" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C16" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D16" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E16" t="n">
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G16" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I16" t="n">
         <v>1488515</v>
       </c>
       <c r="K16" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M16" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N16" t="n">
         <v>214475</v>
@@ -84006,7 +84100,7 @@
         <v>247857</v>
       </c>
       <c r="P16" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q16" t="n">
         <v>738429</v>
@@ -84014,34 +84108,34 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B17" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C17" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D17" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E17" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G17" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I17" t="n">
         <v>1488515</v>
       </c>
       <c r="K17" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M17" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N17" t="n">
         <v>214475</v>
@@ -84050,7 +84144,7 @@
         <v>247857</v>
       </c>
       <c r="P17" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q17" t="n">
         <v>738429</v>
@@ -84058,78 +84152,78 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B18" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C18" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D18" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E18" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F18" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G18" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I18" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K18" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M18" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N18" t="n">
         <v>214475</v>
       </c>
       <c r="O18" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P18" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q18" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B19" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C19" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D19" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E19" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G19" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I19" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K19" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M19" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N19" t="n">
         <v>214475</v>
@@ -84138,42 +84232,42 @@
         <v>264857</v>
       </c>
       <c r="P19" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q19" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B20" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C20" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D20" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E20" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F20" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G20" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I20" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K20" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M20" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N20" t="n">
         <v>214475</v>
@@ -84182,101 +84276,98 @@
         <v>264857</v>
       </c>
       <c r="P20" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q20" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B21" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C21" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D21" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E21" t="n">
         <v>9300</v>
       </c>
       <c r="F21" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G21" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I21" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K21" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M21" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N21" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O21" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P21" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q21" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R21" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B22" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C22" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D22" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E22" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F22" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G22" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I22" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K22" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M22" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N22" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O22" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P22" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q22" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R22" t="n">
         <v>15000</v>
@@ -84284,40 +84375,40 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B23" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C23" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D23" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E23" t="n">
         <v>9100</v>
       </c>
       <c r="F23" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G23" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I23" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K23" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M23" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N23" t="n">
         <v>189475</v>
       </c>
       <c r="O23" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P23" t="n">
         <v>375660</v>
@@ -84326,6 +84417,53 @@
         <v>773586</v>
       </c>
       <c r="R23" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C24" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E24" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K24" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M24" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N24" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O24" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P24" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R24" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -91655,7 +91793,7 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>0.4</v>
+        <v>0.395</v>
       </c>
     </row>
     <row r="652">
@@ -91665,7 +91803,7 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>1.381</v>
+        <v>1.385</v>
       </c>
     </row>
     <row r="653">
@@ -91675,7 +91813,7 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.501</v>
+        <v>2.505</v>
       </c>
     </row>
     <row r="654">
@@ -91695,7 +91833,7 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>0.415</v>
+        <v>0.409</v>
       </c>
     </row>
     <row r="656">
@@ -91715,7 +91853,7 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>3.212</v>
+        <v>3.214</v>
       </c>
     </row>
     <row r="658">
@@ -91725,7 +91863,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.259</v>
+        <v>3.264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feedgas backfill: [ 24/119] 2026-09-04 ~ 13/17 meters metered 12.38 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:21 ~1:25 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80333,9 +80333,36 @@
       <c r="A2440" s="4" t="n">
         <v>46269</v>
       </c>
+      <c r="B2440" t="n">
+        <v>3.405</v>
+      </c>
+      <c r="C2440" t="n">
+        <v>3.204</v>
+      </c>
+      <c r="D2440" t="n">
+        <v>1.474</v>
+      </c>
+      <c r="E2440" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="F2440" t="n">
+        <v>2.571</v>
+      </c>
+      <c r="G2440" t="n">
+        <v>0.438</v>
+      </c>
+      <c r="H2440" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="I2440" t="n">
+        <v>0.671</v>
+      </c>
+      <c r="K2440" t="n">
+        <v>12.376</v>
+      </c>
       <c r="L2440" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81210,7 +81237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81275,57 +81302,57 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B2" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C2" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D2" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E2" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F2" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G2" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H2" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K2" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B3" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C3" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D3" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E3" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F3" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G3" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
@@ -81334,27 +81361,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B4" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C4" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D4" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E4" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F4" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G4" t="n">
         <v>0.437</v>
@@ -81366,178 +81393,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B5" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C5" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D5" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E5" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F5" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G5" t="n">
         <v>0.437</v>
       </c>
       <c r="H5" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I5" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B6" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C6" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D6" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E6" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F6" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G6" t="n">
         <v>0.437</v>
       </c>
       <c r="H6" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I6" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B7" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C7" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D7" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F7" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G7" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K7" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B8" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C8" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D8" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E8" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F8" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G8" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B9" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C9" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D9" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E9" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F9" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G9" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K9" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B10" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C10" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D10" t="n">
         <v>1.44</v>
@@ -81546,7 +81573,7 @@
         <v>0.261</v>
       </c>
       <c r="F10" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G10" t="n">
         <v>0.435</v>
@@ -81555,222 +81582,222 @@
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K10" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B11" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C11" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D11" t="n">
         <v>1.44</v>
       </c>
       <c r="E11" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F11" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G11" t="n">
         <v>0.435</v>
       </c>
       <c r="H11" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K11" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B12" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C12" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D12" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E12" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F12" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G12" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H12" t="n">
         <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K12" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B13" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C13" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D13" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F13" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G13" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H13" t="n">
         <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K13" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B14" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C14" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D14" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E14" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G14" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H14" t="n">
         <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K14" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B15" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C15" t="n">
         <v>3.232</v>
       </c>
       <c r="D15" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F15" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G15" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H15" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K15" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B16" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C16" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D16" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E16" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G16" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H16" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I16" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K16" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B17" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C17" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D17" t="n">
         <v>1.435</v>
       </c>
       <c r="E17" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F17" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G17" t="n">
         <v>0.446</v>
@@ -81782,27 +81809,27 @@
         <v>0.712</v>
       </c>
       <c r="K17" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B18" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C18" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D18" t="n">
         <v>1.435</v>
       </c>
       <c r="E18" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F18" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G18" t="n">
         <v>0.446</v>
@@ -81814,59 +81841,59 @@
         <v>0.712</v>
       </c>
       <c r="K18" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B19" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C19" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D19" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E19" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F19" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G19" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H19" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I19" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K19" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B20" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C20" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D20" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E20" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F20" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G20" t="n">
         <v>0.462</v>
@@ -81875,30 +81902,30 @@
         <v>0.343</v>
       </c>
       <c r="I20" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K20" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B21" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C21" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D21" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E21" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F21" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G21" t="n">
         <v>0.462</v>
@@ -81907,100 +81934,97 @@
         <v>0.343</v>
       </c>
       <c r="I21" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K21" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B22" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C22" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D22" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E22" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F22" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G22" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H22" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I22" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K22" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B23" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C23" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D23" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E23" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F23" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G23" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H23" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I23" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J23" t="n">
         <v>0.014</v>
       </c>
       <c r="K23" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B24" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C24" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D24" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E24" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F24" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G24" t="n">
         <v>0.395</v>
@@ -82015,6 +82039,41 @@
         <v>0.014</v>
       </c>
       <c r="K24" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B25" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K25" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82029,7 +82088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82099,60 +82158,60 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B2" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C2" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D2" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E2" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F2" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G2" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H2" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K2" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L2" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B3" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C3" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D3" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E3" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F3" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G3" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H3" t="n">
         <v>0.367</v>
@@ -82161,30 +82220,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L3" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B4" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C4" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D4" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E4" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F4" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G4" t="n">
         <v>0.437</v>
@@ -82196,196 +82255,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L4" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B5" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C5" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D5" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E5" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F5" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G5" t="n">
         <v>0.437</v>
       </c>
       <c r="H5" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I5" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L5" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B6" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C6" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D6" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E6" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F6" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G6" t="n">
         <v>0.437</v>
       </c>
       <c r="H6" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I6" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L6" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B7" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C7" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D7" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F7" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G7" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K7" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L7" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B8" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C8" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D8" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E8" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F8" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G8" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L8" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B9" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C9" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D9" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E9" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F9" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G9" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K9" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L9" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B10" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C10" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D10" t="n">
         <v>1.44</v>
@@ -82394,7 +82453,7 @@
         <v>0.261</v>
       </c>
       <c r="F10" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G10" t="n">
         <v>0.435</v>
@@ -82403,243 +82462,243 @@
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K10" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L10" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B11" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C11" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D11" t="n">
         <v>1.44</v>
       </c>
       <c r="E11" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F11" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G11" t="n">
         <v>0.435</v>
       </c>
       <c r="H11" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K11" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L11" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B12" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C12" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D12" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E12" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F12" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G12" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H12" t="n">
         <v>0.365</v>
       </c>
       <c r="I12" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K12" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L12" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B13" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C13" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D13" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F13" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G13" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H13" t="n">
         <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K13" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L13" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B14" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C14" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D14" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E14" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G14" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H14" t="n">
         <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K14" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L14" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B15" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C15" t="n">
         <v>3.232</v>
       </c>
       <c r="D15" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F15" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G15" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H15" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K15" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L15" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B16" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C16" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D16" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E16" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G16" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H16" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I16" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K16" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L16" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B17" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C17" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D17" t="n">
         <v>1.435</v>
       </c>
       <c r="E17" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F17" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G17" t="n">
         <v>0.446</v>
@@ -82651,30 +82710,30 @@
         <v>0.712</v>
       </c>
       <c r="K17" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L17" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B18" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C18" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D18" t="n">
         <v>1.435</v>
       </c>
       <c r="E18" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F18" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G18" t="n">
         <v>0.446</v>
@@ -82686,65 +82745,65 @@
         <v>0.712</v>
       </c>
       <c r="K18" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L18" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B19" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C19" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D19" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E19" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F19" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G19" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H19" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I19" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K19" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L19" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B20" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C20" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D20" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E20" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F20" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G20" t="n">
         <v>0.462</v>
@@ -82753,33 +82812,33 @@
         <v>0.343</v>
       </c>
       <c r="I20" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K20" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L20" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B21" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C21" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D21" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E21" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F21" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G21" t="n">
         <v>0.462</v>
@@ -82788,109 +82847,106 @@
         <v>0.343</v>
       </c>
       <c r="I21" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K21" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L21" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B22" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C22" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D22" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E22" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F22" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G22" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H22" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I22" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K22" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L22" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B23" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C23" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D23" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E23" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F23" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G23" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H23" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I23" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J23" t="n">
         <v>0.014</v>
       </c>
       <c r="K23" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L23" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B24" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C24" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D24" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E24" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F24" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G24" t="n">
         <v>0.395</v>
@@ -82905,9 +82961,47 @@
         <v>0.014</v>
       </c>
       <c r="K24" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L24" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B25" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K25" t="n">
         <v>12.277</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L25" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83348,7 +83442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83448,57 +83542,57 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B2" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C2" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D2" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G2" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I2" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K2" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M2" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N2" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P2" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q2" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B3" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C3" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D3" t="n">
         <v>1336369</v>
@@ -83507,28 +83601,28 @@
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G3" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I3" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K3" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M3" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N3" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O3" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P3" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q3" t="n">
         <v>710782</v>
@@ -83536,34 +83630,34 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B4" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C4" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D4" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G4" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I4" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K4" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M4" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
@@ -83572,7 +83666,7 @@
         <v>238857</v>
       </c>
       <c r="P4" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q4" t="n">
         <v>710782</v>
@@ -83580,43 +83674,43 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B5" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C5" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D5" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G5" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I5" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K5" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M5" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N5" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P5" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q5" t="n">
         <v>710782</v>
@@ -83624,201 +83718,201 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B6" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C6" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D6" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G6" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I6" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K6" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M6" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N6" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O6" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P6" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q6" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B7" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C7" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D7" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G7" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I7" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K7" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M7" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N7" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O7" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P7" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q7" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B8" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C8" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D8" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G8" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I8" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K8" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M8" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N8" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P8" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q8" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B9" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C9" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D9" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E9" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G9" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I9" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K9" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M9" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N9" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O9" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P9" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q9" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B10" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C10" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D10" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E10" t="n">
         <v>9400</v>
       </c>
       <c r="F10" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G10" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I10" t="n">
         <v>1493578</v>
@@ -83827,7 +83921,7 @@
         <v>270165</v>
       </c>
       <c r="M10" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
@@ -83839,39 +83933,39 @@
         <v>380581</v>
       </c>
       <c r="Q10" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B11" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C11" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D11" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E11" t="n">
         <v>9400</v>
       </c>
       <c r="F11" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G11" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I11" t="n">
         <v>1493578</v>
       </c>
       <c r="K11" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M11" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
@@ -83880,153 +83974,153 @@
         <v>236857</v>
       </c>
       <c r="P11" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q11" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B12" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C12" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D12" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E12" t="n">
         <v>9400</v>
       </c>
       <c r="F12" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G12" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I12" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K12" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M12" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N12" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P12" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q12" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B13" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C13" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D13" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E13" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F13" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G13" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I13" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K13" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M13" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N13" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O13" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P13" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q13" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B14" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C14" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D14" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G14" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I14" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K14" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M14" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N14" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O14" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P14" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q14" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B15" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C15" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D15" t="n">
         <v>1438502</v>
@@ -84035,107 +84129,107 @@
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G15" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I15" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K15" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M15" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N15" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O15" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P15" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q15" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B16" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C16" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D16" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E16" t="n">
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G16" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I16" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K16" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M16" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N16" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O16" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P16" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q16" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B17" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C17" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D17" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E17" t="n">
         <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G17" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I17" t="n">
         <v>1488515</v>
       </c>
       <c r="K17" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M17" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N17" t="n">
         <v>214475</v>
@@ -84144,7 +84238,7 @@
         <v>247857</v>
       </c>
       <c r="P17" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q17" t="n">
         <v>738429</v>
@@ -84152,34 +84246,34 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B18" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C18" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D18" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E18" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G18" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I18" t="n">
         <v>1488515</v>
       </c>
       <c r="K18" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M18" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N18" t="n">
         <v>214475</v>
@@ -84188,7 +84282,7 @@
         <v>247857</v>
       </c>
       <c r="P18" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q18" t="n">
         <v>738429</v>
@@ -84196,78 +84290,78 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B19" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C19" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D19" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E19" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F19" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G19" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I19" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K19" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M19" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N19" t="n">
         <v>214475</v>
       </c>
       <c r="O19" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P19" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q19" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B20" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C20" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D20" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E20" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F20" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G20" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I20" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K20" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M20" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N20" t="n">
         <v>214475</v>
@@ -84276,42 +84370,42 @@
         <v>264857</v>
       </c>
       <c r="P20" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q20" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B21" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C21" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D21" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E21" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F21" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G21" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I21" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K21" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M21" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N21" t="n">
         <v>214475</v>
@@ -84320,101 +84414,98 @@
         <v>264857</v>
       </c>
       <c r="P21" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q21" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B22" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C22" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D22" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E22" t="n">
         <v>9300</v>
       </c>
       <c r="F22" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G22" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I22" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K22" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M22" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N22" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O22" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P22" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q22" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R22" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B23" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C23" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D23" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E23" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F23" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G23" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I23" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K23" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M23" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N23" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O23" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P23" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q23" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R23" t="n">
         <v>15000</v>
@@ -84422,40 +84513,40 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B24" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C24" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D24" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E24" t="n">
         <v>9100</v>
       </c>
       <c r="F24" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G24" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I24" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K24" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M24" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N24" t="n">
         <v>189475</v>
       </c>
       <c r="O24" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P24" t="n">
         <v>375660</v>
@@ -84464,6 +84555,53 @@
         <v>773586</v>
       </c>
       <c r="R24" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C25" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E25" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K25" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M25" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N25" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O25" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P25" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R25" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -91793,7 +91931,7 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>0.395</v>
+        <v>0.389</v>
       </c>
     </row>
     <row r="652">
@@ -91803,7 +91941,7 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>1.385</v>
+        <v>1.389</v>
       </c>
     </row>
     <row r="653">
@@ -91813,7 +91951,7 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.505</v>
+        <v>2.507</v>
       </c>
     </row>
     <row r="654">
@@ -91833,7 +91971,7 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>0.409</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="656">
@@ -91843,7 +91981,7 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>0.699</v>
+        <v>0.698</v>
       </c>
     </row>
     <row r="657">
@@ -91863,7 +92001,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.264</v>
+        <v>3.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feedgas backfill: [ 25/119] 2026-09-03 ~ 13/17 meters metered 11.79 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:22 ~1:24 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80323,9 +80323,36 @@
       <c r="A2439" s="4" t="n">
         <v>46268</v>
       </c>
+      <c r="B2439" t="n">
+        <v>3.062</v>
+      </c>
+      <c r="C2439" t="n">
+        <v>3.142</v>
+      </c>
+      <c r="D2439" t="n">
+        <v>1.386</v>
+      </c>
+      <c r="E2439" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="F2439" t="n">
+        <v>2.581</v>
+      </c>
+      <c r="G2439" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="H2439" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="I2439" t="n">
+        <v>0.647</v>
+      </c>
+      <c r="K2439" t="n">
+        <v>11.787</v>
+      </c>
       <c r="L2439" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81237,7 +81264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81302,89 +81329,89 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B2" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C2" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D2" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E2" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F2" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G2" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H2" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I2" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K2" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B3" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C3" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D3" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E3" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F3" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G3" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H3" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K3" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B4" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C4" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D4" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E4" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F4" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G4" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
@@ -81393,27 +81420,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B5" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C5" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D5" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E5" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F5" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G5" t="n">
         <v>0.437</v>
@@ -81425,178 +81452,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B6" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C6" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D6" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E6" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F6" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G6" t="n">
         <v>0.437</v>
       </c>
       <c r="H6" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I6" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B7" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C7" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D7" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E7" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F7" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G7" t="n">
         <v>0.437</v>
       </c>
       <c r="H7" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I7" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B8" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C8" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D8" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F8" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G8" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K8" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B9" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C9" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D9" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E9" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F9" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G9" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B10" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C10" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D10" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E10" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F10" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G10" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K10" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B11" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C11" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D11" t="n">
         <v>1.44</v>
@@ -81605,7 +81632,7 @@
         <v>0.261</v>
       </c>
       <c r="F11" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G11" t="n">
         <v>0.435</v>
@@ -81614,222 +81641,222 @@
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K11" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B12" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C12" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D12" t="n">
         <v>1.44</v>
       </c>
       <c r="E12" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F12" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G12" t="n">
         <v>0.435</v>
       </c>
       <c r="H12" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K12" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B13" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C13" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D13" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E13" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F13" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G13" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H13" t="n">
         <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K13" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B14" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C14" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D14" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F14" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G14" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H14" t="n">
         <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K14" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B15" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C15" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D15" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E15" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G15" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H15" t="n">
         <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K15" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B16" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C16" t="n">
         <v>3.232</v>
       </c>
       <c r="D16" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F16" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G16" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H16" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K16" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B17" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C17" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D17" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E17" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G17" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H17" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I17" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K17" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B18" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C18" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D18" t="n">
         <v>1.435</v>
       </c>
       <c r="E18" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F18" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G18" t="n">
         <v>0.446</v>
@@ -81841,27 +81868,27 @@
         <v>0.712</v>
       </c>
       <c r="K18" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B19" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C19" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D19" t="n">
         <v>1.435</v>
       </c>
       <c r="E19" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F19" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G19" t="n">
         <v>0.446</v>
@@ -81873,59 +81900,59 @@
         <v>0.712</v>
       </c>
       <c r="K19" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B20" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C20" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D20" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E20" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F20" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G20" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H20" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I20" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K20" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B21" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C21" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D21" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E21" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F21" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G21" t="n">
         <v>0.462</v>
@@ -81934,30 +81961,30 @@
         <v>0.343</v>
       </c>
       <c r="I21" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K21" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B22" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C22" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D22" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E22" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F22" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G22" t="n">
         <v>0.462</v>
@@ -81966,100 +81993,97 @@
         <v>0.343</v>
       </c>
       <c r="I22" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K22" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B23" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C23" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D23" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E23" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F23" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G23" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H23" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I23" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K23" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B24" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C24" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D24" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E24" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F24" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G24" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H24" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I24" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J24" t="n">
         <v>0.014</v>
       </c>
       <c r="K24" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B25" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C25" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D25" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E25" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F25" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G25" t="n">
         <v>0.395</v>
@@ -82074,6 +82098,41 @@
         <v>0.014</v>
       </c>
       <c r="K25" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B26" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K26" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82088,7 +82147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82158,95 +82217,95 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B2" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C2" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D2" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E2" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F2" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G2" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H2" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I2" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K2" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L2" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B3" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C3" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D3" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E3" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F3" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G3" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H3" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K3" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L3" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B4" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C4" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D4" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E4" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F4" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G4" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H4" t="n">
         <v>0.367</v>
@@ -82255,30 +82314,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L4" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B5" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C5" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D5" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E5" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F5" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G5" t="n">
         <v>0.437</v>
@@ -82290,196 +82349,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L5" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B6" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C6" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D6" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E6" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F6" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G6" t="n">
         <v>0.437</v>
       </c>
       <c r="H6" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I6" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L6" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B7" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C7" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D7" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E7" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F7" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G7" t="n">
         <v>0.437</v>
       </c>
       <c r="H7" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I7" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L7" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B8" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C8" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D8" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F8" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G8" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K8" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L8" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B9" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C9" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D9" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E9" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F9" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G9" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L9" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B10" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C10" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D10" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E10" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F10" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G10" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K10" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L10" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B11" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C11" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D11" t="n">
         <v>1.44</v>
@@ -82488,7 +82547,7 @@
         <v>0.261</v>
       </c>
       <c r="F11" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G11" t="n">
         <v>0.435</v>
@@ -82497,243 +82556,243 @@
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K11" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L11" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B12" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C12" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D12" t="n">
         <v>1.44</v>
       </c>
       <c r="E12" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F12" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G12" t="n">
         <v>0.435</v>
       </c>
       <c r="H12" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K12" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L12" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B13" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C13" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D13" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E13" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F13" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G13" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H13" t="n">
         <v>0.365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K13" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L13" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B14" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C14" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D14" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E14" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F14" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G14" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H14" t="n">
         <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K14" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L14" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B15" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C15" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D15" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E15" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G15" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H15" t="n">
         <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K15" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L15" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B16" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C16" t="n">
         <v>3.232</v>
       </c>
       <c r="D16" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F16" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G16" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H16" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K16" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L16" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B17" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C17" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D17" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E17" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G17" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H17" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I17" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K17" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L17" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B18" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C18" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D18" t="n">
         <v>1.435</v>
       </c>
       <c r="E18" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F18" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G18" t="n">
         <v>0.446</v>
@@ -82745,30 +82804,30 @@
         <v>0.712</v>
       </c>
       <c r="K18" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L18" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B19" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C19" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D19" t="n">
         <v>1.435</v>
       </c>
       <c r="E19" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F19" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G19" t="n">
         <v>0.446</v>
@@ -82780,65 +82839,65 @@
         <v>0.712</v>
       </c>
       <c r="K19" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L19" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B20" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C20" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D20" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E20" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F20" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G20" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H20" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I20" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K20" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L20" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B21" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C21" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D21" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E21" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F21" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G21" t="n">
         <v>0.462</v>
@@ -82847,33 +82906,33 @@
         <v>0.343</v>
       </c>
       <c r="I21" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K21" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L21" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B22" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C22" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D22" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E22" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F22" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G22" t="n">
         <v>0.462</v>
@@ -82882,109 +82941,106 @@
         <v>0.343</v>
       </c>
       <c r="I22" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K22" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L22" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B23" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C23" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D23" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E23" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F23" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G23" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H23" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I23" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K23" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L23" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B24" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C24" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D24" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E24" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F24" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G24" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H24" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I24" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J24" t="n">
         <v>0.014</v>
       </c>
       <c r="K24" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L24" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B25" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C25" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D25" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E25" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F25" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G25" t="n">
         <v>0.395</v>
@@ -82999,9 +83055,47 @@
         <v>0.014</v>
       </c>
       <c r="K25" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L25" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B26" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K26" t="n">
         <v>12.277</v>
       </c>
-      <c r="L25" t="n">
+      <c r="L26" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83442,7 +83536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83542,101 +83636,101 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B2" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C2" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D2" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E2" t="n">
         <v>9200</v>
       </c>
       <c r="F2" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G2" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I2" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K2" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M2" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P2" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q2" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B3" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C3" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D3" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G3" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I3" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K3" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M3" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N3" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P3" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q3" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B4" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C4" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D4" t="n">
         <v>1336369</v>
@@ -83645,28 +83739,28 @@
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G4" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I4" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K4" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M4" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N4" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O4" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P4" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q4" t="n">
         <v>710782</v>
@@ -83674,34 +83768,34 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B5" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C5" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D5" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G5" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I5" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K5" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M5" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
@@ -83710,7 +83804,7 @@
         <v>238857</v>
       </c>
       <c r="P5" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q5" t="n">
         <v>710782</v>
@@ -83718,43 +83812,43 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B6" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C6" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D6" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G6" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I6" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K6" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M6" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N6" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P6" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q6" t="n">
         <v>710782</v>
@@ -83762,201 +83856,201 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B7" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C7" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D7" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G7" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I7" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K7" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M7" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N7" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O7" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P7" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q7" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B8" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C8" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D8" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G8" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I8" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K8" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M8" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N8" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O8" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P8" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q8" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B9" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C9" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D9" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G9" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I9" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K9" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M9" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N9" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P9" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q9" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B10" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C10" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D10" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E10" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G10" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I10" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K10" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M10" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N10" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O10" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P10" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q10" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B11" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C11" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D11" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E11" t="n">
         <v>9400</v>
       </c>
       <c r="F11" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G11" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I11" t="n">
         <v>1493578</v>
@@ -83965,7 +84059,7 @@
         <v>270165</v>
       </c>
       <c r="M11" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
@@ -83977,39 +84071,39 @@
         <v>380581</v>
       </c>
       <c r="Q11" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B12" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C12" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D12" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E12" t="n">
         <v>9400</v>
       </c>
       <c r="F12" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G12" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I12" t="n">
         <v>1493578</v>
       </c>
       <c r="K12" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M12" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
@@ -84018,153 +84112,153 @@
         <v>236857</v>
       </c>
       <c r="P12" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q12" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B13" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C13" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D13" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E13" t="n">
         <v>9400</v>
       </c>
       <c r="F13" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G13" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I13" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K13" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M13" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N13" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O13" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P13" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q13" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B14" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C14" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D14" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E14" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F14" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G14" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I14" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K14" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M14" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N14" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O14" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P14" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q14" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B15" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C15" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D15" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G15" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I15" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K15" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M15" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N15" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O15" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P15" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q15" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B16" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C16" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D16" t="n">
         <v>1438502</v>
@@ -84173,107 +84267,107 @@
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G16" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I16" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K16" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M16" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N16" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O16" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P16" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q16" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B17" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C17" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D17" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E17" t="n">
         <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G17" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I17" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K17" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M17" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N17" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O17" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P17" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q17" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B18" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C18" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D18" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E18" t="n">
         <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G18" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I18" t="n">
         <v>1488515</v>
       </c>
       <c r="K18" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M18" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N18" t="n">
         <v>214475</v>
@@ -84282,7 +84376,7 @@
         <v>247857</v>
       </c>
       <c r="P18" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q18" t="n">
         <v>738429</v>
@@ -84290,34 +84384,34 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B19" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C19" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D19" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E19" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G19" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I19" t="n">
         <v>1488515</v>
       </c>
       <c r="K19" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M19" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N19" t="n">
         <v>214475</v>
@@ -84326,7 +84420,7 @@
         <v>247857</v>
       </c>
       <c r="P19" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q19" t="n">
         <v>738429</v>
@@ -84334,78 +84428,78 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B20" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C20" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D20" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E20" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F20" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G20" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I20" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K20" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M20" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N20" t="n">
         <v>214475</v>
       </c>
       <c r="O20" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P20" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q20" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B21" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C21" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D21" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E21" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F21" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G21" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I21" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K21" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M21" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N21" t="n">
         <v>214475</v>
@@ -84414,42 +84508,42 @@
         <v>264857</v>
       </c>
       <c r="P21" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q21" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B22" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C22" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D22" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E22" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F22" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G22" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I22" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K22" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M22" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N22" t="n">
         <v>214475</v>
@@ -84458,101 +84552,98 @@
         <v>264857</v>
       </c>
       <c r="P22" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q22" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B23" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C23" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D23" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E23" t="n">
         <v>9300</v>
       </c>
       <c r="F23" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G23" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I23" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K23" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M23" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N23" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O23" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P23" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q23" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R23" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B24" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C24" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D24" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E24" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F24" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G24" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I24" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K24" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M24" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N24" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O24" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P24" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q24" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R24" t="n">
         <v>15000</v>
@@ -84560,40 +84651,40 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B25" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C25" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D25" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E25" t="n">
         <v>9100</v>
       </c>
       <c r="F25" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G25" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I25" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K25" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M25" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N25" t="n">
         <v>189475</v>
       </c>
       <c r="O25" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P25" t="n">
         <v>375660</v>
@@ -84602,6 +84693,53 @@
         <v>773586</v>
       </c>
       <c r="R25" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C26" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E26" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K26" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M26" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N26" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O26" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P26" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R26" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -91931,7 +92069,7 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>0.389</v>
+        <v>0.382</v>
       </c>
     </row>
     <row r="652">
@@ -91951,7 +92089,7 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.507</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="654">
@@ -91961,7 +92099,7 @@
         </is>
       </c>
       <c r="D654" t="n">
-        <v>0.36</v>
+        <v>0.359</v>
       </c>
     </row>
     <row r="655">
@@ -91971,7 +92109,7 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>0.41</v>
+        <v>0.411</v>
       </c>
     </row>
     <row r="656">
@@ -91981,7 +92119,7 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>0.698</v>
+        <v>0.696</v>
       </c>
     </row>
     <row r="657">
@@ -91991,7 +92129,7 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>3.214</v>
+        <v>3.211</v>
       </c>
     </row>
     <row r="658">
@@ -92001,7 +92139,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.27</v>
+        <v>3.262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feedgas backfill: [ 26/119] 2026-09-02 ~ 13/17 meters metered 11.34 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:23 ~1:23 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80313,9 +80313,36 @@
       <c r="A2438" s="4" t="n">
         <v>46267</v>
       </c>
+      <c r="B2438" t="n">
+        <v>2.659</v>
+      </c>
+      <c r="C2438" t="n">
+        <v>3.117</v>
+      </c>
+      <c r="D2438" t="n">
+        <v>1.454</v>
+      </c>
+      <c r="E2438" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="F2438" t="n">
+        <v>2.632</v>
+      </c>
+      <c r="G2438" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="H2438" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="I2438" t="n">
+        <v>0.491</v>
+      </c>
+      <c r="K2438" t="n">
+        <v>11.345</v>
+      </c>
       <c r="L2438" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81264,7 +81291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81329,121 +81356,121 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B2" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C2" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D2" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E2" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F2" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G2" t="n">
         <v>0.444</v>
       </c>
       <c r="H2" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I2" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K2" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B3" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C3" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D3" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E3" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F3" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G3" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H3" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I3" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K3" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B4" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C4" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D4" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E4" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F4" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G4" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H4" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K4" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B5" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C5" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D5" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E5" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F5" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G5" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
@@ -81452,27 +81479,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B6" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C6" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D6" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E6" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F6" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G6" t="n">
         <v>0.437</v>
@@ -81484,178 +81511,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B7" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C7" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D7" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E7" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F7" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G7" t="n">
         <v>0.437</v>
       </c>
       <c r="H7" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I7" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B8" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C8" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D8" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E8" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F8" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G8" t="n">
         <v>0.437</v>
       </c>
       <c r="H8" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I8" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B9" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C9" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D9" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F9" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G9" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K9" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B10" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C10" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D10" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E10" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F10" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G10" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B11" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C11" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D11" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E11" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F11" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G11" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K11" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B12" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C12" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D12" t="n">
         <v>1.44</v>
@@ -81664,7 +81691,7 @@
         <v>0.261</v>
       </c>
       <c r="F12" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G12" t="n">
         <v>0.435</v>
@@ -81673,222 +81700,222 @@
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K12" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B13" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C13" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D13" t="n">
         <v>1.44</v>
       </c>
       <c r="E13" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F13" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G13" t="n">
         <v>0.435</v>
       </c>
       <c r="H13" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K13" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B14" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C14" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D14" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E14" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F14" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G14" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H14" t="n">
         <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K14" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B15" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C15" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D15" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F15" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G15" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H15" t="n">
         <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K15" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B16" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C16" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D16" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E16" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G16" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H16" t="n">
         <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K16" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B17" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C17" t="n">
         <v>3.232</v>
       </c>
       <c r="D17" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F17" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G17" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H17" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K17" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B18" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C18" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D18" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E18" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G18" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H18" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I18" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K18" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B19" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C19" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D19" t="n">
         <v>1.435</v>
       </c>
       <c r="E19" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F19" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G19" t="n">
         <v>0.446</v>
@@ -81900,27 +81927,27 @@
         <v>0.712</v>
       </c>
       <c r="K19" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B20" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C20" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D20" t="n">
         <v>1.435</v>
       </c>
       <c r="E20" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F20" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G20" t="n">
         <v>0.446</v>
@@ -81932,59 +81959,59 @@
         <v>0.712</v>
       </c>
       <c r="K20" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B21" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C21" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D21" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E21" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F21" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G21" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H21" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I21" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K21" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B22" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C22" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D22" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E22" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F22" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G22" t="n">
         <v>0.462</v>
@@ -81993,30 +82020,30 @@
         <v>0.343</v>
       </c>
       <c r="I22" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K22" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B23" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C23" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D23" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E23" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F23" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G23" t="n">
         <v>0.462</v>
@@ -82025,100 +82052,97 @@
         <v>0.343</v>
       </c>
       <c r="I23" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K23" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B24" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C24" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D24" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E24" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F24" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G24" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H24" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I24" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K24" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B25" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C25" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D25" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E25" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F25" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G25" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H25" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I25" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J25" t="n">
         <v>0.014</v>
       </c>
       <c r="K25" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B26" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C26" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D26" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E26" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F26" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G26" t="n">
         <v>0.395</v>
@@ -82133,6 +82157,41 @@
         <v>0.014</v>
       </c>
       <c r="K26" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B27" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K27" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82147,7 +82206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82217,130 +82276,130 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B2" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C2" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D2" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E2" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F2" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G2" t="n">
         <v>0.444</v>
       </c>
       <c r="H2" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I2" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K2" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L2" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B3" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C3" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D3" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E3" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F3" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G3" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H3" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I3" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K3" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L3" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B4" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C4" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D4" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E4" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F4" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G4" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H4" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K4" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L4" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B5" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C5" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D5" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E5" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F5" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G5" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H5" t="n">
         <v>0.367</v>
@@ -82349,30 +82408,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L5" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B6" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C6" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D6" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E6" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F6" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G6" t="n">
         <v>0.437</v>
@@ -82384,196 +82443,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L6" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B7" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C7" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D7" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E7" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F7" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G7" t="n">
         <v>0.437</v>
       </c>
       <c r="H7" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I7" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L7" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B8" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C8" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D8" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E8" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F8" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G8" t="n">
         <v>0.437</v>
       </c>
       <c r="H8" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I8" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L8" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B9" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C9" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D9" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F9" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G9" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K9" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L9" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B10" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C10" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D10" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E10" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F10" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G10" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L10" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B11" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C11" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D11" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E11" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F11" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G11" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K11" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L11" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B12" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C12" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D12" t="n">
         <v>1.44</v>
@@ -82582,7 +82641,7 @@
         <v>0.261</v>
       </c>
       <c r="F12" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G12" t="n">
         <v>0.435</v>
@@ -82591,243 +82650,243 @@
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K12" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L12" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B13" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C13" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D13" t="n">
         <v>1.44</v>
       </c>
       <c r="E13" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F13" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G13" t="n">
         <v>0.435</v>
       </c>
       <c r="H13" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K13" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L13" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B14" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C14" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D14" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E14" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F14" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G14" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H14" t="n">
         <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K14" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L14" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B15" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C15" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D15" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F15" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G15" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H15" t="n">
         <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K15" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L15" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B16" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C16" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D16" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E16" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G16" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H16" t="n">
         <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K16" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L16" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B17" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C17" t="n">
         <v>3.232</v>
       </c>
       <c r="D17" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F17" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G17" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H17" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K17" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L17" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B18" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C18" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D18" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E18" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G18" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H18" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I18" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K18" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L18" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B19" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C19" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D19" t="n">
         <v>1.435</v>
       </c>
       <c r="E19" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F19" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G19" t="n">
         <v>0.446</v>
@@ -82839,30 +82898,30 @@
         <v>0.712</v>
       </c>
       <c r="K19" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L19" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B20" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C20" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D20" t="n">
         <v>1.435</v>
       </c>
       <c r="E20" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F20" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G20" t="n">
         <v>0.446</v>
@@ -82874,65 +82933,65 @@
         <v>0.712</v>
       </c>
       <c r="K20" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L20" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B21" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C21" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D21" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E21" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F21" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G21" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H21" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I21" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K21" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L21" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B22" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C22" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D22" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E22" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F22" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G22" t="n">
         <v>0.462</v>
@@ -82941,33 +83000,33 @@
         <v>0.343</v>
       </c>
       <c r="I22" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K22" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L22" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B23" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C23" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D23" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E23" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F23" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G23" t="n">
         <v>0.462</v>
@@ -82976,109 +83035,106 @@
         <v>0.343</v>
       </c>
       <c r="I23" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K23" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L23" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B24" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C24" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D24" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E24" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F24" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G24" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H24" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I24" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K24" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L24" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B25" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C25" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D25" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E25" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F25" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G25" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H25" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I25" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J25" t="n">
         <v>0.014</v>
       </c>
       <c r="K25" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L25" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B26" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C26" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D26" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E26" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F26" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G26" t="n">
         <v>0.395</v>
@@ -83093,9 +83149,47 @@
         <v>0.014</v>
       </c>
       <c r="K26" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L26" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B27" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K27" t="n">
         <v>12.277</v>
       </c>
-      <c r="L26" t="n">
+      <c r="L27" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83536,7 +83630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83636,145 +83730,145 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B2" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C2" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D2" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E2" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F2" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G2" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I2" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K2" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M2" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P2" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q2" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B3" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C3" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D3" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E3" t="n">
         <v>9200</v>
       </c>
       <c r="F3" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G3" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I3" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K3" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M3" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P3" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q3" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B4" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C4" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D4" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G4" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I4" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K4" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M4" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N4" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P4" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q4" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B5" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C5" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D5" t="n">
         <v>1336369</v>
@@ -83783,28 +83877,28 @@
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G5" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I5" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K5" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M5" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N5" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O5" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P5" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q5" t="n">
         <v>710782</v>
@@ -83812,34 +83906,34 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B6" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C6" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D6" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G6" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I6" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K6" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M6" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
@@ -83848,7 +83942,7 @@
         <v>238857</v>
       </c>
       <c r="P6" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q6" t="n">
         <v>710782</v>
@@ -83856,43 +83950,43 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B7" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C7" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D7" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G7" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I7" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K7" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M7" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N7" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P7" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q7" t="n">
         <v>710782</v>
@@ -83900,201 +83994,201 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B8" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C8" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D8" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G8" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I8" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K8" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M8" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N8" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O8" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P8" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q8" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B9" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C9" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D9" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G9" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I9" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K9" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M9" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N9" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O9" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P9" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q9" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B10" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C10" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D10" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G10" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I10" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K10" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M10" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N10" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P10" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q10" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B11" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C11" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D11" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E11" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G11" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I11" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K11" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M11" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N11" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O11" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P11" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q11" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B12" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C12" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D12" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E12" t="n">
         <v>9400</v>
       </c>
       <c r="F12" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G12" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I12" t="n">
         <v>1493578</v>
@@ -84103,7 +84197,7 @@
         <v>270165</v>
       </c>
       <c r="M12" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
@@ -84115,39 +84209,39 @@
         <v>380581</v>
       </c>
       <c r="Q12" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B13" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C13" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D13" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E13" t="n">
         <v>9400</v>
       </c>
       <c r="F13" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G13" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I13" t="n">
         <v>1493578</v>
       </c>
       <c r="K13" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M13" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
@@ -84156,153 +84250,153 @@
         <v>236857</v>
       </c>
       <c r="P13" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q13" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B14" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C14" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D14" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E14" t="n">
         <v>9400</v>
       </c>
       <c r="F14" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G14" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I14" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K14" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M14" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N14" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O14" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P14" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q14" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B15" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C15" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D15" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E15" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F15" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G15" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I15" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K15" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M15" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N15" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O15" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P15" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q15" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B16" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C16" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D16" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E16" t="n">
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G16" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I16" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K16" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M16" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N16" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O16" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P16" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q16" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B17" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C17" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D17" t="n">
         <v>1438502</v>
@@ -84311,107 +84405,107 @@
         <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G17" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I17" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K17" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M17" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N17" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O17" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P17" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q17" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B18" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C18" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D18" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E18" t="n">
         <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G18" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I18" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K18" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M18" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N18" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O18" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P18" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q18" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B19" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C19" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D19" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E19" t="n">
         <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G19" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I19" t="n">
         <v>1488515</v>
       </c>
       <c r="K19" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M19" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N19" t="n">
         <v>214475</v>
@@ -84420,7 +84514,7 @@
         <v>247857</v>
       </c>
       <c r="P19" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q19" t="n">
         <v>738429</v>
@@ -84428,34 +84522,34 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B20" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C20" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D20" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E20" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F20" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G20" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I20" t="n">
         <v>1488515</v>
       </c>
       <c r="K20" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M20" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N20" t="n">
         <v>214475</v>
@@ -84464,7 +84558,7 @@
         <v>247857</v>
       </c>
       <c r="P20" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q20" t="n">
         <v>738429</v>
@@ -84472,78 +84566,78 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B21" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C21" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D21" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E21" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F21" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G21" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I21" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K21" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M21" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N21" t="n">
         <v>214475</v>
       </c>
       <c r="O21" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P21" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q21" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B22" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C22" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D22" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E22" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F22" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G22" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I22" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K22" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M22" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N22" t="n">
         <v>214475</v>
@@ -84552,42 +84646,42 @@
         <v>264857</v>
       </c>
       <c r="P22" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q22" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B23" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C23" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D23" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E23" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F23" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G23" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I23" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K23" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M23" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N23" t="n">
         <v>214475</v>
@@ -84596,101 +84690,98 @@
         <v>264857</v>
       </c>
       <c r="P23" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q23" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B24" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C24" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D24" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E24" t="n">
         <v>9300</v>
       </c>
       <c r="F24" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G24" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I24" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K24" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M24" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N24" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O24" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P24" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q24" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R24" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B25" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C25" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D25" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E25" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F25" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G25" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I25" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K25" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M25" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N25" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O25" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P25" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q25" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R25" t="n">
         <v>15000</v>
@@ -84698,40 +84789,40 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B26" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C26" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D26" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E26" t="n">
         <v>9100</v>
       </c>
       <c r="F26" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G26" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I26" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K26" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M26" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N26" t="n">
         <v>189475</v>
       </c>
       <c r="O26" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P26" t="n">
         <v>375660</v>
@@ -84740,6 +84831,53 @@
         <v>773586</v>
       </c>
       <c r="R26" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C27" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E27" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K27" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M27" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N27" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O27" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P27" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R27" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -92069,7 +92207,7 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>0.382</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="652">
@@ -92079,7 +92217,7 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>1.389</v>
+        <v>1.391</v>
       </c>
     </row>
     <row r="653">
@@ -92089,7 +92227,7 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.51</v>
+        <v>2.515</v>
       </c>
     </row>
     <row r="654">
@@ -92099,7 +92237,7 @@
         </is>
       </c>
       <c r="D654" t="n">
-        <v>0.359</v>
+        <v>0.358</v>
       </c>
     </row>
     <row r="655">
@@ -92109,7 +92247,7 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>0.411</v>
+        <v>0.412</v>
       </c>
     </row>
     <row r="656">
@@ -92119,7 +92257,7 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>0.696</v>
+        <v>0.6879999999999999</v>
       </c>
     </row>
     <row r="657">
@@ -92129,7 +92267,7 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>3.211</v>
+        <v>3.207</v>
       </c>
     </row>
     <row r="658">
@@ -92139,7 +92277,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.262</v>
+        <v>3.239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feedgas backfill: [ 27/119] 2026-09-01 ~ 13/17 meters metered 12.11 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:23 ~1:21 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80303,9 +80303,36 @@
       <c r="A2437" s="4" t="n">
         <v>46266</v>
       </c>
+      <c r="B2437" t="n">
+        <v>3.163</v>
+      </c>
+      <c r="C2437" t="n">
+        <v>3.205</v>
+      </c>
+      <c r="D2437" t="n">
+        <v>1.472</v>
+      </c>
+      <c r="E2437" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="F2437" t="n">
+        <v>2.634</v>
+      </c>
+      <c r="G2437" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="H2437" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="I2437" t="n">
+        <v>0.593</v>
+      </c>
+      <c r="K2437" t="n">
+        <v>12.109</v>
+      </c>
       <c r="L2437" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81291,7 +81318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81356,153 +81383,153 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B2" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C2" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D2" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E2" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F2" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G2" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H2" t="n">
         <v>0.342</v>
       </c>
       <c r="I2" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K2" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B3" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C3" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D3" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E3" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F3" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G3" t="n">
         <v>0.444</v>
       </c>
       <c r="H3" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I3" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K3" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B4" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C4" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D4" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E4" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F4" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G4" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H4" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I4" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K4" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B5" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C5" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D5" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E5" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F5" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G5" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H5" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K5" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B6" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C6" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D6" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E6" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F6" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G6" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
@@ -81511,27 +81538,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B7" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C7" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D7" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E7" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F7" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G7" t="n">
         <v>0.437</v>
@@ -81543,178 +81570,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B8" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C8" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D8" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E8" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F8" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G8" t="n">
         <v>0.437</v>
       </c>
       <c r="H8" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I8" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B9" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C9" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D9" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E9" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F9" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G9" t="n">
         <v>0.437</v>
       </c>
       <c r="H9" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I9" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B10" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C10" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D10" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F10" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G10" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K10" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B11" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C11" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D11" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E11" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F11" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G11" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B12" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C12" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D12" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E12" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F12" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G12" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K12" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B13" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C13" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D13" t="n">
         <v>1.44</v>
@@ -81723,7 +81750,7 @@
         <v>0.261</v>
       </c>
       <c r="F13" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G13" t="n">
         <v>0.435</v>
@@ -81732,222 +81759,222 @@
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K13" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B14" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C14" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D14" t="n">
         <v>1.44</v>
       </c>
       <c r="E14" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F14" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G14" t="n">
         <v>0.435</v>
       </c>
       <c r="H14" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K14" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B15" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C15" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D15" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E15" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F15" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G15" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H15" t="n">
         <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K15" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B16" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C16" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D16" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F16" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G16" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H16" t="n">
         <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K16" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B17" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C17" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D17" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E17" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G17" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H17" t="n">
         <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K17" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B18" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C18" t="n">
         <v>3.232</v>
       </c>
       <c r="D18" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F18" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G18" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H18" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K18" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B19" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C19" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D19" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E19" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G19" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H19" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I19" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K19" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B20" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C20" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D20" t="n">
         <v>1.435</v>
       </c>
       <c r="E20" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F20" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G20" t="n">
         <v>0.446</v>
@@ -81959,27 +81986,27 @@
         <v>0.712</v>
       </c>
       <c r="K20" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B21" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C21" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D21" t="n">
         <v>1.435</v>
       </c>
       <c r="E21" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F21" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G21" t="n">
         <v>0.446</v>
@@ -81991,59 +82018,59 @@
         <v>0.712</v>
       </c>
       <c r="K21" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B22" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C22" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D22" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E22" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F22" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G22" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H22" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I22" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K22" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B23" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C23" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D23" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E23" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F23" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G23" t="n">
         <v>0.462</v>
@@ -82052,30 +82079,30 @@
         <v>0.343</v>
       </c>
       <c r="I23" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K23" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B24" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C24" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D24" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E24" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F24" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G24" t="n">
         <v>0.462</v>
@@ -82084,100 +82111,97 @@
         <v>0.343</v>
       </c>
       <c r="I24" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K24" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B25" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C25" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D25" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E25" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F25" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G25" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H25" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I25" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K25" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B26" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C26" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D26" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E26" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F26" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G26" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H26" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I26" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J26" t="n">
         <v>0.014</v>
       </c>
       <c r="K26" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B27" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C27" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D27" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E27" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F27" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G27" t="n">
         <v>0.395</v>
@@ -82192,6 +82216,41 @@
         <v>0.014</v>
       </c>
       <c r="K27" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K28" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82206,7 +82265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82276,165 +82335,165 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B2" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C2" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D2" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E2" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F2" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G2" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H2" t="n">
         <v>0.342</v>
       </c>
       <c r="I2" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K2" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L2" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B3" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C3" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D3" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E3" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F3" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G3" t="n">
         <v>0.444</v>
       </c>
       <c r="H3" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I3" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K3" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L3" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B4" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C4" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D4" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E4" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F4" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G4" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H4" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I4" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K4" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L4" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B5" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C5" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D5" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E5" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F5" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G5" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H5" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K5" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L5" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B6" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C6" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D6" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E6" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F6" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G6" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H6" t="n">
         <v>0.367</v>
@@ -82443,30 +82502,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L6" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B7" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C7" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D7" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E7" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F7" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G7" t="n">
         <v>0.437</v>
@@ -82478,196 +82537,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L7" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B8" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C8" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D8" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E8" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F8" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G8" t="n">
         <v>0.437</v>
       </c>
       <c r="H8" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I8" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L8" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B9" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C9" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D9" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E9" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F9" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G9" t="n">
         <v>0.437</v>
       </c>
       <c r="H9" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I9" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L9" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B10" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C10" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D10" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F10" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G10" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K10" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L10" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B11" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C11" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D11" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E11" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F11" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G11" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L11" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B12" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C12" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D12" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E12" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F12" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G12" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K12" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L12" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B13" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C13" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D13" t="n">
         <v>1.44</v>
@@ -82676,7 +82735,7 @@
         <v>0.261</v>
       </c>
       <c r="F13" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G13" t="n">
         <v>0.435</v>
@@ -82685,243 +82744,243 @@
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K13" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L13" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B14" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C14" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D14" t="n">
         <v>1.44</v>
       </c>
       <c r="E14" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F14" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G14" t="n">
         <v>0.435</v>
       </c>
       <c r="H14" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K14" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L14" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B15" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C15" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D15" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E15" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F15" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G15" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H15" t="n">
         <v>0.365</v>
       </c>
       <c r="I15" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K15" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L15" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B16" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C16" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D16" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F16" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G16" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H16" t="n">
         <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K16" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L16" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B17" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C17" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D17" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E17" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G17" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H17" t="n">
         <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K17" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L17" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B18" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C18" t="n">
         <v>3.232</v>
       </c>
       <c r="D18" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F18" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G18" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H18" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K18" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L18" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B19" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C19" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D19" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E19" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G19" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H19" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I19" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K19" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L19" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B20" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C20" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D20" t="n">
         <v>1.435</v>
       </c>
       <c r="E20" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F20" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G20" t="n">
         <v>0.446</v>
@@ -82933,30 +82992,30 @@
         <v>0.712</v>
       </c>
       <c r="K20" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L20" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B21" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C21" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D21" t="n">
         <v>1.435</v>
       </c>
       <c r="E21" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F21" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G21" t="n">
         <v>0.446</v>
@@ -82968,65 +83027,65 @@
         <v>0.712</v>
       </c>
       <c r="K21" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L21" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B22" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C22" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D22" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E22" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F22" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G22" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H22" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I22" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K22" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L22" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B23" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C23" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D23" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E23" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F23" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G23" t="n">
         <v>0.462</v>
@@ -83035,33 +83094,33 @@
         <v>0.343</v>
       </c>
       <c r="I23" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K23" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L23" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B24" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C24" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D24" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E24" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F24" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G24" t="n">
         <v>0.462</v>
@@ -83070,109 +83129,106 @@
         <v>0.343</v>
       </c>
       <c r="I24" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K24" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L24" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B25" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C25" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D25" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E25" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F25" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G25" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H25" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I25" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K25" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L25" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B26" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C26" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D26" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E26" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F26" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G26" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H26" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I26" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J26" t="n">
         <v>0.014</v>
       </c>
       <c r="K26" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L26" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B27" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C27" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D27" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E27" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F27" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G27" t="n">
         <v>0.395</v>
@@ -83187,9 +83243,47 @@
         <v>0.014</v>
       </c>
       <c r="K27" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L27" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K28" t="n">
         <v>12.277</v>
       </c>
-      <c r="L27" t="n">
+      <c r="L28" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83630,7 +83724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83730,189 +83824,189 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B2" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C2" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D2" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E2" t="n">
         <v>9000</v>
       </c>
       <c r="F2" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G2" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I2" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K2" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M2" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N2" t="n">
         <v>214475</v>
       </c>
       <c r="O2" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P2" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q2" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B3" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C3" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D3" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E3" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F3" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G3" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I3" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K3" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M3" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P3" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q3" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B4" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C4" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D4" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E4" t="n">
         <v>9200</v>
       </c>
       <c r="F4" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G4" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I4" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K4" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M4" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P4" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q4" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B5" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C5" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D5" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G5" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I5" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K5" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M5" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N5" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P5" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q5" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B6" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C6" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D6" t="n">
         <v>1336369</v>
@@ -83921,28 +84015,28 @@
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G6" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I6" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K6" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M6" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N6" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O6" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P6" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q6" t="n">
         <v>710782</v>
@@ -83950,34 +84044,34 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B7" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C7" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D7" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G7" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I7" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K7" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M7" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
@@ -83986,7 +84080,7 @@
         <v>238857</v>
       </c>
       <c r="P7" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q7" t="n">
         <v>710782</v>
@@ -83994,43 +84088,43 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B8" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C8" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D8" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G8" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I8" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K8" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M8" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N8" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P8" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q8" t="n">
         <v>710782</v>
@@ -84038,201 +84132,201 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B9" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C9" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D9" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G9" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I9" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K9" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M9" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N9" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O9" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P9" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q9" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B10" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C10" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D10" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G10" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I10" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K10" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M10" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N10" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O10" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P10" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q10" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B11" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C11" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D11" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G11" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I11" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K11" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M11" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N11" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P11" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q11" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B12" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C12" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D12" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E12" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G12" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I12" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K12" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M12" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N12" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O12" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P12" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q12" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B13" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C13" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D13" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E13" t="n">
         <v>9400</v>
       </c>
       <c r="F13" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G13" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I13" t="n">
         <v>1493578</v>
@@ -84241,7 +84335,7 @@
         <v>270165</v>
       </c>
       <c r="M13" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
@@ -84253,39 +84347,39 @@
         <v>380581</v>
       </c>
       <c r="Q13" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B14" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C14" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D14" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E14" t="n">
         <v>9400</v>
       </c>
       <c r="F14" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G14" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I14" t="n">
         <v>1493578</v>
       </c>
       <c r="K14" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M14" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
@@ -84294,153 +84388,153 @@
         <v>236857</v>
       </c>
       <c r="P14" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q14" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B15" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C15" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D15" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E15" t="n">
         <v>9400</v>
       </c>
       <c r="F15" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G15" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I15" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K15" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M15" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N15" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O15" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P15" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q15" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B16" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C16" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D16" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E16" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F16" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G16" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I16" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K16" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M16" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N16" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O16" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P16" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q16" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B17" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C17" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D17" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E17" t="n">
         <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G17" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I17" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K17" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M17" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N17" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O17" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P17" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q17" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B18" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C18" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D18" t="n">
         <v>1438502</v>
@@ -84449,107 +84543,107 @@
         <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G18" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I18" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K18" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M18" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N18" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O18" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P18" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q18" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B19" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C19" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D19" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E19" t="n">
         <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G19" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I19" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K19" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M19" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N19" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O19" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P19" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q19" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B20" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C20" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D20" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E20" t="n">
         <v>9200</v>
       </c>
       <c r="F20" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G20" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I20" t="n">
         <v>1488515</v>
       </c>
       <c r="K20" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M20" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N20" t="n">
         <v>214475</v>
@@ -84558,7 +84652,7 @@
         <v>247857</v>
       </c>
       <c r="P20" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q20" t="n">
         <v>738429</v>
@@ -84566,34 +84660,34 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B21" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C21" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D21" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E21" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F21" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G21" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I21" t="n">
         <v>1488515</v>
       </c>
       <c r="K21" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M21" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N21" t="n">
         <v>214475</v>
@@ -84602,7 +84696,7 @@
         <v>247857</v>
       </c>
       <c r="P21" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q21" t="n">
         <v>738429</v>
@@ -84610,78 +84704,78 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B22" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C22" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D22" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E22" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F22" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G22" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I22" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K22" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M22" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N22" t="n">
         <v>214475</v>
       </c>
       <c r="O22" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P22" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q22" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B23" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C23" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D23" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E23" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F23" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G23" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I23" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K23" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M23" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N23" t="n">
         <v>214475</v>
@@ -84690,42 +84784,42 @@
         <v>264857</v>
       </c>
       <c r="P23" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q23" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B24" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C24" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D24" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E24" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F24" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G24" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I24" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K24" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M24" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N24" t="n">
         <v>214475</v>
@@ -84734,101 +84828,98 @@
         <v>264857</v>
       </c>
       <c r="P24" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q24" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B25" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C25" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D25" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E25" t="n">
         <v>9300</v>
       </c>
       <c r="F25" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G25" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I25" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K25" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M25" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N25" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O25" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P25" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q25" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R25" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B26" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C26" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D26" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E26" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F26" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G26" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I26" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K26" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M26" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N26" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O26" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P26" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q26" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R26" t="n">
         <v>15000</v>
@@ -84836,40 +84927,40 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B27" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C27" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D27" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E27" t="n">
         <v>9100</v>
       </c>
       <c r="F27" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G27" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I27" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K27" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M27" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N27" t="n">
         <v>189475</v>
       </c>
       <c r="O27" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P27" t="n">
         <v>375660</v>
@@ -84878,6 +84969,53 @@
         <v>773586</v>
       </c>
       <c r="R27" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B28" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C28" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E28" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K28" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M28" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N28" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O28" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P28" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R28" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -92207,7 +92345,7 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>0.375</v>
+        <v>0.371</v>
       </c>
     </row>
     <row r="652">
@@ -92217,7 +92355,7 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>1.391</v>
+        <v>1.394</v>
       </c>
     </row>
     <row r="653">
@@ -92227,7 +92365,7 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>2.515</v>
+        <v>2.519</v>
       </c>
     </row>
     <row r="654">
@@ -92237,7 +92375,7 @@
         </is>
       </c>
       <c r="D654" t="n">
-        <v>0.358</v>
+        <v>0.357</v>
       </c>
     </row>
     <row r="655">
@@ -92247,7 +92385,7 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>0.412</v>
+        <v>0.413</v>
       </c>
     </row>
     <row r="656">
@@ -92257,7 +92395,7 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.6840000000000001</v>
       </c>
     </row>
     <row r="657">
@@ -92277,7 +92415,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>3.239</v>
+        <v>3.236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feedgas backfill: [ 28/119] 2026-08-31 ~ 13/17 meters metered 12.53 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:24 ~1:20 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80293,9 +80293,36 @@
       <c r="A2436" s="4" t="n">
         <v>46265</v>
       </c>
+      <c r="B2436" t="n">
+        <v>3.392</v>
+      </c>
+      <c r="C2436" t="n">
+        <v>3.207</v>
+      </c>
+      <c r="D2436" t="n">
+        <v>1.476</v>
+      </c>
+      <c r="E2436" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="F2436" t="n">
+        <v>2.512</v>
+      </c>
+      <c r="G2436" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="H2436" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="I2436" t="n">
+        <v>0.723</v>
+      </c>
+      <c r="K2436" t="n">
+        <v>12.534</v>
+      </c>
       <c r="L2436" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81318,7 +81345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81383,185 +81410,185 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B2" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C2" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D2" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E2" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F2" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G2" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H2" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I2" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K2" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B3" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C3" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D3" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E3" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F3" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G3" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H3" t="n">
         <v>0.342</v>
       </c>
       <c r="I3" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K3" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B4" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C4" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D4" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E4" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F4" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G4" t="n">
         <v>0.444</v>
       </c>
       <c r="H4" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I4" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K4" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B5" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C5" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D5" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E5" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F5" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G5" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H5" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I5" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K5" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B6" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C6" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D6" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E6" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F6" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G6" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H6" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K6" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B7" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C7" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D7" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E7" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F7" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G7" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
@@ -81570,27 +81597,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B8" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C8" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D8" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E8" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F8" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G8" t="n">
         <v>0.437</v>
@@ -81602,178 +81629,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B9" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C9" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D9" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E9" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F9" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G9" t="n">
         <v>0.437</v>
       </c>
       <c r="H9" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I9" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B10" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C10" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D10" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E10" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F10" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G10" t="n">
         <v>0.437</v>
       </c>
       <c r="H10" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I10" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B11" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C11" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D11" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F11" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G11" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K11" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B12" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C12" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D12" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E12" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F12" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G12" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B13" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C13" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D13" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E13" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F13" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G13" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K13" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B14" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C14" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D14" t="n">
         <v>1.44</v>
@@ -81782,7 +81809,7 @@
         <v>0.261</v>
       </c>
       <c r="F14" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G14" t="n">
         <v>0.435</v>
@@ -81791,222 +81818,222 @@
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K14" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B15" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C15" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D15" t="n">
         <v>1.44</v>
       </c>
       <c r="E15" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F15" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G15" t="n">
         <v>0.435</v>
       </c>
       <c r="H15" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K15" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B16" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C16" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D16" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E16" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F16" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G16" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H16" t="n">
         <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K16" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B17" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C17" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D17" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F17" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G17" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H17" t="n">
         <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K17" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B18" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C18" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D18" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E18" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G18" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H18" t="n">
         <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K18" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B19" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C19" t="n">
         <v>3.232</v>
       </c>
       <c r="D19" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F19" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G19" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H19" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K19" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B20" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C20" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D20" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E20" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G20" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H20" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I20" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K20" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B21" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C21" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D21" t="n">
         <v>1.435</v>
       </c>
       <c r="E21" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F21" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G21" t="n">
         <v>0.446</v>
@@ -82018,27 +82045,27 @@
         <v>0.712</v>
       </c>
       <c r="K21" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B22" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C22" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D22" t="n">
         <v>1.435</v>
       </c>
       <c r="E22" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F22" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G22" t="n">
         <v>0.446</v>
@@ -82050,59 +82077,59 @@
         <v>0.712</v>
       </c>
       <c r="K22" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B23" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C23" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D23" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E23" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F23" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G23" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H23" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I23" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K23" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B24" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C24" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D24" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E24" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F24" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G24" t="n">
         <v>0.462</v>
@@ -82111,30 +82138,30 @@
         <v>0.343</v>
       </c>
       <c r="I24" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K24" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B25" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C25" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D25" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E25" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F25" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G25" t="n">
         <v>0.462</v>
@@ -82143,100 +82170,97 @@
         <v>0.343</v>
       </c>
       <c r="I25" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K25" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B26" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C26" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D26" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E26" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F26" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G26" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H26" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I26" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K26" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B27" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C27" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D27" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E27" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F27" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G27" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H27" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I27" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J27" t="n">
         <v>0.014</v>
       </c>
       <c r="K27" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B28" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C28" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D28" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F28" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G28" t="n">
         <v>0.395</v>
@@ -82251,6 +82275,41 @@
         <v>0.014</v>
       </c>
       <c r="K28" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B29" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K29" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82265,7 +82324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82335,200 +82394,200 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B2" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C2" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D2" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E2" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F2" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G2" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H2" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I2" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K2" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L2" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B3" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C3" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D3" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E3" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F3" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G3" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H3" t="n">
         <v>0.342</v>
       </c>
       <c r="I3" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K3" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L3" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B4" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C4" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D4" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E4" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F4" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G4" t="n">
         <v>0.444</v>
       </c>
       <c r="H4" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I4" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K4" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L4" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B5" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C5" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D5" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E5" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F5" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G5" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H5" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I5" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K5" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L5" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B6" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C6" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D6" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E6" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F6" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G6" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H6" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K6" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L6" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B7" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C7" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D7" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E7" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F7" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G7" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H7" t="n">
         <v>0.367</v>
@@ -82537,30 +82596,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L7" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B8" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C8" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D8" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E8" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F8" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G8" t="n">
         <v>0.437</v>
@@ -82572,196 +82631,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L8" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B9" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C9" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D9" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E9" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F9" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G9" t="n">
         <v>0.437</v>
       </c>
       <c r="H9" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I9" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L9" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B10" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C10" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D10" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E10" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F10" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G10" t="n">
         <v>0.437</v>
       </c>
       <c r="H10" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I10" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L10" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B11" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C11" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D11" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F11" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G11" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K11" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L11" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B12" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C12" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D12" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E12" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F12" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G12" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L12" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B13" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C13" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D13" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E13" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F13" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G13" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K13" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L13" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B14" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C14" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D14" t="n">
         <v>1.44</v>
@@ -82770,7 +82829,7 @@
         <v>0.261</v>
       </c>
       <c r="F14" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G14" t="n">
         <v>0.435</v>
@@ -82779,243 +82838,243 @@
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K14" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L14" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B15" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C15" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D15" t="n">
         <v>1.44</v>
       </c>
       <c r="E15" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F15" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G15" t="n">
         <v>0.435</v>
       </c>
       <c r="H15" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K15" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L15" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B16" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C16" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D16" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E16" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F16" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G16" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H16" t="n">
         <v>0.365</v>
       </c>
       <c r="I16" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K16" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L16" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B17" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C17" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D17" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F17" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G17" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H17" t="n">
         <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K17" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L17" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B18" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C18" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D18" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E18" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G18" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H18" t="n">
         <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K18" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L18" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B19" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C19" t="n">
         <v>3.232</v>
       </c>
       <c r="D19" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F19" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G19" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H19" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K19" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L19" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B20" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C20" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D20" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E20" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G20" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H20" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I20" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K20" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L20" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B21" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C21" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D21" t="n">
         <v>1.435</v>
       </c>
       <c r="E21" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F21" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G21" t="n">
         <v>0.446</v>
@@ -83027,30 +83086,30 @@
         <v>0.712</v>
       </c>
       <c r="K21" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L21" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B22" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C22" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D22" t="n">
         <v>1.435</v>
       </c>
       <c r="E22" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F22" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G22" t="n">
         <v>0.446</v>
@@ -83062,65 +83121,65 @@
         <v>0.712</v>
       </c>
       <c r="K22" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L22" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B23" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C23" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D23" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E23" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F23" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G23" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H23" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I23" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K23" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L23" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B24" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C24" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D24" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E24" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F24" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G24" t="n">
         <v>0.462</v>
@@ -83129,33 +83188,33 @@
         <v>0.343</v>
       </c>
       <c r="I24" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K24" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L24" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B25" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C25" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D25" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E25" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F25" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G25" t="n">
         <v>0.462</v>
@@ -83164,109 +83223,106 @@
         <v>0.343</v>
       </c>
       <c r="I25" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K25" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L25" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B26" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C26" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D26" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E26" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F26" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G26" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H26" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I26" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K26" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L26" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B27" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C27" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D27" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E27" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F27" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G27" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H27" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I27" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J27" t="n">
         <v>0.014</v>
       </c>
       <c r="K27" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L27" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B28" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C28" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D28" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F28" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G28" t="n">
         <v>0.395</v>
@@ -83281,9 +83337,47 @@
         <v>0.014</v>
       </c>
       <c r="K28" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L28" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B29" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K29" t="n">
         <v>12.277</v>
       </c>
-      <c r="L28" t="n">
+      <c r="L29" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83724,7 +83818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83824,233 +83918,233 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B2" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C2" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D2" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E2" t="n">
         <v>9000</v>
       </c>
       <c r="F2" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G2" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I2" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K2" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M2" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N2" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O2" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P2" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q2" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B3" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C3" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D3" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E3" t="n">
         <v>9000</v>
       </c>
       <c r="F3" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G3" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I3" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K3" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M3" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N3" t="n">
         <v>214475</v>
       </c>
       <c r="O3" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P3" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q3" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B4" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C4" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D4" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E4" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F4" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G4" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I4" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K4" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M4" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P4" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q4" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B5" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C5" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D5" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E5" t="n">
         <v>9200</v>
       </c>
       <c r="F5" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G5" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I5" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K5" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M5" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P5" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q5" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B6" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C6" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D6" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G6" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I6" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K6" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M6" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N6" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P6" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q6" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B7" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C7" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D7" t="n">
         <v>1336369</v>
@@ -84059,28 +84153,28 @@
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G7" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I7" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K7" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M7" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N7" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O7" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P7" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q7" t="n">
         <v>710782</v>
@@ -84088,34 +84182,34 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B8" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C8" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D8" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G8" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I8" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K8" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M8" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
@@ -84124,7 +84218,7 @@
         <v>238857</v>
       </c>
       <c r="P8" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q8" t="n">
         <v>710782</v>
@@ -84132,43 +84226,43 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B9" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C9" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D9" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G9" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I9" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K9" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M9" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N9" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P9" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q9" t="n">
         <v>710782</v>
@@ -84176,201 +84270,201 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B10" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C10" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D10" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G10" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I10" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K10" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M10" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N10" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O10" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P10" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q10" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B11" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C11" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D11" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G11" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I11" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K11" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M11" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N11" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O11" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P11" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q11" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B12" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C12" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D12" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G12" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I12" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K12" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M12" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N12" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P12" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q12" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B13" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C13" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D13" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E13" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G13" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I13" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K13" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M13" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N13" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O13" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P13" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q13" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B14" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C14" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D14" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E14" t="n">
         <v>9400</v>
       </c>
       <c r="F14" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G14" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I14" t="n">
         <v>1493578</v>
@@ -84379,7 +84473,7 @@
         <v>270165</v>
       </c>
       <c r="M14" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
@@ -84391,39 +84485,39 @@
         <v>380581</v>
       </c>
       <c r="Q14" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B15" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C15" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D15" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E15" t="n">
         <v>9400</v>
       </c>
       <c r="F15" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G15" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I15" t="n">
         <v>1493578</v>
       </c>
       <c r="K15" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M15" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
@@ -84432,153 +84526,153 @@
         <v>236857</v>
       </c>
       <c r="P15" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q15" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B16" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C16" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D16" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E16" t="n">
         <v>9400</v>
       </c>
       <c r="F16" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G16" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I16" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K16" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M16" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N16" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O16" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P16" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q16" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B17" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C17" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D17" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E17" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F17" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G17" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I17" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K17" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M17" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N17" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O17" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P17" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q17" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B18" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C18" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D18" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E18" t="n">
         <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G18" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I18" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K18" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M18" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N18" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O18" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P18" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q18" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B19" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C19" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D19" t="n">
         <v>1438502</v>
@@ -84587,107 +84681,107 @@
         <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G19" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I19" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K19" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M19" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N19" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O19" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P19" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q19" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B20" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C20" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D20" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E20" t="n">
         <v>9200</v>
       </c>
       <c r="F20" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G20" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I20" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K20" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M20" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N20" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O20" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P20" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q20" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B21" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C21" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D21" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E21" t="n">
         <v>9200</v>
       </c>
       <c r="F21" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G21" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I21" t="n">
         <v>1488515</v>
       </c>
       <c r="K21" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M21" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N21" t="n">
         <v>214475</v>
@@ -84696,7 +84790,7 @@
         <v>247857</v>
       </c>
       <c r="P21" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q21" t="n">
         <v>738429</v>
@@ -84704,34 +84798,34 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B22" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C22" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D22" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E22" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F22" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G22" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I22" t="n">
         <v>1488515</v>
       </c>
       <c r="K22" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M22" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N22" t="n">
         <v>214475</v>
@@ -84740,7 +84834,7 @@
         <v>247857</v>
       </c>
       <c r="P22" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q22" t="n">
         <v>738429</v>
@@ -84748,78 +84842,78 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B23" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C23" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D23" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E23" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F23" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G23" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I23" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K23" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M23" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N23" t="n">
         <v>214475</v>
       </c>
       <c r="O23" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P23" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q23" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B24" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C24" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D24" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E24" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F24" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G24" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I24" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K24" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M24" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N24" t="n">
         <v>214475</v>
@@ -84828,42 +84922,42 @@
         <v>264857</v>
       </c>
       <c r="P24" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q24" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B25" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C25" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D25" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E25" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F25" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G25" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I25" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K25" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M25" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N25" t="n">
         <v>214475</v>
@@ -84872,101 +84966,98 @@
         <v>264857</v>
       </c>
       <c r="P25" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q25" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B26" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C26" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D26" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E26" t="n">
         <v>9300</v>
       </c>
       <c r="F26" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G26" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I26" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K26" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M26" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N26" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O26" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P26" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q26" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R26" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B27" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C27" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D27" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E27" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F27" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G27" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I27" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K27" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M27" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N27" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O27" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P27" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q27" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R27" t="n">
         <v>15000</v>
@@ -84974,40 +85065,40 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B28" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C28" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D28" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E28" t="n">
         <v>9100</v>
       </c>
       <c r="F28" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G28" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I28" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K28" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M28" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N28" t="n">
         <v>189475</v>
       </c>
       <c r="O28" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P28" t="n">
         <v>375660</v>
@@ -85016,6 +85107,53 @@
         <v>773586</v>
       </c>
       <c r="R28" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B29" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C29" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E29" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K29" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M29" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N29" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O29" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P29" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R29" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 29/119] 2026-08-30 ~ 13/17 meters metered 12.43 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:25 ~1:19 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80283,9 +80283,36 @@
       <c r="A2435" s="4" t="n">
         <v>46264</v>
       </c>
+      <c r="B2435" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="C2435" t="n">
+        <v>3.115</v>
+      </c>
+      <c r="D2435" t="n">
+        <v>1.463</v>
+      </c>
+      <c r="E2435" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="F2435" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="G2435" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="H2435" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="I2435" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="K2435" t="n">
+        <v>12.429</v>
+      </c>
       <c r="L2435" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81345,7 +81372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81410,217 +81437,217 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B2" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C2" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D2" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E2" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F2" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G2" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H2" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K2" t="n">
-        <v>12.534</v>
+        <v>12.428</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B3" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C3" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D3" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E3" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F3" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G3" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H3" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I3" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K3" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B4" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C4" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D4" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E4" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F4" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G4" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H4" t="n">
         <v>0.342</v>
       </c>
       <c r="I4" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K4" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B5" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C5" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D5" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E5" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F5" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G5" t="n">
         <v>0.444</v>
       </c>
       <c r="H5" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I5" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K5" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B6" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C6" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D6" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E6" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F6" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G6" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H6" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I6" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K6" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B7" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C7" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D7" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E7" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F7" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G7" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H7" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K7" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B8" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C8" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D8" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E8" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F8" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G8" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
@@ -81629,27 +81656,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B9" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C9" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D9" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E9" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F9" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G9" t="n">
         <v>0.437</v>
@@ -81661,178 +81688,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B10" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C10" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D10" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E10" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F10" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G10" t="n">
         <v>0.437</v>
       </c>
       <c r="H10" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I10" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B11" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C11" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D11" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E11" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F11" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G11" t="n">
         <v>0.437</v>
       </c>
       <c r="H11" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I11" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B12" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C12" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D12" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F12" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G12" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K12" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B13" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C13" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D13" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E13" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F13" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G13" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B14" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C14" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D14" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E14" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F14" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G14" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K14" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B15" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C15" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D15" t="n">
         <v>1.44</v>
@@ -81841,7 +81868,7 @@
         <v>0.261</v>
       </c>
       <c r="F15" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G15" t="n">
         <v>0.435</v>
@@ -81850,222 +81877,222 @@
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K15" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B16" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C16" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D16" t="n">
         <v>1.44</v>
       </c>
       <c r="E16" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F16" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G16" t="n">
         <v>0.435</v>
       </c>
       <c r="H16" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K16" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B17" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C17" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D17" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E17" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F17" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G17" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H17" t="n">
         <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K17" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B18" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C18" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D18" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F18" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G18" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H18" t="n">
         <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K18" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B19" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C19" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D19" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E19" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G19" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H19" t="n">
         <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K19" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B20" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C20" t="n">
         <v>3.232</v>
       </c>
       <c r="D20" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F20" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G20" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H20" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K20" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B21" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C21" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D21" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E21" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G21" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H21" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I21" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K21" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B22" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C22" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D22" t="n">
         <v>1.435</v>
       </c>
       <c r="E22" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F22" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G22" t="n">
         <v>0.446</v>
@@ -82077,27 +82104,27 @@
         <v>0.712</v>
       </c>
       <c r="K22" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B23" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C23" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D23" t="n">
         <v>1.435</v>
       </c>
       <c r="E23" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F23" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G23" t="n">
         <v>0.446</v>
@@ -82109,59 +82136,59 @@
         <v>0.712</v>
       </c>
       <c r="K23" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B24" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C24" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D24" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E24" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F24" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G24" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H24" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I24" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K24" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B25" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C25" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D25" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E25" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F25" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G25" t="n">
         <v>0.462</v>
@@ -82170,30 +82197,30 @@
         <v>0.343</v>
       </c>
       <c r="I25" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K25" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B26" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C26" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D26" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E26" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F26" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G26" t="n">
         <v>0.462</v>
@@ -82202,100 +82229,97 @@
         <v>0.343</v>
       </c>
       <c r="I26" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K26" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B27" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C27" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D27" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E27" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F27" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G27" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H27" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I27" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K27" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B28" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C28" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D28" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E28" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F28" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G28" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H28" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I28" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J28" t="n">
         <v>0.014</v>
       </c>
       <c r="K28" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B29" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C29" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D29" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E29" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F29" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G29" t="n">
         <v>0.395</v>
@@ -82310,6 +82334,41 @@
         <v>0.014</v>
       </c>
       <c r="K29" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B30" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K30" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82324,7 +82383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82394,235 +82453,235 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B2" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C2" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D2" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E2" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F2" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G2" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H2" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K2" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
       <c r="L2" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B3" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C3" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D3" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E3" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F3" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G3" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H3" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I3" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K3" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L3" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B4" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C4" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D4" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E4" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F4" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G4" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H4" t="n">
         <v>0.342</v>
       </c>
       <c r="I4" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K4" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L4" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B5" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C5" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D5" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E5" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F5" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G5" t="n">
         <v>0.444</v>
       </c>
       <c r="H5" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I5" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K5" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L5" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B6" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C6" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D6" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E6" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F6" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G6" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H6" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I6" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K6" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L6" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B7" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C7" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D7" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E7" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F7" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G7" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H7" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K7" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L7" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B8" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C8" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D8" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E8" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F8" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G8" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H8" t="n">
         <v>0.367</v>
@@ -82631,30 +82690,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L8" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B9" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C9" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D9" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E9" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F9" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G9" t="n">
         <v>0.437</v>
@@ -82666,196 +82725,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L9" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B10" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C10" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D10" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E10" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F10" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G10" t="n">
         <v>0.437</v>
       </c>
       <c r="H10" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I10" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L10" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B11" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C11" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D11" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E11" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F11" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G11" t="n">
         <v>0.437</v>
       </c>
       <c r="H11" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I11" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L11" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B12" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C12" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D12" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F12" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G12" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K12" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L12" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B13" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C13" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D13" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E13" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F13" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G13" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L13" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B14" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C14" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D14" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E14" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F14" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G14" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K14" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L14" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B15" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C15" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D15" t="n">
         <v>1.44</v>
@@ -82864,7 +82923,7 @@
         <v>0.261</v>
       </c>
       <c r="F15" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G15" t="n">
         <v>0.435</v>
@@ -82873,243 +82932,243 @@
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K15" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L15" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B16" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C16" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D16" t="n">
         <v>1.44</v>
       </c>
       <c r="E16" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F16" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G16" t="n">
         <v>0.435</v>
       </c>
       <c r="H16" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K16" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L16" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B17" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C17" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D17" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E17" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F17" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G17" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H17" t="n">
         <v>0.365</v>
       </c>
       <c r="I17" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K17" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L17" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B18" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C18" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D18" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F18" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G18" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H18" t="n">
         <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K18" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L18" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B19" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C19" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D19" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E19" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G19" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H19" t="n">
         <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K19" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L19" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B20" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C20" t="n">
         <v>3.232</v>
       </c>
       <c r="D20" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F20" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G20" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H20" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K20" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L20" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B21" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C21" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D21" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E21" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G21" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H21" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I21" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K21" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L21" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B22" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C22" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D22" t="n">
         <v>1.435</v>
       </c>
       <c r="E22" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F22" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G22" t="n">
         <v>0.446</v>
@@ -83121,30 +83180,30 @@
         <v>0.712</v>
       </c>
       <c r="K22" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L22" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B23" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C23" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D23" t="n">
         <v>1.435</v>
       </c>
       <c r="E23" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F23" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G23" t="n">
         <v>0.446</v>
@@ -83156,65 +83215,65 @@
         <v>0.712</v>
       </c>
       <c r="K23" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L23" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B24" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C24" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D24" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E24" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F24" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G24" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H24" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I24" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K24" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L24" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B25" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C25" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D25" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E25" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F25" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G25" t="n">
         <v>0.462</v>
@@ -83223,33 +83282,33 @@
         <v>0.343</v>
       </c>
       <c r="I25" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K25" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L25" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B26" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C26" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D26" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E26" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F26" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G26" t="n">
         <v>0.462</v>
@@ -83258,109 +83317,106 @@
         <v>0.343</v>
       </c>
       <c r="I26" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K26" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L26" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B27" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C27" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D27" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E27" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F27" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G27" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H27" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I27" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K27" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L27" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B28" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C28" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D28" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E28" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F28" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G28" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H28" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I28" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J28" t="n">
         <v>0.014</v>
       </c>
       <c r="K28" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L28" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B29" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C29" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D29" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E29" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F29" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G29" t="n">
         <v>0.395</v>
@@ -83375,9 +83431,47 @@
         <v>0.014</v>
       </c>
       <c r="K29" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L29" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B30" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K30" t="n">
         <v>12.277</v>
       </c>
-      <c r="L29" t="n">
+      <c r="L30" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83818,7 +83912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83918,277 +84012,277 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B2" t="n">
-        <v>1453305</v>
+        <v>1428345</v>
       </c>
       <c r="C2" t="n">
-        <v>660021</v>
+        <v>613887</v>
       </c>
       <c r="D2" t="n">
-        <v>1394810</v>
+        <v>1360335</v>
       </c>
       <c r="E2" t="n">
         <v>9000</v>
       </c>
       <c r="F2" t="n">
-        <v>1966997</v>
+        <v>2000629</v>
       </c>
       <c r="G2" t="n">
-        <v>1358589</v>
+        <v>1229134</v>
       </c>
       <c r="I2" t="n">
-        <v>1530881</v>
+        <v>1516881</v>
       </c>
       <c r="K2" t="n">
-        <v>224505</v>
+        <v>265281</v>
       </c>
       <c r="M2" t="n">
-        <v>2605275</v>
+        <v>2655010</v>
       </c>
       <c r="N2" t="n">
-        <v>273068</v>
+        <v>275644</v>
       </c>
       <c r="O2" t="n">
-        <v>402811</v>
+        <v>405391</v>
       </c>
       <c r="P2" t="n">
-        <v>368707</v>
+        <v>393345</v>
       </c>
       <c r="Q2" t="n">
-        <v>750038</v>
+        <v>735394</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B3" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C3" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D3" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E3" t="n">
         <v>9000</v>
       </c>
       <c r="F3" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G3" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I3" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K3" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M3" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N3" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O3" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P3" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q3" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B4" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C4" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D4" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E4" t="n">
         <v>9000</v>
       </c>
       <c r="F4" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G4" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I4" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K4" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M4" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N4" t="n">
         <v>214475</v>
       </c>
       <c r="O4" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P4" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q4" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B5" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C5" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D5" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E5" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G5" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I5" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K5" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M5" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P5" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q5" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B6" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C6" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D6" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E6" t="n">
         <v>9200</v>
       </c>
       <c r="F6" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G6" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I6" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K6" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M6" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P6" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q6" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B7" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C7" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D7" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G7" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I7" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K7" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M7" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N7" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P7" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q7" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B8" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C8" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D8" t="n">
         <v>1336369</v>
@@ -84197,28 +84291,28 @@
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G8" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I8" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K8" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M8" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N8" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O8" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P8" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q8" t="n">
         <v>710782</v>
@@ -84226,34 +84320,34 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B9" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C9" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D9" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G9" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I9" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K9" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M9" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
@@ -84262,7 +84356,7 @@
         <v>238857</v>
       </c>
       <c r="P9" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q9" t="n">
         <v>710782</v>
@@ -84270,43 +84364,43 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B10" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C10" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D10" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G10" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I10" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K10" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M10" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N10" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P10" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q10" t="n">
         <v>710782</v>
@@ -84314,201 +84408,201 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B11" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C11" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D11" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G11" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I11" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K11" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M11" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N11" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O11" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P11" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q11" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B12" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C12" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D12" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G12" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I12" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K12" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M12" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N12" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O12" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P12" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q12" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B13" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C13" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D13" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G13" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I13" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K13" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M13" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N13" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O13" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P13" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q13" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B14" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C14" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D14" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E14" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G14" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I14" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K14" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M14" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N14" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O14" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P14" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q14" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B15" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C15" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D15" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E15" t="n">
         <v>9400</v>
       </c>
       <c r="F15" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G15" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I15" t="n">
         <v>1493578</v>
@@ -84517,7 +84611,7 @@
         <v>270165</v>
       </c>
       <c r="M15" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
@@ -84529,39 +84623,39 @@
         <v>380581</v>
       </c>
       <c r="Q15" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B16" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C16" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D16" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E16" t="n">
         <v>9400</v>
       </c>
       <c r="F16" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G16" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I16" t="n">
         <v>1493578</v>
       </c>
       <c r="K16" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M16" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N16" t="n">
         <v>214475</v>
@@ -84570,153 +84664,153 @@
         <v>236857</v>
       </c>
       <c r="P16" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q16" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B17" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C17" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D17" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E17" t="n">
         <v>9400</v>
       </c>
       <c r="F17" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G17" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I17" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K17" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M17" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N17" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O17" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P17" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q17" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B18" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C18" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D18" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E18" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F18" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G18" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I18" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K18" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M18" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N18" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O18" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P18" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q18" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B19" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C19" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D19" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E19" t="n">
         <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G19" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I19" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K19" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M19" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N19" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O19" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P19" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q19" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B20" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C20" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D20" t="n">
         <v>1438502</v>
@@ -84725,107 +84819,107 @@
         <v>9200</v>
       </c>
       <c r="F20" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G20" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I20" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K20" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M20" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N20" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O20" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P20" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q20" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B21" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C21" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D21" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E21" t="n">
         <v>9200</v>
       </c>
       <c r="F21" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G21" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I21" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K21" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M21" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N21" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O21" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P21" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q21" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B22" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C22" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D22" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E22" t="n">
         <v>9200</v>
       </c>
       <c r="F22" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G22" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I22" t="n">
         <v>1488515</v>
       </c>
       <c r="K22" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M22" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N22" t="n">
         <v>214475</v>
@@ -84834,7 +84928,7 @@
         <v>247857</v>
       </c>
       <c r="P22" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q22" t="n">
         <v>738429</v>
@@ -84842,34 +84936,34 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B23" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C23" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D23" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E23" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F23" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G23" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I23" t="n">
         <v>1488515</v>
       </c>
       <c r="K23" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M23" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N23" t="n">
         <v>214475</v>
@@ -84878,7 +84972,7 @@
         <v>247857</v>
       </c>
       <c r="P23" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q23" t="n">
         <v>738429</v>
@@ -84886,78 +84980,78 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B24" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C24" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D24" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E24" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F24" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G24" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I24" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K24" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M24" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N24" t="n">
         <v>214475</v>
       </c>
       <c r="O24" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P24" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q24" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B25" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C25" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D25" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E25" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F25" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G25" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I25" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K25" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M25" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N25" t="n">
         <v>214475</v>
@@ -84966,42 +85060,42 @@
         <v>264857</v>
       </c>
       <c r="P25" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q25" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B26" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C26" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D26" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E26" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F26" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G26" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I26" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K26" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M26" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N26" t="n">
         <v>214475</v>
@@ -85010,101 +85104,98 @@
         <v>264857</v>
       </c>
       <c r="P26" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q26" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B27" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C27" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D27" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E27" t="n">
         <v>9300</v>
       </c>
       <c r="F27" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G27" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I27" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K27" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M27" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N27" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O27" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P27" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q27" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R27" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B28" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C28" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D28" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E28" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F28" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G28" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I28" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K28" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M28" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N28" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O28" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P28" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q28" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R28" t="n">
         <v>15000</v>
@@ -85112,40 +85203,40 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B29" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C29" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D29" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E29" t="n">
         <v>9100</v>
       </c>
       <c r="F29" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G29" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I29" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K29" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M29" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N29" t="n">
         <v>189475</v>
       </c>
       <c r="O29" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P29" t="n">
         <v>375660</v>
@@ -85154,6 +85245,53 @@
         <v>773586</v>
       </c>
       <c r="R29" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B30" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C30" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E30" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K30" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M30" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N30" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O30" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P30" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R30" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 30/119] 2026-08-29 ~ 13/17 meters metered 12.14 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:26 ~1:18 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80273,9 +80273,36 @@
       <c r="A2434" s="4" t="n">
         <v>46263</v>
       </c>
+      <c r="B2434" t="n">
+        <v>3.404</v>
+      </c>
+      <c r="C2434" t="n">
+        <v>3.112</v>
+      </c>
+      <c r="D2434" t="n">
+        <v>1.472</v>
+      </c>
+      <c r="E2434" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="F2434" t="n">
+        <v>2.233</v>
+      </c>
+      <c r="G2434" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="H2434" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="I2434" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="K2434" t="n">
+        <v>12.136</v>
+      </c>
       <c r="L2434" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81372,7 +81399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81437,249 +81464,249 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B2" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C2" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D2" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E2" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F2" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G2" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H2" t="n">
         <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K2" t="n">
-        <v>12.428</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B3" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C3" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D3" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E3" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F3" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G3" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H3" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K3" t="n">
-        <v>12.534</v>
+        <v>12.428</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B4" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C4" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D4" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E4" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F4" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G4" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H4" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I4" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K4" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B5" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C5" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D5" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E5" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F5" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G5" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H5" t="n">
         <v>0.342</v>
       </c>
       <c r="I5" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K5" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B6" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C6" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D6" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E6" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F6" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G6" t="n">
         <v>0.444</v>
       </c>
       <c r="H6" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I6" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K6" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B7" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C7" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D7" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E7" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F7" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G7" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H7" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I7" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K7" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B8" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C8" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D8" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E8" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F8" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G8" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H8" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K8" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B9" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C9" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D9" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E9" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F9" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G9" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
@@ -81688,27 +81715,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B10" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C10" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D10" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E10" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F10" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G10" t="n">
         <v>0.437</v>
@@ -81720,178 +81747,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B11" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C11" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D11" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E11" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F11" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G11" t="n">
         <v>0.437</v>
       </c>
       <c r="H11" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I11" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B12" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C12" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D12" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E12" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F12" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G12" t="n">
         <v>0.437</v>
       </c>
       <c r="H12" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I12" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B13" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C13" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D13" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F13" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G13" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K13" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B14" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C14" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D14" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E14" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F14" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G14" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B15" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C15" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D15" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E15" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F15" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G15" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H15" t="n">
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K15" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B16" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C16" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D16" t="n">
         <v>1.44</v>
@@ -81900,7 +81927,7 @@
         <v>0.261</v>
       </c>
       <c r="F16" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G16" t="n">
         <v>0.435</v>
@@ -81909,222 +81936,222 @@
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K16" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B17" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C17" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D17" t="n">
         <v>1.44</v>
       </c>
       <c r="E17" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F17" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G17" t="n">
         <v>0.435</v>
       </c>
       <c r="H17" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K17" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B18" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C18" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D18" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E18" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F18" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G18" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H18" t="n">
         <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K18" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B19" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C19" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D19" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F19" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G19" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H19" t="n">
         <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K19" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B20" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C20" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D20" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E20" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G20" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H20" t="n">
         <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K20" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B21" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C21" t="n">
         <v>3.232</v>
       </c>
       <c r="D21" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F21" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G21" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H21" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K21" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B22" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C22" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D22" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E22" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G22" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H22" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I22" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K22" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B23" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C23" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D23" t="n">
         <v>1.435</v>
       </c>
       <c r="E23" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F23" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G23" t="n">
         <v>0.446</v>
@@ -82136,27 +82163,27 @@
         <v>0.712</v>
       </c>
       <c r="K23" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B24" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C24" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D24" t="n">
         <v>1.435</v>
       </c>
       <c r="E24" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F24" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G24" t="n">
         <v>0.446</v>
@@ -82168,59 +82195,59 @@
         <v>0.712</v>
       </c>
       <c r="K24" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B25" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C25" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D25" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E25" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F25" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G25" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H25" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I25" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K25" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B26" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C26" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D26" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E26" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F26" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G26" t="n">
         <v>0.462</v>
@@ -82229,30 +82256,30 @@
         <v>0.343</v>
       </c>
       <c r="I26" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K26" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B27" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C27" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D27" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E27" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F27" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G27" t="n">
         <v>0.462</v>
@@ -82261,100 +82288,97 @@
         <v>0.343</v>
       </c>
       <c r="I27" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K27" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B28" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C28" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D28" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E28" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F28" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G28" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H28" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I28" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K28" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B29" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C29" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D29" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E29" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F29" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G29" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H29" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I29" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J29" t="n">
         <v>0.014</v>
       </c>
       <c r="K29" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B30" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C30" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D30" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E30" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F30" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G30" t="n">
         <v>0.395</v>
@@ -82369,6 +82393,41 @@
         <v>0.014</v>
       </c>
       <c r="K30" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B31" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K31" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82383,7 +82442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82453,270 +82512,270 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B2" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C2" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D2" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E2" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F2" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G2" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H2" t="n">
         <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K2" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
       <c r="L2" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B3" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C3" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D3" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E3" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F3" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G3" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H3" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K3" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
       <c r="L3" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B4" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C4" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D4" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E4" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F4" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G4" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H4" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I4" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K4" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L4" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B5" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C5" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D5" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E5" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F5" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G5" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H5" t="n">
         <v>0.342</v>
       </c>
       <c r="I5" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K5" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L5" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B6" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C6" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D6" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E6" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F6" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G6" t="n">
         <v>0.444</v>
       </c>
       <c r="H6" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I6" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K6" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L6" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B7" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C7" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D7" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E7" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F7" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G7" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H7" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I7" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K7" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L7" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B8" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C8" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D8" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E8" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F8" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G8" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H8" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K8" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L8" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B9" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C9" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D9" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E9" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F9" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G9" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H9" t="n">
         <v>0.367</v>
@@ -82725,30 +82784,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L9" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B10" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C10" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D10" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E10" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F10" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G10" t="n">
         <v>0.437</v>
@@ -82760,196 +82819,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L10" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B11" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C11" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D11" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E11" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F11" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G11" t="n">
         <v>0.437</v>
       </c>
       <c r="H11" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I11" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L11" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B12" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C12" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D12" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E12" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F12" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G12" t="n">
         <v>0.437</v>
       </c>
       <c r="H12" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I12" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L12" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B13" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C13" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D13" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F13" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G13" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K13" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L13" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B14" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C14" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D14" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E14" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F14" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G14" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L14" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B15" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C15" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D15" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E15" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F15" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G15" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H15" t="n">
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K15" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L15" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B16" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C16" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D16" t="n">
         <v>1.44</v>
@@ -82958,7 +83017,7 @@
         <v>0.261</v>
       </c>
       <c r="F16" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G16" t="n">
         <v>0.435</v>
@@ -82967,243 +83026,243 @@
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K16" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L16" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B17" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C17" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D17" t="n">
         <v>1.44</v>
       </c>
       <c r="E17" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F17" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G17" t="n">
         <v>0.435</v>
       </c>
       <c r="H17" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K17" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L17" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B18" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C18" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D18" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E18" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F18" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G18" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H18" t="n">
         <v>0.365</v>
       </c>
       <c r="I18" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K18" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L18" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B19" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C19" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D19" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F19" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G19" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H19" t="n">
         <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K19" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L19" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B20" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C20" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D20" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E20" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G20" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H20" t="n">
         <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K20" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L20" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B21" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C21" t="n">
         <v>3.232</v>
       </c>
       <c r="D21" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F21" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G21" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H21" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K21" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L21" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B22" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C22" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D22" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E22" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G22" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H22" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I22" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K22" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L22" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B23" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C23" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D23" t="n">
         <v>1.435</v>
       </c>
       <c r="E23" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F23" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G23" t="n">
         <v>0.446</v>
@@ -83215,30 +83274,30 @@
         <v>0.712</v>
       </c>
       <c r="K23" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L23" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B24" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C24" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D24" t="n">
         <v>1.435</v>
       </c>
       <c r="E24" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F24" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G24" t="n">
         <v>0.446</v>
@@ -83250,65 +83309,65 @@
         <v>0.712</v>
       </c>
       <c r="K24" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L24" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B25" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C25" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D25" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E25" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F25" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G25" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H25" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I25" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K25" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L25" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B26" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C26" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D26" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E26" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F26" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G26" t="n">
         <v>0.462</v>
@@ -83317,33 +83376,33 @@
         <v>0.343</v>
       </c>
       <c r="I26" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K26" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L26" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B27" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C27" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D27" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E27" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F27" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G27" t="n">
         <v>0.462</v>
@@ -83352,109 +83411,106 @@
         <v>0.343</v>
       </c>
       <c r="I27" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K27" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L27" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B28" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C28" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D28" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E28" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F28" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G28" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H28" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I28" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K28" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L28" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B29" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C29" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D29" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E29" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F29" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G29" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H29" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I29" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J29" t="n">
         <v>0.014</v>
       </c>
       <c r="K29" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L29" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B30" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C30" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D30" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E30" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F30" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G30" t="n">
         <v>0.395</v>
@@ -83469,9 +83525,47 @@
         <v>0.014</v>
       </c>
       <c r="K30" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L30" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B31" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K31" t="n">
         <v>12.277</v>
       </c>
-      <c r="L30" t="n">
+      <c r="L31" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -83912,7 +84006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84012,321 +84106,321 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B2" t="n">
-        <v>1428345</v>
+        <v>1453284</v>
       </c>
       <c r="C2" t="n">
-        <v>613887</v>
+        <v>668222</v>
       </c>
       <c r="D2" t="n">
-        <v>1360335</v>
+        <v>1399375</v>
       </c>
       <c r="E2" t="n">
         <v>9000</v>
       </c>
       <c r="F2" t="n">
-        <v>2000629</v>
+        <v>1997673</v>
       </c>
       <c r="G2" t="n">
-        <v>1229134</v>
+        <v>1229304</v>
       </c>
       <c r="I2" t="n">
-        <v>1516881</v>
+        <v>1526881</v>
       </c>
       <c r="K2" t="n">
-        <v>265281</v>
+        <v>210710</v>
       </c>
       <c r="M2" t="n">
-        <v>2655010</v>
+        <v>2315158</v>
       </c>
       <c r="N2" t="n">
-        <v>275644</v>
+        <v>274632</v>
       </c>
       <c r="O2" t="n">
-        <v>405391</v>
+        <v>404378</v>
       </c>
       <c r="P2" t="n">
         <v>393345</v>
       </c>
       <c r="Q2" t="n">
-        <v>735394</v>
+        <v>702775</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B3" t="n">
-        <v>1453305</v>
+        <v>1428345</v>
       </c>
       <c r="C3" t="n">
-        <v>660021</v>
+        <v>613887</v>
       </c>
       <c r="D3" t="n">
-        <v>1394810</v>
+        <v>1360335</v>
       </c>
       <c r="E3" t="n">
         <v>9000</v>
       </c>
       <c r="F3" t="n">
-        <v>1966997</v>
+        <v>2000629</v>
       </c>
       <c r="G3" t="n">
-        <v>1358589</v>
+        <v>1229134</v>
       </c>
       <c r="I3" t="n">
-        <v>1530881</v>
+        <v>1516881</v>
       </c>
       <c r="K3" t="n">
-        <v>224505</v>
+        <v>265281</v>
       </c>
       <c r="M3" t="n">
-        <v>2605275</v>
+        <v>2655010</v>
       </c>
       <c r="N3" t="n">
-        <v>273068</v>
+        <v>275644</v>
       </c>
       <c r="O3" t="n">
-        <v>402811</v>
+        <v>405391</v>
       </c>
       <c r="P3" t="n">
-        <v>368707</v>
+        <v>393345</v>
       </c>
       <c r="Q3" t="n">
-        <v>750038</v>
+        <v>735394</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B4" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C4" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D4" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E4" t="n">
         <v>9000</v>
       </c>
       <c r="F4" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G4" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I4" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K4" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M4" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N4" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O4" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P4" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q4" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B5" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C5" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D5" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E5" t="n">
         <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G5" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I5" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K5" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M5" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N5" t="n">
         <v>214475</v>
       </c>
       <c r="O5" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P5" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q5" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B6" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C6" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D6" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E6" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F6" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G6" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I6" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K6" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M6" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P6" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q6" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B7" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C7" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D7" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E7" t="n">
         <v>9200</v>
       </c>
       <c r="F7" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G7" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I7" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K7" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M7" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P7" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q7" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B8" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C8" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D8" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G8" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I8" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K8" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M8" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N8" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P8" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q8" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B9" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C9" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D9" t="n">
         <v>1336369</v>
@@ -84335,28 +84429,28 @@
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G9" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I9" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K9" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M9" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N9" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O9" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P9" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q9" t="n">
         <v>710782</v>
@@ -84364,34 +84458,34 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B10" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C10" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D10" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G10" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I10" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K10" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M10" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
@@ -84400,7 +84494,7 @@
         <v>238857</v>
       </c>
       <c r="P10" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q10" t="n">
         <v>710782</v>
@@ -84408,43 +84502,43 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B11" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C11" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D11" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G11" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I11" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K11" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M11" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N11" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P11" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q11" t="n">
         <v>710782</v>
@@ -84452,201 +84546,201 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B12" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C12" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D12" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G12" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I12" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K12" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M12" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N12" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O12" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P12" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q12" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B13" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C13" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D13" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G13" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I13" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K13" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M13" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N13" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O13" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P13" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q13" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B14" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C14" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D14" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G14" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I14" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K14" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M14" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N14" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O14" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P14" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q14" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B15" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C15" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D15" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E15" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G15" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I15" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K15" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M15" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N15" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O15" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P15" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q15" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B16" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C16" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D16" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E16" t="n">
         <v>9400</v>
       </c>
       <c r="F16" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G16" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I16" t="n">
         <v>1493578</v>
@@ -84655,7 +84749,7 @@
         <v>270165</v>
       </c>
       <c r="M16" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N16" t="n">
         <v>214475</v>
@@ -84667,39 +84761,39 @@
         <v>380581</v>
       </c>
       <c r="Q16" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B17" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C17" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D17" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E17" t="n">
         <v>9400</v>
       </c>
       <c r="F17" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G17" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I17" t="n">
         <v>1493578</v>
       </c>
       <c r="K17" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M17" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N17" t="n">
         <v>214475</v>
@@ -84708,153 +84802,153 @@
         <v>236857</v>
       </c>
       <c r="P17" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q17" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B18" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C18" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D18" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E18" t="n">
         <v>9400</v>
       </c>
       <c r="F18" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G18" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I18" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K18" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M18" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N18" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O18" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P18" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q18" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B19" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C19" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D19" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E19" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F19" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G19" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I19" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K19" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M19" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N19" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O19" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P19" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q19" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B20" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C20" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D20" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E20" t="n">
         <v>9200</v>
       </c>
       <c r="F20" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G20" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I20" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K20" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M20" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N20" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O20" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P20" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q20" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B21" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C21" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D21" t="n">
         <v>1438502</v>
@@ -84863,107 +84957,107 @@
         <v>9200</v>
       </c>
       <c r="F21" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G21" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I21" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K21" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M21" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N21" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O21" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P21" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q21" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B22" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C22" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D22" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E22" t="n">
         <v>9200</v>
       </c>
       <c r="F22" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G22" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I22" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K22" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M22" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N22" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O22" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P22" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q22" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B23" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C23" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D23" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E23" t="n">
         <v>9200</v>
       </c>
       <c r="F23" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G23" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I23" t="n">
         <v>1488515</v>
       </c>
       <c r="K23" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M23" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N23" t="n">
         <v>214475</v>
@@ -84972,7 +85066,7 @@
         <v>247857</v>
       </c>
       <c r="P23" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q23" t="n">
         <v>738429</v>
@@ -84980,34 +85074,34 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B24" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C24" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D24" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E24" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F24" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G24" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I24" t="n">
         <v>1488515</v>
       </c>
       <c r="K24" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M24" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N24" t="n">
         <v>214475</v>
@@ -85016,7 +85110,7 @@
         <v>247857</v>
       </c>
       <c r="P24" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q24" t="n">
         <v>738429</v>
@@ -85024,78 +85118,78 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B25" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C25" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D25" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E25" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F25" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G25" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I25" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K25" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M25" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N25" t="n">
         <v>214475</v>
       </c>
       <c r="O25" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P25" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q25" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B26" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C26" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D26" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E26" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F26" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G26" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I26" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K26" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M26" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N26" t="n">
         <v>214475</v>
@@ -85104,42 +85198,42 @@
         <v>264857</v>
       </c>
       <c r="P26" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q26" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B27" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C27" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D27" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E27" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F27" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G27" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I27" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K27" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M27" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N27" t="n">
         <v>214475</v>
@@ -85148,101 +85242,98 @@
         <v>264857</v>
       </c>
       <c r="P27" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q27" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B28" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C28" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D28" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E28" t="n">
         <v>9300</v>
       </c>
       <c r="F28" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G28" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I28" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K28" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M28" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N28" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O28" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P28" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q28" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R28" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B29" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C29" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D29" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E29" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F29" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G29" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I29" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K29" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M29" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N29" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O29" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P29" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q29" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R29" t="n">
         <v>15000</v>
@@ -85250,40 +85341,40 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B30" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C30" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D30" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E30" t="n">
         <v>9100</v>
       </c>
       <c r="F30" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G30" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I30" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K30" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M30" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N30" t="n">
         <v>189475</v>
       </c>
       <c r="O30" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P30" t="n">
         <v>375660</v>
@@ -85292,6 +85383,53 @@
         <v>773586</v>
       </c>
       <c r="R30" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B31" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C31" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E31" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K31" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M31" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N31" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O31" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P31" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R31" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 31/119] 2026-08-28 ~ 13/17 meters metered 12.27 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:27 ~1:18 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80263,9 +80263,36 @@
       <c r="A2433" s="4" t="n">
         <v>46262</v>
       </c>
+      <c r="B2433" t="n">
+        <v>3.236</v>
+      </c>
+      <c r="C2433" t="n">
+        <v>3.017</v>
+      </c>
+      <c r="D2433" t="n">
+        <v>1.456</v>
+      </c>
+      <c r="E2433" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="F2433" t="n">
+        <v>2.543</v>
+      </c>
+      <c r="G2433" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H2433" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="I2433" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="K2433" t="n">
+        <v>12.267</v>
+      </c>
       <c r="L2433" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81399,7 +81426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81464,281 +81491,281 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B2" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C2" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D2" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E2" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F2" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G2" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H2" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I2" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>12.136</v>
+        <v>12.269</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B3" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C3" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D3" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E3" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F3" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G3" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H3" t="n">
         <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K3" t="n">
-        <v>12.428</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B4" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C4" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D4" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E4" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F4" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G4" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H4" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K4" t="n">
-        <v>12.534</v>
+        <v>12.428</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B5" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C5" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D5" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E5" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F5" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G5" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H5" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I5" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K5" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B6" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C6" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D6" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E6" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F6" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G6" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H6" t="n">
         <v>0.342</v>
       </c>
       <c r="I6" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K6" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B7" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C7" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D7" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E7" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F7" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G7" t="n">
         <v>0.444</v>
       </c>
       <c r="H7" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I7" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K7" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B8" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C8" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D8" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E8" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F8" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G8" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H8" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I8" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K8" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B9" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C9" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D9" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E9" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F9" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G9" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H9" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K9" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B10" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C10" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D10" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E10" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F10" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G10" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
@@ -81747,27 +81774,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B11" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C11" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D11" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E11" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F11" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G11" t="n">
         <v>0.437</v>
@@ -81779,178 +81806,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B12" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C12" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D12" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E12" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F12" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G12" t="n">
         <v>0.437</v>
       </c>
       <c r="H12" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I12" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B13" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C13" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D13" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E13" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F13" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G13" t="n">
         <v>0.437</v>
       </c>
       <c r="H13" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I13" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B14" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C14" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D14" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F14" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G14" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K14" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B15" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C15" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D15" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E15" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F15" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G15" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H15" t="n">
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B16" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C16" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D16" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E16" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F16" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G16" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H16" t="n">
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K16" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B17" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C17" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D17" t="n">
         <v>1.44</v>
@@ -81959,7 +81986,7 @@
         <v>0.261</v>
       </c>
       <c r="F17" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G17" t="n">
         <v>0.435</v>
@@ -81968,222 +81995,222 @@
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K17" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B18" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C18" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D18" t="n">
         <v>1.44</v>
       </c>
       <c r="E18" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F18" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G18" t="n">
         <v>0.435</v>
       </c>
       <c r="H18" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K18" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B19" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C19" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D19" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E19" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F19" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G19" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H19" t="n">
         <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K19" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B20" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C20" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D20" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F20" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G20" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H20" t="n">
         <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K20" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B21" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C21" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D21" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E21" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G21" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H21" t="n">
         <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K21" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B22" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C22" t="n">
         <v>3.232</v>
       </c>
       <c r="D22" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F22" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G22" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H22" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K22" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B23" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C23" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D23" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E23" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G23" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H23" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I23" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K23" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B24" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C24" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D24" t="n">
         <v>1.435</v>
       </c>
       <c r="E24" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F24" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G24" t="n">
         <v>0.446</v>
@@ -82195,27 +82222,27 @@
         <v>0.712</v>
       </c>
       <c r="K24" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B25" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C25" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D25" t="n">
         <v>1.435</v>
       </c>
       <c r="E25" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F25" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G25" t="n">
         <v>0.446</v>
@@ -82227,59 +82254,59 @@
         <v>0.712</v>
       </c>
       <c r="K25" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B26" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C26" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D26" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E26" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F26" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G26" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H26" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I26" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K26" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B27" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C27" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D27" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E27" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F27" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G27" t="n">
         <v>0.462</v>
@@ -82288,30 +82315,30 @@
         <v>0.343</v>
       </c>
       <c r="I27" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K27" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B28" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C28" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D28" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E28" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F28" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G28" t="n">
         <v>0.462</v>
@@ -82320,100 +82347,97 @@
         <v>0.343</v>
       </c>
       <c r="I28" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K28" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B29" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C29" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D29" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E29" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F29" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G29" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H29" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I29" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K29" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B30" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C30" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D30" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E30" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F30" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G30" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H30" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I30" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J30" t="n">
         <v>0.014</v>
       </c>
       <c r="K30" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B31" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C31" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D31" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E31" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F31" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G31" t="n">
         <v>0.395</v>
@@ -82428,6 +82452,41 @@
         <v>0.014</v>
       </c>
       <c r="K31" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B32" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K32" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82442,7 +82501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82512,305 +82571,305 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B2" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C2" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D2" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E2" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F2" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G2" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H2" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I2" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
       <c r="L2" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B3" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C3" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D3" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E3" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F3" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G3" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H3" t="n">
         <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K3" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
       <c r="L3" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B4" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C4" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D4" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E4" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F4" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G4" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H4" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K4" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
       <c r="L4" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B5" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C5" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D5" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E5" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F5" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G5" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H5" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I5" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K5" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L5" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B6" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C6" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D6" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E6" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F6" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G6" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H6" t="n">
         <v>0.342</v>
       </c>
       <c r="I6" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K6" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L6" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B7" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C7" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D7" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E7" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F7" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G7" t="n">
         <v>0.444</v>
       </c>
       <c r="H7" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I7" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K7" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L7" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B8" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C8" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D8" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E8" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F8" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G8" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H8" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I8" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K8" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L8" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B9" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C9" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D9" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E9" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F9" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G9" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H9" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K9" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L9" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B10" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C10" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D10" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E10" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F10" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G10" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H10" t="n">
         <v>0.367</v>
@@ -82819,30 +82878,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L10" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B11" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C11" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D11" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E11" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F11" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G11" t="n">
         <v>0.437</v>
@@ -82854,196 +82913,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L11" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B12" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C12" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D12" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E12" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F12" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G12" t="n">
         <v>0.437</v>
       </c>
       <c r="H12" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I12" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L12" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B13" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C13" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D13" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E13" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F13" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G13" t="n">
         <v>0.437</v>
       </c>
       <c r="H13" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I13" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L13" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B14" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C14" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D14" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F14" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G14" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
       </c>
       <c r="I14" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K14" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L14" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B15" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C15" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D15" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E15" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F15" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G15" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H15" t="n">
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L15" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B16" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C16" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D16" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E16" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F16" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G16" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H16" t="n">
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K16" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L16" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B17" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C17" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D17" t="n">
         <v>1.44</v>
@@ -83052,7 +83111,7 @@
         <v>0.261</v>
       </c>
       <c r="F17" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G17" t="n">
         <v>0.435</v>
@@ -83061,243 +83120,243 @@
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K17" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L17" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B18" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C18" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D18" t="n">
         <v>1.44</v>
       </c>
       <c r="E18" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F18" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G18" t="n">
         <v>0.435</v>
       </c>
       <c r="H18" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K18" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L18" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B19" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C19" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D19" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E19" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F19" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G19" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H19" t="n">
         <v>0.365</v>
       </c>
       <c r="I19" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K19" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L19" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B20" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C20" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D20" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F20" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G20" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H20" t="n">
         <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K20" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L20" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B21" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C21" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D21" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E21" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G21" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H21" t="n">
         <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K21" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L21" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B22" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C22" t="n">
         <v>3.232</v>
       </c>
       <c r="D22" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F22" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G22" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H22" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K22" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L22" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B23" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C23" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D23" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E23" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G23" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H23" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I23" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K23" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L23" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B24" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C24" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D24" t="n">
         <v>1.435</v>
       </c>
       <c r="E24" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F24" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G24" t="n">
         <v>0.446</v>
@@ -83309,30 +83368,30 @@
         <v>0.712</v>
       </c>
       <c r="K24" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L24" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B25" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C25" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D25" t="n">
         <v>1.435</v>
       </c>
       <c r="E25" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F25" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G25" t="n">
         <v>0.446</v>
@@ -83344,65 +83403,65 @@
         <v>0.712</v>
       </c>
       <c r="K25" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L25" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B26" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C26" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D26" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E26" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F26" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G26" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H26" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I26" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K26" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L26" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B27" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C27" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D27" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E27" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F27" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G27" t="n">
         <v>0.462</v>
@@ -83411,33 +83470,33 @@
         <v>0.343</v>
       </c>
       <c r="I27" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K27" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L27" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B28" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C28" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D28" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E28" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F28" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G28" t="n">
         <v>0.462</v>
@@ -83446,109 +83505,106 @@
         <v>0.343</v>
       </c>
       <c r="I28" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K28" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L28" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B29" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C29" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D29" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E29" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F29" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G29" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H29" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I29" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K29" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L29" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B30" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C30" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D30" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E30" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F30" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G30" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H30" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I30" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J30" t="n">
         <v>0.014</v>
       </c>
       <c r="K30" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L30" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B31" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C31" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D31" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E31" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F31" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G31" t="n">
         <v>0.395</v>
@@ -83563,9 +83619,47 @@
         <v>0.014</v>
       </c>
       <c r="K31" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L31" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B32" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K32" t="n">
         <v>12.277</v>
       </c>
-      <c r="L31" t="n">
+      <c r="L32" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -84006,7 +84100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84106,365 +84200,365 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B2" t="n">
-        <v>1453284</v>
+        <v>1326845</v>
       </c>
       <c r="C2" t="n">
-        <v>668222</v>
+        <v>630343</v>
       </c>
       <c r="D2" t="n">
-        <v>1399375</v>
+        <v>1389820</v>
       </c>
       <c r="E2" t="n">
         <v>9000</v>
       </c>
       <c r="F2" t="n">
-        <v>1997673</v>
+        <v>1898634</v>
       </c>
       <c r="G2" t="n">
-        <v>1229304</v>
+        <v>1230443</v>
       </c>
       <c r="I2" t="n">
-        <v>1526881</v>
+        <v>1509954</v>
       </c>
       <c r="K2" t="n">
-        <v>210710</v>
+        <v>223405</v>
       </c>
       <c r="M2" t="n">
-        <v>2315158</v>
+        <v>2637144</v>
       </c>
       <c r="N2" t="n">
-        <v>274632</v>
+        <v>322000</v>
       </c>
       <c r="O2" t="n">
-        <v>404378</v>
+        <v>445186</v>
       </c>
       <c r="P2" t="n">
-        <v>393345</v>
+        <v>392284</v>
       </c>
       <c r="Q2" t="n">
-        <v>702775</v>
+        <v>707427</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B3" t="n">
-        <v>1428345</v>
+        <v>1453284</v>
       </c>
       <c r="C3" t="n">
-        <v>613887</v>
+        <v>668222</v>
       </c>
       <c r="D3" t="n">
-        <v>1360335</v>
+        <v>1399375</v>
       </c>
       <c r="E3" t="n">
         <v>9000</v>
       </c>
       <c r="F3" t="n">
-        <v>2000629</v>
+        <v>1997673</v>
       </c>
       <c r="G3" t="n">
-        <v>1229134</v>
+        <v>1229304</v>
       </c>
       <c r="I3" t="n">
-        <v>1516881</v>
+        <v>1526881</v>
       </c>
       <c r="K3" t="n">
-        <v>265281</v>
+        <v>210710</v>
       </c>
       <c r="M3" t="n">
-        <v>2655010</v>
+        <v>2315158</v>
       </c>
       <c r="N3" t="n">
-        <v>275644</v>
+        <v>274632</v>
       </c>
       <c r="O3" t="n">
-        <v>405391</v>
+        <v>404378</v>
       </c>
       <c r="P3" t="n">
         <v>393345</v>
       </c>
       <c r="Q3" t="n">
-        <v>735394</v>
+        <v>702775</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B4" t="n">
-        <v>1453305</v>
+        <v>1428345</v>
       </c>
       <c r="C4" t="n">
-        <v>660021</v>
+        <v>613887</v>
       </c>
       <c r="D4" t="n">
-        <v>1394810</v>
+        <v>1360335</v>
       </c>
       <c r="E4" t="n">
         <v>9000</v>
       </c>
       <c r="F4" t="n">
-        <v>1966997</v>
+        <v>2000629</v>
       </c>
       <c r="G4" t="n">
-        <v>1358589</v>
+        <v>1229134</v>
       </c>
       <c r="I4" t="n">
-        <v>1530881</v>
+        <v>1516881</v>
       </c>
       <c r="K4" t="n">
-        <v>224505</v>
+        <v>265281</v>
       </c>
       <c r="M4" t="n">
-        <v>2605275</v>
+        <v>2655010</v>
       </c>
       <c r="N4" t="n">
-        <v>273068</v>
+        <v>275644</v>
       </c>
       <c r="O4" t="n">
-        <v>402811</v>
+        <v>405391</v>
       </c>
       <c r="P4" t="n">
-        <v>368707</v>
+        <v>393345</v>
       </c>
       <c r="Q4" t="n">
-        <v>750038</v>
+        <v>735394</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B5" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C5" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D5" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E5" t="n">
         <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G5" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I5" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K5" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M5" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N5" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O5" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P5" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q5" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B6" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C6" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D6" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E6" t="n">
         <v>9000</v>
       </c>
       <c r="F6" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G6" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I6" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K6" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M6" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N6" t="n">
         <v>214475</v>
       </c>
       <c r="O6" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P6" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q6" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B7" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C7" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D7" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E7" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F7" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G7" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I7" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K7" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M7" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P7" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q7" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B8" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C8" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D8" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E8" t="n">
         <v>9200</v>
       </c>
       <c r="F8" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G8" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I8" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K8" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M8" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P8" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q8" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B9" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C9" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D9" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G9" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I9" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K9" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M9" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N9" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P9" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q9" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B10" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C10" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D10" t="n">
         <v>1336369</v>
@@ -84473,28 +84567,28 @@
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G10" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I10" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K10" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M10" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N10" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O10" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P10" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q10" t="n">
         <v>710782</v>
@@ -84502,34 +84596,34 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B11" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C11" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D11" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G11" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I11" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K11" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M11" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
@@ -84538,7 +84632,7 @@
         <v>238857</v>
       </c>
       <c r="P11" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q11" t="n">
         <v>710782</v>
@@ -84546,43 +84640,43 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B12" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C12" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D12" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G12" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I12" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K12" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M12" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N12" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P12" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q12" t="n">
         <v>710782</v>
@@ -84590,201 +84684,201 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B13" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C13" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D13" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G13" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I13" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K13" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M13" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N13" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O13" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P13" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q13" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B14" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C14" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D14" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G14" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I14" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K14" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M14" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N14" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O14" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P14" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q14" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B15" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C15" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D15" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G15" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I15" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K15" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M15" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N15" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O15" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P15" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q15" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B16" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C16" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D16" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E16" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G16" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I16" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K16" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M16" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N16" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O16" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P16" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q16" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B17" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C17" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D17" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E17" t="n">
         <v>9400</v>
       </c>
       <c r="F17" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G17" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I17" t="n">
         <v>1493578</v>
@@ -84793,7 +84887,7 @@
         <v>270165</v>
       </c>
       <c r="M17" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N17" t="n">
         <v>214475</v>
@@ -84805,39 +84899,39 @@
         <v>380581</v>
       </c>
       <c r="Q17" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B18" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C18" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D18" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E18" t="n">
         <v>9400</v>
       </c>
       <c r="F18" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G18" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I18" t="n">
         <v>1493578</v>
       </c>
       <c r="K18" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M18" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N18" t="n">
         <v>214475</v>
@@ -84846,153 +84940,153 @@
         <v>236857</v>
       </c>
       <c r="P18" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q18" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B19" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C19" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D19" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E19" t="n">
         <v>9400</v>
       </c>
       <c r="F19" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G19" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I19" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K19" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M19" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N19" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O19" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P19" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q19" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B20" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C20" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D20" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E20" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F20" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G20" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I20" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K20" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M20" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N20" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O20" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P20" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q20" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B21" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C21" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D21" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E21" t="n">
         <v>9200</v>
       </c>
       <c r="F21" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G21" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I21" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K21" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M21" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N21" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O21" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P21" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q21" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B22" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C22" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D22" t="n">
         <v>1438502</v>
@@ -85001,107 +85095,107 @@
         <v>9200</v>
       </c>
       <c r="F22" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G22" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I22" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K22" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M22" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N22" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O22" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P22" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q22" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B23" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C23" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D23" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E23" t="n">
         <v>9200</v>
       </c>
       <c r="F23" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G23" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I23" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K23" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M23" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N23" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O23" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P23" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q23" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B24" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C24" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D24" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E24" t="n">
         <v>9200</v>
       </c>
       <c r="F24" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G24" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I24" t="n">
         <v>1488515</v>
       </c>
       <c r="K24" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M24" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N24" t="n">
         <v>214475</v>
@@ -85110,7 +85204,7 @@
         <v>247857</v>
       </c>
       <c r="P24" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q24" t="n">
         <v>738429</v>
@@ -85118,34 +85212,34 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B25" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C25" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D25" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E25" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F25" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G25" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I25" t="n">
         <v>1488515</v>
       </c>
       <c r="K25" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M25" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N25" t="n">
         <v>214475</v>
@@ -85154,7 +85248,7 @@
         <v>247857</v>
       </c>
       <c r="P25" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q25" t="n">
         <v>738429</v>
@@ -85162,78 +85256,78 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B26" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C26" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D26" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E26" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F26" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G26" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I26" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K26" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M26" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N26" t="n">
         <v>214475</v>
       </c>
       <c r="O26" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P26" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q26" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B27" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C27" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D27" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E27" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F27" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G27" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I27" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K27" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M27" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N27" t="n">
         <v>214475</v>
@@ -85242,42 +85336,42 @@
         <v>264857</v>
       </c>
       <c r="P27" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q27" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B28" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C28" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D28" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E28" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F28" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G28" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I28" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K28" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M28" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N28" t="n">
         <v>214475</v>
@@ -85286,101 +85380,98 @@
         <v>264857</v>
       </c>
       <c r="P28" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q28" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B29" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C29" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D29" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E29" t="n">
         <v>9300</v>
       </c>
       <c r="F29" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G29" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I29" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K29" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M29" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N29" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O29" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P29" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q29" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R29" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B30" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C30" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D30" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E30" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F30" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G30" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I30" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K30" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M30" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N30" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O30" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P30" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q30" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R30" t="n">
         <v>15000</v>
@@ -85388,40 +85479,40 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B31" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C31" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D31" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E31" t="n">
         <v>9100</v>
       </c>
       <c r="F31" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G31" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I31" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K31" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M31" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N31" t="n">
         <v>189475</v>
       </c>
       <c r="O31" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P31" t="n">
         <v>375660</v>
@@ -85430,6 +85521,53 @@
         <v>773586</v>
       </c>
       <c r="R31" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B32" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C32" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E32" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K32" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M32" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N32" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O32" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P32" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R32" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 32/119] 2026-08-27 ~ 13/17 meters metered 12.53 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:28 ~1:17 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80253,9 +80253,36 @@
       <c r="A2432" s="4" t="n">
         <v>46261</v>
       </c>
+      <c r="B2432" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="C2432" t="n">
+        <v>3.254</v>
+      </c>
+      <c r="D2432" t="n">
+        <v>1.491</v>
+      </c>
+      <c r="E2432" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F2432" t="n">
+        <v>2.594</v>
+      </c>
+      <c r="G2432" t="n">
+        <v>0.715</v>
+      </c>
+      <c r="H2432" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="I2432" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="K2432" t="n">
+        <v>12.526</v>
+      </c>
       <c r="L2432" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81426,7 +81453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81491,313 +81518,313 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B2" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C2" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D2" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E2" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F2" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G2" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H2" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K2" t="n">
-        <v>12.269</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B3" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C3" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D3" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E3" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F3" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G3" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H3" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I3" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>12.136</v>
+        <v>12.269</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B4" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C4" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D4" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E4" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F4" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G4" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H4" t="n">
         <v>0.379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K4" t="n">
-        <v>12.428</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B5" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C5" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D5" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E5" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F5" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G5" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H5" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I5" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K5" t="n">
-        <v>12.534</v>
+        <v>12.428</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B6" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C6" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D6" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E6" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F6" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G6" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H6" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I6" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K6" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B7" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C7" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D7" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E7" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F7" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G7" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H7" t="n">
         <v>0.342</v>
       </c>
       <c r="I7" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K7" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B8" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C8" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D8" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E8" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F8" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G8" t="n">
         <v>0.444</v>
       </c>
       <c r="H8" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I8" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K8" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B9" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C9" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D9" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E9" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F9" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G9" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H9" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I9" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K9" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B10" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C10" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D10" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E10" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F10" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G10" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H10" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K10" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B11" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C11" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D11" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E11" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F11" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G11" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
@@ -81806,27 +81833,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B12" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C12" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D12" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E12" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F12" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G12" t="n">
         <v>0.437</v>
@@ -81838,178 +81865,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B13" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C13" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D13" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E13" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F13" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G13" t="n">
         <v>0.437</v>
       </c>
       <c r="H13" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I13" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B14" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C14" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D14" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E14" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F14" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G14" t="n">
         <v>0.437</v>
       </c>
       <c r="H14" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I14" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B15" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C15" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D15" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F15" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G15" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H15" t="n">
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K15" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B16" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C16" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D16" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E16" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F16" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G16" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H16" t="n">
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B17" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C17" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D17" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E17" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F17" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G17" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H17" t="n">
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K17" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B18" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C18" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D18" t="n">
         <v>1.44</v>
@@ -82018,7 +82045,7 @@
         <v>0.261</v>
       </c>
       <c r="F18" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G18" t="n">
         <v>0.435</v>
@@ -82027,222 +82054,222 @@
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K18" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B19" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C19" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D19" t="n">
         <v>1.44</v>
       </c>
       <c r="E19" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F19" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G19" t="n">
         <v>0.435</v>
       </c>
       <c r="H19" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K19" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B20" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C20" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D20" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E20" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F20" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G20" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H20" t="n">
         <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K20" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B21" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C21" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D21" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F21" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G21" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H21" t="n">
         <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K21" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B22" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C22" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D22" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E22" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G22" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H22" t="n">
         <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K22" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B23" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C23" t="n">
         <v>3.232</v>
       </c>
       <c r="D23" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F23" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G23" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H23" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K23" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B24" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C24" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D24" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E24" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G24" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H24" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I24" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K24" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B25" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C25" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D25" t="n">
         <v>1.435</v>
       </c>
       <c r="E25" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F25" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G25" t="n">
         <v>0.446</v>
@@ -82254,27 +82281,27 @@
         <v>0.712</v>
       </c>
       <c r="K25" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B26" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C26" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D26" t="n">
         <v>1.435</v>
       </c>
       <c r="E26" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F26" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G26" t="n">
         <v>0.446</v>
@@ -82286,59 +82313,59 @@
         <v>0.712</v>
       </c>
       <c r="K26" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B27" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C27" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D27" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E27" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F27" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G27" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H27" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I27" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K27" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B28" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C28" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D28" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E28" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F28" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G28" t="n">
         <v>0.462</v>
@@ -82347,30 +82374,30 @@
         <v>0.343</v>
       </c>
       <c r="I28" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K28" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B29" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C29" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D29" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E29" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F29" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G29" t="n">
         <v>0.462</v>
@@ -82379,100 +82406,97 @@
         <v>0.343</v>
       </c>
       <c r="I29" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K29" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B30" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C30" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D30" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E30" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F30" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G30" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H30" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I30" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K30" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B31" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C31" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D31" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E31" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F31" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G31" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H31" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I31" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J31" t="n">
         <v>0.014</v>
       </c>
       <c r="K31" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B32" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C32" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D32" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E32" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F32" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G32" t="n">
         <v>0.395</v>
@@ -82487,6 +82511,41 @@
         <v>0.014</v>
       </c>
       <c r="K32" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B33" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C33" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K33" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82501,7 +82560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82571,340 +82630,340 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B2" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C2" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D2" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E2" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F2" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G2" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H2" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K2" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
       <c r="L2" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B3" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C3" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D3" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E3" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F3" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G3" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H3" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I3" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
       <c r="L3" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B4" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C4" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D4" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E4" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F4" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G4" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H4" t="n">
         <v>0.379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K4" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
       <c r="L4" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B5" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C5" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D5" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E5" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F5" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G5" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H5" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I5" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K5" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
       <c r="L5" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B6" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C6" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D6" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E6" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F6" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G6" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H6" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I6" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K6" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L6" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B7" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C7" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D7" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E7" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F7" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G7" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H7" t="n">
         <v>0.342</v>
       </c>
       <c r="I7" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K7" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L7" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B8" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C8" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D8" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E8" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F8" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G8" t="n">
         <v>0.444</v>
       </c>
       <c r="H8" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I8" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K8" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L8" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B9" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C9" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D9" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E9" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F9" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G9" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H9" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I9" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K9" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L9" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B10" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C10" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D10" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E10" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F10" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G10" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H10" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K10" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L10" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B11" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C11" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D11" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E11" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F11" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G11" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H11" t="n">
         <v>0.367</v>
@@ -82913,30 +82972,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L11" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B12" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C12" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D12" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E12" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F12" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G12" t="n">
         <v>0.437</v>
@@ -82948,196 +83007,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L12" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B13" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C13" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D13" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E13" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F13" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G13" t="n">
         <v>0.437</v>
       </c>
       <c r="H13" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I13" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L13" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B14" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C14" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D14" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E14" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F14" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G14" t="n">
         <v>0.437</v>
       </c>
       <c r="H14" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I14" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L14" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B15" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C15" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D15" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F15" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G15" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H15" t="n">
         <v>0.367</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K15" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L15" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B16" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C16" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D16" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E16" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F16" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G16" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H16" t="n">
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L16" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B17" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C17" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D17" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E17" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F17" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G17" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H17" t="n">
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K17" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L17" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B18" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C18" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D18" t="n">
         <v>1.44</v>
@@ -83146,7 +83205,7 @@
         <v>0.261</v>
       </c>
       <c r="F18" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G18" t="n">
         <v>0.435</v>
@@ -83155,243 +83214,243 @@
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K18" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L18" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B19" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C19" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D19" t="n">
         <v>1.44</v>
       </c>
       <c r="E19" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F19" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G19" t="n">
         <v>0.435</v>
       </c>
       <c r="H19" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K19" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L19" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B20" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C20" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D20" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E20" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F20" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G20" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H20" t="n">
         <v>0.365</v>
       </c>
       <c r="I20" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K20" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L20" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B21" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C21" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D21" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F21" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G21" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H21" t="n">
         <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K21" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L21" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B22" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C22" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D22" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E22" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G22" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H22" t="n">
         <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K22" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L22" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B23" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C23" t="n">
         <v>3.232</v>
       </c>
       <c r="D23" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F23" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G23" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H23" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K23" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L23" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B24" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C24" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D24" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E24" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G24" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H24" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I24" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K24" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L24" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B25" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C25" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D25" t="n">
         <v>1.435</v>
       </c>
       <c r="E25" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F25" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G25" t="n">
         <v>0.446</v>
@@ -83403,30 +83462,30 @@
         <v>0.712</v>
       </c>
       <c r="K25" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L25" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B26" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C26" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D26" t="n">
         <v>1.435</v>
       </c>
       <c r="E26" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F26" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G26" t="n">
         <v>0.446</v>
@@ -83438,65 +83497,65 @@
         <v>0.712</v>
       </c>
       <c r="K26" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L26" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B27" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C27" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D27" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E27" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F27" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G27" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H27" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I27" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K27" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L27" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B28" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C28" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D28" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E28" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F28" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G28" t="n">
         <v>0.462</v>
@@ -83505,33 +83564,33 @@
         <v>0.343</v>
       </c>
       <c r="I28" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K28" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L28" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B29" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C29" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D29" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E29" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F29" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G29" t="n">
         <v>0.462</v>
@@ -83540,109 +83599,106 @@
         <v>0.343</v>
       </c>
       <c r="I29" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K29" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L29" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B30" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C30" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D30" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E30" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F30" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G30" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H30" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I30" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K30" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L30" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B31" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C31" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D31" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E31" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F31" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G31" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H31" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I31" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J31" t="n">
         <v>0.014</v>
       </c>
       <c r="K31" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L31" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B32" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C32" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D32" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E32" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F32" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G32" t="n">
         <v>0.395</v>
@@ -83657,9 +83713,47 @@
         <v>0.014</v>
       </c>
       <c r="K32" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L32" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B33" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C33" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K33" t="n">
         <v>12.277</v>
       </c>
-      <c r="L32" t="n">
+      <c r="L33" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -84100,7 +84194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84200,409 +84294,409 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B2" t="n">
-        <v>1326845</v>
+        <v>1383237</v>
       </c>
       <c r="C2" t="n">
-        <v>630343</v>
+        <v>642612</v>
       </c>
       <c r="D2" t="n">
-        <v>1389820</v>
+        <v>1376983</v>
       </c>
       <c r="E2" t="n">
         <v>9000</v>
       </c>
       <c r="F2" t="n">
-        <v>1898634</v>
+        <v>1886772</v>
       </c>
       <c r="G2" t="n">
-        <v>1230443</v>
+        <v>1487288</v>
       </c>
       <c r="I2" t="n">
-        <v>1509954</v>
+        <v>1545952</v>
       </c>
       <c r="K2" t="n">
-        <v>223405</v>
+        <v>145193</v>
       </c>
       <c r="M2" t="n">
-        <v>2637144</v>
+        <v>2689526</v>
       </c>
       <c r="N2" t="n">
-        <v>322000</v>
+        <v>309125</v>
       </c>
       <c r="O2" t="n">
-        <v>445186</v>
+        <v>432534</v>
       </c>
       <c r="P2" t="n">
-        <v>392284</v>
+        <v>399049</v>
       </c>
       <c r="Q2" t="n">
-        <v>707427</v>
+        <v>681693</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B3" t="n">
-        <v>1453284</v>
+        <v>1326845</v>
       </c>
       <c r="C3" t="n">
-        <v>668222</v>
+        <v>630343</v>
       </c>
       <c r="D3" t="n">
-        <v>1399375</v>
+        <v>1389820</v>
       </c>
       <c r="E3" t="n">
         <v>9000</v>
       </c>
       <c r="F3" t="n">
-        <v>1997673</v>
+        <v>1898634</v>
       </c>
       <c r="G3" t="n">
-        <v>1229304</v>
+        <v>1230443</v>
       </c>
       <c r="I3" t="n">
-        <v>1526881</v>
+        <v>1509954</v>
       </c>
       <c r="K3" t="n">
-        <v>210710</v>
+        <v>223405</v>
       </c>
       <c r="M3" t="n">
-        <v>2315158</v>
+        <v>2637144</v>
       </c>
       <c r="N3" t="n">
-        <v>274632</v>
+        <v>322000</v>
       </c>
       <c r="O3" t="n">
-        <v>404378</v>
+        <v>445186</v>
       </c>
       <c r="P3" t="n">
-        <v>393345</v>
+        <v>392284</v>
       </c>
       <c r="Q3" t="n">
-        <v>702775</v>
+        <v>707427</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B4" t="n">
-        <v>1428345</v>
+        <v>1453284</v>
       </c>
       <c r="C4" t="n">
-        <v>613887</v>
+        <v>668222</v>
       </c>
       <c r="D4" t="n">
-        <v>1360335</v>
+        <v>1399375</v>
       </c>
       <c r="E4" t="n">
         <v>9000</v>
       </c>
       <c r="F4" t="n">
-        <v>2000629</v>
+        <v>1997673</v>
       </c>
       <c r="G4" t="n">
-        <v>1229134</v>
+        <v>1229304</v>
       </c>
       <c r="I4" t="n">
-        <v>1516881</v>
+        <v>1526881</v>
       </c>
       <c r="K4" t="n">
-        <v>265281</v>
+        <v>210710</v>
       </c>
       <c r="M4" t="n">
-        <v>2655010</v>
+        <v>2315158</v>
       </c>
       <c r="N4" t="n">
-        <v>275644</v>
+        <v>274632</v>
       </c>
       <c r="O4" t="n">
-        <v>405391</v>
+        <v>404378</v>
       </c>
       <c r="P4" t="n">
         <v>393345</v>
       </c>
       <c r="Q4" t="n">
-        <v>735394</v>
+        <v>702775</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B5" t="n">
-        <v>1453305</v>
+        <v>1428345</v>
       </c>
       <c r="C5" t="n">
-        <v>660021</v>
+        <v>613887</v>
       </c>
       <c r="D5" t="n">
-        <v>1394810</v>
+        <v>1360335</v>
       </c>
       <c r="E5" t="n">
         <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>1966997</v>
+        <v>2000629</v>
       </c>
       <c r="G5" t="n">
-        <v>1358589</v>
+        <v>1229134</v>
       </c>
       <c r="I5" t="n">
-        <v>1530881</v>
+        <v>1516881</v>
       </c>
       <c r="K5" t="n">
-        <v>224505</v>
+        <v>265281</v>
       </c>
       <c r="M5" t="n">
-        <v>2605275</v>
+        <v>2655010</v>
       </c>
       <c r="N5" t="n">
-        <v>273068</v>
+        <v>275644</v>
       </c>
       <c r="O5" t="n">
-        <v>402811</v>
+        <v>405391</v>
       </c>
       <c r="P5" t="n">
-        <v>368707</v>
+        <v>393345</v>
       </c>
       <c r="Q5" t="n">
-        <v>750038</v>
+        <v>735394</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B6" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C6" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D6" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E6" t="n">
         <v>9000</v>
       </c>
       <c r="F6" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G6" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I6" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K6" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M6" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N6" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O6" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P6" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q6" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B7" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C7" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D7" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E7" t="n">
         <v>9000</v>
       </c>
       <c r="F7" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G7" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I7" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K7" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M7" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N7" t="n">
         <v>214475</v>
       </c>
       <c r="O7" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P7" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q7" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B8" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C8" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D8" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E8" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F8" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G8" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I8" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K8" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M8" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P8" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q8" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B9" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C9" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D9" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E9" t="n">
         <v>9200</v>
       </c>
       <c r="F9" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G9" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I9" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K9" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M9" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P9" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q9" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B10" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C10" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D10" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G10" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I10" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K10" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M10" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N10" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P10" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q10" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B11" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C11" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D11" t="n">
         <v>1336369</v>
@@ -84611,28 +84705,28 @@
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G11" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I11" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K11" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M11" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N11" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O11" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P11" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q11" t="n">
         <v>710782</v>
@@ -84640,34 +84734,34 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B12" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C12" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D12" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G12" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I12" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K12" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M12" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
@@ -84676,7 +84770,7 @@
         <v>238857</v>
       </c>
       <c r="P12" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q12" t="n">
         <v>710782</v>
@@ -84684,43 +84778,43 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B13" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C13" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D13" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G13" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I13" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K13" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M13" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N13" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O13" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P13" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q13" t="n">
         <v>710782</v>
@@ -84728,201 +84822,201 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B14" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C14" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D14" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G14" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I14" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K14" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M14" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N14" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O14" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P14" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q14" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B15" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C15" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D15" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G15" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I15" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K15" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M15" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N15" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O15" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P15" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q15" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B16" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C16" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D16" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E16" t="n">
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G16" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I16" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K16" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M16" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N16" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O16" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P16" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q16" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B17" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C17" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D17" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E17" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G17" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I17" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K17" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M17" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N17" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O17" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P17" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q17" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B18" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C18" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D18" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E18" t="n">
         <v>9400</v>
       </c>
       <c r="F18" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G18" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I18" t="n">
         <v>1493578</v>
@@ -84931,7 +85025,7 @@
         <v>270165</v>
       </c>
       <c r="M18" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N18" t="n">
         <v>214475</v>
@@ -84943,39 +85037,39 @@
         <v>380581</v>
       </c>
       <c r="Q18" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B19" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C19" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D19" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E19" t="n">
         <v>9400</v>
       </c>
       <c r="F19" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G19" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I19" t="n">
         <v>1493578</v>
       </c>
       <c r="K19" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M19" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N19" t="n">
         <v>214475</v>
@@ -84984,153 +85078,153 @@
         <v>236857</v>
       </c>
       <c r="P19" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q19" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B20" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C20" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D20" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E20" t="n">
         <v>9400</v>
       </c>
       <c r="F20" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G20" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I20" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K20" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M20" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N20" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O20" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P20" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q20" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B21" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C21" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D21" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E21" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F21" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G21" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I21" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K21" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M21" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N21" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O21" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P21" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q21" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B22" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C22" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D22" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E22" t="n">
         <v>9200</v>
       </c>
       <c r="F22" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G22" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I22" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K22" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M22" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N22" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O22" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P22" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q22" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B23" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C23" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D23" t="n">
         <v>1438502</v>
@@ -85139,107 +85233,107 @@
         <v>9200</v>
       </c>
       <c r="F23" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G23" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I23" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K23" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M23" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N23" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O23" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P23" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q23" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B24" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C24" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D24" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E24" t="n">
         <v>9200</v>
       </c>
       <c r="F24" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G24" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I24" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K24" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M24" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N24" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O24" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P24" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q24" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B25" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C25" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D25" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E25" t="n">
         <v>9200</v>
       </c>
       <c r="F25" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G25" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I25" t="n">
         <v>1488515</v>
       </c>
       <c r="K25" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M25" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N25" t="n">
         <v>214475</v>
@@ -85248,7 +85342,7 @@
         <v>247857</v>
       </c>
       <c r="P25" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q25" t="n">
         <v>738429</v>
@@ -85256,34 +85350,34 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B26" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C26" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D26" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E26" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F26" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G26" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I26" t="n">
         <v>1488515</v>
       </c>
       <c r="K26" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M26" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N26" t="n">
         <v>214475</v>
@@ -85292,7 +85386,7 @@
         <v>247857</v>
       </c>
       <c r="P26" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q26" t="n">
         <v>738429</v>
@@ -85300,78 +85394,78 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B27" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C27" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D27" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E27" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F27" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G27" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I27" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K27" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M27" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N27" t="n">
         <v>214475</v>
       </c>
       <c r="O27" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P27" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q27" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B28" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C28" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D28" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E28" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F28" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G28" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I28" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K28" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M28" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N28" t="n">
         <v>214475</v>
@@ -85380,42 +85474,42 @@
         <v>264857</v>
       </c>
       <c r="P28" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q28" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B29" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C29" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D29" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E29" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F29" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G29" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I29" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K29" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M29" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N29" t="n">
         <v>214475</v>
@@ -85424,101 +85518,98 @@
         <v>264857</v>
       </c>
       <c r="P29" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q29" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B30" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C30" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D30" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E30" t="n">
         <v>9300</v>
       </c>
       <c r="F30" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G30" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I30" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K30" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M30" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N30" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O30" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P30" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q30" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R30" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B31" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C31" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D31" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E31" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F31" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G31" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I31" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K31" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M31" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N31" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O31" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P31" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q31" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R31" t="n">
         <v>15000</v>
@@ -85526,40 +85617,40 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B32" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C32" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D32" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E32" t="n">
         <v>9100</v>
       </c>
       <c r="F32" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G32" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I32" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K32" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M32" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N32" t="n">
         <v>189475</v>
       </c>
       <c r="O32" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P32" t="n">
         <v>375660</v>
@@ -85568,6 +85659,53 @@
         <v>773586</v>
       </c>
       <c r="R32" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C33" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K33" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M33" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N33" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O33" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P33" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R33" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 33/119] 2026-08-26 ~ 13/17 meters metered 11.96 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:29 ~1:16 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80243,9 +80243,36 @@
       <c r="A2431" s="4" t="n">
         <v>46260</v>
       </c>
+      <c r="B2431" t="n">
+        <v>3.184</v>
+      </c>
+      <c r="C2431" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="D2431" t="n">
+        <v>1.444</v>
+      </c>
+      <c r="E2431" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="F2431" t="n">
+        <v>2.596</v>
+      </c>
+      <c r="G2431" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="H2431" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="I2431" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="K2431" t="n">
+        <v>11.964</v>
+      </c>
       <c r="L2431" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81453,7 +81480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81518,345 +81545,345 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B2" t="n">
-        <v>3.29</v>
+        <v>3.184</v>
       </c>
       <c r="C2" t="n">
-        <v>3.254</v>
+        <v>3.08</v>
       </c>
       <c r="D2" t="n">
-        <v>1.491</v>
+        <v>1.444</v>
       </c>
       <c r="E2" t="n">
-        <v>0.14</v>
+        <v>0.235</v>
       </c>
       <c r="F2" t="n">
-        <v>2.594</v>
+        <v>2.596</v>
       </c>
       <c r="G2" t="n">
-        <v>0.715</v>
+        <v>0.404</v>
       </c>
       <c r="H2" t="n">
-        <v>0.385</v>
+        <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.657</v>
+        <v>0.642</v>
       </c>
       <c r="K2" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B3" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C3" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D3" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E3" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F3" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G3" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H3" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K3" t="n">
-        <v>12.269</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B4" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C4" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D4" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E4" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F4" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G4" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H4" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I4" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>12.136</v>
+        <v>12.269</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B5" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C5" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D5" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E5" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F5" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G5" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H5" t="n">
         <v>0.379</v>
       </c>
       <c r="I5" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K5" t="n">
-        <v>12.428</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B6" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C6" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D6" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E6" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F6" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G6" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H6" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I6" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K6" t="n">
-        <v>12.534</v>
+        <v>12.428</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B7" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C7" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D7" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E7" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F7" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G7" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H7" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I7" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K7" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B8" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C8" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D8" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E8" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F8" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G8" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H8" t="n">
         <v>0.342</v>
       </c>
       <c r="I8" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K8" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B9" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C9" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D9" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E9" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F9" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G9" t="n">
         <v>0.444</v>
       </c>
       <c r="H9" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I9" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K9" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B10" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C10" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D10" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E10" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F10" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G10" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H10" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I10" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K10" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B11" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C11" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D11" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E11" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F11" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G11" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H11" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K11" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B12" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C12" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D12" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E12" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F12" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G12" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
@@ -81865,27 +81892,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B13" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C13" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D13" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E13" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F13" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G13" t="n">
         <v>0.437</v>
@@ -81897,178 +81924,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B14" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C14" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D14" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E14" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F14" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G14" t="n">
         <v>0.437</v>
       </c>
       <c r="H14" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I14" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B15" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C15" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D15" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E15" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F15" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G15" t="n">
         <v>0.437</v>
       </c>
       <c r="H15" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I15" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B16" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C16" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D16" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F16" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G16" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H16" t="n">
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K16" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B17" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C17" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D17" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E17" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F17" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G17" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H17" t="n">
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B18" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C18" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D18" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E18" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F18" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G18" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H18" t="n">
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K18" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B19" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C19" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D19" t="n">
         <v>1.44</v>
@@ -82077,7 +82104,7 @@
         <v>0.261</v>
       </c>
       <c r="F19" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G19" t="n">
         <v>0.435</v>
@@ -82086,222 +82113,222 @@
         <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K19" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B20" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C20" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D20" t="n">
         <v>1.44</v>
       </c>
       <c r="E20" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F20" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G20" t="n">
         <v>0.435</v>
       </c>
       <c r="H20" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I20" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K20" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B21" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C21" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D21" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E21" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F21" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G21" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H21" t="n">
         <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K21" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B22" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C22" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D22" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F22" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G22" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H22" t="n">
         <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K22" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B23" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C23" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D23" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E23" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G23" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H23" t="n">
         <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K23" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B24" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C24" t="n">
         <v>3.232</v>
       </c>
       <c r="D24" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F24" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G24" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H24" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I24" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K24" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B25" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C25" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D25" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E25" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F25" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G25" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H25" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I25" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K25" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B26" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C26" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D26" t="n">
         <v>1.435</v>
       </c>
       <c r="E26" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F26" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G26" t="n">
         <v>0.446</v>
@@ -82313,27 +82340,27 @@
         <v>0.712</v>
       </c>
       <c r="K26" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B27" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C27" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D27" t="n">
         <v>1.435</v>
       </c>
       <c r="E27" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F27" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G27" t="n">
         <v>0.446</v>
@@ -82345,59 +82372,59 @@
         <v>0.712</v>
       </c>
       <c r="K27" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B28" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C28" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D28" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E28" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F28" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G28" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H28" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I28" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K28" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B29" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C29" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D29" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E29" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F29" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G29" t="n">
         <v>0.462</v>
@@ -82406,30 +82433,30 @@
         <v>0.343</v>
       </c>
       <c r="I29" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K29" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B30" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C30" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D30" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E30" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F30" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G30" t="n">
         <v>0.462</v>
@@ -82438,100 +82465,97 @@
         <v>0.343</v>
       </c>
       <c r="I30" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K30" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B31" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C31" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D31" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E31" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F31" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G31" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H31" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I31" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K31" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B32" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C32" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D32" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E32" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F32" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G32" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H32" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I32" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J32" t="n">
         <v>0.014</v>
       </c>
       <c r="K32" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B33" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C33" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D33" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E33" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F33" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G33" t="n">
         <v>0.395</v>
@@ -82546,6 +82570,41 @@
         <v>0.014</v>
       </c>
       <c r="K33" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B34" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K34" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82560,7 +82619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82630,375 +82689,375 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B2" t="n">
-        <v>3.29</v>
+        <v>3.184</v>
       </c>
       <c r="C2" t="n">
-        <v>3.254</v>
+        <v>3.08</v>
       </c>
       <c r="D2" t="n">
-        <v>1.491</v>
+        <v>1.444</v>
       </c>
       <c r="E2" t="n">
-        <v>0.14</v>
+        <v>0.235</v>
       </c>
       <c r="F2" t="n">
-        <v>2.594</v>
+        <v>2.596</v>
       </c>
       <c r="G2" t="n">
-        <v>0.715</v>
+        <v>0.404</v>
       </c>
       <c r="H2" t="n">
-        <v>0.385</v>
+        <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.657</v>
+        <v>0.642</v>
       </c>
       <c r="K2" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
       <c r="L2" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B3" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C3" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D3" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E3" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F3" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G3" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H3" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K3" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
       <c r="L3" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B4" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C4" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D4" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E4" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F4" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G4" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H4" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I4" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
       <c r="L4" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B5" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C5" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D5" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E5" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F5" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G5" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H5" t="n">
         <v>0.379</v>
       </c>
       <c r="I5" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K5" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
       <c r="L5" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B6" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C6" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D6" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E6" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F6" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G6" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H6" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I6" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K6" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
       <c r="L6" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B7" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C7" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D7" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E7" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F7" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G7" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H7" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I7" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K7" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L7" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B8" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C8" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D8" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E8" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F8" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G8" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H8" t="n">
         <v>0.342</v>
       </c>
       <c r="I8" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K8" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L8" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B9" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C9" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D9" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E9" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F9" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G9" t="n">
         <v>0.444</v>
       </c>
       <c r="H9" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I9" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K9" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L9" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B10" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C10" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D10" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E10" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F10" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G10" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H10" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I10" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K10" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L10" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B11" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C11" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D11" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E11" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F11" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G11" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H11" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K11" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L11" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B12" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C12" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D12" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E12" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F12" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G12" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H12" t="n">
         <v>0.367</v>
@@ -83007,30 +83066,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L12" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B13" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C13" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D13" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E13" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F13" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G13" t="n">
         <v>0.437</v>
@@ -83042,196 +83101,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L13" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B14" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C14" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D14" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E14" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F14" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G14" t="n">
         <v>0.437</v>
       </c>
       <c r="H14" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I14" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L14" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B15" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C15" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D15" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E15" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F15" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G15" t="n">
         <v>0.437</v>
       </c>
       <c r="H15" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I15" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L15" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B16" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C16" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D16" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F16" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G16" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H16" t="n">
         <v>0.367</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K16" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L16" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B17" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C17" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D17" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E17" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F17" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G17" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H17" t="n">
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L17" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B18" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C18" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D18" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E18" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F18" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G18" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H18" t="n">
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K18" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L18" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B19" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C19" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D19" t="n">
         <v>1.44</v>
@@ -83240,7 +83299,7 @@
         <v>0.261</v>
       </c>
       <c r="F19" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G19" t="n">
         <v>0.435</v>
@@ -83249,243 +83308,243 @@
         <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K19" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L19" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B20" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C20" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D20" t="n">
         <v>1.44</v>
       </c>
       <c r="E20" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F20" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G20" t="n">
         <v>0.435</v>
       </c>
       <c r="H20" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I20" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K20" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L20" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B21" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C21" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D21" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E21" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F21" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G21" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H21" t="n">
         <v>0.365</v>
       </c>
       <c r="I21" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K21" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L21" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B22" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C22" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D22" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F22" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G22" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H22" t="n">
         <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K22" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L22" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B23" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C23" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D23" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E23" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G23" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H23" t="n">
         <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K23" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L23" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B24" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C24" t="n">
         <v>3.232</v>
       </c>
       <c r="D24" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F24" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G24" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H24" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I24" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K24" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L24" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B25" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C25" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D25" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E25" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F25" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G25" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H25" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I25" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K25" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L25" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B26" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C26" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D26" t="n">
         <v>1.435</v>
       </c>
       <c r="E26" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F26" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G26" t="n">
         <v>0.446</v>
@@ -83497,30 +83556,30 @@
         <v>0.712</v>
       </c>
       <c r="K26" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L26" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B27" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C27" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D27" t="n">
         <v>1.435</v>
       </c>
       <c r="E27" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F27" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G27" t="n">
         <v>0.446</v>
@@ -83532,65 +83591,65 @@
         <v>0.712</v>
       </c>
       <c r="K27" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L27" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B28" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C28" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D28" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E28" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F28" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G28" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H28" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I28" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K28" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L28" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B29" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C29" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D29" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E29" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F29" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G29" t="n">
         <v>0.462</v>
@@ -83599,33 +83658,33 @@
         <v>0.343</v>
       </c>
       <c r="I29" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K29" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L29" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B30" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C30" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D30" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E30" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F30" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G30" t="n">
         <v>0.462</v>
@@ -83634,109 +83693,106 @@
         <v>0.343</v>
       </c>
       <c r="I30" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K30" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L30" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B31" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C31" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D31" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E31" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F31" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G31" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H31" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I31" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K31" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L31" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B32" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C32" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D32" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E32" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F32" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G32" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H32" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I32" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J32" t="n">
         <v>0.014</v>
       </c>
       <c r="K32" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L32" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B33" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C33" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D33" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E33" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F33" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G33" t="n">
         <v>0.395</v>
@@ -83751,9 +83807,47 @@
         <v>0.014</v>
       </c>
       <c r="K33" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L33" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B34" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K34" t="n">
         <v>12.277</v>
       </c>
-      <c r="L33" t="n">
+      <c r="L34" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -84194,7 +84288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R33"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84294,453 +84388,453 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B2" t="n">
-        <v>1383237</v>
+        <v>1372566</v>
       </c>
       <c r="C2" t="n">
-        <v>642612</v>
+        <v>535686</v>
       </c>
       <c r="D2" t="n">
-        <v>1376983</v>
+        <v>1384220</v>
       </c>
       <c r="E2" t="n">
-        <v>9000</v>
+        <v>9500</v>
       </c>
       <c r="F2" t="n">
-        <v>1886772</v>
+        <v>1750778</v>
       </c>
       <c r="G2" t="n">
-        <v>1487288</v>
+        <v>1443098</v>
       </c>
       <c r="I2" t="n">
-        <v>1545952</v>
+        <v>1497314</v>
       </c>
       <c r="K2" t="n">
-        <v>145193</v>
+        <v>243577</v>
       </c>
       <c r="M2" t="n">
-        <v>2689526</v>
+        <v>2692467</v>
       </c>
       <c r="N2" t="n">
-        <v>309125</v>
+        <v>188088</v>
       </c>
       <c r="O2" t="n">
-        <v>432534</v>
+        <v>230944</v>
       </c>
       <c r="P2" t="n">
-        <v>399049</v>
+        <v>393254</v>
       </c>
       <c r="Q2" t="n">
-        <v>681693</v>
+        <v>665576</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B3" t="n">
-        <v>1326845</v>
+        <v>1383237</v>
       </c>
       <c r="C3" t="n">
-        <v>630343</v>
+        <v>642612</v>
       </c>
       <c r="D3" t="n">
-        <v>1389820</v>
+        <v>1376983</v>
       </c>
       <c r="E3" t="n">
         <v>9000</v>
       </c>
       <c r="F3" t="n">
-        <v>1898634</v>
+        <v>1886772</v>
       </c>
       <c r="G3" t="n">
-        <v>1230443</v>
+        <v>1487288</v>
       </c>
       <c r="I3" t="n">
-        <v>1509954</v>
+        <v>1545952</v>
       </c>
       <c r="K3" t="n">
-        <v>223405</v>
+        <v>145193</v>
       </c>
       <c r="M3" t="n">
-        <v>2637144</v>
+        <v>2689526</v>
       </c>
       <c r="N3" t="n">
-        <v>322000</v>
+        <v>309125</v>
       </c>
       <c r="O3" t="n">
-        <v>445186</v>
+        <v>432534</v>
       </c>
       <c r="P3" t="n">
-        <v>392284</v>
+        <v>399049</v>
       </c>
       <c r="Q3" t="n">
-        <v>707427</v>
+        <v>681693</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B4" t="n">
-        <v>1453284</v>
+        <v>1326845</v>
       </c>
       <c r="C4" t="n">
-        <v>668222</v>
+        <v>630343</v>
       </c>
       <c r="D4" t="n">
-        <v>1399375</v>
+        <v>1389820</v>
       </c>
       <c r="E4" t="n">
         <v>9000</v>
       </c>
       <c r="F4" t="n">
-        <v>1997673</v>
+        <v>1898634</v>
       </c>
       <c r="G4" t="n">
-        <v>1229304</v>
+        <v>1230443</v>
       </c>
       <c r="I4" t="n">
-        <v>1526881</v>
+        <v>1509954</v>
       </c>
       <c r="K4" t="n">
-        <v>210710</v>
+        <v>223405</v>
       </c>
       <c r="M4" t="n">
-        <v>2315158</v>
+        <v>2637144</v>
       </c>
       <c r="N4" t="n">
-        <v>274632</v>
+        <v>322000</v>
       </c>
       <c r="O4" t="n">
-        <v>404378</v>
+        <v>445186</v>
       </c>
       <c r="P4" t="n">
-        <v>393345</v>
+        <v>392284</v>
       </c>
       <c r="Q4" t="n">
-        <v>702775</v>
+        <v>707427</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B5" t="n">
-        <v>1428345</v>
+        <v>1453284</v>
       </c>
       <c r="C5" t="n">
-        <v>613887</v>
+        <v>668222</v>
       </c>
       <c r="D5" t="n">
-        <v>1360335</v>
+        <v>1399375</v>
       </c>
       <c r="E5" t="n">
         <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>2000629</v>
+        <v>1997673</v>
       </c>
       <c r="G5" t="n">
-        <v>1229134</v>
+        <v>1229304</v>
       </c>
       <c r="I5" t="n">
-        <v>1516881</v>
+        <v>1526881</v>
       </c>
       <c r="K5" t="n">
-        <v>265281</v>
+        <v>210710</v>
       </c>
       <c r="M5" t="n">
-        <v>2655010</v>
+        <v>2315158</v>
       </c>
       <c r="N5" t="n">
-        <v>275644</v>
+        <v>274632</v>
       </c>
       <c r="O5" t="n">
-        <v>405391</v>
+        <v>404378</v>
       </c>
       <c r="P5" t="n">
         <v>393345</v>
       </c>
       <c r="Q5" t="n">
-        <v>735394</v>
+        <v>702775</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B6" t="n">
-        <v>1453305</v>
+        <v>1428345</v>
       </c>
       <c r="C6" t="n">
-        <v>660021</v>
+        <v>613887</v>
       </c>
       <c r="D6" t="n">
-        <v>1394810</v>
+        <v>1360335</v>
       </c>
       <c r="E6" t="n">
         <v>9000</v>
       </c>
       <c r="F6" t="n">
-        <v>1966997</v>
+        <v>2000629</v>
       </c>
       <c r="G6" t="n">
-        <v>1358589</v>
+        <v>1229134</v>
       </c>
       <c r="I6" t="n">
-        <v>1530881</v>
+        <v>1516881</v>
       </c>
       <c r="K6" t="n">
-        <v>224505</v>
+        <v>265281</v>
       </c>
       <c r="M6" t="n">
-        <v>2605275</v>
+        <v>2655010</v>
       </c>
       <c r="N6" t="n">
-        <v>273068</v>
+        <v>275644</v>
       </c>
       <c r="O6" t="n">
-        <v>402811</v>
+        <v>405391</v>
       </c>
       <c r="P6" t="n">
-        <v>368707</v>
+        <v>393345</v>
       </c>
       <c r="Q6" t="n">
-        <v>750038</v>
+        <v>735394</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B7" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C7" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D7" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E7" t="n">
         <v>9000</v>
       </c>
       <c r="F7" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G7" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I7" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K7" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M7" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N7" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O7" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P7" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q7" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B8" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C8" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D8" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E8" t="n">
         <v>9000</v>
       </c>
       <c r="F8" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G8" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I8" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K8" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M8" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N8" t="n">
         <v>214475</v>
       </c>
       <c r="O8" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P8" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q8" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B9" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C9" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D9" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E9" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F9" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G9" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I9" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K9" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M9" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P9" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q9" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B10" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C10" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D10" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E10" t="n">
         <v>9200</v>
       </c>
       <c r="F10" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G10" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I10" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K10" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M10" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P10" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q10" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B11" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C11" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D11" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G11" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I11" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K11" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M11" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N11" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P11" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q11" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B12" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C12" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D12" t="n">
         <v>1336369</v>
@@ -84749,28 +84843,28 @@
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G12" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I12" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K12" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M12" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N12" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O12" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P12" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q12" t="n">
         <v>710782</v>
@@ -84778,34 +84872,34 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B13" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C13" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D13" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G13" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I13" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K13" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M13" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N13" t="n">
         <v>214475</v>
@@ -84814,7 +84908,7 @@
         <v>238857</v>
       </c>
       <c r="P13" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q13" t="n">
         <v>710782</v>
@@ -84822,43 +84916,43 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B14" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C14" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D14" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G14" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I14" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K14" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M14" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N14" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O14" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P14" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q14" t="n">
         <v>710782</v>
@@ -84866,201 +84960,201 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B15" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C15" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D15" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G15" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I15" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K15" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M15" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N15" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O15" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P15" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q15" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B16" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C16" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D16" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E16" t="n">
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G16" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I16" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K16" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M16" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N16" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O16" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P16" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q16" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B17" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C17" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D17" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E17" t="n">
         <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G17" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I17" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K17" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M17" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N17" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O17" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P17" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q17" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B18" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C18" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D18" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E18" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G18" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I18" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K18" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M18" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N18" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O18" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P18" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q18" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B19" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C19" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D19" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E19" t="n">
         <v>9400</v>
       </c>
       <c r="F19" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G19" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I19" t="n">
         <v>1493578</v>
@@ -85069,7 +85163,7 @@
         <v>270165</v>
       </c>
       <c r="M19" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N19" t="n">
         <v>214475</v>
@@ -85081,39 +85175,39 @@
         <v>380581</v>
       </c>
       <c r="Q19" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B20" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C20" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D20" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E20" t="n">
         <v>9400</v>
       </c>
       <c r="F20" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G20" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I20" t="n">
         <v>1493578</v>
       </c>
       <c r="K20" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M20" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N20" t="n">
         <v>214475</v>
@@ -85122,153 +85216,153 @@
         <v>236857</v>
       </c>
       <c r="P20" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q20" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B21" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C21" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D21" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E21" t="n">
         <v>9400</v>
       </c>
       <c r="F21" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G21" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I21" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K21" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M21" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N21" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O21" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P21" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q21" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B22" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C22" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D22" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E22" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F22" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G22" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I22" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K22" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M22" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N22" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O22" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P22" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q22" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B23" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C23" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D23" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E23" t="n">
         <v>9200</v>
       </c>
       <c r="F23" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G23" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I23" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K23" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M23" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N23" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O23" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P23" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q23" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B24" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C24" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D24" t="n">
         <v>1438502</v>
@@ -85277,107 +85371,107 @@
         <v>9200</v>
       </c>
       <c r="F24" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G24" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I24" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K24" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M24" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N24" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O24" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P24" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q24" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B25" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C25" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D25" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E25" t="n">
         <v>9200</v>
       </c>
       <c r="F25" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G25" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I25" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K25" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M25" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N25" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O25" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P25" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q25" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B26" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C26" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D26" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E26" t="n">
         <v>9200</v>
       </c>
       <c r="F26" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G26" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I26" t="n">
         <v>1488515</v>
       </c>
       <c r="K26" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M26" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N26" t="n">
         <v>214475</v>
@@ -85386,7 +85480,7 @@
         <v>247857</v>
       </c>
       <c r="P26" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q26" t="n">
         <v>738429</v>
@@ -85394,34 +85488,34 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B27" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C27" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D27" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E27" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F27" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G27" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I27" t="n">
         <v>1488515</v>
       </c>
       <c r="K27" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M27" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N27" t="n">
         <v>214475</v>
@@ -85430,7 +85524,7 @@
         <v>247857</v>
       </c>
       <c r="P27" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q27" t="n">
         <v>738429</v>
@@ -85438,78 +85532,78 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B28" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C28" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D28" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E28" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F28" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G28" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I28" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K28" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M28" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N28" t="n">
         <v>214475</v>
       </c>
       <c r="O28" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P28" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q28" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B29" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C29" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D29" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E29" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F29" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G29" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I29" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K29" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M29" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N29" t="n">
         <v>214475</v>
@@ -85518,42 +85612,42 @@
         <v>264857</v>
       </c>
       <c r="P29" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q29" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B30" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C30" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D30" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E30" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F30" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G30" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I30" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K30" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M30" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N30" t="n">
         <v>214475</v>
@@ -85562,101 +85656,98 @@
         <v>264857</v>
       </c>
       <c r="P30" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q30" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B31" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C31" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D31" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E31" t="n">
         <v>9300</v>
       </c>
       <c r="F31" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G31" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I31" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K31" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M31" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N31" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O31" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P31" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q31" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R31" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B32" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C32" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D32" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E32" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F32" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G32" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I32" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K32" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M32" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N32" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O32" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P32" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q32" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R32" t="n">
         <v>15000</v>
@@ -85664,40 +85755,40 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B33" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C33" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D33" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E33" t="n">
         <v>9100</v>
       </c>
       <c r="F33" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G33" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I33" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K33" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M33" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N33" t="n">
         <v>189475</v>
       </c>
       <c r="O33" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P33" t="n">
         <v>375660</v>
@@ -85706,6 +85797,53 @@
         <v>773586</v>
       </c>
       <c r="R33" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B34" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C34" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E34" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K34" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M34" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N34" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O34" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P34" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R34" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 34/119] 2026-08-25 ~ 13/17 meters metered 10.95 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:30 ~1:15 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80233,9 +80233,36 @@
       <c r="A2430" s="4" t="n">
         <v>46259</v>
       </c>
+      <c r="B2430" t="n">
+        <v>3.172</v>
+      </c>
+      <c r="C2430" t="n">
+        <v>3.056</v>
+      </c>
+      <c r="D2430" t="n">
+        <v>1.453</v>
+      </c>
+      <c r="E2430" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="F2430" t="n">
+        <v>1.921</v>
+      </c>
+      <c r="G2430" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="H2430" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="I2430" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="K2430" t="n">
+        <v>10.954</v>
+      </c>
       <c r="L2430" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81480,7 +81507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81545,377 +81572,377 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="B2" t="n">
-        <v>3.184</v>
+        <v>3.172</v>
       </c>
       <c r="C2" t="n">
-        <v>3.08</v>
+        <v>3.056</v>
       </c>
       <c r="D2" t="n">
-        <v>1.444</v>
+        <v>1.453</v>
       </c>
       <c r="E2" t="n">
-        <v>0.235</v>
+        <v>0.29</v>
       </c>
       <c r="F2" t="n">
-        <v>2.596</v>
+        <v>1.921</v>
       </c>
       <c r="G2" t="n">
-        <v>0.404</v>
+        <v>0.222</v>
       </c>
       <c r="H2" t="n">
         <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.642</v>
+        <v>0.461</v>
       </c>
       <c r="K2" t="n">
-        <v>11.964</v>
+        <v>10.954</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B3" t="n">
-        <v>3.29</v>
+        <v>3.184</v>
       </c>
       <c r="C3" t="n">
-        <v>3.254</v>
+        <v>3.08</v>
       </c>
       <c r="D3" t="n">
-        <v>1.491</v>
+        <v>1.444</v>
       </c>
       <c r="E3" t="n">
-        <v>0.14</v>
+        <v>0.235</v>
       </c>
       <c r="F3" t="n">
-        <v>2.594</v>
+        <v>2.596</v>
       </c>
       <c r="G3" t="n">
-        <v>0.715</v>
+        <v>0.404</v>
       </c>
       <c r="H3" t="n">
-        <v>0.385</v>
+        <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.657</v>
+        <v>0.642</v>
       </c>
       <c r="K3" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B4" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C4" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D4" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E4" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F4" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G4" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H4" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K4" t="n">
-        <v>12.269</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B5" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C5" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D5" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E5" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F5" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G5" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H5" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I5" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>12.136</v>
+        <v>12.269</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B6" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C6" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D6" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E6" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F6" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G6" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H6" t="n">
         <v>0.379</v>
       </c>
       <c r="I6" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K6" t="n">
-        <v>12.428</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B7" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C7" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D7" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E7" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F7" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G7" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H7" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I7" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K7" t="n">
-        <v>12.534</v>
+        <v>12.428</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B8" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C8" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D8" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E8" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F8" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G8" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H8" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I8" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K8" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B9" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C9" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D9" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E9" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F9" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G9" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H9" t="n">
         <v>0.342</v>
       </c>
       <c r="I9" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K9" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B10" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C10" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D10" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E10" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F10" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G10" t="n">
         <v>0.444</v>
       </c>
       <c r="H10" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I10" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K10" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B11" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C11" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D11" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E11" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F11" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G11" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H11" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I11" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K11" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B12" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C12" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D12" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E12" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F12" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G12" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H12" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K12" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B13" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C13" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D13" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E13" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F13" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G13" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
@@ -81924,27 +81951,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B14" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C14" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D14" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E14" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F14" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G14" t="n">
         <v>0.437</v>
@@ -81956,178 +81983,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B15" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C15" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D15" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E15" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F15" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G15" t="n">
         <v>0.437</v>
       </c>
       <c r="H15" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I15" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B16" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C16" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D16" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E16" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F16" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G16" t="n">
         <v>0.437</v>
       </c>
       <c r="H16" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I16" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B17" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C17" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D17" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F17" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G17" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H17" t="n">
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K17" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B18" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C18" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D18" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E18" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F18" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G18" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H18" t="n">
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B19" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C19" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D19" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E19" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F19" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G19" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H19" t="n">
         <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K19" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B20" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C20" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D20" t="n">
         <v>1.44</v>
@@ -82136,7 +82163,7 @@
         <v>0.261</v>
       </c>
       <c r="F20" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G20" t="n">
         <v>0.435</v>
@@ -82145,222 +82172,222 @@
         <v>0.367</v>
       </c>
       <c r="I20" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K20" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B21" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C21" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D21" t="n">
         <v>1.44</v>
       </c>
       <c r="E21" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F21" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G21" t="n">
         <v>0.435</v>
       </c>
       <c r="H21" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I21" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K21" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B22" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C22" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D22" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E22" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F22" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G22" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H22" t="n">
         <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K22" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B23" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C23" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D23" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F23" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G23" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H23" t="n">
         <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K23" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B24" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C24" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D24" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E24" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G24" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H24" t="n">
         <v>0.365</v>
       </c>
       <c r="I24" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K24" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B25" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C25" t="n">
         <v>3.232</v>
       </c>
       <c r="D25" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F25" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G25" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H25" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I25" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K25" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B26" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C26" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D26" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E26" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F26" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G26" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H26" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I26" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K26" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B27" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C27" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D27" t="n">
         <v>1.435</v>
       </c>
       <c r="E27" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F27" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G27" t="n">
         <v>0.446</v>
@@ -82372,27 +82399,27 @@
         <v>0.712</v>
       </c>
       <c r="K27" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B28" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C28" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D28" t="n">
         <v>1.435</v>
       </c>
       <c r="E28" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F28" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G28" t="n">
         <v>0.446</v>
@@ -82404,59 +82431,59 @@
         <v>0.712</v>
       </c>
       <c r="K28" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B29" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C29" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D29" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E29" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F29" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G29" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H29" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I29" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K29" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B30" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C30" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D30" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E30" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F30" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G30" t="n">
         <v>0.462</v>
@@ -82465,30 +82492,30 @@
         <v>0.343</v>
       </c>
       <c r="I30" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K30" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B31" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C31" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D31" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E31" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F31" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G31" t="n">
         <v>0.462</v>
@@ -82497,100 +82524,97 @@
         <v>0.343</v>
       </c>
       <c r="I31" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K31" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B32" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C32" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D32" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E32" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F32" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G32" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H32" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I32" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J32" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K32" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B33" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C33" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D33" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E33" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F33" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G33" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H33" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I33" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J33" t="n">
         <v>0.014</v>
       </c>
       <c r="K33" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B34" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C34" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D34" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E34" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F34" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G34" t="n">
         <v>0.395</v>
@@ -82605,6 +82629,41 @@
         <v>0.014</v>
       </c>
       <c r="K34" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B35" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C35" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K35" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82619,7 +82678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82689,410 +82748,410 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="B2" t="n">
-        <v>3.184</v>
+        <v>3.172</v>
       </c>
       <c r="C2" t="n">
-        <v>3.08</v>
+        <v>3.056</v>
       </c>
       <c r="D2" t="n">
-        <v>1.444</v>
+        <v>1.453</v>
       </c>
       <c r="E2" t="n">
-        <v>0.235</v>
+        <v>0.29</v>
       </c>
       <c r="F2" t="n">
-        <v>2.596</v>
+        <v>1.921</v>
       </c>
       <c r="G2" t="n">
-        <v>0.404</v>
+        <v>0.222</v>
       </c>
       <c r="H2" t="n">
         <v>0.379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.642</v>
+        <v>0.461</v>
       </c>
       <c r="K2" t="n">
-        <v>11.964</v>
+        <v>10.954</v>
       </c>
       <c r="L2" t="n">
-        <v>11.964</v>
+        <v>10.954</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B3" t="n">
-        <v>3.29</v>
+        <v>3.184</v>
       </c>
       <c r="C3" t="n">
-        <v>3.254</v>
+        <v>3.08</v>
       </c>
       <c r="D3" t="n">
-        <v>1.491</v>
+        <v>1.444</v>
       </c>
       <c r="E3" t="n">
-        <v>0.14</v>
+        <v>0.235</v>
       </c>
       <c r="F3" t="n">
-        <v>2.594</v>
+        <v>2.596</v>
       </c>
       <c r="G3" t="n">
-        <v>0.715</v>
+        <v>0.404</v>
       </c>
       <c r="H3" t="n">
-        <v>0.385</v>
+        <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.657</v>
+        <v>0.642</v>
       </c>
       <c r="K3" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
       <c r="L3" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B4" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C4" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D4" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E4" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F4" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G4" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H4" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K4" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
       <c r="L4" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B5" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C5" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D5" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E5" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F5" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G5" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H5" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I5" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
       <c r="L5" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B6" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C6" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D6" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E6" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F6" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G6" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H6" t="n">
         <v>0.379</v>
       </c>
       <c r="I6" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K6" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
       <c r="L6" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B7" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C7" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D7" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E7" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F7" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G7" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H7" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I7" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K7" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
       <c r="L7" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B8" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C8" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D8" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E8" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F8" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G8" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H8" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I8" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K8" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L8" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B9" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C9" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D9" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E9" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F9" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G9" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H9" t="n">
         <v>0.342</v>
       </c>
       <c r="I9" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K9" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L9" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B10" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C10" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D10" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E10" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F10" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G10" t="n">
         <v>0.444</v>
       </c>
       <c r="H10" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I10" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K10" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L10" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B11" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C11" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D11" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E11" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F11" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G11" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H11" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I11" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K11" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L11" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B12" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C12" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D12" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E12" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F12" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G12" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H12" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K12" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L12" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B13" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C13" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D13" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E13" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F13" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G13" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H13" t="n">
         <v>0.367</v>
@@ -83101,30 +83160,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L13" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B14" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C14" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D14" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E14" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F14" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G14" t="n">
         <v>0.437</v>
@@ -83136,196 +83195,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L14" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B15" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C15" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D15" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E15" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F15" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G15" t="n">
         <v>0.437</v>
       </c>
       <c r="H15" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I15" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L15" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B16" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C16" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D16" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E16" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F16" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G16" t="n">
         <v>0.437</v>
       </c>
       <c r="H16" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I16" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L16" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B17" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C17" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D17" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F17" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G17" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H17" t="n">
         <v>0.367</v>
       </c>
       <c r="I17" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K17" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L17" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B18" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C18" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D18" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E18" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F18" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G18" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H18" t="n">
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L18" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B19" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C19" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D19" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E19" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F19" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G19" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H19" t="n">
         <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K19" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L19" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B20" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C20" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D20" t="n">
         <v>1.44</v>
@@ -83334,7 +83393,7 @@
         <v>0.261</v>
       </c>
       <c r="F20" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G20" t="n">
         <v>0.435</v>
@@ -83343,243 +83402,243 @@
         <v>0.367</v>
       </c>
       <c r="I20" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K20" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L20" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B21" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C21" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D21" t="n">
         <v>1.44</v>
       </c>
       <c r="E21" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F21" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G21" t="n">
         <v>0.435</v>
       </c>
       <c r="H21" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I21" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K21" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L21" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B22" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C22" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D22" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E22" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F22" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G22" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H22" t="n">
         <v>0.365</v>
       </c>
       <c r="I22" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K22" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L22" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B23" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C23" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D23" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F23" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G23" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H23" t="n">
         <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K23" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L23" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B24" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C24" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D24" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E24" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G24" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H24" t="n">
         <v>0.365</v>
       </c>
       <c r="I24" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K24" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L24" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B25" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C25" t="n">
         <v>3.232</v>
       </c>
       <c r="D25" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F25" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G25" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H25" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I25" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K25" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L25" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B26" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C26" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D26" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E26" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F26" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G26" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H26" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I26" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K26" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L26" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B27" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C27" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D27" t="n">
         <v>1.435</v>
       </c>
       <c r="E27" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F27" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G27" t="n">
         <v>0.446</v>
@@ -83591,30 +83650,30 @@
         <v>0.712</v>
       </c>
       <c r="K27" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L27" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B28" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C28" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D28" t="n">
         <v>1.435</v>
       </c>
       <c r="E28" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F28" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G28" t="n">
         <v>0.446</v>
@@ -83626,65 +83685,65 @@
         <v>0.712</v>
       </c>
       <c r="K28" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L28" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B29" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C29" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D29" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E29" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F29" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G29" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H29" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I29" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K29" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L29" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B30" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C30" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D30" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E30" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F30" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G30" t="n">
         <v>0.462</v>
@@ -83693,33 +83752,33 @@
         <v>0.343</v>
       </c>
       <c r="I30" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K30" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L30" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B31" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C31" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D31" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E31" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F31" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G31" t="n">
         <v>0.462</v>
@@ -83728,109 +83787,106 @@
         <v>0.343</v>
       </c>
       <c r="I31" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K31" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L31" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B32" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C32" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D32" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E32" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F32" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G32" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H32" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I32" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J32" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K32" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L32" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B33" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C33" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D33" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E33" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F33" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G33" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H33" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I33" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J33" t="n">
         <v>0.014</v>
       </c>
       <c r="K33" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L33" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B34" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C34" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D34" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E34" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F34" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G34" t="n">
         <v>0.395</v>
@@ -83845,9 +83901,47 @@
         <v>0.014</v>
       </c>
       <c r="K34" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L34" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B35" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C35" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K35" t="n">
         <v>12.277</v>
       </c>
-      <c r="L34" t="n">
+      <c r="L35" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -84288,7 +84382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R34"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84388,497 +84482,497 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="B2" t="n">
-        <v>1372566</v>
+        <v>1423202</v>
       </c>
       <c r="C2" t="n">
-        <v>535686</v>
+        <v>455161</v>
       </c>
       <c r="D2" t="n">
-        <v>1384220</v>
+        <v>1401725</v>
       </c>
       <c r="E2" t="n">
         <v>9500</v>
       </c>
       <c r="F2" t="n">
-        <v>1750778</v>
+        <v>1790742</v>
       </c>
       <c r="G2" t="n">
-        <v>1443098</v>
+        <v>1378077</v>
       </c>
       <c r="I2" t="n">
-        <v>1497314</v>
+        <v>1506700</v>
       </c>
       <c r="K2" t="n">
-        <v>243577</v>
+        <v>300344</v>
       </c>
       <c r="M2" t="n">
-        <v>2692467</v>
+        <v>1992032</v>
       </c>
       <c r="N2" t="n">
-        <v>188088</v>
+        <v>92394</v>
       </c>
       <c r="O2" t="n">
-        <v>230944</v>
+        <v>137551</v>
       </c>
       <c r="P2" t="n">
-        <v>393254</v>
+        <v>393389</v>
       </c>
       <c r="Q2" t="n">
-        <v>665576</v>
+        <v>478122</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B3" t="n">
-        <v>1383237</v>
+        <v>1372566</v>
       </c>
       <c r="C3" t="n">
-        <v>642612</v>
+        <v>535686</v>
       </c>
       <c r="D3" t="n">
-        <v>1376983</v>
+        <v>1384220</v>
       </c>
       <c r="E3" t="n">
-        <v>9000</v>
+        <v>9500</v>
       </c>
       <c r="F3" t="n">
-        <v>1886772</v>
+        <v>1750778</v>
       </c>
       <c r="G3" t="n">
-        <v>1487288</v>
+        <v>1443098</v>
       </c>
       <c r="I3" t="n">
-        <v>1545952</v>
+        <v>1497314</v>
       </c>
       <c r="K3" t="n">
-        <v>145193</v>
+        <v>243577</v>
       </c>
       <c r="M3" t="n">
-        <v>2689526</v>
+        <v>2692467</v>
       </c>
       <c r="N3" t="n">
-        <v>309125</v>
+        <v>188088</v>
       </c>
       <c r="O3" t="n">
-        <v>432534</v>
+        <v>230944</v>
       </c>
       <c r="P3" t="n">
-        <v>399049</v>
+        <v>393254</v>
       </c>
       <c r="Q3" t="n">
-        <v>681693</v>
+        <v>665576</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B4" t="n">
-        <v>1326845</v>
+        <v>1383237</v>
       </c>
       <c r="C4" t="n">
-        <v>630343</v>
+        <v>642612</v>
       </c>
       <c r="D4" t="n">
-        <v>1389820</v>
+        <v>1376983</v>
       </c>
       <c r="E4" t="n">
         <v>9000</v>
       </c>
       <c r="F4" t="n">
-        <v>1898634</v>
+        <v>1886772</v>
       </c>
       <c r="G4" t="n">
-        <v>1230443</v>
+        <v>1487288</v>
       </c>
       <c r="I4" t="n">
-        <v>1509954</v>
+        <v>1545952</v>
       </c>
       <c r="K4" t="n">
-        <v>223405</v>
+        <v>145193</v>
       </c>
       <c r="M4" t="n">
-        <v>2637144</v>
+        <v>2689526</v>
       </c>
       <c r="N4" t="n">
-        <v>322000</v>
+        <v>309125</v>
       </c>
       <c r="O4" t="n">
-        <v>445186</v>
+        <v>432534</v>
       </c>
       <c r="P4" t="n">
-        <v>392284</v>
+        <v>399049</v>
       </c>
       <c r="Q4" t="n">
-        <v>707427</v>
+        <v>681693</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B5" t="n">
-        <v>1453284</v>
+        <v>1326845</v>
       </c>
       <c r="C5" t="n">
-        <v>668222</v>
+        <v>630343</v>
       </c>
       <c r="D5" t="n">
-        <v>1399375</v>
+        <v>1389820</v>
       </c>
       <c r="E5" t="n">
         <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>1997673</v>
+        <v>1898634</v>
       </c>
       <c r="G5" t="n">
-        <v>1229304</v>
+        <v>1230443</v>
       </c>
       <c r="I5" t="n">
-        <v>1526881</v>
+        <v>1509954</v>
       </c>
       <c r="K5" t="n">
-        <v>210710</v>
+        <v>223405</v>
       </c>
       <c r="M5" t="n">
-        <v>2315158</v>
+        <v>2637144</v>
       </c>
       <c r="N5" t="n">
-        <v>274632</v>
+        <v>322000</v>
       </c>
       <c r="O5" t="n">
-        <v>404378</v>
+        <v>445186</v>
       </c>
       <c r="P5" t="n">
-        <v>393345</v>
+        <v>392284</v>
       </c>
       <c r="Q5" t="n">
-        <v>702775</v>
+        <v>707427</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B6" t="n">
-        <v>1428345</v>
+        <v>1453284</v>
       </c>
       <c r="C6" t="n">
-        <v>613887</v>
+        <v>668222</v>
       </c>
       <c r="D6" t="n">
-        <v>1360335</v>
+        <v>1399375</v>
       </c>
       <c r="E6" t="n">
         <v>9000</v>
       </c>
       <c r="F6" t="n">
-        <v>2000629</v>
+        <v>1997673</v>
       </c>
       <c r="G6" t="n">
-        <v>1229134</v>
+        <v>1229304</v>
       </c>
       <c r="I6" t="n">
-        <v>1516881</v>
+        <v>1526881</v>
       </c>
       <c r="K6" t="n">
-        <v>265281</v>
+        <v>210710</v>
       </c>
       <c r="M6" t="n">
-        <v>2655010</v>
+        <v>2315158</v>
       </c>
       <c r="N6" t="n">
-        <v>275644</v>
+        <v>274632</v>
       </c>
       <c r="O6" t="n">
-        <v>405391</v>
+        <v>404378</v>
       </c>
       <c r="P6" t="n">
         <v>393345</v>
       </c>
       <c r="Q6" t="n">
-        <v>735394</v>
+        <v>702775</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B7" t="n">
-        <v>1453305</v>
+        <v>1428345</v>
       </c>
       <c r="C7" t="n">
-        <v>660021</v>
+        <v>613887</v>
       </c>
       <c r="D7" t="n">
-        <v>1394810</v>
+        <v>1360335</v>
       </c>
       <c r="E7" t="n">
         <v>9000</v>
       </c>
       <c r="F7" t="n">
-        <v>1966997</v>
+        <v>2000629</v>
       </c>
       <c r="G7" t="n">
-        <v>1358589</v>
+        <v>1229134</v>
       </c>
       <c r="I7" t="n">
-        <v>1530881</v>
+        <v>1516881</v>
       </c>
       <c r="K7" t="n">
-        <v>224505</v>
+        <v>265281</v>
       </c>
       <c r="M7" t="n">
-        <v>2605275</v>
+        <v>2655010</v>
       </c>
       <c r="N7" t="n">
-        <v>273068</v>
+        <v>275644</v>
       </c>
       <c r="O7" t="n">
-        <v>402811</v>
+        <v>405391</v>
       </c>
       <c r="P7" t="n">
-        <v>368707</v>
+        <v>393345</v>
       </c>
       <c r="Q7" t="n">
-        <v>750038</v>
+        <v>735394</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B8" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C8" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D8" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E8" t="n">
         <v>9000</v>
       </c>
       <c r="F8" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G8" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I8" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K8" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M8" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N8" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O8" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P8" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q8" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B9" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C9" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D9" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E9" t="n">
         <v>9000</v>
       </c>
       <c r="F9" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G9" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I9" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K9" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M9" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N9" t="n">
         <v>214475</v>
       </c>
       <c r="O9" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P9" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q9" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B10" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C10" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D10" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E10" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F10" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G10" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I10" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K10" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M10" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P10" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q10" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B11" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C11" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D11" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E11" t="n">
         <v>9200</v>
       </c>
       <c r="F11" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G11" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I11" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K11" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M11" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P11" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q11" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B12" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C12" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D12" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G12" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I12" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K12" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M12" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N12" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P12" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q12" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B13" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C13" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D13" t="n">
         <v>1336369</v>
@@ -84887,28 +84981,28 @@
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G13" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I13" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K13" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M13" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N13" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O13" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P13" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q13" t="n">
         <v>710782</v>
@@ -84916,34 +85010,34 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B14" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C14" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D14" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E14" t="n">
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G14" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I14" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K14" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M14" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N14" t="n">
         <v>214475</v>
@@ -84952,7 +85046,7 @@
         <v>238857</v>
       </c>
       <c r="P14" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q14" t="n">
         <v>710782</v>
@@ -84960,43 +85054,43 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B15" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C15" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D15" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G15" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I15" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K15" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M15" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N15" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O15" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P15" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q15" t="n">
         <v>710782</v>
@@ -85004,201 +85098,201 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B16" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C16" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D16" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E16" t="n">
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G16" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I16" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K16" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M16" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N16" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O16" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P16" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q16" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B17" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C17" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D17" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E17" t="n">
         <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G17" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I17" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K17" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M17" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N17" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O17" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P17" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q17" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B18" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C18" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D18" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E18" t="n">
         <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G18" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I18" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K18" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M18" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N18" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O18" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P18" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q18" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B19" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C19" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D19" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E19" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G19" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I19" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K19" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M19" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N19" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O19" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P19" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q19" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B20" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C20" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D20" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E20" t="n">
         <v>9400</v>
       </c>
       <c r="F20" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G20" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I20" t="n">
         <v>1493578</v>
@@ -85207,7 +85301,7 @@
         <v>270165</v>
       </c>
       <c r="M20" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N20" t="n">
         <v>214475</v>
@@ -85219,39 +85313,39 @@
         <v>380581</v>
       </c>
       <c r="Q20" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B21" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C21" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D21" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E21" t="n">
         <v>9400</v>
       </c>
       <c r="F21" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G21" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I21" t="n">
         <v>1493578</v>
       </c>
       <c r="K21" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M21" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N21" t="n">
         <v>214475</v>
@@ -85260,153 +85354,153 @@
         <v>236857</v>
       </c>
       <c r="P21" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q21" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B22" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C22" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D22" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E22" t="n">
         <v>9400</v>
       </c>
       <c r="F22" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G22" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I22" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K22" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M22" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N22" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O22" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P22" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q22" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B23" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C23" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D23" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E23" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F23" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G23" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I23" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K23" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M23" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N23" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O23" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P23" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q23" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B24" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C24" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D24" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E24" t="n">
         <v>9200</v>
       </c>
       <c r="F24" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G24" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I24" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K24" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M24" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N24" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O24" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P24" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q24" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B25" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C25" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D25" t="n">
         <v>1438502</v>
@@ -85415,107 +85509,107 @@
         <v>9200</v>
       </c>
       <c r="F25" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G25" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I25" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K25" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M25" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N25" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O25" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P25" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q25" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B26" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C26" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D26" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E26" t="n">
         <v>9200</v>
       </c>
       <c r="F26" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G26" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I26" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K26" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M26" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N26" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O26" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P26" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q26" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B27" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C27" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D27" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E27" t="n">
         <v>9200</v>
       </c>
       <c r="F27" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G27" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I27" t="n">
         <v>1488515</v>
       </c>
       <c r="K27" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M27" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N27" t="n">
         <v>214475</v>
@@ -85524,7 +85618,7 @@
         <v>247857</v>
       </c>
       <c r="P27" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q27" t="n">
         <v>738429</v>
@@ -85532,34 +85626,34 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B28" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C28" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D28" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E28" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F28" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G28" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I28" t="n">
         <v>1488515</v>
       </c>
       <c r="K28" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M28" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N28" t="n">
         <v>214475</v>
@@ -85568,7 +85662,7 @@
         <v>247857</v>
       </c>
       <c r="P28" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q28" t="n">
         <v>738429</v>
@@ -85576,78 +85670,78 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B29" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C29" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D29" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E29" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F29" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G29" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I29" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K29" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M29" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N29" t="n">
         <v>214475</v>
       </c>
       <c r="O29" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P29" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q29" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B30" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C30" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D30" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E30" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F30" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G30" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I30" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K30" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M30" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N30" t="n">
         <v>214475</v>
@@ -85656,42 +85750,42 @@
         <v>264857</v>
       </c>
       <c r="P30" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q30" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B31" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C31" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D31" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E31" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F31" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G31" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I31" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K31" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M31" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N31" t="n">
         <v>214475</v>
@@ -85700,101 +85794,98 @@
         <v>264857</v>
       </c>
       <c r="P31" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q31" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B32" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C32" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D32" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E32" t="n">
         <v>9300</v>
       </c>
       <c r="F32" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G32" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I32" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K32" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M32" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N32" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O32" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P32" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q32" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R32" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B33" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C33" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D33" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E33" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F33" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G33" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I33" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K33" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M33" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N33" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O33" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P33" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q33" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R33" t="n">
         <v>15000</v>
@@ -85802,40 +85893,40 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B34" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C34" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D34" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E34" t="n">
         <v>9100</v>
       </c>
       <c r="F34" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G34" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I34" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K34" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M34" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N34" t="n">
         <v>189475</v>
       </c>
       <c r="O34" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P34" t="n">
         <v>375660</v>
@@ -85844,6 +85935,53 @@
         <v>773586</v>
       </c>
       <c r="R34" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B35" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C35" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E35" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K35" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M35" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N35" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O35" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P35" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R35" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feedgas backfill: [ 35/119] 2026-08-24 ~ 13/17 meters metered 10.91 Bcf/d missing: Calcasieu Pass (ANR), Cameron (CGT), Cove Point (cpl), Plaquemines (CGT) | elapsed 0:31 ~1:14 left
</commit_message>
<xml_diff>
--- a/americas/feedgas_ebb/lng_feedgas_daily.xlsx
+++ b/americas/feedgas_ebb/lng_feedgas_daily.xlsx
@@ -80223,9 +80223,36 @@
       <c r="A2429" s="4" t="n">
         <v>46258</v>
       </c>
+      <c r="B2429" t="n">
+        <v>3.171</v>
+      </c>
+      <c r="C2429" t="n">
+        <v>3.166</v>
+      </c>
+      <c r="D2429" t="n">
+        <v>1.453</v>
+      </c>
+      <c r="E2429" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="F2429" t="n">
+        <v>1.648</v>
+      </c>
+      <c r="G2429" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="H2429" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="I2429" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="K2429" t="n">
+        <v>10.913</v>
+      </c>
       <c r="L2429" t="inlineStr">
         <is>
-          <t>no data yet (EIA runs 2-3 months behind)</t>
+          <t>metered</t>
         </is>
       </c>
     </row>
@@ -81507,7 +81534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81572,409 +81599,409 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B2" t="n">
-        <v>3.172</v>
+        <v>3.171</v>
       </c>
       <c r="C2" t="n">
-        <v>3.056</v>
+        <v>3.166</v>
       </c>
       <c r="D2" t="n">
         <v>1.453</v>
       </c>
       <c r="E2" t="n">
-        <v>0.29</v>
+        <v>0.175</v>
       </c>
       <c r="F2" t="n">
-        <v>1.921</v>
+        <v>1.648</v>
       </c>
       <c r="G2" t="n">
-        <v>0.222</v>
+        <v>0.198</v>
       </c>
       <c r="H2" t="n">
-        <v>0.379</v>
+        <v>0.381</v>
       </c>
       <c r="I2" t="n">
-        <v>0.461</v>
+        <v>0.721</v>
       </c>
       <c r="K2" t="n">
-        <v>10.954</v>
+        <v>10.912</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="B3" t="n">
-        <v>3.184</v>
+        <v>3.172</v>
       </c>
       <c r="C3" t="n">
-        <v>3.08</v>
+        <v>3.056</v>
       </c>
       <c r="D3" t="n">
-        <v>1.444</v>
+        <v>1.453</v>
       </c>
       <c r="E3" t="n">
-        <v>0.235</v>
+        <v>0.29</v>
       </c>
       <c r="F3" t="n">
-        <v>2.596</v>
+        <v>1.921</v>
       </c>
       <c r="G3" t="n">
-        <v>0.404</v>
+        <v>0.222</v>
       </c>
       <c r="H3" t="n">
         <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.642</v>
+        <v>0.461</v>
       </c>
       <c r="K3" t="n">
-        <v>11.964</v>
+        <v>10.954</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B4" t="n">
-        <v>3.29</v>
+        <v>3.184</v>
       </c>
       <c r="C4" t="n">
-        <v>3.254</v>
+        <v>3.08</v>
       </c>
       <c r="D4" t="n">
-        <v>1.491</v>
+        <v>1.444</v>
       </c>
       <c r="E4" t="n">
-        <v>0.14</v>
+        <v>0.235</v>
       </c>
       <c r="F4" t="n">
-        <v>2.594</v>
+        <v>2.596</v>
       </c>
       <c r="G4" t="n">
-        <v>0.715</v>
+        <v>0.404</v>
       </c>
       <c r="H4" t="n">
-        <v>0.385</v>
+        <v>0.379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.657</v>
+        <v>0.642</v>
       </c>
       <c r="K4" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B5" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C5" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D5" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E5" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F5" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G5" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H5" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K5" t="n">
-        <v>12.269</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B6" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C6" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D6" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E6" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F6" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G6" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H6" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I6" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>12.136</v>
+        <v>12.269</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B7" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C7" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D7" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E7" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F7" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G7" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H7" t="n">
         <v>0.379</v>
       </c>
       <c r="I7" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K7" t="n">
-        <v>12.428</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B8" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C8" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D8" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E8" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F8" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G8" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H8" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I8" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K8" t="n">
-        <v>12.534</v>
+        <v>12.428</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B9" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C9" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D9" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E9" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F9" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G9" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H9" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I9" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K9" t="n">
-        <v>12.108</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B10" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C10" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D10" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E10" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F10" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G10" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H10" t="n">
         <v>0.342</v>
       </c>
       <c r="I10" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K10" t="n">
-        <v>11.344</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B11" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C11" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D11" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E11" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F11" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G11" t="n">
         <v>0.444</v>
       </c>
       <c r="H11" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I11" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K11" t="n">
-        <v>11.786</v>
+        <v>11.344</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B12" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C12" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D12" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E12" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F12" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G12" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H12" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I12" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K12" t="n">
-        <v>12.376</v>
+        <v>11.786</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B13" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C13" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D13" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E13" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F13" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G13" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H13" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K13" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B14" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C14" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D14" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E14" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F14" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G14" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
@@ -81983,27 +82010,27 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B15" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C15" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D15" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E15" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F15" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G15" t="n">
         <v>0.437</v>
@@ -82015,178 +82042,178 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>11.937</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B16" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C16" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D16" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E16" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F16" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G16" t="n">
         <v>0.437</v>
       </c>
       <c r="H16" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I16" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>11.964</v>
+        <v>11.937</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B17" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C17" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D17" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E17" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F17" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G17" t="n">
         <v>0.437</v>
       </c>
       <c r="H17" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I17" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>12.126</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B18" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C18" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D18" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F18" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G18" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H18" t="n">
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K18" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B19" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C19" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D19" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E19" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F19" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G19" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H19" t="n">
         <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B20" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C20" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D20" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E20" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F20" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G20" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H20" t="n">
         <v>0.367</v>
       </c>
       <c r="I20" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K20" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B21" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C21" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D21" t="n">
         <v>1.44</v>
@@ -82195,7 +82222,7 @@
         <v>0.261</v>
       </c>
       <c r="F21" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G21" t="n">
         <v>0.435</v>
@@ -82204,222 +82231,222 @@
         <v>0.367</v>
       </c>
       <c r="I21" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K21" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B22" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C22" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D22" t="n">
         <v>1.44</v>
       </c>
       <c r="E22" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F22" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G22" t="n">
         <v>0.435</v>
       </c>
       <c r="H22" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I22" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K22" t="n">
-        <v>12.228</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B23" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C23" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D23" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E23" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F23" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G23" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H23" t="n">
         <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K23" t="n">
-        <v>12.021</v>
+        <v>12.228</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B24" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C24" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D24" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F24" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G24" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H24" t="n">
         <v>0.365</v>
       </c>
       <c r="I24" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K24" t="n">
-        <v>12.107</v>
+        <v>12.021</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B25" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C25" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D25" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E25" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F25" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G25" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H25" t="n">
         <v>0.365</v>
       </c>
       <c r="I25" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K25" t="n">
-        <v>12.271</v>
+        <v>12.107</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B26" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C26" t="n">
         <v>3.232</v>
       </c>
       <c r="D26" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F26" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G26" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H26" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I26" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K26" t="n">
-        <v>12.632</v>
+        <v>12.271</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B27" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C27" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D27" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E27" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F27" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G27" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H27" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I27" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K27" t="n">
-        <v>12.569</v>
+        <v>12.632</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B28" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C28" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D28" t="n">
         <v>1.435</v>
       </c>
       <c r="E28" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F28" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G28" t="n">
         <v>0.446</v>
@@ -82431,27 +82458,27 @@
         <v>0.712</v>
       </c>
       <c r="K28" t="n">
-        <v>12.277</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B29" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C29" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D29" t="n">
         <v>1.435</v>
       </c>
       <c r="E29" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F29" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G29" t="n">
         <v>0.446</v>
@@ -82463,59 +82490,59 @@
         <v>0.712</v>
       </c>
       <c r="K29" t="n">
-        <v>12.223</v>
+        <v>12.277</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B30" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C30" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D30" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E30" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F30" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G30" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H30" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I30" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K30" t="n">
-        <v>12.187</v>
+        <v>12.223</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B31" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C31" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D31" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E31" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F31" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G31" t="n">
         <v>0.462</v>
@@ -82524,30 +82551,30 @@
         <v>0.343</v>
       </c>
       <c r="I31" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K31" t="n">
-        <v>12.079</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B32" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C32" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D32" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E32" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F32" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G32" t="n">
         <v>0.462</v>
@@ -82556,100 +82583,97 @@
         <v>0.343</v>
       </c>
       <c r="I32" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K32" t="n">
-        <v>12.117</v>
+        <v>12.079</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B33" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C33" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D33" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E33" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F33" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G33" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H33" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I33" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K33" t="n">
-        <v>12.374</v>
+        <v>12.117</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B34" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C34" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D34" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E34" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F34" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G34" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H34" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I34" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J34" t="n">
         <v>0.014</v>
       </c>
       <c r="K34" t="n">
-        <v>12.643</v>
+        <v>12.374</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B35" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C35" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D35" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E35" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F35" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G35" t="n">
         <v>0.395</v>
@@ -82664,6 +82688,41 @@
         <v>0.014</v>
       </c>
       <c r="K35" t="n">
+        <v>12.643</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B36" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K36" t="n">
         <v>12.278</v>
       </c>
     </row>
@@ -82678,7 +82737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82748,445 +82807,445 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B2" t="n">
-        <v>3.172</v>
+        <v>3.171</v>
       </c>
       <c r="C2" t="n">
-        <v>3.056</v>
+        <v>3.166</v>
       </c>
       <c r="D2" t="n">
         <v>1.453</v>
       </c>
       <c r="E2" t="n">
-        <v>0.29</v>
+        <v>0.175</v>
       </c>
       <c r="F2" t="n">
-        <v>1.921</v>
+        <v>1.648</v>
       </c>
       <c r="G2" t="n">
-        <v>0.222</v>
+        <v>0.198</v>
       </c>
       <c r="H2" t="n">
-        <v>0.379</v>
+        <v>0.381</v>
       </c>
       <c r="I2" t="n">
-        <v>0.461</v>
+        <v>0.721</v>
       </c>
       <c r="K2" t="n">
-        <v>10.954</v>
+        <v>10.913</v>
       </c>
       <c r="L2" t="n">
-        <v>10.954</v>
+        <v>10.913</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="B3" t="n">
-        <v>3.184</v>
+        <v>3.172</v>
       </c>
       <c r="C3" t="n">
-        <v>3.08</v>
+        <v>3.056</v>
       </c>
       <c r="D3" t="n">
-        <v>1.444</v>
+        <v>1.453</v>
       </c>
       <c r="E3" t="n">
-        <v>0.235</v>
+        <v>0.29</v>
       </c>
       <c r="F3" t="n">
-        <v>2.596</v>
+        <v>1.921</v>
       </c>
       <c r="G3" t="n">
-        <v>0.404</v>
+        <v>0.222</v>
       </c>
       <c r="H3" t="n">
         <v>0.379</v>
       </c>
       <c r="I3" t="n">
-        <v>0.642</v>
+        <v>0.461</v>
       </c>
       <c r="K3" t="n">
-        <v>11.964</v>
+        <v>10.954</v>
       </c>
       <c r="L3" t="n">
-        <v>11.964</v>
+        <v>10.954</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B4" t="n">
-        <v>3.29</v>
+        <v>3.184</v>
       </c>
       <c r="C4" t="n">
-        <v>3.254</v>
+        <v>3.08</v>
       </c>
       <c r="D4" t="n">
-        <v>1.491</v>
+        <v>1.444</v>
       </c>
       <c r="E4" t="n">
-        <v>0.14</v>
+        <v>0.235</v>
       </c>
       <c r="F4" t="n">
-        <v>2.594</v>
+        <v>2.596</v>
       </c>
       <c r="G4" t="n">
-        <v>0.715</v>
+        <v>0.404</v>
       </c>
       <c r="H4" t="n">
-        <v>0.385</v>
+        <v>0.379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.657</v>
+        <v>0.642</v>
       </c>
       <c r="K4" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
       <c r="L4" t="n">
-        <v>12.526</v>
+        <v>11.964</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B5" t="n">
-        <v>3.236</v>
+        <v>3.29</v>
       </c>
       <c r="C5" t="n">
-        <v>3.017</v>
+        <v>3.254</v>
       </c>
       <c r="D5" t="n">
-        <v>1.456</v>
+        <v>1.491</v>
       </c>
       <c r="E5" t="n">
-        <v>0.215</v>
+        <v>0.14</v>
       </c>
       <c r="F5" t="n">
-        <v>2.543</v>
+        <v>2.594</v>
       </c>
       <c r="G5" t="n">
-        <v>0.74</v>
+        <v>0.715</v>
       </c>
       <c r="H5" t="n">
-        <v>0.378</v>
+        <v>0.385</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.657</v>
       </c>
       <c r="K5" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
       <c r="L5" t="n">
-        <v>12.267</v>
+        <v>12.526</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B6" t="n">
-        <v>3.404</v>
+        <v>3.236</v>
       </c>
       <c r="C6" t="n">
-        <v>3.112</v>
+        <v>3.017</v>
       </c>
       <c r="D6" t="n">
-        <v>1.472</v>
+        <v>1.456</v>
       </c>
       <c r="E6" t="n">
-        <v>0.203</v>
+        <v>0.215</v>
       </c>
       <c r="F6" t="n">
-        <v>2.233</v>
+        <v>2.543</v>
       </c>
       <c r="G6" t="n">
-        <v>0.655</v>
+        <v>0.74</v>
       </c>
       <c r="H6" t="n">
-        <v>0.379</v>
+        <v>0.378</v>
       </c>
       <c r="I6" t="n">
-        <v>0.678</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
       <c r="L6" t="n">
-        <v>12.136</v>
+        <v>12.267</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B7" t="n">
-        <v>3.29</v>
+        <v>3.404</v>
       </c>
       <c r="C7" t="n">
-        <v>3.115</v>
+        <v>3.112</v>
       </c>
       <c r="D7" t="n">
-        <v>1.463</v>
+        <v>1.472</v>
       </c>
       <c r="E7" t="n">
-        <v>0.256</v>
+        <v>0.203</v>
       </c>
       <c r="F7" t="n">
-        <v>2.56</v>
+        <v>2.233</v>
       </c>
       <c r="G7" t="n">
-        <v>0.657</v>
+        <v>0.655</v>
       </c>
       <c r="H7" t="n">
         <v>0.379</v>
       </c>
       <c r="I7" t="n">
-        <v>0.709</v>
+        <v>0.678</v>
       </c>
       <c r="K7" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
       <c r="L7" t="n">
-        <v>12.429</v>
+        <v>12.136</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B8" t="n">
-        <v>3.392</v>
+        <v>3.29</v>
       </c>
       <c r="C8" t="n">
-        <v>3.207</v>
+        <v>3.115</v>
       </c>
       <c r="D8" t="n">
-        <v>1.476</v>
+        <v>1.463</v>
       </c>
       <c r="E8" t="n">
-        <v>0.216</v>
+        <v>0.256</v>
       </c>
       <c r="F8" t="n">
-        <v>2.512</v>
+        <v>2.56</v>
       </c>
       <c r="G8" t="n">
-        <v>0.652</v>
+        <v>0.657</v>
       </c>
       <c r="H8" t="n">
-        <v>0.356</v>
+        <v>0.379</v>
       </c>
       <c r="I8" t="n">
-        <v>0.723</v>
+        <v>0.709</v>
       </c>
       <c r="K8" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
       <c r="L8" t="n">
-        <v>12.534</v>
+        <v>12.429</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B9" t="n">
-        <v>3.163</v>
+        <v>3.392</v>
       </c>
       <c r="C9" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="D9" t="n">
-        <v>1.472</v>
+        <v>1.476</v>
       </c>
       <c r="E9" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F9" t="n">
-        <v>2.634</v>
+        <v>2.512</v>
       </c>
       <c r="G9" t="n">
-        <v>0.424</v>
+        <v>0.652</v>
       </c>
       <c r="H9" t="n">
-        <v>0.342</v>
+        <v>0.356</v>
       </c>
       <c r="I9" t="n">
-        <v>0.593</v>
+        <v>0.723</v>
       </c>
       <c r="K9" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
       <c r="L9" t="n">
-        <v>12.109</v>
+        <v>12.534</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B10" t="n">
-        <v>2.659</v>
+        <v>3.163</v>
       </c>
       <c r="C10" t="n">
-        <v>3.117</v>
+        <v>3.205</v>
       </c>
       <c r="D10" t="n">
-        <v>1.454</v>
+        <v>1.472</v>
       </c>
       <c r="E10" t="n">
-        <v>0.206</v>
+        <v>0.276</v>
       </c>
       <c r="F10" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G10" t="n">
-        <v>0.444</v>
+        <v>0.424</v>
       </c>
       <c r="H10" t="n">
         <v>0.342</v>
       </c>
       <c r="I10" t="n">
-        <v>0.491</v>
+        <v>0.593</v>
       </c>
       <c r="K10" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
       <c r="L10" t="n">
-        <v>11.345</v>
+        <v>12.109</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B11" t="n">
-        <v>3.062</v>
+        <v>2.659</v>
       </c>
       <c r="C11" t="n">
-        <v>3.142</v>
+        <v>3.117</v>
       </c>
       <c r="D11" t="n">
-        <v>1.386</v>
+        <v>1.454</v>
       </c>
       <c r="E11" t="n">
-        <v>0.205</v>
+        <v>0.206</v>
       </c>
       <c r="F11" t="n">
-        <v>2.581</v>
+        <v>2.632</v>
       </c>
       <c r="G11" t="n">
         <v>0.444</v>
       </c>
       <c r="H11" t="n">
-        <v>0.32</v>
+        <v>0.342</v>
       </c>
       <c r="I11" t="n">
-        <v>0.647</v>
+        <v>0.491</v>
       </c>
       <c r="K11" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
       <c r="L11" t="n">
-        <v>11.787</v>
+        <v>11.345</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B12" t="n">
-        <v>3.405</v>
+        <v>3.062</v>
       </c>
       <c r="C12" t="n">
-        <v>3.204</v>
+        <v>3.142</v>
       </c>
       <c r="D12" t="n">
-        <v>1.474</v>
+        <v>1.386</v>
       </c>
       <c r="E12" t="n">
-        <v>0.247</v>
+        <v>0.205</v>
       </c>
       <c r="F12" t="n">
-        <v>2.571</v>
+        <v>2.581</v>
       </c>
       <c r="G12" t="n">
-        <v>0.438</v>
+        <v>0.444</v>
       </c>
       <c r="H12" t="n">
-        <v>0.366</v>
+        <v>0.32</v>
       </c>
       <c r="I12" t="n">
-        <v>0.671</v>
+        <v>0.647</v>
       </c>
       <c r="K12" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
       <c r="L12" t="n">
-        <v>12.376</v>
+        <v>11.787</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B13" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="C13" t="n">
-        <v>3.261</v>
+        <v>3.204</v>
       </c>
       <c r="D13" t="n">
-        <v>1.478</v>
+        <v>1.474</v>
       </c>
       <c r="E13" t="n">
-        <v>0.297</v>
+        <v>0.247</v>
       </c>
       <c r="F13" t="n">
-        <v>2.592</v>
+        <v>2.571</v>
       </c>
       <c r="G13" t="n">
-        <v>0.27</v>
+        <v>0.438</v>
       </c>
       <c r="H13" t="n">
-        <v>0.367</v>
+        <v>0.366</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.671</v>
       </c>
       <c r="K13" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
       <c r="L13" t="n">
-        <v>12.341</v>
+        <v>12.376</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B14" t="n">
-        <v>3.177</v>
+        <v>3.391</v>
       </c>
       <c r="C14" t="n">
-        <v>2.859</v>
+        <v>3.261</v>
       </c>
       <c r="D14" t="n">
-        <v>1.485</v>
+        <v>1.478</v>
       </c>
       <c r="E14" t="n">
-        <v>0.335</v>
+        <v>0.297</v>
       </c>
       <c r="F14" t="n">
-        <v>2.586</v>
+        <v>2.592</v>
       </c>
       <c r="G14" t="n">
-        <v>0.437</v>
+        <v>0.27</v>
       </c>
       <c r="H14" t="n">
         <v>0.367</v>
@@ -83195,30 +83254,30 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
       <c r="L14" t="n">
-        <v>11.931</v>
+        <v>12.341</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B15" t="n">
-        <v>3.227</v>
+        <v>3.177</v>
       </c>
       <c r="C15" t="n">
-        <v>3.139</v>
+        <v>2.859</v>
       </c>
       <c r="D15" t="n">
-        <v>1.24</v>
+        <v>1.485</v>
       </c>
       <c r="E15" t="n">
-        <v>0.287</v>
+        <v>0.335</v>
       </c>
       <c r="F15" t="n">
-        <v>2.554</v>
+        <v>2.586</v>
       </c>
       <c r="G15" t="n">
         <v>0.437</v>
@@ -83230,196 +83289,196 @@
         <v>0.6850000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
       <c r="L15" t="n">
-        <v>11.936</v>
+        <v>11.931</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B16" t="n">
-        <v>3.205</v>
+        <v>3.227</v>
       </c>
       <c r="C16" t="n">
-        <v>3.213</v>
+        <v>3.139</v>
       </c>
       <c r="D16" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="E16" t="n">
-        <v>0.205</v>
+        <v>0.287</v>
       </c>
       <c r="F16" t="n">
-        <v>2.58</v>
+        <v>2.554</v>
       </c>
       <c r="G16" t="n">
         <v>0.437</v>
       </c>
       <c r="H16" t="n">
-        <v>0.361</v>
+        <v>0.367</v>
       </c>
       <c r="I16" t="n">
         <v>0.6850000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
       <c r="L16" t="n">
-        <v>11.961</v>
+        <v>11.936</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B17" t="n">
-        <v>3.215</v>
+        <v>3.205</v>
       </c>
       <c r="C17" t="n">
-        <v>3.214</v>
+        <v>3.213</v>
       </c>
       <c r="D17" t="n">
-        <v>1.464</v>
+        <v>1.275</v>
       </c>
       <c r="E17" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="F17" t="n">
-        <v>2.594</v>
+        <v>2.58</v>
       </c>
       <c r="G17" t="n">
         <v>0.437</v>
       </c>
       <c r="H17" t="n">
-        <v>0.367</v>
+        <v>0.361</v>
       </c>
       <c r="I17" t="n">
-        <v>0.627</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
       <c r="L17" t="n">
-        <v>12.126</v>
+        <v>11.961</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B18" t="n">
-        <v>3.334</v>
+        <v>3.215</v>
       </c>
       <c r="C18" t="n">
-        <v>3.234</v>
+        <v>3.214</v>
       </c>
       <c r="D18" t="n">
-        <v>1.361</v>
+        <v>1.464</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3</v>
+        <v>0.208</v>
       </c>
       <c r="F18" t="n">
-        <v>2.609</v>
+        <v>2.594</v>
       </c>
       <c r="G18" t="n">
-        <v>0.457</v>
+        <v>0.437</v>
       </c>
       <c r="H18" t="n">
         <v>0.367</v>
       </c>
       <c r="I18" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.627</v>
       </c>
       <c r="K18" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
       <c r="L18" t="n">
-        <v>12.347</v>
+        <v>12.126</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B19" t="n">
-        <v>3.287</v>
+        <v>3.334</v>
       </c>
       <c r="C19" t="n">
-        <v>3.198</v>
+        <v>3.234</v>
       </c>
       <c r="D19" t="n">
-        <v>1.48</v>
+        <v>1.361</v>
       </c>
       <c r="E19" t="n">
-        <v>0.278</v>
+        <v>0.3</v>
       </c>
       <c r="F19" t="n">
-        <v>2.607</v>
+        <v>2.609</v>
       </c>
       <c r="G19" t="n">
-        <v>0.288</v>
+        <v>0.457</v>
       </c>
       <c r="H19" t="n">
         <v>0.367</v>
       </c>
       <c r="I19" t="n">
-        <v>0.666</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
       <c r="L19" t="n">
-        <v>12.171</v>
+        <v>12.347</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B20" t="n">
-        <v>3.244</v>
+        <v>3.287</v>
       </c>
       <c r="C20" t="n">
-        <v>3.247</v>
+        <v>3.198</v>
       </c>
       <c r="D20" t="n">
-        <v>1.44</v>
+        <v>1.48</v>
       </c>
       <c r="E20" t="n">
-        <v>0.261</v>
+        <v>0.278</v>
       </c>
       <c r="F20" t="n">
-        <v>2.638</v>
+        <v>2.607</v>
       </c>
       <c r="G20" t="n">
-        <v>0.435</v>
+        <v>0.288</v>
       </c>
       <c r="H20" t="n">
         <v>0.367</v>
       </c>
       <c r="I20" t="n">
-        <v>0.662</v>
+        <v>0.666</v>
       </c>
       <c r="K20" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
       <c r="L20" t="n">
-        <v>12.294</v>
+        <v>12.171</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B21" t="n">
-        <v>3.218</v>
+        <v>3.244</v>
       </c>
       <c r="C21" t="n">
-        <v>3.218</v>
+        <v>3.247</v>
       </c>
       <c r="D21" t="n">
         <v>1.44</v>
@@ -83428,7 +83487,7 @@
         <v>0.261</v>
       </c>
       <c r="F21" t="n">
-        <v>2.635</v>
+        <v>2.638</v>
       </c>
       <c r="G21" t="n">
         <v>0.435</v>
@@ -83437,243 +83496,243 @@
         <v>0.367</v>
       </c>
       <c r="I21" t="n">
-        <v>0.659</v>
+        <v>0.662</v>
       </c>
       <c r="K21" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
       <c r="L21" t="n">
-        <v>12.233</v>
+        <v>12.294</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B22" t="n">
-        <v>3.21</v>
+        <v>3.218</v>
       </c>
       <c r="C22" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="D22" t="n">
         <v>1.44</v>
       </c>
       <c r="E22" t="n">
-        <v>0.28</v>
+        <v>0.261</v>
       </c>
       <c r="F22" t="n">
-        <v>2.609</v>
+        <v>2.635</v>
       </c>
       <c r="G22" t="n">
         <v>0.435</v>
       </c>
       <c r="H22" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="I22" t="n">
-        <v>0.671</v>
+        <v>0.659</v>
       </c>
       <c r="K22" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
       <c r="L22" t="n">
-        <v>12.229</v>
+        <v>12.233</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B23" t="n">
-        <v>3.223</v>
+        <v>3.21</v>
       </c>
       <c r="C23" t="n">
-        <v>3.299</v>
+        <v>3.219</v>
       </c>
       <c r="D23" t="n">
-        <v>1.188</v>
+        <v>1.44</v>
       </c>
       <c r="E23" t="n">
-        <v>0.322</v>
+        <v>0.28</v>
       </c>
       <c r="F23" t="n">
-        <v>2.549</v>
+        <v>2.609</v>
       </c>
       <c r="G23" t="n">
-        <v>0.371</v>
+        <v>0.435</v>
       </c>
       <c r="H23" t="n">
         <v>0.365</v>
       </c>
       <c r="I23" t="n">
-        <v>0.703</v>
+        <v>0.671</v>
       </c>
       <c r="K23" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
       <c r="L23" t="n">
-        <v>12.02</v>
+        <v>12.229</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B24" t="n">
-        <v>3.195</v>
+        <v>3.223</v>
       </c>
       <c r="C24" t="n">
-        <v>3.193</v>
+        <v>3.299</v>
       </c>
       <c r="D24" t="n">
-        <v>0.947</v>
+        <v>1.188</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.322</v>
       </c>
       <c r="F24" t="n">
-        <v>2.577</v>
+        <v>2.549</v>
       </c>
       <c r="G24" t="n">
-        <v>0.437</v>
+        <v>0.371</v>
       </c>
       <c r="H24" t="n">
         <v>0.365</v>
       </c>
       <c r="I24" t="n">
-        <v>0.709</v>
+        <v>0.703</v>
       </c>
       <c r="K24" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
       <c r="L24" t="n">
-        <v>12.108</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B25" t="n">
-        <v>3.196</v>
+        <v>3.195</v>
       </c>
       <c r="C25" t="n">
-        <v>3.232</v>
+        <v>3.193</v>
       </c>
       <c r="D25" t="n">
-        <v>1.246</v>
+        <v>0.947</v>
       </c>
       <c r="E25" t="n">
-        <v>0.677</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F25" t="n">
-        <v>2.543</v>
+        <v>2.577</v>
       </c>
       <c r="G25" t="n">
-        <v>0.281</v>
+        <v>0.437</v>
       </c>
       <c r="H25" t="n">
         <v>0.365</v>
       </c>
       <c r="I25" t="n">
-        <v>0.732</v>
+        <v>0.709</v>
       </c>
       <c r="K25" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
       <c r="L25" t="n">
-        <v>12.272</v>
+        <v>12.108</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B26" t="n">
-        <v>3.307</v>
+        <v>3.196</v>
       </c>
       <c r="C26" t="n">
         <v>3.232</v>
       </c>
       <c r="D26" t="n">
-        <v>1.484</v>
+        <v>1.246</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="F26" t="n">
-        <v>2.598</v>
+        <v>2.543</v>
       </c>
       <c r="G26" t="n">
-        <v>0.288</v>
+        <v>0.281</v>
       </c>
       <c r="H26" t="n">
-        <v>0.36</v>
+        <v>0.365</v>
       </c>
       <c r="I26" t="n">
-        <v>0.676</v>
+        <v>0.732</v>
       </c>
       <c r="K26" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
       <c r="L26" t="n">
-        <v>12.634</v>
+        <v>12.272</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B27" t="n">
-        <v>3.176</v>
+        <v>3.307</v>
       </c>
       <c r="C27" t="n">
-        <v>3.163</v>
+        <v>3.232</v>
       </c>
       <c r="D27" t="n">
-        <v>1.435</v>
+        <v>1.484</v>
       </c>
       <c r="E27" t="n">
-        <v>0.674</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="F27" t="n">
-        <v>2.607</v>
+        <v>2.598</v>
       </c>
       <c r="G27" t="n">
-        <v>0.446</v>
+        <v>0.288</v>
       </c>
       <c r="H27" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="I27" t="n">
-        <v>0.712</v>
+        <v>0.676</v>
       </c>
       <c r="K27" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
       <c r="L27" t="n">
-        <v>12.569</v>
+        <v>12.634</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B28" t="n">
-        <v>3.232</v>
+        <v>3.176</v>
       </c>
       <c r="C28" t="n">
-        <v>3.162</v>
+        <v>3.163</v>
       </c>
       <c r="D28" t="n">
         <v>1.435</v>
       </c>
       <c r="E28" t="n">
-        <v>0.609</v>
+        <v>0.674</v>
       </c>
       <c r="F28" t="n">
-        <v>2.324</v>
+        <v>2.607</v>
       </c>
       <c r="G28" t="n">
         <v>0.446</v>
@@ -83685,30 +83744,30 @@
         <v>0.712</v>
       </c>
       <c r="K28" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
       <c r="L28" t="n">
-        <v>12.276</v>
+        <v>12.569</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B29" t="n">
-        <v>3.263</v>
+        <v>3.232</v>
       </c>
       <c r="C29" t="n">
-        <v>3.261</v>
+        <v>3.162</v>
       </c>
       <c r="D29" t="n">
         <v>1.435</v>
       </c>
       <c r="E29" t="n">
-        <v>0.554</v>
+        <v>0.609</v>
       </c>
       <c r="F29" t="n">
-        <v>2.197</v>
+        <v>2.324</v>
       </c>
       <c r="G29" t="n">
         <v>0.446</v>
@@ -83720,65 +83779,65 @@
         <v>0.712</v>
       </c>
       <c r="K29" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
       <c r="L29" t="n">
-        <v>12.224</v>
+        <v>12.276</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B30" t="n">
-        <v>3.259</v>
+        <v>3.263</v>
       </c>
       <c r="C30" t="n">
-        <v>3.268</v>
+        <v>3.261</v>
       </c>
       <c r="D30" t="n">
-        <v>1.449</v>
+        <v>1.435</v>
       </c>
       <c r="E30" t="n">
-        <v>0.399</v>
+        <v>0.554</v>
       </c>
       <c r="F30" t="n">
-        <v>2.276</v>
+        <v>2.197</v>
       </c>
       <c r="G30" t="n">
-        <v>0.462</v>
+        <v>0.446</v>
       </c>
       <c r="H30" t="n">
-        <v>0.343</v>
+        <v>0.356</v>
       </c>
       <c r="I30" t="n">
-        <v>0.731</v>
+        <v>0.712</v>
       </c>
       <c r="K30" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
       <c r="L30" t="n">
-        <v>12.187</v>
+        <v>12.224</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B31" t="n">
-        <v>3.277</v>
+        <v>3.259</v>
       </c>
       <c r="C31" t="n">
-        <v>3.153</v>
+        <v>3.268</v>
       </c>
       <c r="D31" t="n">
-        <v>1.426</v>
+        <v>1.449</v>
       </c>
       <c r="E31" t="n">
-        <v>0.237</v>
+        <v>0.399</v>
       </c>
       <c r="F31" t="n">
-        <v>2.454</v>
+        <v>2.276</v>
       </c>
       <c r="G31" t="n">
         <v>0.462</v>
@@ -83787,33 +83846,33 @@
         <v>0.343</v>
       </c>
       <c r="I31" t="n">
-        <v>0.728</v>
+        <v>0.731</v>
       </c>
       <c r="K31" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
       <c r="L31" t="n">
-        <v>12.08</v>
+        <v>12.187</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B32" t="n">
-        <v>3.365</v>
+        <v>3.277</v>
       </c>
       <c r="C32" t="n">
-        <v>3.197</v>
+        <v>3.153</v>
       </c>
       <c r="D32" t="n">
-        <v>1.44</v>
+        <v>1.426</v>
       </c>
       <c r="E32" t="n">
-        <v>0.253</v>
+        <v>0.237</v>
       </c>
       <c r="F32" t="n">
-        <v>2.354</v>
+        <v>2.454</v>
       </c>
       <c r="G32" t="n">
         <v>0.462</v>
@@ -83822,109 +83881,106 @@
         <v>0.343</v>
       </c>
       <c r="I32" t="n">
-        <v>0.704</v>
+        <v>0.728</v>
       </c>
       <c r="K32" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
       <c r="L32" t="n">
-        <v>12.118</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B33" t="n">
-        <v>3.412</v>
+        <v>3.365</v>
       </c>
       <c r="C33" t="n">
-        <v>3.251</v>
+        <v>3.197</v>
       </c>
       <c r="D33" t="n">
-        <v>1.484</v>
+        <v>1.44</v>
       </c>
       <c r="E33" t="n">
-        <v>0.408</v>
+        <v>0.253</v>
       </c>
       <c r="F33" t="n">
-        <v>2.274</v>
+        <v>2.354</v>
       </c>
       <c r="G33" t="n">
-        <v>0.439</v>
+        <v>0.462</v>
       </c>
       <c r="H33" t="n">
-        <v>0.34</v>
+        <v>0.343</v>
       </c>
       <c r="I33" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0.014</v>
+        <v>0.704</v>
       </c>
       <c r="K33" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
       <c r="L33" t="n">
-        <v>12.373</v>
+        <v>12.118</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B34" t="n">
-        <v>3.361</v>
+        <v>3.412</v>
       </c>
       <c r="C34" t="n">
-        <v>3.372</v>
+        <v>3.251</v>
       </c>
       <c r="D34" t="n">
-        <v>1.406</v>
+        <v>1.484</v>
       </c>
       <c r="E34" t="n">
-        <v>0.569</v>
+        <v>0.408</v>
       </c>
       <c r="F34" t="n">
-        <v>2.417</v>
+        <v>2.274</v>
       </c>
       <c r="G34" t="n">
-        <v>0.395</v>
+        <v>0.439</v>
       </c>
       <c r="H34" t="n">
-        <v>0.362</v>
+        <v>0.34</v>
       </c>
       <c r="I34" t="n">
-        <v>0.746</v>
+        <v>0.751</v>
       </c>
       <c r="J34" t="n">
         <v>0.014</v>
       </c>
       <c r="K34" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
       <c r="L34" t="n">
-        <v>12.642</v>
+        <v>12.373</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B35" t="n">
-        <v>3.307</v>
+        <v>3.361</v>
       </c>
       <c r="C35" t="n">
-        <v>3.344</v>
+        <v>3.372</v>
       </c>
       <c r="D35" t="n">
-        <v>1.377</v>
+        <v>1.406</v>
       </c>
       <c r="E35" t="n">
-        <v>0.3</v>
+        <v>0.569</v>
       </c>
       <c r="F35" t="n">
-        <v>2.432</v>
+        <v>2.417</v>
       </c>
       <c r="G35" t="n">
         <v>0.395</v>
@@ -83939,9 +83995,47 @@
         <v>0.014</v>
       </c>
       <c r="K35" t="n">
+        <v>12.642</v>
+      </c>
+      <c r="L35" t="n">
+        <v>12.642</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B36" t="n">
+        <v>3.307</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3.344</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2.432</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K36" t="n">
         <v>12.277</v>
       </c>
-      <c r="L35" t="n">
+      <c r="L36" t="n">
         <v>12.277</v>
       </c>
     </row>
@@ -84382,7 +84476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84482,541 +84576,541 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B2" t="n">
-        <v>1423202</v>
+        <v>1303673</v>
       </c>
       <c r="C2" t="n">
-        <v>455161</v>
+        <v>551434</v>
       </c>
       <c r="D2" t="n">
-        <v>1401725</v>
+        <v>1423476</v>
       </c>
       <c r="E2" t="n">
         <v>9500</v>
       </c>
       <c r="F2" t="n">
-        <v>1790742</v>
+        <v>1876323</v>
       </c>
       <c r="G2" t="n">
-        <v>1378077</v>
+        <v>1407165</v>
       </c>
       <c r="I2" t="n">
-        <v>1506700</v>
+        <v>1506352</v>
       </c>
       <c r="K2" t="n">
-        <v>300344</v>
+        <v>181857</v>
       </c>
       <c r="M2" t="n">
-        <v>1992032</v>
+        <v>1708871</v>
       </c>
       <c r="N2" t="n">
         <v>92394</v>
       </c>
       <c r="O2" t="n">
-        <v>137551</v>
+        <v>112465</v>
       </c>
       <c r="P2" t="n">
-        <v>393389</v>
+        <v>394639</v>
       </c>
       <c r="Q2" t="n">
-        <v>478122</v>
+        <v>748069</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="B3" t="n">
-        <v>1372566</v>
+        <v>1423202</v>
       </c>
       <c r="C3" t="n">
-        <v>535686</v>
+        <v>455161</v>
       </c>
       <c r="D3" t="n">
-        <v>1384220</v>
+        <v>1401725</v>
       </c>
       <c r="E3" t="n">
         <v>9500</v>
       </c>
       <c r="F3" t="n">
-        <v>1750778</v>
+        <v>1790742</v>
       </c>
       <c r="G3" t="n">
-        <v>1443098</v>
+        <v>1378077</v>
       </c>
       <c r="I3" t="n">
-        <v>1497314</v>
+        <v>1506700</v>
       </c>
       <c r="K3" t="n">
-        <v>243577</v>
+        <v>300344</v>
       </c>
       <c r="M3" t="n">
-        <v>2692467</v>
+        <v>1992032</v>
       </c>
       <c r="N3" t="n">
-        <v>188088</v>
+        <v>92394</v>
       </c>
       <c r="O3" t="n">
-        <v>230944</v>
+        <v>137551</v>
       </c>
       <c r="P3" t="n">
-        <v>393254</v>
+        <v>393389</v>
       </c>
       <c r="Q3" t="n">
-        <v>665576</v>
+        <v>478122</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B4" t="n">
-        <v>1383237</v>
+        <v>1372566</v>
       </c>
       <c r="C4" t="n">
-        <v>642612</v>
+        <v>535686</v>
       </c>
       <c r="D4" t="n">
-        <v>1376983</v>
+        <v>1384220</v>
       </c>
       <c r="E4" t="n">
-        <v>9000</v>
+        <v>9500</v>
       </c>
       <c r="F4" t="n">
-        <v>1886772</v>
+        <v>1750778</v>
       </c>
       <c r="G4" t="n">
-        <v>1487288</v>
+        <v>1443098</v>
       </c>
       <c r="I4" t="n">
-        <v>1545952</v>
+        <v>1497314</v>
       </c>
       <c r="K4" t="n">
-        <v>145193</v>
+        <v>243577</v>
       </c>
       <c r="M4" t="n">
-        <v>2689526</v>
+        <v>2692467</v>
       </c>
       <c r="N4" t="n">
-        <v>309125</v>
+        <v>188088</v>
       </c>
       <c r="O4" t="n">
-        <v>432534</v>
+        <v>230944</v>
       </c>
       <c r="P4" t="n">
-        <v>399049</v>
+        <v>393254</v>
       </c>
       <c r="Q4" t="n">
-        <v>681693</v>
+        <v>665576</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B5" t="n">
-        <v>1326845</v>
+        <v>1383237</v>
       </c>
       <c r="C5" t="n">
-        <v>630343</v>
+        <v>642612</v>
       </c>
       <c r="D5" t="n">
-        <v>1389820</v>
+        <v>1376983</v>
       </c>
       <c r="E5" t="n">
         <v>9000</v>
       </c>
       <c r="F5" t="n">
-        <v>1898634</v>
+        <v>1886772</v>
       </c>
       <c r="G5" t="n">
-        <v>1230443</v>
+        <v>1487288</v>
       </c>
       <c r="I5" t="n">
-        <v>1509954</v>
+        <v>1545952</v>
       </c>
       <c r="K5" t="n">
-        <v>223405</v>
+        <v>145193</v>
       </c>
       <c r="M5" t="n">
-        <v>2637144</v>
+        <v>2689526</v>
       </c>
       <c r="N5" t="n">
-        <v>322000</v>
+        <v>309125</v>
       </c>
       <c r="O5" t="n">
-        <v>445186</v>
+        <v>432534</v>
       </c>
       <c r="P5" t="n">
-        <v>392284</v>
+        <v>399049</v>
       </c>
       <c r="Q5" t="n">
-        <v>707427</v>
+        <v>681693</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B6" t="n">
-        <v>1453284</v>
+        <v>1326845</v>
       </c>
       <c r="C6" t="n">
-        <v>668222</v>
+        <v>630343</v>
       </c>
       <c r="D6" t="n">
-        <v>1399375</v>
+        <v>1389820</v>
       </c>
       <c r="E6" t="n">
         <v>9000</v>
       </c>
       <c r="F6" t="n">
-        <v>1997673</v>
+        <v>1898634</v>
       </c>
       <c r="G6" t="n">
-        <v>1229304</v>
+        <v>1230443</v>
       </c>
       <c r="I6" t="n">
-        <v>1526881</v>
+        <v>1509954</v>
       </c>
       <c r="K6" t="n">
-        <v>210710</v>
+        <v>223405</v>
       </c>
       <c r="M6" t="n">
-        <v>2315158</v>
+        <v>2637144</v>
       </c>
       <c r="N6" t="n">
-        <v>274632</v>
+        <v>322000</v>
       </c>
       <c r="O6" t="n">
-        <v>404378</v>
+        <v>445186</v>
       </c>
       <c r="P6" t="n">
-        <v>393345</v>
+        <v>392284</v>
       </c>
       <c r="Q6" t="n">
-        <v>702775</v>
+        <v>707427</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B7" t="n">
-        <v>1428345</v>
+        <v>1453284</v>
       </c>
       <c r="C7" t="n">
-        <v>613887</v>
+        <v>668222</v>
       </c>
       <c r="D7" t="n">
-        <v>1360335</v>
+        <v>1399375</v>
       </c>
       <c r="E7" t="n">
         <v>9000</v>
       </c>
       <c r="F7" t="n">
-        <v>2000629</v>
+        <v>1997673</v>
       </c>
       <c r="G7" t="n">
-        <v>1229134</v>
+        <v>1229304</v>
       </c>
       <c r="I7" t="n">
-        <v>1516881</v>
+        <v>1526881</v>
       </c>
       <c r="K7" t="n">
-        <v>265281</v>
+        <v>210710</v>
       </c>
       <c r="M7" t="n">
-        <v>2655010</v>
+        <v>2315158</v>
       </c>
       <c r="N7" t="n">
-        <v>275644</v>
+        <v>274632</v>
       </c>
       <c r="O7" t="n">
-        <v>405391</v>
+        <v>404378</v>
       </c>
       <c r="P7" t="n">
         <v>393345</v>
       </c>
       <c r="Q7" t="n">
-        <v>735394</v>
+        <v>702775</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B8" t="n">
-        <v>1453305</v>
+        <v>1428345</v>
       </c>
       <c r="C8" t="n">
-        <v>660021</v>
+        <v>613887</v>
       </c>
       <c r="D8" t="n">
-        <v>1394810</v>
+        <v>1360335</v>
       </c>
       <c r="E8" t="n">
         <v>9000</v>
       </c>
       <c r="F8" t="n">
-        <v>1966997</v>
+        <v>2000629</v>
       </c>
       <c r="G8" t="n">
-        <v>1358589</v>
+        <v>1229134</v>
       </c>
       <c r="I8" t="n">
-        <v>1530881</v>
+        <v>1516881</v>
       </c>
       <c r="K8" t="n">
-        <v>224505</v>
+        <v>265281</v>
       </c>
       <c r="M8" t="n">
-        <v>2605275</v>
+        <v>2655010</v>
       </c>
       <c r="N8" t="n">
-        <v>273068</v>
+        <v>275644</v>
       </c>
       <c r="O8" t="n">
-        <v>402811</v>
+        <v>405391</v>
       </c>
       <c r="P8" t="n">
-        <v>368707</v>
+        <v>393345</v>
       </c>
       <c r="Q8" t="n">
-        <v>750038</v>
+        <v>735394</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B9" t="n">
-        <v>1104818</v>
+        <v>1453305</v>
       </c>
       <c r="C9" t="n">
-        <v>667392</v>
+        <v>660021</v>
       </c>
       <c r="D9" t="n">
-        <v>1498652</v>
+        <v>1394810</v>
       </c>
       <c r="E9" t="n">
         <v>9000</v>
       </c>
       <c r="F9" t="n">
-        <v>1894575</v>
+        <v>1966997</v>
       </c>
       <c r="G9" t="n">
-        <v>1428865</v>
+        <v>1358589</v>
       </c>
       <c r="I9" t="n">
-        <v>1526911</v>
+        <v>1530881</v>
       </c>
       <c r="K9" t="n">
-        <v>285753</v>
+        <v>224505</v>
       </c>
       <c r="M9" t="n">
-        <v>2731003</v>
+        <v>2605275</v>
       </c>
       <c r="N9" t="n">
-        <v>214475</v>
+        <v>273068</v>
       </c>
       <c r="O9" t="n">
-        <v>224840</v>
+        <v>402811</v>
       </c>
       <c r="P9" t="n">
-        <v>355073</v>
+        <v>368707</v>
       </c>
       <c r="Q9" t="n">
-        <v>614624</v>
+        <v>750038</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B10" t="n">
-        <v>977033</v>
+        <v>1104818</v>
       </c>
       <c r="C10" t="n">
-        <v>493347</v>
+        <v>667392</v>
       </c>
       <c r="D10" t="n">
-        <v>1277653</v>
+        <v>1498652</v>
       </c>
       <c r="E10" t="n">
         <v>9000</v>
       </c>
       <c r="F10" t="n">
-        <v>1875666</v>
+        <v>1894575</v>
       </c>
       <c r="G10" t="n">
-        <v>1356150</v>
+        <v>1428865</v>
       </c>
       <c r="I10" t="n">
-        <v>1507739</v>
+        <v>1526911</v>
       </c>
       <c r="K10" t="n">
-        <v>213692</v>
+        <v>285753</v>
       </c>
       <c r="M10" t="n">
-        <v>2729375</v>
+        <v>2731003</v>
       </c>
       <c r="N10" t="n">
         <v>214475</v>
       </c>
       <c r="O10" t="n">
-        <v>246357</v>
+        <v>224840</v>
       </c>
       <c r="P10" t="n">
-        <v>354625</v>
+        <v>355073</v>
       </c>
       <c r="Q10" t="n">
-        <v>508923</v>
+        <v>614624</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B11" t="n">
-        <v>1222754</v>
+        <v>977033</v>
       </c>
       <c r="C11" t="n">
-        <v>600260</v>
+        <v>493347</v>
       </c>
       <c r="D11" t="n">
-        <v>1343521</v>
+        <v>1277653</v>
       </c>
       <c r="E11" t="n">
-        <v>9200</v>
+        <v>9000</v>
       </c>
       <c r="F11" t="n">
-        <v>1872474</v>
+        <v>1875666</v>
       </c>
       <c r="G11" t="n">
-        <v>1385603</v>
+        <v>1356150</v>
       </c>
       <c r="I11" t="n">
-        <v>1436775</v>
+        <v>1507739</v>
       </c>
       <c r="K11" t="n">
-        <v>212263</v>
+        <v>213692</v>
       </c>
       <c r="M11" t="n">
-        <v>2676981</v>
+        <v>2729375</v>
       </c>
       <c r="N11" t="n">
         <v>214475</v>
       </c>
       <c r="O11" t="n">
-        <v>245565</v>
+        <v>246357</v>
       </c>
       <c r="P11" t="n">
-        <v>331850</v>
+        <v>354625</v>
       </c>
       <c r="Q11" t="n">
-        <v>670444</v>
+        <v>508923</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B12" t="n">
-        <v>1347666</v>
+        <v>1222754</v>
       </c>
       <c r="C12" t="n">
-        <v>711291</v>
+        <v>600260</v>
       </c>
       <c r="D12" t="n">
-        <v>1463104</v>
+        <v>1343521</v>
       </c>
       <c r="E12" t="n">
         <v>9200</v>
       </c>
       <c r="F12" t="n">
-        <v>1917047</v>
+        <v>1872474</v>
       </c>
       <c r="G12" t="n">
-        <v>1405212</v>
+        <v>1385603</v>
       </c>
       <c r="I12" t="n">
-        <v>1528739</v>
+        <v>1436775</v>
       </c>
       <c r="K12" t="n">
-        <v>256281</v>
+        <v>212263</v>
       </c>
       <c r="M12" t="n">
-        <v>2665641</v>
+        <v>2676981</v>
       </c>
       <c r="N12" t="n">
         <v>214475</v>
       </c>
       <c r="O12" t="n">
-        <v>239857</v>
+        <v>245565</v>
       </c>
       <c r="P12" t="n">
-        <v>379888</v>
+        <v>331850</v>
       </c>
       <c r="Q12" t="n">
-        <v>696003</v>
+        <v>670444</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B13" t="n">
-        <v>1371402</v>
+        <v>1347666</v>
       </c>
       <c r="C13" t="n">
-        <v>799313</v>
+        <v>711291</v>
       </c>
       <c r="D13" t="n">
-        <v>1336369</v>
+        <v>1463104</v>
       </c>
       <c r="E13" t="n">
         <v>9200</v>
       </c>
       <c r="F13" t="n">
-        <v>1938280</v>
+        <v>1917047</v>
       </c>
       <c r="G13" t="n">
-        <v>1443483</v>
+        <v>1405212</v>
       </c>
       <c r="I13" t="n">
-        <v>1532739</v>
+        <v>1528739</v>
       </c>
       <c r="K13" t="n">
-        <v>307648</v>
+        <v>256281</v>
       </c>
       <c r="M13" t="n">
-        <v>2687880</v>
+        <v>2665641</v>
       </c>
       <c r="N13" t="n">
-        <v>127995</v>
+        <v>214475</v>
       </c>
       <c r="O13" t="n">
-        <v>152230</v>
+        <v>239857</v>
       </c>
       <c r="P13" t="n">
-        <v>380516</v>
+        <v>379888</v>
       </c>
       <c r="Q13" t="n">
-        <v>710782</v>
+        <v>696003</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B14" t="n">
-        <v>1222188</v>
+        <v>1371402</v>
       </c>
       <c r="C14" t="n">
-        <v>726662</v>
+        <v>799313</v>
       </c>
       <c r="D14" t="n">
         <v>1336369</v>
@@ -85025,28 +85119,28 @@
         <v>9200</v>
       </c>
       <c r="F14" t="n">
-        <v>1819723</v>
+        <v>1938280</v>
       </c>
       <c r="G14" t="n">
-        <v>1144716</v>
+        <v>1443483</v>
       </c>
       <c r="I14" t="n">
-        <v>1539739</v>
+        <v>1532739</v>
       </c>
       <c r="K14" t="n">
-        <v>347698</v>
+        <v>307648</v>
       </c>
       <c r="M14" t="n">
-        <v>2681880</v>
+        <v>2687880</v>
       </c>
       <c r="N14" t="n">
-        <v>214475</v>
+        <v>127995</v>
       </c>
       <c r="O14" t="n">
-        <v>238857</v>
+        <v>152230</v>
       </c>
       <c r="P14" t="n">
-        <v>380595</v>
+        <v>380516</v>
       </c>
       <c r="Q14" t="n">
         <v>710782</v>
@@ -85054,34 +85148,34 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B15" t="n">
-        <v>1245221</v>
+        <v>1222188</v>
       </c>
       <c r="C15" t="n">
-        <v>748948</v>
+        <v>726662</v>
       </c>
       <c r="D15" t="n">
-        <v>1343138</v>
+        <v>1336369</v>
       </c>
       <c r="E15" t="n">
         <v>9200</v>
       </c>
       <c r="F15" t="n">
-        <v>1828741</v>
+        <v>1819723</v>
       </c>
       <c r="G15" t="n">
-        <v>1426853</v>
+        <v>1144716</v>
       </c>
       <c r="I15" t="n">
-        <v>1286120</v>
+        <v>1539739</v>
       </c>
       <c r="K15" t="n">
-        <v>297542</v>
+        <v>347698</v>
       </c>
       <c r="M15" t="n">
-        <v>2648485</v>
+        <v>2681880</v>
       </c>
       <c r="N15" t="n">
         <v>214475</v>
@@ -85090,7 +85184,7 @@
         <v>238857</v>
       </c>
       <c r="P15" t="n">
-        <v>380596</v>
+        <v>380595</v>
       </c>
       <c r="Q15" t="n">
         <v>710782</v>
@@ -85098,43 +85192,43 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B16" t="n">
-        <v>1270655</v>
+        <v>1245221</v>
       </c>
       <c r="C16" t="n">
-        <v>720759</v>
+        <v>748948</v>
       </c>
       <c r="D16" t="n">
-        <v>1323318</v>
+        <v>1343138</v>
       </c>
       <c r="E16" t="n">
         <v>9200</v>
       </c>
       <c r="F16" t="n">
-        <v>1887685</v>
+        <v>1828741</v>
       </c>
       <c r="G16" t="n">
-        <v>1444684</v>
+        <v>1426853</v>
       </c>
       <c r="I16" t="n">
-        <v>1322407</v>
+        <v>1286120</v>
       </c>
       <c r="K16" t="n">
-        <v>212971</v>
+        <v>297542</v>
       </c>
       <c r="M16" t="n">
-        <v>2675880</v>
+        <v>2648485</v>
       </c>
       <c r="N16" t="n">
-        <v>217075</v>
+        <v>214475</v>
       </c>
       <c r="O16" t="n">
-        <v>236445</v>
+        <v>238857</v>
       </c>
       <c r="P16" t="n">
-        <v>374416</v>
+        <v>380596</v>
       </c>
       <c r="Q16" t="n">
         <v>710782</v>
@@ -85142,201 +85236,201 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B17" t="n">
-        <v>1312169</v>
+        <v>1270655</v>
       </c>
       <c r="C17" t="n">
-        <v>724772</v>
+        <v>720759</v>
       </c>
       <c r="D17" t="n">
-        <v>1287902</v>
+        <v>1323318</v>
       </c>
       <c r="E17" t="n">
         <v>9200</v>
       </c>
       <c r="F17" t="n">
-        <v>1901259</v>
+        <v>1887685</v>
       </c>
       <c r="G17" t="n">
-        <v>1431569</v>
+        <v>1444684</v>
       </c>
       <c r="I17" t="n">
-        <v>1517739</v>
+        <v>1322407</v>
       </c>
       <c r="K17" t="n">
-        <v>215710</v>
+        <v>212971</v>
       </c>
       <c r="M17" t="n">
-        <v>2690149</v>
+        <v>2675880</v>
       </c>
       <c r="N17" t="n">
-        <v>212599</v>
+        <v>217075</v>
       </c>
       <c r="O17" t="n">
-        <v>240961</v>
+        <v>236445</v>
       </c>
       <c r="P17" t="n">
-        <v>380562</v>
+        <v>374416</v>
       </c>
       <c r="Q17" t="n">
-        <v>650000</v>
+        <v>710782</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B18" t="n">
-        <v>1329569</v>
+        <v>1312169</v>
       </c>
       <c r="C18" t="n">
-        <v>762468</v>
+        <v>724772</v>
       </c>
       <c r="D18" t="n">
-        <v>1356602</v>
+        <v>1287902</v>
       </c>
       <c r="E18" t="n">
         <v>9200</v>
       </c>
       <c r="F18" t="n">
-        <v>1904492</v>
+        <v>1901259</v>
       </c>
       <c r="G18" t="n">
-        <v>1449343</v>
+        <v>1431569</v>
       </c>
       <c r="I18" t="n">
-        <v>1411819</v>
+        <v>1517739</v>
       </c>
       <c r="K18" t="n">
-        <v>310810</v>
+        <v>215710</v>
       </c>
       <c r="M18" t="n">
-        <v>2705056</v>
+        <v>2690149</v>
       </c>
       <c r="N18" t="n">
-        <v>214475</v>
+        <v>212599</v>
       </c>
       <c r="O18" t="n">
-        <v>259857</v>
+        <v>240961</v>
       </c>
       <c r="P18" t="n">
-        <v>380664</v>
+        <v>380562</v>
       </c>
       <c r="Q18" t="n">
-        <v>709873</v>
+        <v>650000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B19" t="n">
-        <v>1270354</v>
+        <v>1329569</v>
       </c>
       <c r="C19" t="n">
-        <v>650008</v>
+        <v>762468</v>
       </c>
       <c r="D19" t="n">
-        <v>1478806</v>
+        <v>1356602</v>
       </c>
       <c r="E19" t="n">
         <v>9200</v>
       </c>
       <c r="F19" t="n">
-        <v>1835055</v>
+        <v>1904492</v>
       </c>
       <c r="G19" t="n">
-        <v>1481786</v>
+        <v>1449343</v>
       </c>
       <c r="I19" t="n">
-        <v>1534739</v>
+        <v>1411819</v>
       </c>
       <c r="K19" t="n">
-        <v>288093</v>
+        <v>310810</v>
       </c>
       <c r="M19" t="n">
-        <v>2703043</v>
+        <v>2705056</v>
       </c>
       <c r="N19" t="n">
-        <v>131771</v>
+        <v>214475</v>
       </c>
       <c r="O19" t="n">
-        <v>167012</v>
+        <v>259857</v>
       </c>
       <c r="P19" t="n">
-        <v>380459</v>
+        <v>380664</v>
       </c>
       <c r="Q19" t="n">
-        <v>690681</v>
+        <v>709873</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B20" t="n">
-        <v>1291024</v>
+        <v>1270354</v>
       </c>
       <c r="C20" t="n">
-        <v>625316</v>
+        <v>650008</v>
       </c>
       <c r="D20" t="n">
-        <v>1438301</v>
+        <v>1478806</v>
       </c>
       <c r="E20" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F20" t="n">
-        <v>1882671</v>
+        <v>1835055</v>
       </c>
       <c r="G20" t="n">
-        <v>1484709</v>
+        <v>1481786</v>
       </c>
       <c r="I20" t="n">
-        <v>1493578</v>
+        <v>1534739</v>
       </c>
       <c r="K20" t="n">
-        <v>270165</v>
+        <v>288093</v>
       </c>
       <c r="M20" t="n">
-        <v>2735408</v>
+        <v>2703043</v>
       </c>
       <c r="N20" t="n">
-        <v>214475</v>
+        <v>131771</v>
       </c>
       <c r="O20" t="n">
-        <v>236857</v>
+        <v>167012</v>
       </c>
       <c r="P20" t="n">
-        <v>380581</v>
+        <v>380459</v>
       </c>
       <c r="Q20" t="n">
-        <v>686237</v>
+        <v>690681</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B21" t="n">
-        <v>1240901</v>
+        <v>1291024</v>
       </c>
       <c r="C21" t="n">
-        <v>663382</v>
+        <v>625316</v>
       </c>
       <c r="D21" t="n">
-        <v>1423376</v>
+        <v>1438301</v>
       </c>
       <c r="E21" t="n">
         <v>9400</v>
       </c>
       <c r="F21" t="n">
-        <v>1882670</v>
+        <v>1882671</v>
       </c>
       <c r="G21" t="n">
-        <v>1454791</v>
+        <v>1484709</v>
       </c>
       <c r="I21" t="n">
         <v>1493578</v>
@@ -85345,7 +85439,7 @@
         <v>270165</v>
       </c>
       <c r="M21" t="n">
-        <v>2732297</v>
+        <v>2735408</v>
       </c>
       <c r="N21" t="n">
         <v>214475</v>
@@ -85357,39 +85451,39 @@
         <v>380581</v>
       </c>
       <c r="Q21" t="n">
-        <v>683510</v>
+        <v>686237</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B22" t="n">
-        <v>1257633</v>
+        <v>1240901</v>
       </c>
       <c r="C22" t="n">
-        <v>611578</v>
+        <v>663382</v>
       </c>
       <c r="D22" t="n">
-        <v>1449703</v>
+        <v>1423376</v>
       </c>
       <c r="E22" t="n">
         <v>9400</v>
       </c>
       <c r="F22" t="n">
-        <v>1882647</v>
+        <v>1882670</v>
       </c>
       <c r="G22" t="n">
-        <v>1455299</v>
+        <v>1454791</v>
       </c>
       <c r="I22" t="n">
         <v>1493578</v>
       </c>
       <c r="K22" t="n">
-        <v>290165</v>
+        <v>270165</v>
       </c>
       <c r="M22" t="n">
-        <v>2705287</v>
+        <v>2732297</v>
       </c>
       <c r="N22" t="n">
         <v>214475</v>
@@ -85398,153 +85492,153 @@
         <v>236857</v>
       </c>
       <c r="P22" t="n">
-        <v>378153</v>
+        <v>380581</v>
       </c>
       <c r="Q22" t="n">
-        <v>696137</v>
+        <v>683510</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B23" t="n">
-        <v>1271516</v>
+        <v>1257633</v>
       </c>
       <c r="C23" t="n">
-        <v>597877</v>
+        <v>611578</v>
       </c>
       <c r="D23" t="n">
-        <v>1463300</v>
+        <v>1449703</v>
       </c>
       <c r="E23" t="n">
         <v>9400</v>
       </c>
       <c r="F23" t="n">
-        <v>1948739</v>
+        <v>1882647</v>
       </c>
       <c r="G23" t="n">
-        <v>1472527</v>
+        <v>1455299</v>
       </c>
       <c r="I23" t="n">
-        <v>1232047</v>
+        <v>1493578</v>
       </c>
       <c r="K23" t="n">
-        <v>334269</v>
+        <v>290165</v>
       </c>
       <c r="M23" t="n">
-        <v>2643426</v>
+        <v>2705287</v>
       </c>
       <c r="N23" t="n">
-        <v>186552</v>
+        <v>214475</v>
       </c>
       <c r="O23" t="n">
-        <v>197887</v>
+        <v>236857</v>
       </c>
       <c r="P23" t="n">
-        <v>378590</v>
+        <v>378153</v>
       </c>
       <c r="Q23" t="n">
-        <v>729365</v>
+        <v>696137</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B24" t="n">
-        <v>1274678</v>
+        <v>1271516</v>
       </c>
       <c r="C24" t="n">
-        <v>523874</v>
+        <v>597877</v>
       </c>
       <c r="D24" t="n">
-        <v>1505828</v>
+        <v>1463300</v>
       </c>
       <c r="E24" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F24" t="n">
-        <v>1900789</v>
+        <v>1948739</v>
       </c>
       <c r="G24" t="n">
-        <v>1409855</v>
+        <v>1472527</v>
       </c>
       <c r="I24" t="n">
-        <v>981796</v>
+        <v>1232047</v>
       </c>
       <c r="K24" t="n">
-        <v>709874</v>
+        <v>334269</v>
       </c>
       <c r="M24" t="n">
-        <v>2672575</v>
+        <v>2643426</v>
       </c>
       <c r="N24" t="n">
-        <v>214475</v>
+        <v>186552</v>
       </c>
       <c r="O24" t="n">
-        <v>238857</v>
+        <v>197887</v>
       </c>
       <c r="P24" t="n">
-        <v>378233</v>
+        <v>378590</v>
       </c>
       <c r="Q24" t="n">
-        <v>735025</v>
+        <v>729365</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B25" t="n">
-        <v>1291480</v>
+        <v>1274678</v>
       </c>
       <c r="C25" t="n">
-        <v>574586</v>
+        <v>523874</v>
       </c>
       <c r="D25" t="n">
-        <v>1438502</v>
+        <v>1505828</v>
       </c>
       <c r="E25" t="n">
         <v>9200</v>
       </c>
       <c r="F25" t="n">
-        <v>1868644</v>
+        <v>1900789</v>
       </c>
       <c r="G25" t="n">
-        <v>1482710</v>
+        <v>1409855</v>
       </c>
       <c r="I25" t="n">
-        <v>1291683</v>
+        <v>981796</v>
       </c>
       <c r="K25" t="n">
-        <v>702469</v>
+        <v>709874</v>
       </c>
       <c r="M25" t="n">
-        <v>2637080</v>
+        <v>2672575</v>
       </c>
       <c r="N25" t="n">
-        <v>135639</v>
+        <v>214475</v>
       </c>
       <c r="O25" t="n">
-        <v>155887</v>
+        <v>238857</v>
       </c>
       <c r="P25" t="n">
-        <v>378140</v>
+        <v>378233</v>
       </c>
       <c r="Q25" t="n">
-        <v>759291</v>
+        <v>735025</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="B26" t="n">
-        <v>1344999</v>
+        <v>1291480</v>
       </c>
       <c r="C26" t="n">
-        <v>636735</v>
+        <v>574586</v>
       </c>
       <c r="D26" t="n">
         <v>1438502</v>
@@ -85553,107 +85647,107 @@
         <v>9200</v>
       </c>
       <c r="F26" t="n">
-        <v>1892344</v>
+        <v>1868644</v>
       </c>
       <c r="G26" t="n">
-        <v>1459196</v>
+        <v>1482710</v>
       </c>
       <c r="I26" t="n">
-        <v>1538980</v>
+        <v>1291683</v>
       </c>
       <c r="K26" t="n">
-        <v>714270</v>
+        <v>702469</v>
       </c>
       <c r="M26" t="n">
-        <v>2693673</v>
+        <v>2637080</v>
       </c>
       <c r="N26" t="n">
-        <v>131452</v>
+        <v>135639</v>
       </c>
       <c r="O26" t="n">
-        <v>166693</v>
+        <v>155887</v>
       </c>
       <c r="P26" t="n">
-        <v>373275</v>
+        <v>378140</v>
       </c>
       <c r="Q26" t="n">
-        <v>700532</v>
+        <v>759291</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B27" t="n">
-        <v>1208720</v>
+        <v>1344999</v>
       </c>
       <c r="C27" t="n">
-        <v>615524</v>
+        <v>636735</v>
       </c>
       <c r="D27" t="n">
-        <v>1460388</v>
+        <v>1438502</v>
       </c>
       <c r="E27" t="n">
         <v>9200</v>
       </c>
       <c r="F27" t="n">
-        <v>1787948</v>
+        <v>1892344</v>
       </c>
       <c r="G27" t="n">
-        <v>1492147</v>
+        <v>1459196</v>
       </c>
       <c r="I27" t="n">
-        <v>1488515</v>
+        <v>1538980</v>
       </c>
       <c r="K27" t="n">
-        <v>698623</v>
+        <v>714270</v>
       </c>
       <c r="M27" t="n">
-        <v>2703143</v>
+        <v>2693673</v>
       </c>
       <c r="N27" t="n">
-        <v>214475</v>
+        <v>131452</v>
       </c>
       <c r="O27" t="n">
-        <v>247857</v>
+        <v>166693</v>
       </c>
       <c r="P27" t="n">
-        <v>369576</v>
+        <v>373275</v>
       </c>
       <c r="Q27" t="n">
-        <v>738429</v>
+        <v>700532</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B28" t="n">
-        <v>1255158</v>
+        <v>1208720</v>
       </c>
       <c r="C28" t="n">
-        <v>621535</v>
+        <v>615524</v>
       </c>
       <c r="D28" t="n">
-        <v>1465868</v>
+        <v>1460388</v>
       </c>
       <c r="E28" t="n">
         <v>9200</v>
       </c>
       <c r="F28" t="n">
-        <v>1787951</v>
+        <v>1787948</v>
       </c>
       <c r="G28" t="n">
-        <v>1491513</v>
+        <v>1492147</v>
       </c>
       <c r="I28" t="n">
         <v>1488515</v>
       </c>
       <c r="K28" t="n">
-        <v>631586</v>
+        <v>698623</v>
       </c>
       <c r="M28" t="n">
-        <v>2409537</v>
+        <v>2703143</v>
       </c>
       <c r="N28" t="n">
         <v>214475</v>
@@ -85662,7 +85756,7 @@
         <v>247857</v>
       </c>
       <c r="P28" t="n">
-        <v>369120</v>
+        <v>369576</v>
       </c>
       <c r="Q28" t="n">
         <v>738429</v>
@@ -85670,34 +85764,34 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B29" t="n">
-        <v>1268054</v>
+        <v>1255158</v>
       </c>
       <c r="C29" t="n">
-        <v>646819</v>
+        <v>621535</v>
       </c>
       <c r="D29" t="n">
-        <v>1458973</v>
+        <v>1465868</v>
       </c>
       <c r="E29" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F29" t="n">
-        <v>1892157</v>
+        <v>1787951</v>
       </c>
       <c r="G29" t="n">
-        <v>1489325</v>
+        <v>1491513</v>
       </c>
       <c r="I29" t="n">
         <v>1488515</v>
       </c>
       <c r="K29" t="n">
-        <v>574363</v>
+        <v>631586</v>
       </c>
       <c r="M29" t="n">
-        <v>2277986</v>
+        <v>2409537</v>
       </c>
       <c r="N29" t="n">
         <v>214475</v>
@@ -85706,7 +85800,7 @@
         <v>247857</v>
       </c>
       <c r="P29" t="n">
-        <v>369082</v>
+        <v>369120</v>
       </c>
       <c r="Q29" t="n">
         <v>738429</v>
@@ -85714,78 +85808,78 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B30" t="n">
-        <v>1294415</v>
+        <v>1268054</v>
       </c>
       <c r="C30" t="n">
-        <v>622563</v>
+        <v>646819</v>
       </c>
       <c r="D30" t="n">
-        <v>1452901</v>
+        <v>1458973</v>
       </c>
       <c r="E30" t="n">
-        <v>9200</v>
+        <v>9400</v>
       </c>
       <c r="F30" t="n">
-        <v>1896083</v>
+        <v>1892157</v>
       </c>
       <c r="G30" t="n">
-        <v>1492662</v>
+        <v>1489325</v>
       </c>
       <c r="I30" t="n">
-        <v>1502826</v>
+        <v>1488515</v>
       </c>
       <c r="K30" t="n">
-        <v>414091</v>
+        <v>574363</v>
       </c>
       <c r="M30" t="n">
-        <v>2360445</v>
+        <v>2277986</v>
       </c>
       <c r="N30" t="n">
         <v>214475</v>
       </c>
       <c r="O30" t="n">
-        <v>264857</v>
+        <v>247857</v>
       </c>
       <c r="P30" t="n">
-        <v>355841</v>
+        <v>369082</v>
       </c>
       <c r="Q30" t="n">
-        <v>758041</v>
+        <v>738429</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B31" t="n">
-        <v>1287738</v>
+        <v>1294415</v>
       </c>
       <c r="C31" t="n">
-        <v>627470</v>
+        <v>622563</v>
       </c>
       <c r="D31" t="n">
-        <v>1473202</v>
+        <v>1452901</v>
       </c>
       <c r="E31" t="n">
-        <v>9400</v>
+        <v>9200</v>
       </c>
       <c r="F31" t="n">
-        <v>1827111</v>
+        <v>1896083</v>
       </c>
       <c r="G31" t="n">
-        <v>1442936</v>
+        <v>1492662</v>
       </c>
       <c r="I31" t="n">
-        <v>1478756</v>
+        <v>1502826</v>
       </c>
       <c r="K31" t="n">
-        <v>245359</v>
+        <v>414091</v>
       </c>
       <c r="M31" t="n">
-        <v>2544314</v>
+        <v>2360445</v>
       </c>
       <c r="N31" t="n">
         <v>214475</v>
@@ -85794,42 +85888,42 @@
         <v>264857</v>
       </c>
       <c r="P31" t="n">
-        <v>355281</v>
+        <v>355841</v>
       </c>
       <c r="Q31" t="n">
-        <v>755100</v>
+        <v>758041</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B32" t="n">
-        <v>1355779</v>
+        <v>1287738</v>
       </c>
       <c r="C32" t="n">
-        <v>636253</v>
+        <v>627470</v>
       </c>
       <c r="D32" t="n">
-        <v>1488152</v>
+        <v>1473202</v>
       </c>
       <c r="E32" t="n">
-        <v>9300</v>
+        <v>9400</v>
       </c>
       <c r="F32" t="n">
-        <v>1882472</v>
+        <v>1827111</v>
       </c>
       <c r="G32" t="n">
-        <v>1433134</v>
+        <v>1442936</v>
       </c>
       <c r="I32" t="n">
-        <v>1492810</v>
+        <v>1478756</v>
       </c>
       <c r="K32" t="n">
-        <v>262398</v>
+        <v>245359</v>
       </c>
       <c r="M32" t="n">
-        <v>2441130</v>
+        <v>2544314</v>
       </c>
       <c r="N32" t="n">
         <v>214475</v>
@@ -85838,101 +85932,98 @@
         <v>264857</v>
       </c>
       <c r="P32" t="n">
-        <v>355279</v>
+        <v>355281</v>
       </c>
       <c r="Q32" t="n">
-        <v>729723</v>
+        <v>755100</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="B33" t="n">
-        <v>1372528</v>
+        <v>1355779</v>
       </c>
       <c r="C33" t="n">
-        <v>661067</v>
+        <v>636253</v>
       </c>
       <c r="D33" t="n">
-        <v>1495794</v>
+        <v>1488152</v>
       </c>
       <c r="E33" t="n">
         <v>9300</v>
       </c>
       <c r="F33" t="n">
-        <v>1984198</v>
+        <v>1882472</v>
       </c>
       <c r="G33" t="n">
-        <v>1386625</v>
+        <v>1433134</v>
       </c>
       <c r="I33" t="n">
-        <v>1538415</v>
+        <v>1492810</v>
       </c>
       <c r="K33" t="n">
-        <v>423452</v>
+        <v>262398</v>
       </c>
       <c r="M33" t="n">
-        <v>2358379</v>
+        <v>2441130</v>
       </c>
       <c r="N33" t="n">
-        <v>207642</v>
+        <v>214475</v>
       </c>
       <c r="O33" t="n">
-        <v>248013</v>
+        <v>264857</v>
       </c>
       <c r="P33" t="n">
-        <v>352672</v>
+        <v>355279</v>
       </c>
       <c r="Q33" t="n">
-        <v>779164</v>
-      </c>
-      <c r="R33" t="n">
-        <v>15000</v>
+        <v>729723</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B34" t="n">
-        <v>1301942</v>
+        <v>1372528</v>
       </c>
       <c r="C34" t="n">
-        <v>666110</v>
+        <v>661067</v>
       </c>
       <c r="D34" t="n">
-        <v>1508302</v>
+        <v>1495794</v>
       </c>
       <c r="E34" t="n">
-        <v>9100</v>
+        <v>9300</v>
       </c>
       <c r="F34" t="n">
-        <v>2013551</v>
+        <v>1984198</v>
       </c>
       <c r="G34" t="n">
-        <v>1483009</v>
+        <v>1386625</v>
       </c>
       <c r="I34" t="n">
-        <v>1458275</v>
+        <v>1538415</v>
       </c>
       <c r="K34" t="n">
-        <v>590414</v>
+        <v>423452</v>
       </c>
       <c r="M34" t="n">
-        <v>2506388</v>
+        <v>2358379</v>
       </c>
       <c r="N34" t="n">
-        <v>189475</v>
+        <v>207642</v>
       </c>
       <c r="O34" t="n">
-        <v>219815</v>
+        <v>248013</v>
       </c>
       <c r="P34" t="n">
-        <v>375660</v>
+        <v>352672</v>
       </c>
       <c r="Q34" t="n">
-        <v>773586</v>
+        <v>779164</v>
       </c>
       <c r="R34" t="n">
         <v>15000</v>
@@ -85940,40 +86031,40 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B35" t="n">
-        <v>1276064</v>
+        <v>1301942</v>
       </c>
       <c r="C35" t="n">
-        <v>646110</v>
+        <v>666110</v>
       </c>
       <c r="D35" t="n">
-        <v>1498302</v>
+        <v>1508302</v>
       </c>
       <c r="E35" t="n">
         <v>9100</v>
       </c>
       <c r="F35" t="n">
-        <v>1999274</v>
+        <v>2013551</v>
       </c>
       <c r="G35" t="n">
-        <v>1468619</v>
+        <v>1483009</v>
       </c>
       <c r="I35" t="n">
-        <v>1428275</v>
+        <v>1458275</v>
       </c>
       <c r="K35" t="n">
-        <v>310625</v>
+        <v>590414</v>
       </c>
       <c r="M35" t="n">
-        <v>2522392</v>
+        <v>2506388</v>
       </c>
       <c r="N35" t="n">
         <v>189475</v>
       </c>
       <c r="O35" t="n">
-        <v>219811</v>
+        <v>219815</v>
       </c>
       <c r="P35" t="n">
         <v>375660</v>
@@ -85982,6 +86073,53 @@
         <v>773586</v>
       </c>
       <c r="R35" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1276064</v>
+      </c>
+      <c r="C36" t="n">
+        <v>646110</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1498302</v>
+      </c>
+      <c r="E36" t="n">
+        <v>9100</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1999274</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1468619</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1428275</v>
+      </c>
+      <c r="K36" t="n">
+        <v>310625</v>
+      </c>
+      <c r="M36" t="n">
+        <v>2522392</v>
+      </c>
+      <c r="N36" t="n">
+        <v>189475</v>
+      </c>
+      <c r="O36" t="n">
+        <v>219811</v>
+      </c>
+      <c r="P36" t="n">
+        <v>375660</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>773586</v>
+      </c>
+      <c r="R36" t="n">
         <v>15000</v>
       </c>
     </row>

</xml_diff>